<commit_message>
Consol TB report update 2026-03-16
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -1547,7 +1547,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ecdf8a3-112b-4aa8-8637-1edb1ae72ab1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{cbab7bde-197a-4703-981f-662e5746fe30}">
   <dimension ref="A1:I1782"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -1636,7 +1636,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>2.9802322387695312E-8</v>
+        <v>-8.940696716308594E-8</v>
       </c>
       <c r="G3" s="1">
         <v>0.02</v>
@@ -1645,7 +1645,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>-3.519999970197677</v>
+        <v>-3.5200000894069667</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -1787,10 +1787,10 @@
         <v>5.43186561E8</v>
       </c>
       <c r="H8" s="1">
-        <v>2.711028429799999E8</v>
+        <v>2.7110284298E8</v>
       </c>
       <c r="I8" s="1">
-        <v>2.720837180200001E8</v>
+        <v>2.7208371802E8</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="12.75">
@@ -3814,10 +3814,10 @@
         <v>918706</v>
       </c>
       <c r="G78" s="1">
-        <v>4.366243983000001E7</v>
+        <v>4.366243983E7</v>
       </c>
       <c r="H78" s="1">
-        <v>4.3068153200000025E7</v>
+        <v>4.306815320000001E7</v>
       </c>
       <c r="I78" s="1">
         <v>1512992.6299999878</v>
@@ -3898,7 +3898,7 @@
         <v>13</v>
       </c>
       <c r="F81" s="1">
-        <v>0</v>
+        <v>-9.313225746154785E-10</v>
       </c>
       <c r="G81" s="1">
         <v>333614</v>
@@ -3907,7 +3907,7 @@
         <v>333614</v>
       </c>
       <c r="I81" s="1">
-        <v>0</v>
+        <v>-9.313225746154785E-10</v>
       </c>
     </row>
     <row r="82" spans="1:9" ht="12.75">
@@ -6047,13 +6047,13 @@
         <v>0</v>
       </c>
       <c r="G155" s="1">
-        <v>1.907233301E7</v>
+        <v>1.9072333009999998E7</v>
       </c>
       <c r="H155" s="1">
         <v>18680110</v>
       </c>
       <c r="I155" s="1">
-        <v>392223.01000000164</v>
+        <v>392223.0099999979</v>
       </c>
     </row>
     <row r="156" spans="1:9" ht="12.75">
@@ -7671,13 +7671,13 @@
         <v>0</v>
       </c>
       <c r="G211" s="1">
-        <v>61736.97000000001</v>
+        <v>61736.97</v>
       </c>
       <c r="H211" s="1">
         <v>0</v>
       </c>
       <c r="I211" s="1">
-        <v>61736.97000000001</v>
+        <v>61736.97</v>
       </c>
     </row>
     <row r="212" spans="1:9" ht="12.75">
@@ -18343,13 +18343,13 @@
         <v>0</v>
       </c>
       <c r="G579" s="1">
-        <v>892804.57</v>
+        <v>892804.5700000001</v>
       </c>
       <c r="H579" s="1">
         <v>0</v>
       </c>
       <c r="I579" s="1">
-        <v>892804.57</v>
+        <v>892804.5700000001</v>
       </c>
     </row>
     <row r="580" spans="1:9" ht="12.75">
@@ -18575,13 +18575,13 @@
         <v>0</v>
       </c>
       <c r="G587" s="1">
-        <v>2994848.4499999997</v>
+        <v>2994848.45</v>
       </c>
       <c r="H587" s="1">
         <v>14722.75</v>
       </c>
       <c r="I587" s="1">
-        <v>2980125.6999999997</v>
+        <v>2980125.70</v>
       </c>
     </row>
     <row r="588" spans="1:9" ht="12.75">
@@ -18604,13 +18604,13 @@
         <v>0</v>
       </c>
       <c r="G588" s="1">
-        <v>150327.47000000003</v>
+        <v>150327.47</v>
       </c>
       <c r="H588" s="1">
         <v>0</v>
       </c>
       <c r="I588" s="1">
-        <v>150327.47000000003</v>
+        <v>150327.47</v>
       </c>
     </row>
     <row r="589" spans="1:9" ht="12.75">
@@ -19503,13 +19503,13 @@
         <v>0</v>
       </c>
       <c r="G619" s="1">
-        <v>635480.0199999999</v>
+        <v>635480.02</v>
       </c>
       <c r="H619" s="1">
         <v>0</v>
       </c>
       <c r="I619" s="1">
-        <v>635480.0199999999</v>
+        <v>635480.02</v>
       </c>
     </row>
     <row r="620" spans="1:9" ht="12.75">
@@ -19561,13 +19561,13 @@
         <v>0</v>
       </c>
       <c r="G621" s="1">
-        <v>2798165.8900000006</v>
+        <v>2798165.8899999997</v>
       </c>
       <c r="H621" s="1">
         <v>23236.93</v>
       </c>
       <c r="I621" s="1">
-        <v>2774928.9600000004</v>
+        <v>2774928.9599999995</v>
       </c>
     </row>
     <row r="622" spans="1:9" ht="12.75">
@@ -19967,13 +19967,13 @@
         <v>0</v>
       </c>
       <c r="G635" s="1">
-        <v>397731.83</v>
+        <v>397731.82999999996</v>
       </c>
       <c r="H635" s="1">
         <v>0</v>
       </c>
       <c r="I635" s="1">
-        <v>397731.83</v>
+        <v>397731.82999999996</v>
       </c>
     </row>
     <row r="636" spans="1:9" ht="12.75">
@@ -20025,13 +20025,13 @@
         <v>0</v>
       </c>
       <c r="G637" s="1">
-        <v>900877.7399999998</v>
+        <v>900877.74</v>
       </c>
       <c r="H637" s="1">
         <v>0</v>
       </c>
       <c r="I637" s="1">
-        <v>900877.7399999998</v>
+        <v>900877.74</v>
       </c>
     </row>
     <row r="638" spans="1:9" ht="12.75">
@@ -20083,13 +20083,13 @@
         <v>0</v>
       </c>
       <c r="G639" s="1">
-        <v>93486.40000000001</v>
+        <v>93486.40</v>
       </c>
       <c r="H639" s="1">
         <v>0</v>
       </c>
       <c r="I639" s="1">
-        <v>93486.40000000001</v>
+        <v>93486.40</v>
       </c>
     </row>
     <row r="640" spans="1:9" ht="12.75">
@@ -20112,13 +20112,13 @@
         <v>0</v>
       </c>
       <c r="G640" s="1">
-        <v>1595365.7100000002</v>
+        <v>1595365.71</v>
       </c>
       <c r="H640" s="1">
         <v>9049.23</v>
       </c>
       <c r="I640" s="1">
-        <v>1586316.4800000002</v>
+        <v>1586316.48</v>
       </c>
     </row>
     <row r="641" spans="1:9" ht="12.75">
@@ -20170,13 +20170,13 @@
         <v>0</v>
       </c>
       <c r="G642" s="1">
-        <v>516927.00000000006</v>
+        <v>516927</v>
       </c>
       <c r="H642" s="1">
         <v>0</v>
       </c>
       <c r="I642" s="1">
-        <v>516927.00000000006</v>
+        <v>516927</v>
       </c>
     </row>
     <row r="643" spans="1:9" ht="12.75">
@@ -20228,13 +20228,13 @@
         <v>0</v>
       </c>
       <c r="G644" s="1">
-        <v>393958.93999999994</v>
+        <v>393958.94</v>
       </c>
       <c r="H644" s="1">
         <v>0</v>
       </c>
       <c r="I644" s="1">
-        <v>393958.93999999994</v>
+        <v>393958.94</v>
       </c>
     </row>
     <row r="645" spans="1:9" ht="12.75">
@@ -20344,13 +20344,13 @@
         <v>0</v>
       </c>
       <c r="G648" s="1">
-        <v>1824764.4799999997</v>
+        <v>1824764.48</v>
       </c>
       <c r="H648" s="1">
         <v>13850.19</v>
       </c>
       <c r="I648" s="1">
-        <v>1810914.2899999998</v>
+        <v>1810914.29</v>
       </c>
     </row>
     <row r="649" spans="1:9" ht="12.75">
@@ -20431,13 +20431,13 @@
         <v>0</v>
       </c>
       <c r="G651" s="1">
-        <v>264343.41000000003</v>
+        <v>264343.41</v>
       </c>
       <c r="H651" s="1">
         <v>0</v>
       </c>
       <c r="I651" s="1">
-        <v>264343.41000000003</v>
+        <v>264343.41</v>
       </c>
     </row>
     <row r="652" spans="1:9" ht="12.75">
@@ -20721,13 +20721,13 @@
         <v>0</v>
       </c>
       <c r="G661" s="1">
-        <v>171980.19999999998</v>
+        <v>171980.20</v>
       </c>
       <c r="H661" s="1">
         <v>0</v>
       </c>
       <c r="I661" s="1">
-        <v>171980.19999999998</v>
+        <v>171980.20</v>
       </c>
     </row>
     <row r="662" spans="1:9" ht="12.75">
@@ -20895,13 +20895,13 @@
         <v>0</v>
       </c>
       <c r="G667" s="1">
-        <v>780446.0900000001</v>
+        <v>780446.09</v>
       </c>
       <c r="H667" s="1">
         <v>0</v>
       </c>
       <c r="I667" s="1">
-        <v>780446.0900000001</v>
+        <v>780446.09</v>
       </c>
     </row>
     <row r="668" spans="1:9" ht="12.75">
@@ -21939,13 +21939,13 @@
         <v>0</v>
       </c>
       <c r="G703" s="1">
-        <v>906485.9900000001</v>
+        <v>906485.99</v>
       </c>
       <c r="H703" s="1">
         <v>0</v>
       </c>
       <c r="I703" s="1">
-        <v>906485.9900000001</v>
+        <v>906485.99</v>
       </c>
     </row>
     <row r="704" spans="1:9" ht="12.75">
@@ -22026,13 +22026,13 @@
         <v>0</v>
       </c>
       <c r="G706" s="1">
-        <v>5448697.789999999</v>
+        <v>5448697.790000001</v>
       </c>
       <c r="H706" s="1">
         <v>0</v>
       </c>
       <c r="I706" s="1">
-        <v>5448697.789999999</v>
+        <v>5448697.790000001</v>
       </c>
     </row>
     <row r="707" spans="1:9" ht="12.75">
@@ -22403,13 +22403,13 @@
         <v>0</v>
       </c>
       <c r="G719" s="1">
-        <v>253568.64</v>
+        <v>253568.63999999998</v>
       </c>
       <c r="H719" s="1">
         <v>0</v>
       </c>
       <c r="I719" s="1">
-        <v>253568.64</v>
+        <v>253568.63999999998</v>
       </c>
     </row>
     <row r="720" spans="1:9" ht="12.75">
@@ -22432,13 +22432,13 @@
         <v>0</v>
       </c>
       <c r="G720" s="1">
-        <v>2766043.1599999997</v>
+        <v>2766043.16</v>
       </c>
       <c r="H720" s="1">
         <v>0</v>
       </c>
       <c r="I720" s="1">
-        <v>2766043.1599999997</v>
+        <v>2766043.16</v>
       </c>
     </row>
     <row r="721" spans="1:9" ht="12.75">
@@ -22519,13 +22519,13 @@
         <v>0</v>
       </c>
       <c r="G723" s="1">
-        <v>180148.38999999998</v>
+        <v>180148.39</v>
       </c>
       <c r="H723" s="1">
         <v>0</v>
       </c>
       <c r="I723" s="1">
-        <v>180148.38999999998</v>
+        <v>180148.39</v>
       </c>
     </row>
     <row r="724" spans="1:9" ht="12.75">
@@ -22606,13 +22606,13 @@
         <v>0</v>
       </c>
       <c r="G726" s="1">
-        <v>143323.11</v>
+        <v>143323.11000000002</v>
       </c>
       <c r="H726" s="1">
         <v>0</v>
       </c>
       <c r="I726" s="1">
-        <v>143323.11</v>
+        <v>143323.11000000002</v>
       </c>
     </row>
     <row r="727" spans="1:9" ht="12.75">
@@ -22870,10 +22870,10 @@
         <v>0</v>
       </c>
       <c r="H735" s="1">
-        <v>7.258656368E7</v>
+        <v>7.258656367999999E7</v>
       </c>
       <c r="I735" s="1">
-        <v>-7.258656368E7</v>
+        <v>-7.258656367999999E7</v>
       </c>
     </row>
     <row r="736" spans="1:9" ht="12.75">
@@ -44527,16 +44527,16 @@
         <v>13</v>
       </c>
       <c r="F1482" s="1">
-        <v>-19347197</v>
+        <v>-1.934719700000018E7</v>
       </c>
       <c r="G1482" s="1">
-        <v>2.0665386530000034E8</v>
+        <v>2.0665386529999983E8</v>
       </c>
       <c r="H1482" s="1">
-        <v>1.9811070830000022E8</v>
+        <v>1.9811070829999977E8</v>
       </c>
       <c r="I1482" s="1">
-        <v>-1.080403999999988E7</v>
+        <v>-1.080404000000012E7</v>
       </c>
     </row>
     <row r="1483" spans="1:9" ht="12.75">
@@ -45113,10 +45113,10 @@
         <v>556577.47</v>
       </c>
       <c r="H1502" s="1">
-        <v>586448.8999999993</v>
+        <v>586448.90</v>
       </c>
       <c r="I1502" s="1">
-        <v>-29871.429999999353</v>
+        <v>-29871.43000000005</v>
       </c>
     </row>
     <row r="1503" spans="1:9" ht="12.75">
@@ -45171,10 +45171,10 @@
         <v>7533462.2</v>
       </c>
       <c r="H1504" s="1">
-        <v>8502435.920000007</v>
+        <v>8502435.919999998</v>
       </c>
       <c r="I1504" s="1">
-        <v>-968973.7200000072</v>
+        <v>-968973.7199999979</v>
       </c>
     </row>
     <row r="1505" spans="1:9" ht="12.75">
@@ -45194,16 +45194,16 @@
         <v>13</v>
       </c>
       <c r="F1505" s="1">
-        <v>-56796.99999999907</v>
+        <v>-56797.000000011176</v>
       </c>
       <c r="G1505" s="1">
         <v>3227421.94</v>
       </c>
       <c r="H1505" s="1">
-        <v>3631156.9400000004</v>
+        <v>3631156.939999999</v>
       </c>
       <c r="I1505" s="1">
-        <v>-460531.99999999953</v>
+        <v>-460532.00000001024</v>
       </c>
     </row>
     <row r="1506" spans="1:9" ht="12.75">
@@ -45252,16 +45252,16 @@
         <v>13</v>
       </c>
       <c r="F1507" s="1">
-        <v>-5.9604644775390625E-8</v>
+        <v>0</v>
       </c>
       <c r="G1507" s="1">
-        <v>1.1068072367300003E9</v>
+        <v>1.10680723673E9</v>
       </c>
       <c r="H1507" s="1">
-        <v>1.1068072367300022E9</v>
+        <v>1.10680723673E9</v>
       </c>
       <c r="I1507" s="1">
-        <v>-1.9073486328125E-6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1508" spans="1:9" ht="12.75">
@@ -46244,10 +46244,10 @@
         <v>8.56587629E8</v>
       </c>
       <c r="H1541" s="1">
-        <v>3.3588584282E8</v>
+        <v>3.3588584281999993E8</v>
       </c>
       <c r="I1541" s="1">
-        <v>5.2070178618E8</v>
+        <v>5.2070178618000007E8</v>
       </c>
     </row>
     <row r="1542" spans="1:9" ht="12.75">
@@ -49808,13 +49808,13 @@
         <v>0</v>
       </c>
       <c r="G1664" s="1">
-        <v>1910663.0799999996</v>
+        <v>1910663.0799999998</v>
       </c>
       <c r="H1664" s="1">
         <v>0</v>
       </c>
       <c r="I1664" s="1">
-        <v>1910663.0799999996</v>
+        <v>1910663.0799999998</v>
       </c>
     </row>
     <row r="1665" spans="1:9" ht="12.75">
@@ -49837,13 +49837,13 @@
         <v>0</v>
       </c>
       <c r="G1665" s="1">
-        <v>685737.61</v>
+        <v>685737.6099999999</v>
       </c>
       <c r="H1665" s="1">
         <v>0</v>
       </c>
       <c r="I1665" s="1">
-        <v>685737.61</v>
+        <v>685737.6099999999</v>
       </c>
     </row>
     <row r="1666" spans="1:9" ht="12.75">
@@ -53030,10 +53030,10 @@
         <v>37299</v>
       </c>
       <c r="H1775" s="1">
-        <v>185786.19999999998</v>
+        <v>185786.20</v>
       </c>
       <c r="I1775" s="1">
-        <v>-148487.19999999998</v>
+        <v>-148487.20</v>
       </c>
     </row>
     <row r="1776" spans="1:9" ht="12.75">
@@ -53227,16 +53227,16 @@
         <v>361</v>
       </c>
       <c r="F1782" s="1">
-        <v>5.9604644775390625E-8</v>
+        <v>-1.9371509552001953E-7</v>
       </c>
       <c r="G1782" s="1">
-        <v>6.97229419303E9</v>
+        <v>6.972294193029999E9</v>
       </c>
       <c r="H1782" s="1">
-        <v>6.972294193030003E9</v>
+        <v>6.972294193029999E9</v>
       </c>
       <c r="I1782" s="1">
-        <v>-1.9185245037078857E-6</v>
+        <v>-4.880130290985107E-7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-03-17
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8918" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8923" uniqueCount="362">
   <si>
     <t>Book</t>
   </si>
@@ -1547,8 +1547,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{cbab7bde-197a-4703-981f-662e5746fe30}">
-  <dimension ref="A1:I1782"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60a9dc32-2f2a-4db2-8f07-5cd3b9eb1d41}">
+  <dimension ref="A1:I1783"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="14.142857142857142" customWidth="1"/>
@@ -1636,7 +1636,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>-8.940696716308594E-8</v>
+        <v>-2.9802322387695312E-8</v>
       </c>
       <c r="G3" s="1">
         <v>0.02</v>
@@ -1645,7 +1645,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>-3.5200000894069667</v>
+        <v>-3.520000029802322</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -1671,10 +1671,10 @@
         <v>2.4882729998E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.398457705400005E8</v>
+        <v>3.400399935400005E8</v>
       </c>
       <c r="I4" s="1">
-        <v>4.0884281309999526E7</v>
+        <v>4.0690058309999526E7</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -1787,10 +1787,10 @@
         <v>5.43186561E8</v>
       </c>
       <c r="H8" s="1">
-        <v>2.7110284298E8</v>
+        <v>2.7110284297999996E8</v>
       </c>
       <c r="I8" s="1">
-        <v>2.7208371802E8</v>
+        <v>2.7208371802000004E8</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="12.75">
@@ -3814,13 +3814,13 @@
         <v>918706</v>
       </c>
       <c r="G78" s="1">
-        <v>4.366243983E7</v>
+        <v>4.387191483E7</v>
       </c>
       <c r="H78" s="1">
-        <v>4.306815320000001E7</v>
+        <v>4.306815319999997E7</v>
       </c>
       <c r="I78" s="1">
-        <v>1512992.6299999878</v>
+        <v>1722467.630000025</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="12.75">
@@ -3898,7 +3898,7 @@
         <v>13</v>
       </c>
       <c r="F81" s="1">
-        <v>-9.313225746154785E-10</v>
+        <v>0</v>
       </c>
       <c r="G81" s="1">
         <v>333614</v>
@@ -3907,7 +3907,7 @@
         <v>333614</v>
       </c>
       <c r="I81" s="1">
-        <v>-9.313225746154785E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:9" ht="12.75">
@@ -18343,13 +18343,13 @@
         <v>0</v>
       </c>
       <c r="G579" s="1">
-        <v>892804.5700000001</v>
+        <v>892804.57</v>
       </c>
       <c r="H579" s="1">
         <v>0</v>
       </c>
       <c r="I579" s="1">
-        <v>892804.5700000001</v>
+        <v>892804.57</v>
       </c>
     </row>
     <row r="580" spans="1:9" ht="12.75">
@@ -18575,13 +18575,13 @@
         <v>0</v>
       </c>
       <c r="G587" s="1">
-        <v>2994848.45</v>
+        <v>2994848.4499999997</v>
       </c>
       <c r="H587" s="1">
         <v>14722.75</v>
       </c>
       <c r="I587" s="1">
-        <v>2980125.70</v>
+        <v>2980125.6999999997</v>
       </c>
     </row>
     <row r="588" spans="1:9" ht="12.75">
@@ -18604,13 +18604,13 @@
         <v>0</v>
       </c>
       <c r="G588" s="1">
-        <v>150327.47</v>
+        <v>150327.47000000003</v>
       </c>
       <c r="H588" s="1">
         <v>0</v>
       </c>
       <c r="I588" s="1">
-        <v>150327.47</v>
+        <v>150327.47000000003</v>
       </c>
     </row>
     <row r="589" spans="1:9" ht="12.75">
@@ -19561,13 +19561,13 @@
         <v>0</v>
       </c>
       <c r="G621" s="1">
-        <v>2798165.8899999997</v>
+        <v>2798165.89</v>
       </c>
       <c r="H621" s="1">
         <v>23236.93</v>
       </c>
       <c r="I621" s="1">
-        <v>2774928.9599999995</v>
+        <v>2774928.96</v>
       </c>
     </row>
     <row r="622" spans="1:9" ht="12.75">
@@ -19590,13 +19590,13 @@
         <v>0</v>
       </c>
       <c r="G622" s="1">
-        <v>1374964.32</v>
+        <v>1374964.3199999998</v>
       </c>
       <c r="H622" s="1">
         <v>0</v>
       </c>
       <c r="I622" s="1">
-        <v>1374964.32</v>
+        <v>1374964.3199999998</v>
       </c>
     </row>
     <row r="623" spans="1:9" ht="12.75">
@@ -19619,13 +19619,13 @@
         <v>0</v>
       </c>
       <c r="G623" s="1">
-        <v>3046869.40</v>
+        <v>3046869.400000001</v>
       </c>
       <c r="H623" s="1">
         <v>9049.23</v>
       </c>
       <c r="I623" s="1">
-        <v>3037820.17</v>
+        <v>3037820.170000001</v>
       </c>
     </row>
     <row r="624" spans="1:9" ht="12.75">
@@ -19967,13 +19967,13 @@
         <v>0</v>
       </c>
       <c r="G635" s="1">
-        <v>397731.82999999996</v>
+        <v>397731.83</v>
       </c>
       <c r="H635" s="1">
         <v>0</v>
       </c>
       <c r="I635" s="1">
-        <v>397731.82999999996</v>
+        <v>397731.83</v>
       </c>
     </row>
     <row r="636" spans="1:9" ht="12.75">
@@ -20025,13 +20025,13 @@
         <v>0</v>
       </c>
       <c r="G637" s="1">
-        <v>900877.74</v>
+        <v>900877.7399999998</v>
       </c>
       <c r="H637" s="1">
         <v>0</v>
       </c>
       <c r="I637" s="1">
-        <v>900877.74</v>
+        <v>900877.7399999998</v>
       </c>
     </row>
     <row r="638" spans="1:9" ht="12.75">
@@ -20141,13 +20141,13 @@
         <v>0</v>
       </c>
       <c r="G641" s="1">
-        <v>703295.80</v>
+        <v>703295.7999999999</v>
       </c>
       <c r="H641" s="1">
         <v>0</v>
       </c>
       <c r="I641" s="1">
-        <v>703295.80</v>
+        <v>703295.7999999999</v>
       </c>
     </row>
     <row r="642" spans="1:9" ht="12.75">
@@ -20228,13 +20228,13 @@
         <v>0</v>
       </c>
       <c r="G644" s="1">
-        <v>393958.94</v>
+        <v>393958.94000000006</v>
       </c>
       <c r="H644" s="1">
         <v>0</v>
       </c>
       <c r="I644" s="1">
-        <v>393958.94</v>
+        <v>393958.94000000006</v>
       </c>
     </row>
     <row r="645" spans="1:9" ht="12.75">
@@ -20344,13 +20344,13 @@
         <v>0</v>
       </c>
       <c r="G648" s="1">
-        <v>1824764.48</v>
+        <v>1824764.4800000004</v>
       </c>
       <c r="H648" s="1">
         <v>13850.19</v>
       </c>
       <c r="I648" s="1">
-        <v>1810914.29</v>
+        <v>1810914.2900000005</v>
       </c>
     </row>
     <row r="649" spans="1:9" ht="12.75">
@@ -20431,13 +20431,13 @@
         <v>0</v>
       </c>
       <c r="G651" s="1">
-        <v>264343.41</v>
+        <v>264343.41000000003</v>
       </c>
       <c r="H651" s="1">
         <v>0</v>
       </c>
       <c r="I651" s="1">
-        <v>264343.41</v>
+        <v>264343.41000000003</v>
       </c>
     </row>
     <row r="652" spans="1:9" ht="12.75">
@@ -20953,13 +20953,13 @@
         <v>0</v>
       </c>
       <c r="G669" s="1">
-        <v>617404.2000000001</v>
+        <v>617404.20</v>
       </c>
       <c r="H669" s="1">
         <v>0</v>
       </c>
       <c r="I669" s="1">
-        <v>617404.2000000001</v>
+        <v>617404.20</v>
       </c>
     </row>
     <row r="670" spans="1:9" ht="12.75">
@@ -21997,13 +21997,13 @@
         <v>0</v>
       </c>
       <c r="G705" s="1">
-        <v>4420392.420000001</v>
+        <v>4420392.42</v>
       </c>
       <c r="H705" s="1">
         <v>0</v>
       </c>
       <c r="I705" s="1">
-        <v>4420392.420000001</v>
+        <v>4420392.42</v>
       </c>
     </row>
     <row r="706" spans="1:9" ht="12.75">
@@ -22026,13 +22026,13 @@
         <v>0</v>
       </c>
       <c r="G706" s="1">
-        <v>5448697.790000001</v>
+        <v>5448697.789999999</v>
       </c>
       <c r="H706" s="1">
         <v>0</v>
       </c>
       <c r="I706" s="1">
-        <v>5448697.790000001</v>
+        <v>5448697.789999999</v>
       </c>
     </row>
     <row r="707" spans="1:9" ht="12.75">
@@ -22461,13 +22461,13 @@
         <v>0</v>
       </c>
       <c r="G721" s="1">
-        <v>1220232.68</v>
+        <v>1220232.6800000002</v>
       </c>
       <c r="H721" s="1">
         <v>0</v>
       </c>
       <c r="I721" s="1">
-        <v>1220232.68</v>
+        <v>1220232.6800000002</v>
       </c>
     </row>
     <row r="722" spans="1:9" ht="12.75">
@@ -22490,13 +22490,13 @@
         <v>0</v>
       </c>
       <c r="G722" s="1">
-        <v>742650.70</v>
+        <v>742650.7000000001</v>
       </c>
       <c r="H722" s="1">
         <v>0</v>
       </c>
       <c r="I722" s="1">
-        <v>742650.70</v>
+        <v>742650.7000000001</v>
       </c>
     </row>
     <row r="723" spans="1:9" ht="12.75">
@@ -22577,13 +22577,13 @@
         <v>0</v>
       </c>
       <c r="G725" s="1">
-        <v>9665763.799999999</v>
+        <v>9665763.8</v>
       </c>
       <c r="H725" s="1">
         <v>0</v>
       </c>
       <c r="I725" s="1">
-        <v>9665763.799999999</v>
+        <v>9665763.8</v>
       </c>
     </row>
     <row r="726" spans="1:9" ht="12.75">
@@ -22606,13 +22606,13 @@
         <v>0</v>
       </c>
       <c r="G726" s="1">
-        <v>143323.11000000002</v>
+        <v>143323.11</v>
       </c>
       <c r="H726" s="1">
         <v>0</v>
       </c>
       <c r="I726" s="1">
-        <v>143323.11000000002</v>
+        <v>143323.11</v>
       </c>
     </row>
     <row r="727" spans="1:9" ht="12.75">
@@ -22870,10 +22870,10 @@
         <v>0</v>
       </c>
       <c r="H735" s="1">
-        <v>7.258656367999999E7</v>
+        <v>7.258656368E7</v>
       </c>
       <c r="I735" s="1">
-        <v>-7.258656367999999E7</v>
+        <v>-7.258656368E7</v>
       </c>
     </row>
     <row r="736" spans="1:9" ht="12.75">
@@ -38933,13 +38933,13 @@
         <v>0</v>
       </c>
       <c r="G1289" s="1">
-        <v>417310.80</v>
+        <v>417310.80000000005</v>
       </c>
       <c r="H1289" s="1">
         <v>0</v>
       </c>
       <c r="I1289" s="1">
-        <v>417310.80</v>
+        <v>417310.80000000005</v>
       </c>
     </row>
     <row r="1290" spans="1:9" ht="12.75">
@@ -43341,13 +43341,13 @@
         <v>0</v>
       </c>
       <c r="G1441" s="1">
-        <v>1894601.3199999998</v>
+        <v>1894601.32</v>
       </c>
       <c r="H1441" s="1">
         <v>0</v>
       </c>
       <c r="I1441" s="1">
-        <v>1894601.3199999998</v>
+        <v>1894601.32</v>
       </c>
     </row>
     <row r="1442" spans="1:9" ht="12.75">
@@ -44527,16 +44527,16 @@
         <v>13</v>
       </c>
       <c r="F1482" s="1">
-        <v>-1.934719700000018E7</v>
+        <v>-1.934719699999994E7</v>
       </c>
       <c r="G1482" s="1">
-        <v>2.0665386529999983E8</v>
+        <v>2.0665636529999977E8</v>
       </c>
       <c r="H1482" s="1">
-        <v>1.9811070829999977E8</v>
+        <v>1.9811070829999998E8</v>
       </c>
       <c r="I1482" s="1">
-        <v>-1.080404000000012E7</v>
+        <v>-1.0801540000000149E7</v>
       </c>
     </row>
     <row r="1483" spans="1:9" ht="12.75">
@@ -45171,10 +45171,10 @@
         <v>7533462.2</v>
       </c>
       <c r="H1504" s="1">
-        <v>8502435.919999998</v>
+        <v>8520187.920000002</v>
       </c>
       <c r="I1504" s="1">
-        <v>-968973.7199999979</v>
+        <v>-986725.7200000016</v>
       </c>
     </row>
     <row r="1505" spans="1:9" ht="12.75">
@@ -45194,16 +45194,16 @@
         <v>13</v>
       </c>
       <c r="F1505" s="1">
-        <v>-56797.000000011176</v>
+        <v>-56797.000000003725</v>
       </c>
       <c r="G1505" s="1">
         <v>3227421.94</v>
       </c>
       <c r="H1505" s="1">
-        <v>3631156.939999999</v>
+        <v>3631156.9399999967</v>
       </c>
       <c r="I1505" s="1">
-        <v>-460532.00000001024</v>
+        <v>-460532.00000000047</v>
       </c>
     </row>
     <row r="1506" spans="1:9" ht="12.75">
@@ -45258,10 +45258,10 @@
         <v>1.10680723673E9</v>
       </c>
       <c r="H1507" s="1">
-        <v>1.10680723673E9</v>
+        <v>1.1068072367300007E9</v>
       </c>
       <c r="I1507" s="1">
-        <v>0</v>
+        <v>-7.152557373046875E-7</v>
       </c>
     </row>
     <row r="1508" spans="1:9" ht="12.75">
@@ -46157,10 +46157,10 @@
         <v>6.486054004000001E7</v>
       </c>
       <c r="H1538" s="1">
-        <v>6.0772886169999994E7</v>
+        <v>6.077288616999999E7</v>
       </c>
       <c r="I1538" s="1">
-        <v>3.3281362770000003E7</v>
+        <v>3.328136277000001E7</v>
       </c>
     </row>
     <row r="1539" spans="1:9" ht="12.75">
@@ -46244,10 +46244,10 @@
         <v>8.56587629E8</v>
       </c>
       <c r="H1541" s="1">
-        <v>3.3588584281999993E8</v>
+        <v>3.3588584282E8</v>
       </c>
       <c r="I1541" s="1">
-        <v>5.2070178618000007E8</v>
+        <v>5.2070178618E8</v>
       </c>
     </row>
     <row r="1542" spans="1:9" ht="12.75">
@@ -48990,19 +48990,19 @@
         <v>212</v>
       </c>
       <c r="E1636" t="s">
-        <v>329</v>
+        <v>13</v>
       </c>
       <c r="F1636" s="1">
         <v>0</v>
       </c>
       <c r="G1636" s="1">
-        <v>2133376.20</v>
+        <v>98282</v>
       </c>
       <c r="H1636" s="1">
         <v>0</v>
       </c>
       <c r="I1636" s="1">
-        <v>2133376.20</v>
+        <v>98282</v>
       </c>
     </row>
     <row r="1637" spans="1:9" ht="12.75">
@@ -49019,19 +49019,19 @@
         <v>212</v>
       </c>
       <c r="E1637" t="s">
-        <v>348</v>
+        <v>329</v>
       </c>
       <c r="F1637" s="1">
         <v>0</v>
       </c>
       <c r="G1637" s="1">
-        <v>40134</v>
+        <v>2133376.20</v>
       </c>
       <c r="H1637" s="1">
         <v>0</v>
       </c>
       <c r="I1637" s="1">
-        <v>40134</v>
+        <v>2133376.20</v>
       </c>
     </row>
     <row r="1638" spans="1:9" ht="12.75">
@@ -49048,19 +49048,19 @@
         <v>212</v>
       </c>
       <c r="E1638" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="F1638" s="1">
         <v>0</v>
       </c>
       <c r="G1638" s="1">
-        <v>2619977.68</v>
+        <v>40134</v>
       </c>
       <c r="H1638" s="1">
         <v>0</v>
       </c>
       <c r="I1638" s="1">
-        <v>2619977.68</v>
+        <v>40134</v>
       </c>
     </row>
     <row r="1639" spans="1:9" ht="12.75">
@@ -49077,19 +49077,19 @@
         <v>212</v>
       </c>
       <c r="E1639" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1639" s="1">
         <v>0</v>
       </c>
       <c r="G1639" s="1">
-        <v>2449797.92</v>
+        <v>2619977.68</v>
       </c>
       <c r="H1639" s="1">
         <v>0</v>
       </c>
       <c r="I1639" s="1">
-        <v>2449797.92</v>
+        <v>2619977.68</v>
       </c>
     </row>
     <row r="1640" spans="1:9" ht="12.75">
@@ -49106,19 +49106,19 @@
         <v>212</v>
       </c>
       <c r="E1640" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1640" s="1">
         <v>0</v>
       </c>
       <c r="G1640" s="1">
-        <v>578555</v>
+        <v>2449797.92</v>
       </c>
       <c r="H1640" s="1">
         <v>0</v>
       </c>
       <c r="I1640" s="1">
-        <v>578555</v>
+        <v>2449797.92</v>
       </c>
     </row>
     <row r="1641" spans="1:9" ht="12.75">
@@ -49135,19 +49135,19 @@
         <v>212</v>
       </c>
       <c r="E1641" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1641" s="1">
         <v>0</v>
       </c>
       <c r="G1641" s="1">
-        <v>101989</v>
+        <v>589597</v>
       </c>
       <c r="H1641" s="1">
         <v>0</v>
       </c>
       <c r="I1641" s="1">
-        <v>101989</v>
+        <v>589597</v>
       </c>
     </row>
     <row r="1642" spans="1:9" ht="12.75">
@@ -49164,19 +49164,19 @@
         <v>212</v>
       </c>
       <c r="E1642" t="s">
-        <v>349</v>
+        <v>333</v>
       </c>
       <c r="F1642" s="1">
         <v>0</v>
       </c>
       <c r="G1642" s="1">
-        <v>6559</v>
+        <v>101989</v>
       </c>
       <c r="H1642" s="1">
         <v>0</v>
       </c>
       <c r="I1642" s="1">
-        <v>6559</v>
+        <v>101989</v>
       </c>
     </row>
     <row r="1643" spans="1:9" ht="12.75">
@@ -49193,19 +49193,19 @@
         <v>212</v>
       </c>
       <c r="E1643" t="s">
-        <v>334</v>
+        <v>349</v>
       </c>
       <c r="F1643" s="1">
         <v>0</v>
       </c>
       <c r="G1643" s="1">
-        <v>200632</v>
+        <v>6559</v>
       </c>
       <c r="H1643" s="1">
         <v>0</v>
       </c>
       <c r="I1643" s="1">
-        <v>200632</v>
+        <v>6559</v>
       </c>
     </row>
     <row r="1644" spans="1:9" ht="12.75">
@@ -49222,19 +49222,19 @@
         <v>212</v>
       </c>
       <c r="E1644" t="s">
-        <v>350</v>
+        <v>334</v>
       </c>
       <c r="F1644" s="1">
         <v>0</v>
       </c>
       <c r="G1644" s="1">
-        <v>13921</v>
+        <v>200632</v>
       </c>
       <c r="H1644" s="1">
         <v>0</v>
       </c>
       <c r="I1644" s="1">
-        <v>13921</v>
+        <v>200632</v>
       </c>
     </row>
     <row r="1645" spans="1:9" ht="12.75">
@@ -49251,19 +49251,19 @@
         <v>212</v>
       </c>
       <c r="E1645" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="F1645" s="1">
         <v>0</v>
       </c>
       <c r="G1645" s="1">
-        <v>3436</v>
+        <v>13921</v>
       </c>
       <c r="H1645" s="1">
         <v>0</v>
       </c>
       <c r="I1645" s="1">
-        <v>3436</v>
+        <v>13921</v>
       </c>
     </row>
     <row r="1646" spans="1:9" ht="12.75">
@@ -49280,19 +49280,19 @@
         <v>212</v>
       </c>
       <c r="E1646" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="F1646" s="1">
         <v>0</v>
       </c>
       <c r="G1646" s="1">
-        <v>300656</v>
+        <v>3436</v>
       </c>
       <c r="H1646" s="1">
         <v>0</v>
       </c>
       <c r="I1646" s="1">
-        <v>300656</v>
+        <v>3436</v>
       </c>
     </row>
     <row r="1647" spans="1:9" ht="12.75">
@@ -49309,19 +49309,19 @@
         <v>212</v>
       </c>
       <c r="E1647" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="F1647" s="1">
         <v>0</v>
       </c>
       <c r="G1647" s="1">
-        <v>1144422</v>
+        <v>300656</v>
       </c>
       <c r="H1647" s="1">
         <v>0</v>
       </c>
       <c r="I1647" s="1">
-        <v>1144422</v>
+        <v>300656</v>
       </c>
     </row>
     <row r="1648" spans="1:9" ht="12.75">
@@ -49335,22 +49335,22 @@
         <v>105</v>
       </c>
       <c r="D1648" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="E1648" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="F1648" s="1">
         <v>0</v>
       </c>
       <c r="G1648" s="1">
-        <v>1824</v>
+        <v>1144422</v>
       </c>
       <c r="H1648" s="1">
         <v>0</v>
       </c>
       <c r="I1648" s="1">
-        <v>1824</v>
+        <v>1144422</v>
       </c>
     </row>
     <row r="1649" spans="1:9" ht="12.75">
@@ -49367,19 +49367,19 @@
         <v>218</v>
       </c>
       <c r="E1649" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F1649" s="1">
         <v>0</v>
       </c>
       <c r="G1649" s="1">
-        <v>223551</v>
+        <v>1824</v>
       </c>
       <c r="H1649" s="1">
         <v>0</v>
       </c>
       <c r="I1649" s="1">
-        <v>223551</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="1650" spans="1:9" ht="12.75">
@@ -49393,22 +49393,22 @@
         <v>105</v>
       </c>
       <c r="D1650" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E1650" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="F1650" s="1">
         <v>0</v>
       </c>
       <c r="G1650" s="1">
-        <v>49500</v>
+        <v>223551</v>
       </c>
       <c r="H1650" s="1">
         <v>0</v>
       </c>
       <c r="I1650" s="1">
-        <v>49500</v>
+        <v>223551</v>
       </c>
     </row>
     <row r="1651" spans="1:9" ht="12.75">
@@ -49425,19 +49425,19 @@
         <v>219</v>
       </c>
       <c r="E1651" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1651" s="1">
         <v>0</v>
       </c>
       <c r="G1651" s="1">
-        <v>2507503</v>
+        <v>49500</v>
       </c>
       <c r="H1651" s="1">
         <v>0</v>
       </c>
       <c r="I1651" s="1">
-        <v>2507503</v>
+        <v>49500</v>
       </c>
     </row>
     <row r="1652" spans="1:9" ht="12.75">
@@ -49454,19 +49454,19 @@
         <v>219</v>
       </c>
       <c r="E1652" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1652" s="1">
         <v>0</v>
       </c>
       <c r="G1652" s="1">
-        <v>65932</v>
+        <v>2507503</v>
       </c>
       <c r="H1652" s="1">
         <v>0</v>
       </c>
       <c r="I1652" s="1">
-        <v>65932</v>
+        <v>2507503</v>
       </c>
     </row>
     <row r="1653" spans="1:9" ht="12.75">
@@ -49483,19 +49483,19 @@
         <v>219</v>
       </c>
       <c r="E1653" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1653" s="1">
         <v>0</v>
       </c>
       <c r="G1653" s="1">
-        <v>86124</v>
+        <v>65932</v>
       </c>
       <c r="H1653" s="1">
         <v>0</v>
       </c>
       <c r="I1653" s="1">
-        <v>86124</v>
+        <v>65932</v>
       </c>
     </row>
     <row r="1654" spans="1:9" ht="12.75">
@@ -49512,19 +49512,19 @@
         <v>219</v>
       </c>
       <c r="E1654" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1654" s="1">
         <v>0</v>
       </c>
       <c r="G1654" s="1">
-        <v>1021380</v>
+        <v>86124</v>
       </c>
       <c r="H1654" s="1">
         <v>0</v>
       </c>
       <c r="I1654" s="1">
-        <v>1021380</v>
+        <v>86124</v>
       </c>
     </row>
     <row r="1655" spans="1:9" ht="12.75">
@@ -49541,19 +49541,19 @@
         <v>219</v>
       </c>
       <c r="E1655" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1655" s="1">
         <v>0</v>
       </c>
       <c r="G1655" s="1">
-        <v>138789</v>
+        <v>1021380</v>
       </c>
       <c r="H1655" s="1">
         <v>0</v>
       </c>
       <c r="I1655" s="1">
-        <v>138789</v>
+        <v>1021380</v>
       </c>
     </row>
     <row r="1656" spans="1:9" ht="12.75">
@@ -49570,19 +49570,19 @@
         <v>219</v>
       </c>
       <c r="E1656" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F1656" s="1">
         <v>0</v>
       </c>
       <c r="G1656" s="1">
-        <v>8288</v>
+        <v>138789</v>
       </c>
       <c r="H1656" s="1">
         <v>0</v>
       </c>
       <c r="I1656" s="1">
-        <v>8288</v>
+        <v>138789</v>
       </c>
     </row>
     <row r="1657" spans="1:9" ht="12.75">
@@ -49599,19 +49599,19 @@
         <v>219</v>
       </c>
       <c r="E1657" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F1657" s="1">
         <v>0</v>
       </c>
       <c r="G1657" s="1">
-        <v>219258</v>
+        <v>8288</v>
       </c>
       <c r="H1657" s="1">
         <v>0</v>
       </c>
       <c r="I1657" s="1">
-        <v>219258</v>
+        <v>8288</v>
       </c>
     </row>
     <row r="1658" spans="1:9" ht="12.75">
@@ -49628,19 +49628,19 @@
         <v>219</v>
       </c>
       <c r="E1658" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F1658" s="1">
         <v>0</v>
       </c>
       <c r="G1658" s="1">
-        <v>4807583</v>
+        <v>219258</v>
       </c>
       <c r="H1658" s="1">
-        <v>4807583</v>
+        <v>0</v>
       </c>
       <c r="I1658" s="1">
-        <v>0</v>
+        <v>219258</v>
       </c>
     </row>
     <row r="1659" spans="1:9" ht="12.75">
@@ -49657,19 +49657,19 @@
         <v>219</v>
       </c>
       <c r="E1659" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F1659" s="1">
         <v>0</v>
       </c>
       <c r="G1659" s="1">
-        <v>13811</v>
+        <v>4807583</v>
       </c>
       <c r="H1659" s="1">
-        <v>0</v>
+        <v>4807583</v>
       </c>
       <c r="I1659" s="1">
-        <v>13811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1660" spans="1:9" ht="12.75">
@@ -49686,19 +49686,19 @@
         <v>219</v>
       </c>
       <c r="E1660" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F1660" s="1">
         <v>0</v>
       </c>
       <c r="G1660" s="1">
-        <v>729998</v>
+        <v>13811</v>
       </c>
       <c r="H1660" s="1">
         <v>0</v>
       </c>
       <c r="I1660" s="1">
-        <v>729998</v>
+        <v>13811</v>
       </c>
     </row>
     <row r="1661" spans="1:9" ht="12.75">
@@ -49712,22 +49712,22 @@
         <v>105</v>
       </c>
       <c r="D1661" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E1661" t="s">
-        <v>331</v>
+        <v>342</v>
       </c>
       <c r="F1661" s="1">
         <v>0</v>
       </c>
       <c r="G1661" s="1">
-        <v>3734639.23</v>
+        <v>729998</v>
       </c>
       <c r="H1661" s="1">
         <v>0</v>
       </c>
       <c r="I1661" s="1">
-        <v>3734639.23</v>
+        <v>729998</v>
       </c>
     </row>
     <row r="1662" spans="1:9" ht="12.75">
@@ -49744,19 +49744,19 @@
         <v>221</v>
       </c>
       <c r="E1662" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1662" s="1">
         <v>0</v>
       </c>
       <c r="G1662" s="1">
-        <v>289295.48</v>
+        <v>3734639.2299999995</v>
       </c>
       <c r="H1662" s="1">
         <v>0</v>
       </c>
       <c r="I1662" s="1">
-        <v>289295.48</v>
+        <v>3734639.2299999995</v>
       </c>
     </row>
     <row r="1663" spans="1:9" ht="12.75">
@@ -49773,19 +49773,19 @@
         <v>221</v>
       </c>
       <c r="E1663" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1663" s="1">
         <v>0</v>
       </c>
       <c r="G1663" s="1">
-        <v>218609.22000000003</v>
+        <v>289295.48</v>
       </c>
       <c r="H1663" s="1">
         <v>0</v>
       </c>
       <c r="I1663" s="1">
-        <v>218609.22000000003</v>
+        <v>289295.48</v>
       </c>
     </row>
     <row r="1664" spans="1:9" ht="12.75">
@@ -49802,19 +49802,19 @@
         <v>221</v>
       </c>
       <c r="E1664" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1664" s="1">
         <v>0</v>
       </c>
       <c r="G1664" s="1">
-        <v>1910663.0799999998</v>
+        <v>218609.22000000003</v>
       </c>
       <c r="H1664" s="1">
         <v>0</v>
       </c>
       <c r="I1664" s="1">
-        <v>1910663.0799999998</v>
+        <v>218609.22000000003</v>
       </c>
     </row>
     <row r="1665" spans="1:9" ht="12.75">
@@ -49831,19 +49831,19 @@
         <v>221</v>
       </c>
       <c r="E1665" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1665" s="1">
         <v>0</v>
       </c>
       <c r="G1665" s="1">
-        <v>685737.6099999999</v>
+        <v>1910663.0799999996</v>
       </c>
       <c r="H1665" s="1">
         <v>0</v>
       </c>
       <c r="I1665" s="1">
-        <v>685737.6099999999</v>
+        <v>1910663.0799999996</v>
       </c>
     </row>
     <row r="1666" spans="1:9" ht="12.75">
@@ -49860,19 +49860,19 @@
         <v>221</v>
       </c>
       <c r="E1666" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F1666" s="1">
         <v>0</v>
       </c>
       <c r="G1666" s="1">
-        <v>4078.70</v>
+        <v>685737.61</v>
       </c>
       <c r="H1666" s="1">
         <v>0</v>
       </c>
       <c r="I1666" s="1">
-        <v>4078.70</v>
+        <v>685737.61</v>
       </c>
     </row>
     <row r="1667" spans="1:9" ht="12.75">
@@ -49889,19 +49889,19 @@
         <v>221</v>
       </c>
       <c r="E1667" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F1667" s="1">
         <v>0</v>
       </c>
       <c r="G1667" s="1">
-        <v>191355.02000000002</v>
+        <v>4078.70</v>
       </c>
       <c r="H1667" s="1">
         <v>0</v>
       </c>
       <c r="I1667" s="1">
-        <v>191355.02000000002</v>
+        <v>4078.70</v>
       </c>
     </row>
     <row r="1668" spans="1:9" ht="12.75">
@@ -49918,19 +49918,19 @@
         <v>221</v>
       </c>
       <c r="E1668" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F1668" s="1">
         <v>0</v>
       </c>
       <c r="G1668" s="1">
-        <v>381348.32000000007</v>
+        <v>191355.02</v>
       </c>
       <c r="H1668" s="1">
         <v>0</v>
       </c>
       <c r="I1668" s="1">
-        <v>381348.32000000007</v>
+        <v>191355.02</v>
       </c>
     </row>
     <row r="1669" spans="1:9" ht="12.75">
@@ -49947,19 +49947,19 @@
         <v>221</v>
       </c>
       <c r="E1669" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F1669" s="1">
         <v>0</v>
       </c>
       <c r="G1669" s="1">
-        <v>93497</v>
+        <v>381348.32000000007</v>
       </c>
       <c r="H1669" s="1">
         <v>0</v>
       </c>
       <c r="I1669" s="1">
-        <v>93497</v>
+        <v>381348.32000000007</v>
       </c>
     </row>
     <row r="1670" spans="1:9" ht="12.75">
@@ -49976,19 +49976,19 @@
         <v>221</v>
       </c>
       <c r="E1670" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F1670" s="1">
         <v>0</v>
       </c>
       <c r="G1670" s="1">
-        <v>211054</v>
+        <v>93497</v>
       </c>
       <c r="H1670" s="1">
         <v>0</v>
       </c>
       <c r="I1670" s="1">
-        <v>211054</v>
+        <v>93497</v>
       </c>
     </row>
     <row r="1671" spans="1:9" ht="12.75">
@@ -50005,19 +50005,19 @@
         <v>221</v>
       </c>
       <c r="E1671" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F1671" s="1">
         <v>0</v>
       </c>
       <c r="G1671" s="1">
-        <v>1105942</v>
+        <v>211054</v>
       </c>
       <c r="H1671" s="1">
         <v>0</v>
       </c>
       <c r="I1671" s="1">
-        <v>1105942</v>
+        <v>211054</v>
       </c>
     </row>
     <row r="1672" spans="1:9" ht="12.75">
@@ -50031,22 +50031,22 @@
         <v>105</v>
       </c>
       <c r="D1672" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E1672" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="F1672" s="1">
         <v>0</v>
       </c>
       <c r="G1672" s="1">
-        <v>1711047.58</v>
+        <v>1105942</v>
       </c>
       <c r="H1672" s="1">
         <v>0</v>
       </c>
       <c r="I1672" s="1">
-        <v>1711047.58</v>
+        <v>1105942</v>
       </c>
     </row>
     <row r="1673" spans="1:9" ht="12.75">
@@ -50063,19 +50063,19 @@
         <v>222</v>
       </c>
       <c r="E1673" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1673" s="1">
         <v>0</v>
       </c>
       <c r="G1673" s="1">
-        <v>1338867.5899999999</v>
+        <v>1711047.58</v>
       </c>
       <c r="H1673" s="1">
         <v>0</v>
       </c>
       <c r="I1673" s="1">
-        <v>1338867.5899999999</v>
+        <v>1711047.58</v>
       </c>
     </row>
     <row r="1674" spans="1:9" ht="12.75">
@@ -50092,19 +50092,19 @@
         <v>222</v>
       </c>
       <c r="E1674" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1674" s="1">
         <v>0</v>
       </c>
       <c r="G1674" s="1">
-        <v>6084145</v>
+        <v>1338867.5899999999</v>
       </c>
       <c r="H1674" s="1">
         <v>0</v>
       </c>
       <c r="I1674" s="1">
-        <v>6084145</v>
+        <v>1338867.5899999999</v>
       </c>
     </row>
     <row r="1675" spans="1:9" ht="12.75">
@@ -50121,19 +50121,19 @@
         <v>222</v>
       </c>
       <c r="E1675" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1675" s="1">
         <v>0</v>
       </c>
       <c r="G1675" s="1">
-        <v>492996</v>
+        <v>6084145</v>
       </c>
       <c r="H1675" s="1">
         <v>0</v>
       </c>
       <c r="I1675" s="1">
-        <v>492996</v>
+        <v>6084145</v>
       </c>
     </row>
     <row r="1676" spans="1:9" ht="12.75">
@@ -50150,19 +50150,19 @@
         <v>222</v>
       </c>
       <c r="E1676" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1676" s="1">
         <v>0</v>
       </c>
       <c r="G1676" s="1">
-        <v>351533</v>
+        <v>492996</v>
       </c>
       <c r="H1676" s="1">
         <v>0</v>
       </c>
       <c r="I1676" s="1">
-        <v>351533</v>
+        <v>492996</v>
       </c>
     </row>
     <row r="1677" spans="1:9" ht="12.75">
@@ -50179,19 +50179,19 @@
         <v>222</v>
       </c>
       <c r="E1677" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1677" s="1">
         <v>0</v>
       </c>
       <c r="G1677" s="1">
-        <v>10682502</v>
+        <v>351533</v>
       </c>
       <c r="H1677" s="1">
         <v>0</v>
       </c>
       <c r="I1677" s="1">
-        <v>10682502</v>
+        <v>351533</v>
       </c>
     </row>
     <row r="1678" spans="1:9" ht="12.75">
@@ -50208,19 +50208,19 @@
         <v>222</v>
       </c>
       <c r="E1678" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1678" s="1">
         <v>0</v>
       </c>
       <c r="G1678" s="1">
-        <v>992656</v>
+        <v>10682502</v>
       </c>
       <c r="H1678" s="1">
         <v>0</v>
       </c>
       <c r="I1678" s="1">
-        <v>992656</v>
+        <v>10682502</v>
       </c>
     </row>
     <row r="1679" spans="1:9" ht="12.75">
@@ -50237,19 +50237,19 @@
         <v>222</v>
       </c>
       <c r="E1679" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F1679" s="1">
         <v>0</v>
       </c>
       <c r="G1679" s="1">
-        <v>12048</v>
+        <v>992656</v>
       </c>
       <c r="H1679" s="1">
         <v>0</v>
       </c>
       <c r="I1679" s="1">
-        <v>12048</v>
+        <v>992656</v>
       </c>
     </row>
     <row r="1680" spans="1:9" ht="12.75">
@@ -50266,19 +50266,19 @@
         <v>222</v>
       </c>
       <c r="E1680" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="F1680" s="1">
         <v>0</v>
       </c>
       <c r="G1680" s="1">
-        <v>25244</v>
+        <v>12048</v>
       </c>
       <c r="H1680" s="1">
         <v>0</v>
       </c>
       <c r="I1680" s="1">
-        <v>25244</v>
+        <v>12048</v>
       </c>
     </row>
     <row r="1681" spans="1:9" ht="12.75">
@@ -50295,19 +50295,19 @@
         <v>222</v>
       </c>
       <c r="E1681" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="F1681" s="1">
         <v>0</v>
       </c>
       <c r="G1681" s="1">
-        <v>288601</v>
+        <v>25244</v>
       </c>
       <c r="H1681" s="1">
         <v>0</v>
       </c>
       <c r="I1681" s="1">
-        <v>288601</v>
+        <v>25244</v>
       </c>
     </row>
     <row r="1682" spans="1:9" ht="12.75">
@@ -50324,19 +50324,19 @@
         <v>222</v>
       </c>
       <c r="E1682" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F1682" s="1">
         <v>0</v>
       </c>
       <c r="G1682" s="1">
-        <v>1595017</v>
+        <v>288601</v>
       </c>
       <c r="H1682" s="1">
         <v>0</v>
       </c>
       <c r="I1682" s="1">
-        <v>1595017</v>
+        <v>288601</v>
       </c>
     </row>
     <row r="1683" spans="1:9" ht="12.75">
@@ -50353,19 +50353,19 @@
         <v>222</v>
       </c>
       <c r="E1683" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
       <c r="F1683" s="1">
         <v>0</v>
       </c>
       <c r="G1683" s="1">
-        <v>100146</v>
+        <v>1595017</v>
       </c>
       <c r="H1683" s="1">
         <v>0</v>
       </c>
       <c r="I1683" s="1">
-        <v>100146</v>
+        <v>1595017</v>
       </c>
     </row>
     <row r="1684" spans="1:9" ht="12.75">
@@ -50382,19 +50382,19 @@
         <v>222</v>
       </c>
       <c r="E1684" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="F1684" s="1">
         <v>0</v>
       </c>
       <c r="G1684" s="1">
-        <v>279211</v>
+        <v>100146</v>
       </c>
       <c r="H1684" s="1">
         <v>0</v>
       </c>
       <c r="I1684" s="1">
-        <v>279211</v>
+        <v>100146</v>
       </c>
     </row>
     <row r="1685" spans="1:9" ht="12.75">
@@ -50411,19 +50411,19 @@
         <v>222</v>
       </c>
       <c r="E1685" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F1685" s="1">
         <v>0</v>
       </c>
       <c r="G1685" s="1">
-        <v>227931</v>
+        <v>279211</v>
       </c>
       <c r="H1685" s="1">
         <v>0</v>
       </c>
       <c r="I1685" s="1">
-        <v>227931</v>
+        <v>279211</v>
       </c>
     </row>
     <row r="1686" spans="1:9" ht="12.75">
@@ -50440,19 +50440,19 @@
         <v>222</v>
       </c>
       <c r="E1686" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F1686" s="1">
         <v>0</v>
       </c>
       <c r="G1686" s="1">
-        <v>53925</v>
+        <v>227931</v>
       </c>
       <c r="H1686" s="1">
         <v>0</v>
       </c>
       <c r="I1686" s="1">
-        <v>53925</v>
+        <v>227931</v>
       </c>
     </row>
     <row r="1687" spans="1:9" ht="12.75">
@@ -50466,22 +50466,22 @@
         <v>105</v>
       </c>
       <c r="D1687" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E1687" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="F1687" s="1">
         <v>0</v>
       </c>
       <c r="G1687" s="1">
-        <v>0</v>
+        <v>53925</v>
       </c>
       <c r="H1687" s="1">
-        <v>2.423587017E7</v>
+        <v>0</v>
       </c>
       <c r="I1687" s="1">
-        <v>-2.423587017E7</v>
+        <v>53925</v>
       </c>
     </row>
     <row r="1688" spans="1:9" ht="12.75">
@@ -50495,7 +50495,7 @@
         <v>105</v>
       </c>
       <c r="D1688" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E1688" t="s">
         <v>348</v>
@@ -50504,13 +50504,13 @@
         <v>0</v>
       </c>
       <c r="G1688" s="1">
-        <v>119165</v>
+        <v>0</v>
       </c>
       <c r="H1688" s="1">
-        <v>0</v>
+        <v>2.423587017E7</v>
       </c>
       <c r="I1688" s="1">
-        <v>119165</v>
+        <v>-2.423587017E7</v>
       </c>
     </row>
     <row r="1689" spans="1:9" ht="12.75">
@@ -50524,22 +50524,22 @@
         <v>105</v>
       </c>
       <c r="D1689" t="s">
-        <v>307</v>
+        <v>225</v>
       </c>
       <c r="E1689" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="F1689" s="1">
         <v>0</v>
       </c>
       <c r="G1689" s="1">
-        <v>10532</v>
+        <v>119165</v>
       </c>
       <c r="H1689" s="1">
         <v>0</v>
       </c>
       <c r="I1689" s="1">
-        <v>10532</v>
+        <v>119165</v>
       </c>
     </row>
     <row r="1690" spans="1:9" ht="12.75">
@@ -50556,19 +50556,19 @@
         <v>307</v>
       </c>
       <c r="E1690" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1690" s="1">
         <v>0</v>
       </c>
       <c r="G1690" s="1">
-        <v>1417</v>
+        <v>10532</v>
       </c>
       <c r="H1690" s="1">
         <v>0</v>
       </c>
       <c r="I1690" s="1">
-        <v>1417</v>
+        <v>10532</v>
       </c>
     </row>
     <row r="1691" spans="1:9" ht="12.75">
@@ -50585,19 +50585,19 @@
         <v>307</v>
       </c>
       <c r="E1691" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1691" s="1">
         <v>0</v>
       </c>
       <c r="G1691" s="1">
-        <v>88200</v>
+        <v>1417</v>
       </c>
       <c r="H1691" s="1">
         <v>0</v>
       </c>
       <c r="I1691" s="1">
-        <v>88200</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="1692" spans="1:9" ht="12.75">
@@ -50614,19 +50614,19 @@
         <v>307</v>
       </c>
       <c r="E1692" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1692" s="1">
         <v>0</v>
       </c>
       <c r="G1692" s="1">
-        <v>3374</v>
+        <v>88200</v>
       </c>
       <c r="H1692" s="1">
         <v>0</v>
       </c>
       <c r="I1692" s="1">
-        <v>3374</v>
+        <v>88200</v>
       </c>
     </row>
     <row r="1693" spans="1:9" ht="12.75">
@@ -50643,19 +50643,19 @@
         <v>307</v>
       </c>
       <c r="E1693" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1693" s="1">
         <v>0</v>
       </c>
       <c r="G1693" s="1">
-        <v>5996</v>
+        <v>3374</v>
       </c>
       <c r="H1693" s="1">
         <v>0</v>
       </c>
       <c r="I1693" s="1">
-        <v>5996</v>
+        <v>3374</v>
       </c>
     </row>
     <row r="1694" spans="1:9" ht="12.75">
@@ -50672,19 +50672,19 @@
         <v>307</v>
       </c>
       <c r="E1694" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1694" s="1">
         <v>0</v>
       </c>
       <c r="G1694" s="1">
-        <v>22800</v>
+        <v>5996</v>
       </c>
       <c r="H1694" s="1">
         <v>0</v>
       </c>
       <c r="I1694" s="1">
-        <v>22800</v>
+        <v>5996</v>
       </c>
     </row>
     <row r="1695" spans="1:9" ht="12.75">
@@ -50701,19 +50701,19 @@
         <v>307</v>
       </c>
       <c r="E1695" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1695" s="1">
         <v>0</v>
       </c>
       <c r="G1695" s="1">
-        <v>12631</v>
+        <v>22800</v>
       </c>
       <c r="H1695" s="1">
         <v>0</v>
       </c>
       <c r="I1695" s="1">
-        <v>12631</v>
+        <v>22800</v>
       </c>
     </row>
     <row r="1696" spans="1:9" ht="12.75">
@@ -50730,19 +50730,19 @@
         <v>307</v>
       </c>
       <c r="E1696" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F1696" s="1">
         <v>0</v>
       </c>
       <c r="G1696" s="1">
-        <v>179</v>
+        <v>12631</v>
       </c>
       <c r="H1696" s="1">
         <v>0</v>
       </c>
       <c r="I1696" s="1">
-        <v>179</v>
+        <v>12631</v>
       </c>
     </row>
     <row r="1697" spans="1:9" ht="12.75">
@@ -50759,19 +50759,19 @@
         <v>307</v>
       </c>
       <c r="E1697" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F1697" s="1">
         <v>0</v>
       </c>
       <c r="G1697" s="1">
-        <v>1584</v>
+        <v>179</v>
       </c>
       <c r="H1697" s="1">
         <v>0</v>
       </c>
       <c r="I1697" s="1">
-        <v>1584</v>
+        <v>179</v>
       </c>
     </row>
     <row r="1698" spans="1:9" ht="12.75">
@@ -50788,19 +50788,19 @@
         <v>307</v>
       </c>
       <c r="E1698" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F1698" s="1">
         <v>0</v>
       </c>
       <c r="G1698" s="1">
-        <v>10660</v>
+        <v>1584</v>
       </c>
       <c r="H1698" s="1">
         <v>0</v>
       </c>
       <c r="I1698" s="1">
-        <v>10660</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="1699" spans="1:9" ht="12.75">
@@ -50817,19 +50817,19 @@
         <v>307</v>
       </c>
       <c r="E1699" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F1699" s="1">
         <v>0</v>
       </c>
       <c r="G1699" s="1">
-        <v>154499</v>
+        <v>10660</v>
       </c>
       <c r="H1699" s="1">
-        <v>154499</v>
+        <v>0</v>
       </c>
       <c r="I1699" s="1">
-        <v>0</v>
+        <v>10660</v>
       </c>
     </row>
     <row r="1700" spans="1:9" ht="12.75">
@@ -50846,19 +50846,19 @@
         <v>307</v>
       </c>
       <c r="E1700" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F1700" s="1">
         <v>0</v>
       </c>
       <c r="G1700" s="1">
-        <v>249</v>
+        <v>154499</v>
       </c>
       <c r="H1700" s="1">
-        <v>0</v>
+        <v>154499</v>
       </c>
       <c r="I1700" s="1">
-        <v>249</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1701" spans="1:9" ht="12.75">
@@ -50875,19 +50875,19 @@
         <v>307</v>
       </c>
       <c r="E1701" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F1701" s="1">
         <v>0</v>
       </c>
       <c r="G1701" s="1">
-        <v>375</v>
+        <v>249</v>
       </c>
       <c r="H1701" s="1">
         <v>0</v>
       </c>
       <c r="I1701" s="1">
-        <v>375</v>
+        <v>249</v>
       </c>
     </row>
     <row r="1702" spans="1:9" ht="12.75">
@@ -50904,19 +50904,19 @@
         <v>307</v>
       </c>
       <c r="E1702" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F1702" s="1">
         <v>0</v>
       </c>
       <c r="G1702" s="1">
-        <v>667</v>
+        <v>375</v>
       </c>
       <c r="H1702" s="1">
         <v>0</v>
       </c>
       <c r="I1702" s="1">
-        <v>667</v>
+        <v>375</v>
       </c>
     </row>
     <row r="1703" spans="1:9" ht="12.75">
@@ -50930,22 +50930,22 @@
         <v>105</v>
       </c>
       <c r="D1703" t="s">
-        <v>228</v>
+        <v>307</v>
       </c>
       <c r="E1703" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
       <c r="F1703" s="1">
         <v>0</v>
       </c>
       <c r="G1703" s="1">
-        <v>121502</v>
+        <v>667</v>
       </c>
       <c r="H1703" s="1">
         <v>0</v>
       </c>
       <c r="I1703" s="1">
-        <v>121502</v>
+        <v>667</v>
       </c>
     </row>
     <row r="1704" spans="1:9" ht="12.75">
@@ -50959,22 +50959,22 @@
         <v>105</v>
       </c>
       <c r="D1704" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="E1704" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="F1704" s="1">
         <v>0</v>
       </c>
       <c r="G1704" s="1">
-        <v>3500</v>
+        <v>121502</v>
       </c>
       <c r="H1704" s="1">
         <v>0</v>
       </c>
       <c r="I1704" s="1">
-        <v>3500</v>
+        <v>121502</v>
       </c>
     </row>
     <row r="1705" spans="1:9" ht="12.75">
@@ -50988,22 +50988,22 @@
         <v>105</v>
       </c>
       <c r="D1705" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E1705" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
       <c r="F1705" s="1">
         <v>0</v>
       </c>
       <c r="G1705" s="1">
-        <v>9000</v>
+        <v>3500</v>
       </c>
       <c r="H1705" s="1">
         <v>0</v>
       </c>
       <c r="I1705" s="1">
-        <v>9000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="1706" spans="1:9" ht="12.75">
@@ -51020,19 +51020,19 @@
         <v>234</v>
       </c>
       <c r="E1706" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F1706" s="1">
         <v>0</v>
       </c>
       <c r="G1706" s="1">
-        <v>516448</v>
+        <v>9000</v>
       </c>
       <c r="H1706" s="1">
         <v>0</v>
       </c>
       <c r="I1706" s="1">
-        <v>516448</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="1707" spans="1:9" ht="12.75">
@@ -51046,22 +51046,22 @@
         <v>105</v>
       </c>
       <c r="D1707" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E1707" t="s">
-        <v>244</v>
+        <v>339</v>
       </c>
       <c r="F1707" s="1">
         <v>0</v>
       </c>
       <c r="G1707" s="1">
-        <v>853156</v>
+        <v>516448</v>
       </c>
       <c r="H1707" s="1">
         <v>0</v>
       </c>
       <c r="I1707" s="1">
-        <v>853156</v>
+        <v>516448</v>
       </c>
     </row>
     <row r="1708" spans="1:9" ht="12.75">
@@ -51078,19 +51078,19 @@
         <v>235</v>
       </c>
       <c r="E1708" t="s">
-        <v>351</v>
+        <v>244</v>
       </c>
       <c r="F1708" s="1">
         <v>0</v>
       </c>
       <c r="G1708" s="1">
-        <v>1317706</v>
+        <v>853156</v>
       </c>
       <c r="H1708" s="1">
         <v>0</v>
       </c>
       <c r="I1708" s="1">
-        <v>1317706</v>
+        <v>853156</v>
       </c>
     </row>
     <row r="1709" spans="1:9" ht="12.75">
@@ -51107,19 +51107,19 @@
         <v>235</v>
       </c>
       <c r="E1709" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="F1709" s="1">
         <v>0</v>
       </c>
       <c r="G1709" s="1">
-        <v>3665552</v>
+        <v>1317706</v>
       </c>
       <c r="H1709" s="1">
         <v>0</v>
       </c>
       <c r="I1709" s="1">
-        <v>3665552</v>
+        <v>1317706</v>
       </c>
     </row>
     <row r="1710" spans="1:9" ht="12.75">
@@ -51136,19 +51136,19 @@
         <v>235</v>
       </c>
       <c r="E1710" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F1710" s="1">
         <v>0</v>
       </c>
       <c r="G1710" s="1">
-        <v>2999088</v>
+        <v>3665552</v>
       </c>
       <c r="H1710" s="1">
         <v>0</v>
       </c>
       <c r="I1710" s="1">
-        <v>2999088</v>
+        <v>3665552</v>
       </c>
     </row>
     <row r="1711" spans="1:9" ht="12.75">
@@ -51165,19 +51165,19 @@
         <v>235</v>
       </c>
       <c r="E1711" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F1711" s="1">
         <v>0</v>
       </c>
       <c r="G1711" s="1">
-        <v>709534</v>
+        <v>2999088</v>
       </c>
       <c r="H1711" s="1">
         <v>0</v>
       </c>
       <c r="I1711" s="1">
-        <v>709534</v>
+        <v>2999088</v>
       </c>
     </row>
     <row r="1712" spans="1:9" ht="12.75">
@@ -51191,22 +51191,22 @@
         <v>105</v>
       </c>
       <c r="D1712" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E1712" t="s">
-        <v>330</v>
+        <v>354</v>
       </c>
       <c r="F1712" s="1">
         <v>0</v>
       </c>
       <c r="G1712" s="1">
-        <v>31500</v>
+        <v>709534</v>
       </c>
       <c r="H1712" s="1">
         <v>0</v>
       </c>
       <c r="I1712" s="1">
-        <v>31500</v>
+        <v>709534</v>
       </c>
     </row>
     <row r="1713" spans="1:9" ht="12.75">
@@ -51220,22 +51220,22 @@
         <v>105</v>
       </c>
       <c r="D1713" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E1713" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F1713" s="1">
         <v>0</v>
       </c>
       <c r="G1713" s="1">
-        <v>212400</v>
+        <v>32840</v>
       </c>
       <c r="H1713" s="1">
         <v>0</v>
       </c>
       <c r="I1713" s="1">
-        <v>212400</v>
+        <v>32840</v>
       </c>
     </row>
     <row r="1714" spans="1:9" ht="12.75">
@@ -51252,19 +51252,19 @@
         <v>238</v>
       </c>
       <c r="E1714" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1714" s="1">
         <v>0</v>
       </c>
       <c r="G1714" s="1">
-        <v>577360</v>
+        <v>212400</v>
       </c>
       <c r="H1714" s="1">
         <v>0</v>
       </c>
       <c r="I1714" s="1">
-        <v>577360</v>
+        <v>212400</v>
       </c>
     </row>
     <row r="1715" spans="1:9" ht="12.75">
@@ -51281,19 +51281,19 @@
         <v>238</v>
       </c>
       <c r="E1715" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1715" s="1">
         <v>0</v>
       </c>
       <c r="G1715" s="1">
-        <v>518969</v>
+        <v>577360</v>
       </c>
       <c r="H1715" s="1">
         <v>0</v>
       </c>
       <c r="I1715" s="1">
-        <v>518969</v>
+        <v>577360</v>
       </c>
     </row>
     <row r="1716" spans="1:9" ht="12.75">
@@ -51310,19 +51310,19 @@
         <v>238</v>
       </c>
       <c r="E1716" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F1716" s="1">
         <v>0</v>
       </c>
       <c r="G1716" s="1">
-        <v>271070</v>
+        <v>518969</v>
       </c>
       <c r="H1716" s="1">
         <v>0</v>
       </c>
       <c r="I1716" s="1">
-        <v>271070</v>
+        <v>518969</v>
       </c>
     </row>
     <row r="1717" spans="1:9" ht="12.75">
@@ -51339,19 +51339,19 @@
         <v>238</v>
       </c>
       <c r="E1717" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1717" s="1">
         <v>0</v>
       </c>
       <c r="G1717" s="1">
-        <v>137184</v>
+        <v>271070</v>
       </c>
       <c r="H1717" s="1">
         <v>0</v>
       </c>
       <c r="I1717" s="1">
-        <v>137184</v>
+        <v>271070</v>
       </c>
     </row>
     <row r="1718" spans="1:9" ht="12.75">
@@ -51368,19 +51368,19 @@
         <v>238</v>
       </c>
       <c r="E1718" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F1718" s="1">
         <v>0</v>
       </c>
       <c r="G1718" s="1">
-        <v>91456</v>
+        <v>137184</v>
       </c>
       <c r="H1718" s="1">
         <v>0</v>
       </c>
       <c r="I1718" s="1">
-        <v>91456</v>
+        <v>137184</v>
       </c>
     </row>
     <row r="1719" spans="1:9" ht="12.75">
@@ -51397,19 +51397,19 @@
         <v>238</v>
       </c>
       <c r="E1719" t="s">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="F1719" s="1">
         <v>0</v>
       </c>
       <c r="G1719" s="1">
-        <v>8275</v>
+        <v>91456</v>
       </c>
       <c r="H1719" s="1">
         <v>0</v>
       </c>
       <c r="I1719" s="1">
-        <v>8275</v>
+        <v>91456</v>
       </c>
     </row>
     <row r="1720" spans="1:9" ht="12.75">
@@ -51426,19 +51426,19 @@
         <v>238</v>
       </c>
       <c r="E1720" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="F1720" s="1">
         <v>0</v>
       </c>
       <c r="G1720" s="1">
-        <v>104725</v>
+        <v>8275</v>
       </c>
       <c r="H1720" s="1">
         <v>0</v>
       </c>
       <c r="I1720" s="1">
-        <v>104725</v>
+        <v>8275</v>
       </c>
     </row>
     <row r="1721" spans="1:9" ht="12.75">
@@ -51452,22 +51452,22 @@
         <v>105</v>
       </c>
       <c r="D1721" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E1721" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="F1721" s="1">
         <v>0</v>
       </c>
       <c r="G1721" s="1">
-        <v>8770</v>
+        <v>104725</v>
       </c>
       <c r="H1721" s="1">
         <v>0</v>
       </c>
       <c r="I1721" s="1">
-        <v>8770</v>
+        <v>104725</v>
       </c>
     </row>
     <row r="1722" spans="1:9" ht="12.75">
@@ -51481,7 +51481,7 @@
         <v>105</v>
       </c>
       <c r="D1722" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E1722" t="s">
         <v>330</v>
@@ -51490,13 +51490,13 @@
         <v>0</v>
       </c>
       <c r="G1722" s="1">
-        <v>62919.34</v>
+        <v>8770</v>
       </c>
       <c r="H1722" s="1">
         <v>0</v>
       </c>
       <c r="I1722" s="1">
-        <v>62919.34</v>
+        <v>8770</v>
       </c>
     </row>
     <row r="1723" spans="1:9" ht="12.75">
@@ -51510,22 +51510,22 @@
         <v>105</v>
       </c>
       <c r="D1723" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E1723" t="s">
-        <v>13</v>
+        <v>330</v>
       </c>
       <c r="F1723" s="1">
         <v>0</v>
       </c>
       <c r="G1723" s="1">
-        <v>1</v>
+        <v>77798.34</v>
       </c>
       <c r="H1723" s="1">
-        <v>12.20</v>
+        <v>0</v>
       </c>
       <c r="I1723" s="1">
-        <v>-11.20</v>
+        <v>77798.34</v>
       </c>
     </row>
     <row r="1724" spans="1:9" ht="12.75">
@@ -51539,22 +51539,22 @@
         <v>105</v>
       </c>
       <c r="D1724" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E1724" t="s">
-        <v>329</v>
+        <v>13</v>
       </c>
       <c r="F1724" s="1">
         <v>0</v>
       </c>
       <c r="G1724" s="1">
-        <v>8760</v>
+        <v>1</v>
       </c>
       <c r="H1724" s="1">
-        <v>0</v>
+        <v>12.20</v>
       </c>
       <c r="I1724" s="1">
-        <v>8760</v>
+        <v>-11.20</v>
       </c>
     </row>
     <row r="1725" spans="1:9" ht="12.75">
@@ -51571,19 +51571,19 @@
         <v>243</v>
       </c>
       <c r="E1725" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1725" s="1">
         <v>0</v>
       </c>
       <c r="G1725" s="1">
-        <v>1205693</v>
+        <v>8760</v>
       </c>
       <c r="H1725" s="1">
         <v>0</v>
       </c>
       <c r="I1725" s="1">
-        <v>1205693</v>
+        <v>8760</v>
       </c>
     </row>
     <row r="1726" spans="1:9" ht="12.75">
@@ -51600,19 +51600,19 @@
         <v>243</v>
       </c>
       <c r="E1726" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F1726" s="1">
         <v>0</v>
       </c>
       <c r="G1726" s="1">
-        <v>117363390</v>
+        <v>1205693</v>
       </c>
       <c r="H1726" s="1">
         <v>0</v>
       </c>
       <c r="I1726" s="1">
-        <v>117363390</v>
+        <v>1205693</v>
       </c>
     </row>
     <row r="1727" spans="1:9" ht="12.75">
@@ -51629,19 +51629,19 @@
         <v>243</v>
       </c>
       <c r="E1727" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1727" s="1">
         <v>0</v>
       </c>
       <c r="G1727" s="1">
-        <v>10830040</v>
+        <v>117363390</v>
       </c>
       <c r="H1727" s="1">
         <v>0</v>
       </c>
       <c r="I1727" s="1">
-        <v>10830040</v>
+        <v>117363390</v>
       </c>
     </row>
     <row r="1728" spans="1:9" ht="12.75">
@@ -51658,19 +51658,19 @@
         <v>243</v>
       </c>
       <c r="E1728" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="F1728" s="1">
         <v>0</v>
       </c>
       <c r="G1728" s="1">
-        <v>5015000</v>
+        <v>10830040</v>
       </c>
       <c r="H1728" s="1">
         <v>0</v>
       </c>
       <c r="I1728" s="1">
-        <v>5015000</v>
+        <v>10830040</v>
       </c>
     </row>
     <row r="1729" spans="1:9" ht="12.75">
@@ -51687,19 +51687,19 @@
         <v>243</v>
       </c>
       <c r="E1729" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F1729" s="1">
         <v>0</v>
       </c>
       <c r="G1729" s="1">
-        <v>33458322</v>
+        <v>5015000</v>
       </c>
       <c r="H1729" s="1">
         <v>0</v>
       </c>
       <c r="I1729" s="1">
-        <v>33458322</v>
+        <v>5015000</v>
       </c>
     </row>
     <row r="1730" spans="1:9" ht="12.75">
@@ -51716,19 +51716,19 @@
         <v>243</v>
       </c>
       <c r="E1730" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="F1730" s="1">
         <v>0</v>
       </c>
       <c r="G1730" s="1">
-        <v>1194533</v>
+        <v>33458322</v>
       </c>
       <c r="H1730" s="1">
         <v>0</v>
       </c>
       <c r="I1730" s="1">
-        <v>1194533</v>
+        <v>33458322</v>
       </c>
     </row>
     <row r="1731" spans="1:9" ht="12.75">
@@ -51742,22 +51742,22 @@
         <v>105</v>
       </c>
       <c r="D1731" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1731" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="F1731" s="1">
         <v>0</v>
       </c>
       <c r="G1731" s="1">
-        <v>31481</v>
+        <v>1194533</v>
       </c>
       <c r="H1731" s="1">
         <v>0</v>
       </c>
       <c r="I1731" s="1">
-        <v>31481</v>
+        <v>1194533</v>
       </c>
     </row>
     <row r="1732" spans="1:9" ht="12.75">
@@ -51774,19 +51774,19 @@
         <v>246</v>
       </c>
       <c r="E1732" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1732" s="1">
         <v>0</v>
       </c>
       <c r="G1732" s="1">
-        <v>6638</v>
+        <v>31481</v>
       </c>
       <c r="H1732" s="1">
         <v>0</v>
       </c>
       <c r="I1732" s="1">
-        <v>6638</v>
+        <v>31481</v>
       </c>
     </row>
     <row r="1733" spans="1:9" ht="12.75">
@@ -51803,19 +51803,19 @@
         <v>246</v>
       </c>
       <c r="E1733" t="s">
-        <v>355</v>
+        <v>332</v>
       </c>
       <c r="F1733" s="1">
         <v>0</v>
       </c>
       <c r="G1733" s="1">
-        <v>7140</v>
+        <v>6638</v>
       </c>
       <c r="H1733" s="1">
         <v>0</v>
       </c>
       <c r="I1733" s="1">
-        <v>7140</v>
+        <v>6638</v>
       </c>
     </row>
     <row r="1734" spans="1:9" ht="12.75">
@@ -51832,19 +51832,19 @@
         <v>246</v>
       </c>
       <c r="E1734" t="s">
-        <v>338</v>
+        <v>355</v>
       </c>
       <c r="F1734" s="1">
         <v>0</v>
       </c>
       <c r="G1734" s="1">
-        <v>41204</v>
+        <v>7140</v>
       </c>
       <c r="H1734" s="1">
         <v>0</v>
       </c>
       <c r="I1734" s="1">
-        <v>41204</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="1735" spans="1:9" ht="12.75">
@@ -51858,22 +51858,22 @@
         <v>105</v>
       </c>
       <c r="D1735" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E1735" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="F1735" s="1">
         <v>0</v>
       </c>
       <c r="G1735" s="1">
-        <v>77571</v>
+        <v>41204</v>
       </c>
       <c r="H1735" s="1">
         <v>0</v>
       </c>
       <c r="I1735" s="1">
-        <v>77571</v>
+        <v>41204</v>
       </c>
     </row>
     <row r="1736" spans="1:9" ht="12.75">
@@ -51890,19 +51890,19 @@
         <v>247</v>
       </c>
       <c r="E1736" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1736" s="1">
         <v>0</v>
       </c>
       <c r="G1736" s="1">
-        <v>1513824</v>
+        <v>77571</v>
       </c>
       <c r="H1736" s="1">
         <v>0</v>
       </c>
       <c r="I1736" s="1">
-        <v>1513824</v>
+        <v>77571</v>
       </c>
     </row>
     <row r="1737" spans="1:9" ht="12.75">
@@ -51919,19 +51919,19 @@
         <v>247</v>
       </c>
       <c r="E1737" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F1737" s="1">
         <v>0</v>
       </c>
       <c r="G1737" s="1">
-        <v>22538</v>
+        <v>1513824</v>
       </c>
       <c r="H1737" s="1">
         <v>0</v>
       </c>
       <c r="I1737" s="1">
-        <v>22538</v>
+        <v>1513824</v>
       </c>
     </row>
     <row r="1738" spans="1:9" ht="12.75">
@@ -51945,22 +51945,22 @@
         <v>105</v>
       </c>
       <c r="D1738" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E1738" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F1738" s="1">
         <v>0</v>
       </c>
       <c r="G1738" s="1">
-        <v>9676</v>
+        <v>22538</v>
       </c>
       <c r="H1738" s="1">
         <v>0</v>
       </c>
       <c r="I1738" s="1">
-        <v>9676</v>
+        <v>22538</v>
       </c>
     </row>
     <row r="1739" spans="1:9" ht="12.75">
@@ -51974,22 +51974,22 @@
         <v>105</v>
       </c>
       <c r="D1739" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E1739" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F1739" s="1">
         <v>0</v>
       </c>
       <c r="G1739" s="1">
-        <v>3353166</v>
+        <v>9676</v>
       </c>
       <c r="H1739" s="1">
         <v>0</v>
       </c>
       <c r="I1739" s="1">
-        <v>3353166</v>
+        <v>9676</v>
       </c>
     </row>
     <row r="1740" spans="1:9" ht="12.75">
@@ -52006,19 +52006,19 @@
         <v>250</v>
       </c>
       <c r="E1740" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1740" s="1">
         <v>0</v>
       </c>
       <c r="G1740" s="1">
-        <v>662779</v>
+        <v>3353166</v>
       </c>
       <c r="H1740" s="1">
         <v>0</v>
       </c>
       <c r="I1740" s="1">
-        <v>662779</v>
+        <v>3353166</v>
       </c>
     </row>
     <row r="1741" spans="1:9" ht="12.75">
@@ -52035,19 +52035,19 @@
         <v>250</v>
       </c>
       <c r="E1741" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1741" s="1">
         <v>0</v>
       </c>
       <c r="G1741" s="1">
-        <v>31417864</v>
+        <v>662779</v>
       </c>
       <c r="H1741" s="1">
         <v>0</v>
       </c>
       <c r="I1741" s="1">
-        <v>31417864</v>
+        <v>662779</v>
       </c>
     </row>
     <row r="1742" spans="1:9" ht="12.75">
@@ -52064,19 +52064,19 @@
         <v>250</v>
       </c>
       <c r="E1742" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1742" s="1">
         <v>0</v>
       </c>
       <c r="G1742" s="1">
-        <v>2664907</v>
+        <v>31417864</v>
       </c>
       <c r="H1742" s="1">
         <v>0</v>
       </c>
       <c r="I1742" s="1">
-        <v>2664907</v>
+        <v>31417864</v>
       </c>
     </row>
     <row r="1743" spans="1:9" ht="12.75">
@@ -52093,19 +52093,19 @@
         <v>250</v>
       </c>
       <c r="E1743" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1743" s="1">
         <v>0</v>
       </c>
       <c r="G1743" s="1">
-        <v>2021829</v>
+        <v>2664907</v>
       </c>
       <c r="H1743" s="1">
         <v>0</v>
       </c>
       <c r="I1743" s="1">
-        <v>2021829</v>
+        <v>2664907</v>
       </c>
     </row>
     <row r="1744" spans="1:9" ht="12.75">
@@ -52122,19 +52122,19 @@
         <v>250</v>
       </c>
       <c r="E1744" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1744" s="1">
         <v>0</v>
       </c>
       <c r="G1744" s="1">
-        <v>14946353</v>
+        <v>2021829</v>
       </c>
       <c r="H1744" s="1">
         <v>0</v>
       </c>
       <c r="I1744" s="1">
-        <v>14946353</v>
+        <v>2021829</v>
       </c>
     </row>
     <row r="1745" spans="1:9" ht="12.75">
@@ -52151,19 +52151,19 @@
         <v>250</v>
       </c>
       <c r="E1745" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1745" s="1">
         <v>0</v>
       </c>
       <c r="G1745" s="1">
-        <v>5986158</v>
+        <v>14946353</v>
       </c>
       <c r="H1745" s="1">
         <v>0</v>
       </c>
       <c r="I1745" s="1">
-        <v>5986158</v>
+        <v>14946353</v>
       </c>
     </row>
     <row r="1746" spans="1:9" ht="12.75">
@@ -52180,19 +52180,19 @@
         <v>250</v>
       </c>
       <c r="E1746" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F1746" s="1">
         <v>0</v>
       </c>
       <c r="G1746" s="1">
-        <v>30819</v>
+        <v>5986158</v>
       </c>
       <c r="H1746" s="1">
         <v>0</v>
       </c>
       <c r="I1746" s="1">
-        <v>30819</v>
+        <v>5986158</v>
       </c>
     </row>
     <row r="1747" spans="1:9" ht="12.75">
@@ -52209,19 +52209,19 @@
         <v>250</v>
       </c>
       <c r="E1747" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F1747" s="1">
         <v>0</v>
       </c>
       <c r="G1747" s="1">
-        <v>1516559</v>
+        <v>30819</v>
       </c>
       <c r="H1747" s="1">
         <v>0</v>
       </c>
       <c r="I1747" s="1">
-        <v>1516559</v>
+        <v>30819</v>
       </c>
     </row>
     <row r="1748" spans="1:9" ht="12.75">
@@ -52238,19 +52238,19 @@
         <v>250</v>
       </c>
       <c r="E1748" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F1748" s="1">
         <v>0</v>
       </c>
       <c r="G1748" s="1">
-        <v>3492740</v>
+        <v>1516559</v>
       </c>
       <c r="H1748" s="1">
         <v>0</v>
       </c>
       <c r="I1748" s="1">
-        <v>3492740</v>
+        <v>1516559</v>
       </c>
     </row>
     <row r="1749" spans="1:9" ht="12.75">
@@ -52267,19 +52267,19 @@
         <v>250</v>
       </c>
       <c r="E1749" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F1749" s="1">
         <v>0</v>
       </c>
       <c r="G1749" s="1">
-        <v>75917498</v>
+        <v>3492740</v>
       </c>
       <c r="H1749" s="1">
-        <v>75931161</v>
+        <v>0</v>
       </c>
       <c r="I1749" s="1">
-        <v>-13663</v>
+        <v>3492740</v>
       </c>
     </row>
     <row r="1750" spans="1:9" ht="12.75">
@@ -52296,19 +52296,19 @@
         <v>250</v>
       </c>
       <c r="E1750" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F1750" s="1">
         <v>0</v>
       </c>
       <c r="G1750" s="1">
-        <v>747484</v>
+        <v>75917498</v>
       </c>
       <c r="H1750" s="1">
-        <v>0</v>
+        <v>75931161</v>
       </c>
       <c r="I1750" s="1">
-        <v>747484</v>
+        <v>-13663</v>
       </c>
     </row>
     <row r="1751" spans="1:9" ht="12.75">
@@ -52325,19 +52325,19 @@
         <v>250</v>
       </c>
       <c r="E1751" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F1751" s="1">
         <v>0</v>
       </c>
       <c r="G1751" s="1">
-        <v>1826516</v>
+        <v>747484</v>
       </c>
       <c r="H1751" s="1">
         <v>0</v>
       </c>
       <c r="I1751" s="1">
-        <v>1826516</v>
+        <v>747484</v>
       </c>
     </row>
     <row r="1752" spans="1:9" ht="12.75">
@@ -52354,19 +52354,19 @@
         <v>250</v>
       </c>
       <c r="E1752" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F1752" s="1">
         <v>0</v>
       </c>
       <c r="G1752" s="1">
-        <v>9827272</v>
+        <v>1826516</v>
       </c>
       <c r="H1752" s="1">
         <v>0</v>
       </c>
       <c r="I1752" s="1">
-        <v>9827272</v>
+        <v>1826516</v>
       </c>
     </row>
     <row r="1753" spans="1:9" ht="12.75">
@@ -52380,22 +52380,22 @@
         <v>105</v>
       </c>
       <c r="D1753" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E1753" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="F1753" s="1">
         <v>0</v>
       </c>
       <c r="G1753" s="1">
-        <v>0</v>
+        <v>9827272</v>
       </c>
       <c r="H1753" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1753" s="1">
-        <v>-1</v>
+        <v>9827272</v>
       </c>
     </row>
     <row r="1754" spans="1:9" ht="12.75">
@@ -52409,22 +52409,22 @@
         <v>105</v>
       </c>
       <c r="D1754" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E1754" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="F1754" s="1">
         <v>0</v>
       </c>
       <c r="G1754" s="1">
-        <v>148184</v>
+        <v>0</v>
       </c>
       <c r="H1754" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I1754" s="1">
-        <v>148184</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="1755" spans="1:9" ht="12.75">
@@ -52441,19 +52441,19 @@
         <v>257</v>
       </c>
       <c r="E1755" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F1755" s="1">
         <v>0</v>
       </c>
       <c r="G1755" s="1">
-        <v>74092</v>
+        <v>148184</v>
       </c>
       <c r="H1755" s="1">
         <v>0</v>
       </c>
       <c r="I1755" s="1">
-        <v>74092</v>
+        <v>148184</v>
       </c>
     </row>
     <row r="1756" spans="1:9" ht="12.75">
@@ -52470,19 +52470,19 @@
         <v>257</v>
       </c>
       <c r="E1756" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1756" s="1">
         <v>0</v>
       </c>
       <c r="G1756" s="1">
-        <v>74092.80</v>
+        <v>74092</v>
       </c>
       <c r="H1756" s="1">
         <v>0</v>
       </c>
       <c r="I1756" s="1">
-        <v>74092.80</v>
+        <v>74092</v>
       </c>
     </row>
     <row r="1757" spans="1:9" ht="12.75">
@@ -52496,22 +52496,22 @@
         <v>105</v>
       </c>
       <c r="D1757" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E1757" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="F1757" s="1">
         <v>0</v>
       </c>
       <c r="G1757" s="1">
-        <v>137490</v>
+        <v>74092.80</v>
       </c>
       <c r="H1757" s="1">
         <v>0</v>
       </c>
       <c r="I1757" s="1">
-        <v>137490</v>
+        <v>74092.80</v>
       </c>
     </row>
     <row r="1758" spans="1:9" ht="12.75">
@@ -52528,19 +52528,19 @@
         <v>258</v>
       </c>
       <c r="E1758" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1758" s="1">
         <v>0</v>
       </c>
       <c r="G1758" s="1">
-        <v>305648</v>
+        <v>137490</v>
       </c>
       <c r="H1758" s="1">
         <v>0</v>
       </c>
       <c r="I1758" s="1">
-        <v>305648</v>
+        <v>137490</v>
       </c>
     </row>
     <row r="1759" spans="1:9" ht="12.75">
@@ -52557,19 +52557,19 @@
         <v>258</v>
       </c>
       <c r="E1759" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1759" s="1">
         <v>0</v>
       </c>
       <c r="G1759" s="1">
-        <v>484</v>
+        <v>305648</v>
       </c>
       <c r="H1759" s="1">
         <v>0</v>
       </c>
       <c r="I1759" s="1">
-        <v>484</v>
+        <v>305648</v>
       </c>
     </row>
     <row r="1760" spans="1:9" ht="12.75">
@@ -52583,22 +52583,22 @@
         <v>105</v>
       </c>
       <c r="D1760" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E1760" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="F1760" s="1">
         <v>0</v>
       </c>
       <c r="G1760" s="1">
-        <v>24000</v>
+        <v>484</v>
       </c>
       <c r="H1760" s="1">
         <v>0</v>
       </c>
       <c r="I1760" s="1">
-        <v>24000</v>
+        <v>484</v>
       </c>
     </row>
     <row r="1761" spans="1:9" ht="12.75">
@@ -52612,22 +52612,22 @@
         <v>105</v>
       </c>
       <c r="D1761" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E1761" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="F1761" s="1">
         <v>0</v>
       </c>
       <c r="G1761" s="1">
-        <v>1125720</v>
+        <v>24000</v>
       </c>
       <c r="H1761" s="1">
         <v>0</v>
       </c>
       <c r="I1761" s="1">
-        <v>1125720</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="1762" spans="1:9" ht="12.75">
@@ -52644,7 +52644,7 @@
         <v>263</v>
       </c>
       <c r="E1762" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="F1762" s="1">
         <v>0</v>
@@ -52664,28 +52664,28 @@
         <v>312</v>
       </c>
       <c r="B1763" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="C1763" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="D1763" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="E1763" t="s">
-        <v>13</v>
+        <v>338</v>
       </c>
       <c r="F1763" s="1">
         <v>0</v>
       </c>
       <c r="G1763" s="1">
-        <v>0</v>
+        <v>1125720</v>
       </c>
       <c r="H1763" s="1">
-        <v>7351276</v>
+        <v>0</v>
       </c>
       <c r="I1763" s="1">
-        <v>-7351276</v>
+        <v>1125720</v>
       </c>
     </row>
     <row r="1764" spans="1:9" ht="12.75">
@@ -52699,7 +52699,7 @@
         <v>264</v>
       </c>
       <c r="D1764" t="s">
-        <v>308</v>
+        <v>267</v>
       </c>
       <c r="E1764" t="s">
         <v>13</v>
@@ -52711,10 +52711,10 @@
         <v>0</v>
       </c>
       <c r="H1764" s="1">
-        <v>0</v>
+        <v>7351276</v>
       </c>
       <c r="I1764" s="1">
-        <v>0</v>
+        <v>-7351276</v>
       </c>
     </row>
     <row r="1765" spans="1:9" ht="12.75">
@@ -52722,28 +52722,28 @@
         <v>312</v>
       </c>
       <c r="B1765" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C1765" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D1765" t="s">
-        <v>269</v>
+        <v>308</v>
       </c>
       <c r="E1765" t="s">
         <v>13</v>
       </c>
       <c r="F1765" s="1">
-        <v>-5418882</v>
+        <v>0</v>
       </c>
       <c r="G1765" s="1">
-        <v>2.3231524567000002E8</v>
+        <v>0</v>
       </c>
       <c r="H1765" s="1">
-        <v>2.6244316570000005E8</v>
+        <v>0</v>
       </c>
       <c r="I1765" s="1">
-        <v>-3.554680203000003E7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1766" spans="1:9" ht="12.75">
@@ -52754,25 +52754,25 @@
         <v>268</v>
       </c>
       <c r="C1766" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D1766" t="s">
-        <v>356</v>
+        <v>269</v>
       </c>
       <c r="E1766" t="s">
         <v>13</v>
       </c>
       <c r="F1766" s="1">
-        <v>0</v>
+        <v>-5418882</v>
       </c>
       <c r="G1766" s="1">
-        <v>2274999</v>
+        <v>2.3231524567E8</v>
       </c>
       <c r="H1766" s="1">
-        <v>5013786</v>
+        <v>2.6256870870000005E8</v>
       </c>
       <c r="I1766" s="1">
-        <v>-2738787</v>
+        <v>-3.567234503000006E7</v>
       </c>
     </row>
     <row r="1767" spans="1:9" ht="12.75">
@@ -52786,22 +52786,22 @@
         <v>273</v>
       </c>
       <c r="D1767" t="s">
-        <v>278</v>
+        <v>356</v>
       </c>
       <c r="E1767" t="s">
         <v>13</v>
       </c>
       <c r="F1767" s="1">
-        <v>-22030149</v>
+        <v>0</v>
       </c>
       <c r="G1767" s="1">
-        <v>0</v>
+        <v>2274999</v>
       </c>
       <c r="H1767" s="1">
-        <v>9.094276758399999E8</v>
+        <v>5013786</v>
       </c>
       <c r="I1767" s="1">
-        <v>-9.314578248399999E8</v>
+        <v>-2738787</v>
       </c>
     </row>
     <row r="1768" spans="1:9" ht="12.75">
@@ -52815,22 +52815,22 @@
         <v>273</v>
       </c>
       <c r="D1768" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E1768" t="s">
         <v>13</v>
       </c>
       <c r="F1768" s="1">
-        <v>-14989</v>
+        <v>-22030149</v>
       </c>
       <c r="G1768" s="1">
-        <v>5380456</v>
+        <v>0</v>
       </c>
       <c r="H1768" s="1">
-        <v>10165830</v>
+        <v>9.094276758399999E8</v>
       </c>
       <c r="I1768" s="1">
-        <v>-4800363</v>
+        <v>-9.314578248399999E8</v>
       </c>
     </row>
     <row r="1769" spans="1:9" ht="12.75">
@@ -52844,22 +52844,22 @@
         <v>273</v>
       </c>
       <c r="D1769" t="s">
-        <v>357</v>
+        <v>282</v>
       </c>
       <c r="E1769" t="s">
         <v>13</v>
       </c>
       <c r="F1769" s="1">
-        <v>0</v>
+        <v>-14989</v>
       </c>
       <c r="G1769" s="1">
-        <v>2659661</v>
+        <v>5380456</v>
       </c>
       <c r="H1769" s="1">
-        <v>2659660</v>
+        <v>10165830</v>
       </c>
       <c r="I1769" s="1">
-        <v>1</v>
+        <v>-4800363</v>
       </c>
     </row>
     <row r="1770" spans="1:9" ht="12.75">
@@ -52873,7 +52873,7 @@
         <v>273</v>
       </c>
       <c r="D1770" t="s">
-        <v>286</v>
+        <v>357</v>
       </c>
       <c r="E1770" t="s">
         <v>13</v>
@@ -52882,13 +52882,13 @@
         <v>0</v>
       </c>
       <c r="G1770" s="1">
-        <v>0</v>
+        <v>2659661</v>
       </c>
       <c r="H1770" s="1">
-        <v>190424</v>
+        <v>2659660</v>
       </c>
       <c r="I1770" s="1">
-        <v>-190424</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1771" spans="1:9" ht="12.75">
@@ -52902,7 +52902,7 @@
         <v>273</v>
       </c>
       <c r="D1771" t="s">
-        <v>358</v>
+        <v>286</v>
       </c>
       <c r="E1771" t="s">
         <v>13</v>
@@ -52911,13 +52911,13 @@
         <v>0</v>
       </c>
       <c r="G1771" s="1">
-        <v>1966914</v>
+        <v>0</v>
       </c>
       <c r="H1771" s="1">
-        <v>1995881</v>
+        <v>190424</v>
       </c>
       <c r="I1771" s="1">
-        <v>-28967</v>
+        <v>-190424</v>
       </c>
     </row>
     <row r="1772" spans="1:9" ht="12.75">
@@ -52931,7 +52931,7 @@
         <v>273</v>
       </c>
       <c r="D1772" t="s">
-        <v>287</v>
+        <v>358</v>
       </c>
       <c r="E1772" t="s">
         <v>13</v>
@@ -52940,13 +52940,13 @@
         <v>0</v>
       </c>
       <c r="G1772" s="1">
-        <v>46090</v>
+        <v>1966914</v>
       </c>
       <c r="H1772" s="1">
-        <v>70730</v>
+        <v>1995881</v>
       </c>
       <c r="I1772" s="1">
-        <v>-24640</v>
+        <v>-28967</v>
       </c>
     </row>
     <row r="1773" spans="1:9" ht="12.75">
@@ -52960,7 +52960,7 @@
         <v>273</v>
       </c>
       <c r="D1773" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E1773" t="s">
         <v>13</v>
@@ -52969,13 +52969,13 @@
         <v>0</v>
       </c>
       <c r="G1773" s="1">
-        <v>840</v>
+        <v>46090</v>
       </c>
       <c r="H1773" s="1">
-        <v>416</v>
+        <v>70730</v>
       </c>
       <c r="I1773" s="1">
-        <v>424</v>
+        <v>-24640</v>
       </c>
     </row>
     <row r="1774" spans="1:9" ht="12.75">
@@ -52989,7 +52989,7 @@
         <v>273</v>
       </c>
       <c r="D1774" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E1774" t="s">
         <v>13</v>
@@ -52998,13 +52998,13 @@
         <v>0</v>
       </c>
       <c r="G1774" s="1">
-        <v>4.65382019E7</v>
+        <v>840</v>
       </c>
       <c r="H1774" s="1">
-        <v>58379674</v>
+        <v>416</v>
       </c>
       <c r="I1774" s="1">
-        <v>-1.1841472100000001E7</v>
+        <v>424</v>
       </c>
     </row>
     <row r="1775" spans="1:9" ht="12.75">
@@ -53018,7 +53018,7 @@
         <v>273</v>
       </c>
       <c r="D1775" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E1775" t="s">
         <v>13</v>
@@ -53027,13 +53027,13 @@
         <v>0</v>
       </c>
       <c r="G1775" s="1">
-        <v>37299</v>
+        <v>4.65382019E7</v>
       </c>
       <c r="H1775" s="1">
-        <v>185786.20</v>
+        <v>58379674</v>
       </c>
       <c r="I1775" s="1">
-        <v>-148487.20</v>
+        <v>-1.1841472100000001E7</v>
       </c>
     </row>
     <row r="1776" spans="1:9" ht="12.75">
@@ -53047,7 +53047,7 @@
         <v>273</v>
       </c>
       <c r="D1776" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E1776" t="s">
         <v>13</v>
@@ -53056,13 +53056,13 @@
         <v>0</v>
       </c>
       <c r="G1776" s="1">
-        <v>90747</v>
+        <v>37299</v>
       </c>
       <c r="H1776" s="1">
-        <v>498838.90</v>
+        <v>185786.20</v>
       </c>
       <c r="I1776" s="1">
-        <v>-408091.90</v>
+        <v>-148487.20</v>
       </c>
     </row>
     <row r="1777" spans="1:9" ht="12.75">
@@ -53076,7 +53076,7 @@
         <v>273</v>
       </c>
       <c r="D1777" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E1777" t="s">
         <v>13</v>
@@ -53085,13 +53085,13 @@
         <v>0</v>
       </c>
       <c r="G1777" s="1">
-        <v>4109064</v>
+        <v>90747</v>
       </c>
       <c r="H1777" s="1">
-        <v>1.186267109E7</v>
+        <v>498838.90</v>
       </c>
       <c r="I1777" s="1">
-        <v>-7753607.09</v>
+        <v>-408091.90</v>
       </c>
     </row>
     <row r="1778" spans="1:9" ht="12.75">
@@ -53105,7 +53105,7 @@
         <v>273</v>
       </c>
       <c r="D1778" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E1778" t="s">
         <v>13</v>
@@ -53114,13 +53114,13 @@
         <v>0</v>
       </c>
       <c r="G1778" s="1">
-        <v>1758542.24</v>
+        <v>4109064</v>
       </c>
       <c r="H1778" s="1">
-        <v>1153027.74</v>
+        <v>1.186267109E7</v>
       </c>
       <c r="I1778" s="1">
-        <v>605514.50</v>
+        <v>-7753607.09</v>
       </c>
     </row>
     <row r="1779" spans="1:9" ht="12.75">
@@ -53134,7 +53134,7 @@
         <v>273</v>
       </c>
       <c r="D1779" t="s">
-        <v>359</v>
+        <v>294</v>
       </c>
       <c r="E1779" t="s">
         <v>13</v>
@@ -53143,13 +53143,13 @@
         <v>0</v>
       </c>
       <c r="G1779" s="1">
-        <v>8601440</v>
+        <v>1758542.24</v>
       </c>
       <c r="H1779" s="1">
-        <v>18873669</v>
+        <v>1153027.74</v>
       </c>
       <c r="I1779" s="1">
-        <v>-10272229</v>
+        <v>605514.50</v>
       </c>
     </row>
     <row r="1780" spans="1:9" ht="12.75">
@@ -53160,10 +53160,10 @@
         <v>268</v>
       </c>
       <c r="C1780" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="D1780" t="s">
-        <v>297</v>
+        <v>359</v>
       </c>
       <c r="E1780" t="s">
         <v>13</v>
@@ -53172,13 +53172,13 @@
         <v>0</v>
       </c>
       <c r="G1780" s="1">
-        <v>2.2509215249E8</v>
+        <v>8601440</v>
       </c>
       <c r="H1780" s="1">
-        <v>2.2509215249000007E8</v>
+        <v>18873669</v>
       </c>
       <c r="I1780" s="1">
-        <v>-5.9604644775390625E-8</v>
+        <v>-10272229</v>
       </c>
     </row>
     <row r="1781" spans="1:9" ht="12.75">
@@ -53192,7 +53192,7 @@
         <v>296</v>
       </c>
       <c r="D1781" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E1781" t="s">
         <v>13</v>
@@ -53201,42 +53201,71 @@
         <v>0</v>
       </c>
       <c r="G1781" s="1">
-        <v>0</v>
+        <v>2.2509215249E8</v>
       </c>
       <c r="H1781" s="1">
-        <v>8826219.66</v>
+        <v>2.2509215249000007E8</v>
       </c>
       <c r="I1781" s="1">
-        <v>-8826219.66</v>
+        <v>-5.9604644775390625E-8</v>
       </c>
     </row>
     <row r="1782" spans="1:9" ht="12.75">
       <c r="A1782" t="s">
+        <v>312</v>
+      </c>
+      <c r="B1782" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1782" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1782" t="s">
+        <v>298</v>
+      </c>
+      <c r="E1782" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1782" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1782" s="1">
+        <v>0</v>
+      </c>
+      <c r="H1782" s="1">
+        <v>8826219.66</v>
+      </c>
+      <c r="I1782" s="1">
+        <v>-8826219.66</v>
+      </c>
+    </row>
+    <row r="1783" spans="1:9" ht="12.75">
+      <c r="A1783" t="s">
         <v>360</v>
       </c>
-      <c r="B1782" t="s">
+      <c r="B1783" t="s">
         <v>361</v>
       </c>
-      <c r="C1782" t="s">
+      <c r="C1783" t="s">
         <v>361</v>
       </c>
-      <c r="D1782" t="s">
+      <c r="D1783" t="s">
         <v>361</v>
       </c>
-      <c r="E1782" t="s">
+      <c r="E1783" t="s">
         <v>361</v>
       </c>
-      <c r="F1782" s="1">
-        <v>-1.9371509552001953E-7</v>
-      </c>
-      <c r="G1782" s="1">
-        <v>6.972294193029999E9</v>
-      </c>
-      <c r="H1782" s="1">
-        <v>6.972294193029999E9</v>
-      </c>
-      <c r="I1782" s="1">
-        <v>-4.880130290985107E-7</v>
+      <c r="F1783" s="1">
+        <v>5.9604644775390625E-8</v>
+      </c>
+      <c r="G1783" s="1">
+        <v>6.972631711029999E9</v>
+      </c>
+      <c r="H1783" s="1">
+        <v>6.972631711030001E9</v>
+      </c>
+      <c r="I1783" s="1">
+        <v>-1.560896635055542E-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-03-20
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8983" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8988" uniqueCount="362">
   <si>
     <t>Book</t>
   </si>
@@ -1079,6 +1079,9 @@
     <t>AIP-0120-Training Infra and MEL-Waymo-NFC</t>
   </si>
   <si>
+    <t>AIP-0109-Education Innovation-Google Cloud</t>
+  </si>
+  <si>
     <t>AIP-0103-Administration-RFR-NFC</t>
   </si>
   <si>
@@ -1544,8 +1547,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{f20bd0e4-3176-41c4-a8bb-f3bc73c0b63e}">
-  <dimension ref="A1:I1795"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62080ec0-bdc4-4af0-b553-5e86381d06af}">
+  <dimension ref="A1:I1796"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="14.142857142857142" customWidth="1"/>
@@ -1633,7 +1636,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>0</v>
+        <v>-2.9802322387695312E-8</v>
       </c>
       <c r="G3" s="1">
         <v>3.54</v>
@@ -1642,7 +1645,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>4.440892098500626E-16</v>
+        <v>-2.9802321943606103E-8</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -1668,10 +1671,10 @@
         <v>3.9882729998E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.447998005400002E8</v>
+        <v>3.447998005400005E8</v>
       </c>
       <c r="I4" s="1">
-        <v>1.8593025130999982E8</v>
+        <v>1.8593025130999953E8</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -3814,10 +3817,10 @@
         <v>4.406711083E7</v>
       </c>
       <c r="H78" s="1">
-        <v>4.32673492E7</v>
+        <v>4.346434919999997E7</v>
       </c>
       <c r="I78" s="1">
-        <v>1718467.6299999952</v>
+        <v>1521467.630000025</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="12.75">
@@ -3895,7 +3898,7 @@
         <v>13</v>
       </c>
       <c r="F81" s="1">
-        <v>-9.313225746154785E-10</v>
+        <v>0</v>
       </c>
       <c r="G81" s="1">
         <v>333614</v>
@@ -3904,7 +3907,7 @@
         <v>333614</v>
       </c>
       <c r="I81" s="1">
-        <v>-9.313225746154785E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:9" ht="12.75">
@@ -6972,13 +6975,13 @@
         <v>0</v>
       </c>
       <c r="G187" s="1">
-        <v>379</v>
+        <v>86047</v>
       </c>
       <c r="H187" s="1">
         <v>0</v>
       </c>
       <c r="I187" s="1">
-        <v>379</v>
+        <v>86047</v>
       </c>
     </row>
     <row r="188" spans="1:9" ht="12.75">
@@ -12279,13 +12282,13 @@
         <v>0</v>
       </c>
       <c r="G370" s="1">
-        <v>259000</v>
+        <v>660200</v>
       </c>
       <c r="H370" s="1">
         <v>0</v>
       </c>
       <c r="I370" s="1">
-        <v>259000</v>
+        <v>660200</v>
       </c>
     </row>
     <row r="371" spans="1:9" ht="12.75">
@@ -14019,13 +14022,13 @@
         <v>0</v>
       </c>
       <c r="G430" s="1">
-        <v>56936</v>
+        <v>57547</v>
       </c>
       <c r="H430" s="1">
         <v>0</v>
       </c>
       <c r="I430" s="1">
-        <v>56936</v>
+        <v>57547</v>
       </c>
     </row>
     <row r="431" spans="1:9" ht="12.75">
@@ -15034,13 +15037,13 @@
         <v>0</v>
       </c>
       <c r="G465" s="1">
-        <v>1868821.50</v>
+        <v>1870416.50</v>
       </c>
       <c r="H465" s="1">
         <v>9923</v>
       </c>
       <c r="I465" s="1">
-        <v>1858898.50</v>
+        <v>1860493.50</v>
       </c>
     </row>
     <row r="466" spans="1:9" ht="12.75">
@@ -15411,13 +15414,13 @@
         <v>0</v>
       </c>
       <c r="G478" s="1">
-        <v>81248</v>
+        <v>82168</v>
       </c>
       <c r="H478" s="1">
         <v>0</v>
       </c>
       <c r="I478" s="1">
-        <v>81248</v>
+        <v>82168</v>
       </c>
     </row>
     <row r="479" spans="1:9" ht="12.75">
@@ -15469,13 +15472,13 @@
         <v>0</v>
       </c>
       <c r="G480" s="1">
-        <v>350989</v>
+        <v>352761</v>
       </c>
       <c r="H480" s="1">
         <v>0</v>
       </c>
       <c r="I480" s="1">
-        <v>350989</v>
+        <v>352761</v>
       </c>
     </row>
     <row r="481" spans="1:9" ht="12.75">
@@ -19616,13 +19619,13 @@
         <v>0</v>
       </c>
       <c r="G623" s="1">
-        <v>3046869.4000000004</v>
+        <v>3046869.40</v>
       </c>
       <c r="H623" s="1">
         <v>9049.23</v>
       </c>
       <c r="I623" s="1">
-        <v>3037820.1700000004</v>
+        <v>3037820.17</v>
       </c>
     </row>
     <row r="624" spans="1:9" ht="12.75">
@@ -20051,13 +20054,13 @@
         <v>0</v>
       </c>
       <c r="G638" s="1">
-        <v>617359.95</v>
+        <v>617359.9500000001</v>
       </c>
       <c r="H638" s="1">
         <v>0</v>
       </c>
       <c r="I638" s="1">
-        <v>617359.95</v>
+        <v>617359.9500000001</v>
       </c>
     </row>
     <row r="639" spans="1:9" ht="12.75">
@@ -20109,13 +20112,13 @@
         <v>0</v>
       </c>
       <c r="G640" s="1">
-        <v>1595365.71</v>
+        <v>1595365.7100000002</v>
       </c>
       <c r="H640" s="1">
         <v>9049.23</v>
       </c>
       <c r="I640" s="1">
-        <v>1586316.48</v>
+        <v>1586316.4800000002</v>
       </c>
     </row>
     <row r="641" spans="1:9" ht="12.75">
@@ -20167,13 +20170,13 @@
         <v>0</v>
       </c>
       <c r="G642" s="1">
-        <v>516927</v>
+        <v>516927.00000000006</v>
       </c>
       <c r="H642" s="1">
         <v>0</v>
       </c>
       <c r="I642" s="1">
-        <v>516927</v>
+        <v>516927.00000000006</v>
       </c>
     </row>
     <row r="643" spans="1:9" ht="12.75">
@@ -20341,13 +20344,13 @@
         <v>0</v>
       </c>
       <c r="G648" s="1">
-        <v>1824764.4800000004</v>
+        <v>1824764.48</v>
       </c>
       <c r="H648" s="1">
         <v>13850.19</v>
       </c>
       <c r="I648" s="1">
-        <v>1810914.2900000005</v>
+        <v>1810914.29</v>
       </c>
     </row>
     <row r="649" spans="1:9" ht="12.75">
@@ -36088,13 +36091,13 @@
         <v>0</v>
       </c>
       <c r="G1191" s="1">
-        <v>44250</v>
+        <v>177000</v>
       </c>
       <c r="H1191" s="1">
         <v>0</v>
       </c>
       <c r="I1191" s="1">
-        <v>44250</v>
+        <v>177000</v>
       </c>
     </row>
     <row r="1192" spans="1:9" ht="12.75">
@@ -44814,16 +44817,16 @@
         <v>13</v>
       </c>
       <c r="F1492" s="1">
-        <v>-1.934719699999988E7</v>
+        <v>-1.934719699999994E7</v>
       </c>
       <c r="G1492" s="1">
-        <v>2.1142017229999983E8</v>
+        <v>2.1161717229999986E8</v>
       </c>
       <c r="H1492" s="1">
-        <v>1.985679182999999E8</v>
+        <v>1.9916543229999998E8</v>
       </c>
       <c r="I1492" s="1">
-        <v>-6494942.99999994</v>
+        <v>-6895457.00000006</v>
       </c>
     </row>
     <row r="1493" spans="1:9" ht="12.75">
@@ -45400,10 +45403,10 @@
         <v>556908.05</v>
       </c>
       <c r="H1512" s="1">
-        <v>587081.4800000001</v>
+        <v>588533.4800000001</v>
       </c>
       <c r="I1512" s="1">
-        <v>-30173.43000000005</v>
+        <v>-31625.43000000005</v>
       </c>
     </row>
     <row r="1513" spans="1:9" ht="12.75">
@@ -45458,10 +45461,10 @@
         <v>7533462.2</v>
       </c>
       <c r="H1514" s="1">
-        <v>8520187.919999998</v>
+        <v>8545737.919999998</v>
       </c>
       <c r="I1514" s="1">
-        <v>-986725.7199999979</v>
+        <v>-1012275.7199999979</v>
       </c>
     </row>
     <row r="1515" spans="1:9" ht="12.75">
@@ -45481,7 +45484,7 @@
         <v>13</v>
       </c>
       <c r="F1515" s="1">
-        <v>-56797.000000002794</v>
+        <v>-56797.000000003725</v>
       </c>
       <c r="G1515" s="1">
         <v>3227421.94</v>
@@ -45490,7 +45493,7 @@
         <v>3631156.939999996</v>
       </c>
       <c r="I1515" s="1">
-        <v>-460531.99999999907</v>
+        <v>-460532</v>
       </c>
     </row>
     <row r="1516" spans="1:9" ht="12.75">
@@ -45545,10 +45548,10 @@
         <v>1.1068387002800002E9</v>
       </c>
       <c r="H1517" s="1">
-        <v>1.1068387002800007E9</v>
+        <v>1.1068387002800004E9</v>
       </c>
       <c r="I1517" s="1">
-        <v>-4.76837158203125E-7</v>
+        <v>-2.384185791015625E-7</v>
       </c>
     </row>
     <row r="1518" spans="1:9" ht="12.75">
@@ -46441,13 +46444,13 @@
         <v>2.91937089E7</v>
       </c>
       <c r="G1548" s="1">
-        <v>6.486054004000001E7</v>
+        <v>6.515914804E7</v>
       </c>
       <c r="H1548" s="1">
-        <v>6.4471495279999994E7</v>
+        <v>6.724710968E7</v>
       </c>
       <c r="I1548" s="1">
-        <v>2.9582753660000004E7</v>
+        <v>2.710574725999999E7</v>
       </c>
     </row>
     <row r="1549" spans="1:9" ht="12.75">
@@ -46473,10 +46476,10 @@
         <v>0</v>
       </c>
       <c r="H1549" s="1">
-        <v>1969504</v>
+        <v>0</v>
       </c>
       <c r="I1549" s="1">
-        <v>-1969492</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1550" spans="1:9" ht="12.75">
@@ -46531,10 +46534,10 @@
         <v>8.56587629E8</v>
       </c>
       <c r="H1551" s="1">
-        <v>3.6511678777E8</v>
+        <v>3.856976476E8</v>
       </c>
       <c r="I1551" s="1">
-        <v>4.9147084123E8</v>
+        <v>4.708899814E8</v>
       </c>
     </row>
     <row r="1552" spans="1:9" ht="12.75">
@@ -46905,13 +46908,13 @@
         <v>0</v>
       </c>
       <c r="G1564" s="1">
-        <v>2515388</v>
+        <v>2539794</v>
       </c>
       <c r="H1564" s="1">
         <v>2844459</v>
       </c>
       <c r="I1564" s="1">
-        <v>-329071</v>
+        <v>-304665</v>
       </c>
     </row>
     <row r="1565" spans="1:9" ht="12.75">
@@ -48413,13 +48416,13 @@
         <v>0</v>
       </c>
       <c r="G1616" s="1">
-        <v>307964.57</v>
+        <v>307964.56999999995</v>
       </c>
       <c r="H1616" s="1">
         <v>0</v>
       </c>
       <c r="I1616" s="1">
-        <v>307964.57</v>
+        <v>307964.56999999995</v>
       </c>
     </row>
     <row r="1617" spans="1:9" ht="12.75">
@@ -49370,13 +49373,13 @@
         <v>0</v>
       </c>
       <c r="G1649" s="1">
-        <v>2619977.68</v>
+        <v>2619977.6799999997</v>
       </c>
       <c r="H1649" s="1">
         <v>0</v>
       </c>
       <c r="I1649" s="1">
-        <v>2619977.68</v>
+        <v>2619977.6799999997</v>
       </c>
     </row>
     <row r="1650" spans="1:9" ht="12.75">
@@ -49399,13 +49402,13 @@
         <v>0</v>
       </c>
       <c r="G1650" s="1">
-        <v>2559591.92</v>
+        <v>2585749.92</v>
       </c>
       <c r="H1650" s="1">
         <v>0</v>
       </c>
       <c r="I1650" s="1">
-        <v>2559591.92</v>
+        <v>2585749.92</v>
       </c>
     </row>
     <row r="1651" spans="1:9" ht="12.75">
@@ -49428,13 +49431,13 @@
         <v>0</v>
       </c>
       <c r="G1651" s="1">
-        <v>619120</v>
+        <v>652186</v>
       </c>
       <c r="H1651" s="1">
         <v>0</v>
       </c>
       <c r="I1651" s="1">
-        <v>619120</v>
+        <v>652186</v>
       </c>
     </row>
     <row r="1652" spans="1:9" ht="12.75">
@@ -49631,13 +49634,13 @@
         <v>0</v>
       </c>
       <c r="G1658" s="1">
-        <v>15618</v>
+        <v>18528</v>
       </c>
       <c r="H1658" s="1">
         <v>0</v>
       </c>
       <c r="I1658" s="1">
-        <v>15618</v>
+        <v>18528</v>
       </c>
     </row>
     <row r="1659" spans="1:9" ht="12.75">
@@ -49660,13 +49663,13 @@
         <v>0</v>
       </c>
       <c r="G1659" s="1">
-        <v>1163610</v>
+        <v>1164147</v>
       </c>
       <c r="H1659" s="1">
         <v>0</v>
       </c>
       <c r="I1659" s="1">
-        <v>1163610</v>
+        <v>1164147</v>
       </c>
     </row>
     <row r="1660" spans="1:9" ht="12.75">
@@ -50066,13 +50069,13 @@
         <v>0</v>
       </c>
       <c r="G1673" s="1">
-        <v>3734639.2299999995</v>
+        <v>3734639.2300000004</v>
       </c>
       <c r="H1673" s="1">
         <v>0</v>
       </c>
       <c r="I1673" s="1">
-        <v>3734639.2299999995</v>
+        <v>3734639.2300000004</v>
       </c>
     </row>
     <row r="1674" spans="1:9" ht="12.75">
@@ -50124,13 +50127,13 @@
         <v>0</v>
       </c>
       <c r="G1675" s="1">
-        <v>218609.22</v>
+        <v>218609.21999999997</v>
       </c>
       <c r="H1675" s="1">
         <v>0</v>
       </c>
       <c r="I1675" s="1">
-        <v>218609.22</v>
+        <v>218609.21999999997</v>
       </c>
     </row>
     <row r="1676" spans="1:9" ht="12.75">
@@ -50153,13 +50156,13 @@
         <v>0</v>
       </c>
       <c r="G1676" s="1">
-        <v>1910663.0799999996</v>
+        <v>1910663.08</v>
       </c>
       <c r="H1676" s="1">
         <v>0</v>
       </c>
       <c r="I1676" s="1">
-        <v>1910663.0799999996</v>
+        <v>1910663.08</v>
       </c>
     </row>
     <row r="1677" spans="1:9" ht="12.75">
@@ -50182,13 +50185,13 @@
         <v>0</v>
       </c>
       <c r="G1677" s="1">
-        <v>685737.6099999999</v>
+        <v>685737.61</v>
       </c>
       <c r="H1677" s="1">
         <v>0</v>
       </c>
       <c r="I1677" s="1">
-        <v>685737.6099999999</v>
+        <v>685737.61</v>
       </c>
     </row>
     <row r="1678" spans="1:9" ht="12.75">
@@ -50269,13 +50272,13 @@
         <v>0</v>
       </c>
       <c r="G1680" s="1">
-        <v>381348.31999999995</v>
+        <v>381348.32</v>
       </c>
       <c r="H1680" s="1">
         <v>0</v>
       </c>
       <c r="I1680" s="1">
-        <v>381348.31999999995</v>
+        <v>381348.32</v>
       </c>
     </row>
     <row r="1681" spans="1:9" ht="12.75">
@@ -52003,19 +52006,19 @@
         <v>243</v>
       </c>
       <c r="E1740" t="s">
-        <v>337</v>
+        <v>354</v>
       </c>
       <c r="F1740" s="1">
         <v>0</v>
       </c>
       <c r="G1740" s="1">
-        <v>10030000</v>
+        <v>6372000</v>
       </c>
       <c r="H1740" s="1">
         <v>0</v>
       </c>
       <c r="I1740" s="1">
-        <v>10030000</v>
+        <v>6372000</v>
       </c>
     </row>
     <row r="1741" spans="1:9" ht="12.75">
@@ -52032,19 +52035,19 @@
         <v>243</v>
       </c>
       <c r="E1741" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="F1741" s="1">
         <v>0</v>
       </c>
       <c r="G1741" s="1">
-        <v>41158322</v>
+        <v>12266100</v>
       </c>
       <c r="H1741" s="1">
         <v>0</v>
       </c>
       <c r="I1741" s="1">
-        <v>41158322</v>
+        <v>12266100</v>
       </c>
     </row>
     <row r="1742" spans="1:9" ht="12.75">
@@ -52061,19 +52064,19 @@
         <v>243</v>
       </c>
       <c r="E1742" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="F1742" s="1">
         <v>0</v>
       </c>
       <c r="G1742" s="1">
-        <v>1194533</v>
+        <v>41158322</v>
       </c>
       <c r="H1742" s="1">
         <v>0</v>
       </c>
       <c r="I1742" s="1">
-        <v>1194533</v>
+        <v>41158322</v>
       </c>
     </row>
     <row r="1743" spans="1:9" ht="12.75">
@@ -52087,22 +52090,22 @@
         <v>105</v>
       </c>
       <c r="D1743" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1743" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="F1743" s="1">
         <v>0</v>
       </c>
       <c r="G1743" s="1">
-        <v>31481</v>
+        <v>1194533</v>
       </c>
       <c r="H1743" s="1">
         <v>0</v>
       </c>
       <c r="I1743" s="1">
-        <v>31481</v>
+        <v>1194533</v>
       </c>
     </row>
     <row r="1744" spans="1:9" ht="12.75">
@@ -52119,19 +52122,19 @@
         <v>246</v>
       </c>
       <c r="E1744" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1744" s="1">
         <v>0</v>
       </c>
       <c r="G1744" s="1">
-        <v>6638</v>
+        <v>31481</v>
       </c>
       <c r="H1744" s="1">
         <v>0</v>
       </c>
       <c r="I1744" s="1">
-        <v>6638</v>
+        <v>31481</v>
       </c>
     </row>
     <row r="1745" spans="1:9" ht="12.75">
@@ -52148,19 +52151,19 @@
         <v>246</v>
       </c>
       <c r="E1745" t="s">
-        <v>354</v>
+        <v>331</v>
       </c>
       <c r="F1745" s="1">
         <v>0</v>
       </c>
       <c r="G1745" s="1">
-        <v>7140</v>
+        <v>6638</v>
       </c>
       <c r="H1745" s="1">
         <v>0</v>
       </c>
       <c r="I1745" s="1">
-        <v>7140</v>
+        <v>6638</v>
       </c>
     </row>
     <row r="1746" spans="1:9" ht="12.75">
@@ -52177,19 +52180,19 @@
         <v>246</v>
       </c>
       <c r="E1746" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="F1746" s="1">
         <v>0</v>
       </c>
       <c r="G1746" s="1">
-        <v>41204</v>
+        <v>7140</v>
       </c>
       <c r="H1746" s="1">
         <v>0</v>
       </c>
       <c r="I1746" s="1">
-        <v>41204</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="1747" spans="1:9" ht="12.75">
@@ -52203,22 +52206,22 @@
         <v>105</v>
       </c>
       <c r="D1747" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E1747" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="F1747" s="1">
         <v>0</v>
       </c>
       <c r="G1747" s="1">
-        <v>77571</v>
+        <v>41204</v>
       </c>
       <c r="H1747" s="1">
         <v>0</v>
       </c>
       <c r="I1747" s="1">
-        <v>77571</v>
+        <v>41204</v>
       </c>
     </row>
     <row r="1748" spans="1:9" ht="12.75">
@@ -52235,19 +52238,19 @@
         <v>247</v>
       </c>
       <c r="E1748" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F1748" s="1">
         <v>0</v>
       </c>
       <c r="G1748" s="1">
-        <v>1513824</v>
+        <v>77571</v>
       </c>
       <c r="H1748" s="1">
         <v>0</v>
       </c>
       <c r="I1748" s="1">
-        <v>1513824</v>
+        <v>77571</v>
       </c>
     </row>
     <row r="1749" spans="1:9" ht="12.75">
@@ -52264,19 +52267,19 @@
         <v>247</v>
       </c>
       <c r="E1749" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1749" s="1">
         <v>0</v>
       </c>
       <c r="G1749" s="1">
-        <v>22538</v>
+        <v>1513824</v>
       </c>
       <c r="H1749" s="1">
         <v>0</v>
       </c>
       <c r="I1749" s="1">
-        <v>22538</v>
+        <v>1513824</v>
       </c>
     </row>
     <row r="1750" spans="1:9" ht="12.75">
@@ -52290,22 +52293,22 @@
         <v>105</v>
       </c>
       <c r="D1750" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E1750" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F1750" s="1">
         <v>0</v>
       </c>
       <c r="G1750" s="1">
-        <v>9676</v>
+        <v>22538</v>
       </c>
       <c r="H1750" s="1">
         <v>0</v>
       </c>
       <c r="I1750" s="1">
-        <v>9676</v>
+        <v>22538</v>
       </c>
     </row>
     <row r="1751" spans="1:9" ht="12.75">
@@ -52319,22 +52322,22 @@
         <v>105</v>
       </c>
       <c r="D1751" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E1751" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F1751" s="1">
         <v>0</v>
       </c>
       <c r="G1751" s="1">
-        <v>3353166</v>
+        <v>9676</v>
       </c>
       <c r="H1751" s="1">
         <v>0</v>
       </c>
       <c r="I1751" s="1">
-        <v>3353166</v>
+        <v>9676</v>
       </c>
     </row>
     <row r="1752" spans="1:9" ht="12.75">
@@ -52351,19 +52354,19 @@
         <v>250</v>
       </c>
       <c r="E1752" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F1752" s="1">
         <v>0</v>
       </c>
       <c r="G1752" s="1">
-        <v>662779</v>
+        <v>3353166</v>
       </c>
       <c r="H1752" s="1">
         <v>0</v>
       </c>
       <c r="I1752" s="1">
-        <v>662779</v>
+        <v>3353166</v>
       </c>
     </row>
     <row r="1753" spans="1:9" ht="12.75">
@@ -52380,19 +52383,19 @@
         <v>250</v>
       </c>
       <c r="E1753" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1753" s="1">
         <v>0</v>
       </c>
       <c r="G1753" s="1">
-        <v>31417864</v>
+        <v>662779</v>
       </c>
       <c r="H1753" s="1">
         <v>0</v>
       </c>
       <c r="I1753" s="1">
-        <v>31417864</v>
+        <v>662779</v>
       </c>
     </row>
     <row r="1754" spans="1:9" ht="12.75">
@@ -52409,19 +52412,19 @@
         <v>250</v>
       </c>
       <c r="E1754" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1754" s="1">
         <v>0</v>
       </c>
       <c r="G1754" s="1">
-        <v>2664907</v>
+        <v>31417864</v>
       </c>
       <c r="H1754" s="1">
         <v>0</v>
       </c>
       <c r="I1754" s="1">
-        <v>2664907</v>
+        <v>31417864</v>
       </c>
     </row>
     <row r="1755" spans="1:9" ht="12.75">
@@ -52438,19 +52441,19 @@
         <v>250</v>
       </c>
       <c r="E1755" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1755" s="1">
         <v>0</v>
       </c>
       <c r="G1755" s="1">
-        <v>2021829</v>
+        <v>2664907</v>
       </c>
       <c r="H1755" s="1">
         <v>0</v>
       </c>
       <c r="I1755" s="1">
-        <v>2021829</v>
+        <v>2664907</v>
       </c>
     </row>
     <row r="1756" spans="1:9" ht="12.75">
@@ -52467,19 +52470,19 @@
         <v>250</v>
       </c>
       <c r="E1756" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1756" s="1">
         <v>0</v>
       </c>
       <c r="G1756" s="1">
-        <v>14946353</v>
+        <v>2021829</v>
       </c>
       <c r="H1756" s="1">
         <v>0</v>
       </c>
       <c r="I1756" s="1">
-        <v>14946353</v>
+        <v>2021829</v>
       </c>
     </row>
     <row r="1757" spans="1:9" ht="12.75">
@@ -52496,19 +52499,19 @@
         <v>250</v>
       </c>
       <c r="E1757" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1757" s="1">
         <v>0</v>
       </c>
       <c r="G1757" s="1">
-        <v>5986158</v>
+        <v>14946353</v>
       </c>
       <c r="H1757" s="1">
         <v>0</v>
       </c>
       <c r="I1757" s="1">
-        <v>5986158</v>
+        <v>14946353</v>
       </c>
     </row>
     <row r="1758" spans="1:9" ht="12.75">
@@ -52525,19 +52528,19 @@
         <v>250</v>
       </c>
       <c r="E1758" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1758" s="1">
         <v>0</v>
       </c>
       <c r="G1758" s="1">
-        <v>30819</v>
+        <v>5986158</v>
       </c>
       <c r="H1758" s="1">
         <v>0</v>
       </c>
       <c r="I1758" s="1">
-        <v>30819</v>
+        <v>5986158</v>
       </c>
     </row>
     <row r="1759" spans="1:9" ht="12.75">
@@ -52554,19 +52557,19 @@
         <v>250</v>
       </c>
       <c r="E1759" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F1759" s="1">
         <v>0</v>
       </c>
       <c r="G1759" s="1">
-        <v>1516559</v>
+        <v>30819</v>
       </c>
       <c r="H1759" s="1">
         <v>0</v>
       </c>
       <c r="I1759" s="1">
-        <v>1516559</v>
+        <v>30819</v>
       </c>
     </row>
     <row r="1760" spans="1:9" ht="12.75">
@@ -52583,19 +52586,19 @@
         <v>250</v>
       </c>
       <c r="E1760" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F1760" s="1">
         <v>0</v>
       </c>
       <c r="G1760" s="1">
-        <v>3492740</v>
+        <v>1516559</v>
       </c>
       <c r="H1760" s="1">
         <v>0</v>
       </c>
       <c r="I1760" s="1">
-        <v>3492740</v>
+        <v>1516559</v>
       </c>
     </row>
     <row r="1761" spans="1:9" ht="12.75">
@@ -52612,19 +52615,19 @@
         <v>250</v>
       </c>
       <c r="E1761" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F1761" s="1">
         <v>0</v>
       </c>
       <c r="G1761" s="1">
-        <v>75917498</v>
+        <v>3492740</v>
       </c>
       <c r="H1761" s="1">
-        <v>75931161</v>
+        <v>0</v>
       </c>
       <c r="I1761" s="1">
-        <v>-13663</v>
+        <v>3492740</v>
       </c>
     </row>
     <row r="1762" spans="1:9" ht="12.75">
@@ -52641,19 +52644,19 @@
         <v>250</v>
       </c>
       <c r="E1762" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F1762" s="1">
         <v>0</v>
       </c>
       <c r="G1762" s="1">
-        <v>747484</v>
+        <v>75917498</v>
       </c>
       <c r="H1762" s="1">
-        <v>0</v>
+        <v>75931161</v>
       </c>
       <c r="I1762" s="1">
-        <v>747484</v>
+        <v>-13663</v>
       </c>
     </row>
     <row r="1763" spans="1:9" ht="12.75">
@@ -52670,19 +52673,19 @@
         <v>250</v>
       </c>
       <c r="E1763" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F1763" s="1">
         <v>0</v>
       </c>
       <c r="G1763" s="1">
-        <v>1826516</v>
+        <v>747484</v>
       </c>
       <c r="H1763" s="1">
         <v>0</v>
       </c>
       <c r="I1763" s="1">
-        <v>1826516</v>
+        <v>747484</v>
       </c>
     </row>
     <row r="1764" spans="1:9" ht="12.75">
@@ -52699,19 +52702,19 @@
         <v>250</v>
       </c>
       <c r="E1764" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F1764" s="1">
         <v>0</v>
       </c>
       <c r="G1764" s="1">
-        <v>9827272</v>
+        <v>1826516</v>
       </c>
       <c r="H1764" s="1">
         <v>0</v>
       </c>
       <c r="I1764" s="1">
-        <v>9827272</v>
+        <v>1826516</v>
       </c>
     </row>
     <row r="1765" spans="1:9" ht="12.75">
@@ -52725,22 +52728,22 @@
         <v>105</v>
       </c>
       <c r="D1765" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E1765" t="s">
-        <v>13</v>
+        <v>341</v>
       </c>
       <c r="F1765" s="1">
         <v>0</v>
       </c>
       <c r="G1765" s="1">
-        <v>0.15</v>
+        <v>9827272</v>
       </c>
       <c r="H1765" s="1">
         <v>0</v>
       </c>
       <c r="I1765" s="1">
-        <v>0.15</v>
+        <v>9827272</v>
       </c>
     </row>
     <row r="1766" spans="1:9" ht="12.75">
@@ -52757,19 +52760,19 @@
         <v>253</v>
       </c>
       <c r="E1766" t="s">
-        <v>338</v>
+        <v>13</v>
       </c>
       <c r="F1766" s="1">
         <v>0</v>
       </c>
       <c r="G1766" s="1">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="H1766" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1766" s="1">
-        <v>-1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="1767" spans="1:9" ht="12.75">
@@ -52783,22 +52786,22 @@
         <v>105</v>
       </c>
       <c r="D1767" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E1767" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="F1767" s="1">
         <v>0</v>
       </c>
       <c r="G1767" s="1">
-        <v>148184</v>
+        <v>0</v>
       </c>
       <c r="H1767" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I1767" s="1">
-        <v>148184</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="1768" spans="1:9" ht="12.75">
@@ -52815,19 +52818,19 @@
         <v>257</v>
       </c>
       <c r="E1768" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="F1768" s="1">
         <v>0</v>
       </c>
       <c r="G1768" s="1">
-        <v>74092</v>
+        <v>148184</v>
       </c>
       <c r="H1768" s="1">
         <v>0</v>
       </c>
       <c r="I1768" s="1">
-        <v>74092</v>
+        <v>148184</v>
       </c>
     </row>
     <row r="1769" spans="1:9" ht="12.75">
@@ -52844,19 +52847,19 @@
         <v>257</v>
       </c>
       <c r="E1769" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1769" s="1">
         <v>0</v>
       </c>
       <c r="G1769" s="1">
-        <v>74092.80</v>
+        <v>74092</v>
       </c>
       <c r="H1769" s="1">
         <v>0</v>
       </c>
       <c r="I1769" s="1">
-        <v>74092.80</v>
+        <v>74092</v>
       </c>
     </row>
     <row r="1770" spans="1:9" ht="12.75">
@@ -52870,22 +52873,22 @@
         <v>105</v>
       </c>
       <c r="D1770" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E1770" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="F1770" s="1">
         <v>0</v>
       </c>
       <c r="G1770" s="1">
-        <v>137490</v>
+        <v>74092.80</v>
       </c>
       <c r="H1770" s="1">
         <v>0</v>
       </c>
       <c r="I1770" s="1">
-        <v>137490</v>
+        <v>74092.80</v>
       </c>
     </row>
     <row r="1771" spans="1:9" ht="12.75">
@@ -52902,19 +52905,19 @@
         <v>258</v>
       </c>
       <c r="E1771" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F1771" s="1">
         <v>0</v>
       </c>
       <c r="G1771" s="1">
-        <v>305648</v>
+        <v>137490</v>
       </c>
       <c r="H1771" s="1">
         <v>0</v>
       </c>
       <c r="I1771" s="1">
-        <v>305648</v>
+        <v>137490</v>
       </c>
     </row>
     <row r="1772" spans="1:9" ht="12.75">
@@ -52931,19 +52934,19 @@
         <v>258</v>
       </c>
       <c r="E1772" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1772" s="1">
         <v>0</v>
       </c>
       <c r="G1772" s="1">
-        <v>484</v>
+        <v>305648</v>
       </c>
       <c r="H1772" s="1">
         <v>0</v>
       </c>
       <c r="I1772" s="1">
-        <v>484</v>
+        <v>305648</v>
       </c>
     </row>
     <row r="1773" spans="1:9" ht="12.75">
@@ -52957,22 +52960,22 @@
         <v>105</v>
       </c>
       <c r="D1773" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E1773" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="F1773" s="1">
         <v>0</v>
       </c>
       <c r="G1773" s="1">
-        <v>24000</v>
+        <v>484</v>
       </c>
       <c r="H1773" s="1">
         <v>0</v>
       </c>
       <c r="I1773" s="1">
-        <v>24000</v>
+        <v>484</v>
       </c>
     </row>
     <row r="1774" spans="1:9" ht="12.75">
@@ -52986,22 +52989,22 @@
         <v>105</v>
       </c>
       <c r="D1774" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E1774" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="F1774" s="1">
         <v>0</v>
       </c>
       <c r="G1774" s="1">
-        <v>1125720</v>
+        <v>24000</v>
       </c>
       <c r="H1774" s="1">
         <v>0</v>
       </c>
       <c r="I1774" s="1">
-        <v>1125720</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="1775" spans="1:9" ht="12.75">
@@ -53018,19 +53021,19 @@
         <v>263</v>
       </c>
       <c r="E1775" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="F1775" s="1">
         <v>0</v>
       </c>
       <c r="G1775" s="1">
-        <v>1688580</v>
+        <v>1125720</v>
       </c>
       <c r="H1775" s="1">
         <v>0</v>
       </c>
       <c r="I1775" s="1">
-        <v>1688580</v>
+        <v>1125720</v>
       </c>
     </row>
     <row r="1776" spans="1:9" ht="12.75">
@@ -53038,28 +53041,28 @@
         <v>312</v>
       </c>
       <c r="B1776" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="C1776" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="D1776" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="E1776" t="s">
-        <v>13</v>
+        <v>337</v>
       </c>
       <c r="F1776" s="1">
         <v>0</v>
       </c>
       <c r="G1776" s="1">
-        <v>0</v>
+        <v>1688580</v>
       </c>
       <c r="H1776" s="1">
-        <v>7351276</v>
+        <v>0</v>
       </c>
       <c r="I1776" s="1">
-        <v>-7351276</v>
+        <v>1688580</v>
       </c>
     </row>
     <row r="1777" spans="1:9" ht="12.75">
@@ -53073,7 +53076,7 @@
         <v>264</v>
       </c>
       <c r="D1777" t="s">
-        <v>308</v>
+        <v>267</v>
       </c>
       <c r="E1777" t="s">
         <v>13</v>
@@ -53085,10 +53088,10 @@
         <v>0</v>
       </c>
       <c r="H1777" s="1">
-        <v>0</v>
+        <v>7351276</v>
       </c>
       <c r="I1777" s="1">
-        <v>0</v>
+        <v>-7351276</v>
       </c>
     </row>
     <row r="1778" spans="1:9" ht="12.75">
@@ -53096,28 +53099,28 @@
         <v>312</v>
       </c>
       <c r="B1778" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C1778" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D1778" t="s">
-        <v>269</v>
+        <v>308</v>
       </c>
       <c r="E1778" t="s">
         <v>13</v>
       </c>
       <c r="F1778" s="1">
-        <v>-5418882</v>
+        <v>0</v>
       </c>
       <c r="G1778" s="1">
-        <v>2.6231209744E8</v>
+        <v>0</v>
       </c>
       <c r="H1778" s="1">
-        <v>2.8301954077E8</v>
+        <v>0</v>
       </c>
       <c r="I1778" s="1">
-        <v>-2.6126325329999983E7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1779" spans="1:9" ht="12.75">
@@ -53128,25 +53131,25 @@
         <v>268</v>
       </c>
       <c r="C1779" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D1779" t="s">
-        <v>355</v>
+        <v>269</v>
       </c>
       <c r="E1779" t="s">
         <v>13</v>
       </c>
       <c r="F1779" s="1">
-        <v>0</v>
+        <v>-5418882</v>
       </c>
       <c r="G1779" s="1">
-        <v>2274999</v>
+        <v>2.8291444627E8</v>
       </c>
       <c r="H1779" s="1">
-        <v>5013786</v>
+        <v>2.9112331177E8</v>
       </c>
       <c r="I1779" s="1">
-        <v>-2738787</v>
+        <v>-1.36277475E7</v>
       </c>
     </row>
     <row r="1780" spans="1:9" ht="12.75">
@@ -53160,22 +53163,22 @@
         <v>273</v>
       </c>
       <c r="D1780" t="s">
-        <v>278</v>
+        <v>356</v>
       </c>
       <c r="E1780" t="s">
         <v>13</v>
       </c>
       <c r="F1780" s="1">
-        <v>-22030149</v>
+        <v>0</v>
       </c>
       <c r="G1780" s="1">
-        <v>9625806</v>
+        <v>2274999</v>
       </c>
       <c r="H1780" s="1">
-        <v>9.094276758399999E8</v>
+        <v>5013786</v>
       </c>
       <c r="I1780" s="1">
-        <v>-9.218320188399999E8</v>
+        <v>-2738787</v>
       </c>
     </row>
     <row r="1781" spans="1:9" ht="12.75">
@@ -53189,22 +53192,22 @@
         <v>273</v>
       </c>
       <c r="D1781" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E1781" t="s">
         <v>13</v>
       </c>
       <c r="F1781" s="1">
-        <v>-14989</v>
+        <v>-22030149</v>
       </c>
       <c r="G1781" s="1">
-        <v>5439991</v>
+        <v>7656302</v>
       </c>
       <c r="H1781" s="1">
-        <v>10165830</v>
+        <v>9.094276758399999E8</v>
       </c>
       <c r="I1781" s="1">
-        <v>-4740828</v>
+        <v>-9.238015228399999E8</v>
       </c>
     </row>
     <row r="1782" spans="1:9" ht="12.75">
@@ -53218,22 +53221,22 @@
         <v>273</v>
       </c>
       <c r="D1782" t="s">
-        <v>356</v>
+        <v>282</v>
       </c>
       <c r="E1782" t="s">
         <v>13</v>
       </c>
       <c r="F1782" s="1">
-        <v>0</v>
+        <v>-14989</v>
       </c>
       <c r="G1782" s="1">
-        <v>2659661</v>
+        <v>5515449</v>
       </c>
       <c r="H1782" s="1">
-        <v>2659660</v>
+        <v>10165830</v>
       </c>
       <c r="I1782" s="1">
-        <v>1</v>
+        <v>-4665370</v>
       </c>
     </row>
     <row r="1783" spans="1:9" ht="12.75">
@@ -53247,7 +53250,7 @@
         <v>273</v>
       </c>
       <c r="D1783" t="s">
-        <v>286</v>
+        <v>357</v>
       </c>
       <c r="E1783" t="s">
         <v>13</v>
@@ -53256,13 +53259,13 @@
         <v>0</v>
       </c>
       <c r="G1783" s="1">
-        <v>0</v>
+        <v>2659661</v>
       </c>
       <c r="H1783" s="1">
-        <v>190424</v>
+        <v>2659660</v>
       </c>
       <c r="I1783" s="1">
-        <v>-190424</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1784" spans="1:9" ht="12.75">
@@ -53276,7 +53279,7 @@
         <v>273</v>
       </c>
       <c r="D1784" t="s">
-        <v>357</v>
+        <v>286</v>
       </c>
       <c r="E1784" t="s">
         <v>13</v>
@@ -53285,13 +53288,13 @@
         <v>0</v>
       </c>
       <c r="G1784" s="1">
-        <v>1981165</v>
+        <v>0</v>
       </c>
       <c r="H1784" s="1">
-        <v>1995881</v>
+        <v>190424</v>
       </c>
       <c r="I1784" s="1">
-        <v>-14716</v>
+        <v>-190424</v>
       </c>
     </row>
     <row r="1785" spans="1:9" ht="12.75">
@@ -53305,7 +53308,7 @@
         <v>273</v>
       </c>
       <c r="D1785" t="s">
-        <v>287</v>
+        <v>358</v>
       </c>
       <c r="E1785" t="s">
         <v>13</v>
@@ -53314,13 +53317,13 @@
         <v>0</v>
       </c>
       <c r="G1785" s="1">
-        <v>48290</v>
+        <v>2279773</v>
       </c>
       <c r="H1785" s="1">
-        <v>70730</v>
+        <v>2294489</v>
       </c>
       <c r="I1785" s="1">
-        <v>-22440</v>
+        <v>-14716</v>
       </c>
     </row>
     <row r="1786" spans="1:9" ht="12.75">
@@ -53334,7 +53337,7 @@
         <v>273</v>
       </c>
       <c r="D1786" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E1786" t="s">
         <v>13</v>
@@ -53343,13 +53346,13 @@
         <v>0</v>
       </c>
       <c r="G1786" s="1">
-        <v>840</v>
+        <v>48730</v>
       </c>
       <c r="H1786" s="1">
-        <v>416</v>
+        <v>70730</v>
       </c>
       <c r="I1786" s="1">
-        <v>424</v>
+        <v>-22000</v>
       </c>
     </row>
     <row r="1787" spans="1:9" ht="12.75">
@@ -53363,7 +53366,7 @@
         <v>273</v>
       </c>
       <c r="D1787" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E1787" t="s">
         <v>13</v>
@@ -53372,13 +53375,13 @@
         <v>0</v>
       </c>
       <c r="G1787" s="1">
-        <v>4.74855129E7</v>
+        <v>840</v>
       </c>
       <c r="H1787" s="1">
-        <v>58379674</v>
+        <v>416</v>
       </c>
       <c r="I1787" s="1">
-        <v>-1.0894161100000001E7</v>
+        <v>424</v>
       </c>
     </row>
     <row r="1788" spans="1:9" ht="12.75">
@@ -53392,7 +53395,7 @@
         <v>273</v>
       </c>
       <c r="D1788" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E1788" t="s">
         <v>13</v>
@@ -53401,13 +53404,13 @@
         <v>0</v>
       </c>
       <c r="G1788" s="1">
-        <v>52444</v>
+        <v>4.89969833E7</v>
       </c>
       <c r="H1788" s="1">
-        <v>199075.79</v>
+        <v>58379674</v>
       </c>
       <c r="I1788" s="1">
-        <v>-146631.79</v>
+        <v>-9382690.700000003</v>
       </c>
     </row>
     <row r="1789" spans="1:9" ht="12.75">
@@ -53421,7 +53424,7 @@
         <v>273</v>
       </c>
       <c r="D1789" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E1789" t="s">
         <v>13</v>
@@ -53430,13 +53433,13 @@
         <v>0</v>
       </c>
       <c r="G1789" s="1">
-        <v>99271</v>
+        <v>55944</v>
       </c>
       <c r="H1789" s="1">
-        <v>498838.90</v>
+        <v>199075.78999999998</v>
       </c>
       <c r="I1789" s="1">
-        <v>-399567.90</v>
+        <v>-143131.78999999998</v>
       </c>
     </row>
     <row r="1790" spans="1:9" ht="12.75">
@@ -53450,7 +53453,7 @@
         <v>273</v>
       </c>
       <c r="D1790" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E1790" t="s">
         <v>13</v>
@@ -53459,13 +53462,13 @@
         <v>0</v>
       </c>
       <c r="G1790" s="1">
-        <v>4415952</v>
+        <v>105045</v>
       </c>
       <c r="H1790" s="1">
-        <v>1.365706809E7</v>
+        <v>498838.90</v>
       </c>
       <c r="I1790" s="1">
-        <v>-9241116.09</v>
+        <v>-393793.90</v>
       </c>
     </row>
     <row r="1791" spans="1:9" ht="12.75">
@@ -53479,7 +53482,7 @@
         <v>273</v>
       </c>
       <c r="D1791" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E1791" t="s">
         <v>13</v>
@@ -53488,13 +53491,13 @@
         <v>0</v>
       </c>
       <c r="G1791" s="1">
-        <v>1758542.24</v>
+        <v>4687449</v>
       </c>
       <c r="H1791" s="1">
-        <v>1153027.74</v>
+        <v>1.422406809E7</v>
       </c>
       <c r="I1791" s="1">
-        <v>605514.50</v>
+        <v>-9536619.09</v>
       </c>
     </row>
     <row r="1792" spans="1:9" ht="12.75">
@@ -53508,7 +53511,7 @@
         <v>273</v>
       </c>
       <c r="D1792" t="s">
-        <v>358</v>
+        <v>294</v>
       </c>
       <c r="E1792" t="s">
         <v>13</v>
@@ -53517,13 +53520,13 @@
         <v>0</v>
       </c>
       <c r="G1792" s="1">
-        <v>8658949</v>
+        <v>1758542.24</v>
       </c>
       <c r="H1792" s="1">
-        <v>18873669</v>
+        <v>1153027.7400000002</v>
       </c>
       <c r="I1792" s="1">
-        <v>-10214720</v>
+        <v>605514.4999999998</v>
       </c>
     </row>
     <row r="1793" spans="1:9" ht="12.75">
@@ -53534,10 +53537,10 @@
         <v>268</v>
       </c>
       <c r="C1793" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="D1793" t="s">
-        <v>297</v>
+        <v>359</v>
       </c>
       <c r="E1793" t="s">
         <v>13</v>
@@ -53546,13 +53549,13 @@
         <v>0</v>
       </c>
       <c r="G1793" s="1">
-        <v>2.2509215249E8</v>
+        <v>9251007</v>
       </c>
       <c r="H1793" s="1">
-        <v>2.2509215249000007E8</v>
+        <v>18902755</v>
       </c>
       <c r="I1793" s="1">
-        <v>-5.9604644775390625E-8</v>
+        <v>-9651748</v>
       </c>
     </row>
     <row r="1794" spans="1:9" ht="12.75">
@@ -53566,7 +53569,7 @@
         <v>296</v>
       </c>
       <c r="D1794" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E1794" t="s">
         <v>13</v>
@@ -53575,42 +53578,71 @@
         <v>0</v>
       </c>
       <c r="G1794" s="1">
-        <v>0</v>
+        <v>2.2518876449E8</v>
       </c>
       <c r="H1794" s="1">
-        <v>8826219.66</v>
+        <v>2.2518876449E8</v>
       </c>
       <c r="I1794" s="1">
-        <v>-8826219.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1795" spans="1:9" ht="12.75">
       <c r="A1795" t="s">
-        <v>359</v>
+        <v>312</v>
       </c>
       <c r="B1795" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1795" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1795" t="s">
+        <v>298</v>
+      </c>
+      <c r="E1795" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1795" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1795" s="1">
+        <v>0</v>
+      </c>
+      <c r="H1795" s="1">
+        <v>8826219.66</v>
+      </c>
+      <c r="I1795" s="1">
+        <v>-8826219.66</v>
+      </c>
+    </row>
+    <row r="1796" spans="1:9" ht="12.75">
+      <c r="A1796" t="s">
         <v>360</v>
       </c>
-      <c r="C1795" t="s">
-        <v>360</v>
-      </c>
-      <c r="D1795" t="s">
-        <v>360</v>
-      </c>
-      <c r="E1795" t="s">
-        <v>360</v>
-      </c>
-      <c r="F1795" s="1">
-        <v>1.1920928955078125E-7</v>
-      </c>
-      <c r="G1795" s="1">
-        <v>7.191002696809998E9</v>
-      </c>
-      <c r="H1795" s="1">
-        <v>7.1910026968099985E9</v>
-      </c>
-      <c r="I1795" s="1">
-        <v>-3.3527612686157227E-7</v>
+      <c r="B1796" t="s">
+        <v>361</v>
+      </c>
+      <c r="C1796" t="s">
+        <v>361</v>
+      </c>
+      <c r="D1796" t="s">
+        <v>361</v>
+      </c>
+      <c r="E1796" t="s">
+        <v>361</v>
+      </c>
+      <c r="F1796" s="1">
+        <v>5.9604644775390625E-8</v>
+      </c>
+      <c r="G1796" s="1">
+        <v>7.222306260039998E9</v>
+      </c>
+      <c r="H1796" s="1">
+        <v>7.222306260040002E9</v>
+      </c>
+      <c r="I1796" s="1">
+        <v>-3.725290298461914E-7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-03-21
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8988" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8993" uniqueCount="362">
   <si>
     <t>Book</t>
   </si>
@@ -1547,8 +1547,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62080ec0-bdc4-4af0-b553-5e86381d06af}">
-  <dimension ref="A1:I1796"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{d3efb514-2c25-46c6-9ab6-fc30dac3ba8f}">
+  <dimension ref="A1:I1797"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="14.142857142857142" customWidth="1"/>
@@ -47085,7 +47085,7 @@
         <v>1243234.22</v>
       </c>
       <c r="H1570" s="1">
-        <v>218466.36</v>
+        <v>218466.36000000002</v>
       </c>
       <c r="I1570" s="1">
         <v>1024767.86</v>
@@ -48619,13 +48619,13 @@
         <v>0</v>
       </c>
       <c r="G1623" s="1">
-        <v>1072113</v>
+        <v>1750251</v>
       </c>
       <c r="H1623" s="1">
         <v>0</v>
       </c>
       <c r="I1623" s="1">
-        <v>1072113</v>
+        <v>1750251</v>
       </c>
     </row>
     <row r="1624" spans="1:9" ht="12.75">
@@ -48648,13 +48648,13 @@
         <v>0</v>
       </c>
       <c r="G1624" s="1">
-        <v>145140</v>
+        <v>484209</v>
       </c>
       <c r="H1624" s="1">
         <v>0</v>
       </c>
       <c r="I1624" s="1">
-        <v>145140</v>
+        <v>484209</v>
       </c>
     </row>
     <row r="1625" spans="1:9" ht="12.75">
@@ -48677,13 +48677,13 @@
         <v>0</v>
       </c>
       <c r="G1625" s="1">
-        <v>145140</v>
+        <v>484209</v>
       </c>
       <c r="H1625" s="1">
         <v>0</v>
       </c>
       <c r="I1625" s="1">
-        <v>145140</v>
+        <v>484209</v>
       </c>
     </row>
     <row r="1626" spans="1:9" ht="12.75">
@@ -48706,13 +48706,13 @@
         <v>0</v>
       </c>
       <c r="G1626" s="1">
-        <v>72570</v>
+        <v>242105</v>
       </c>
       <c r="H1626" s="1">
         <v>0</v>
       </c>
       <c r="I1626" s="1">
-        <v>72570</v>
+        <v>242105</v>
       </c>
     </row>
     <row r="1627" spans="1:9" ht="12.75">
@@ -48735,13 +48735,13 @@
         <v>0</v>
       </c>
       <c r="G1627" s="1">
-        <v>72570</v>
+        <v>253467</v>
       </c>
       <c r="H1627" s="1">
         <v>0</v>
       </c>
       <c r="I1627" s="1">
-        <v>72570</v>
+        <v>253467</v>
       </c>
     </row>
     <row r="1628" spans="1:9" ht="12.75">
@@ -50127,13 +50127,13 @@
         <v>0</v>
       </c>
       <c r="G1675" s="1">
-        <v>218609.21999999997</v>
+        <v>218609.22000000003</v>
       </c>
       <c r="H1675" s="1">
         <v>0</v>
       </c>
       <c r="I1675" s="1">
-        <v>218609.21999999997</v>
+        <v>218609.22000000003</v>
       </c>
     </row>
     <row r="1676" spans="1:9" ht="12.75">
@@ -50156,13 +50156,13 @@
         <v>0</v>
       </c>
       <c r="G1676" s="1">
-        <v>1910663.08</v>
+        <v>1910663.0799999998</v>
       </c>
       <c r="H1676" s="1">
         <v>0</v>
       </c>
       <c r="I1676" s="1">
-        <v>1910663.08</v>
+        <v>1910663.0799999998</v>
       </c>
     </row>
     <row r="1677" spans="1:9" ht="12.75">
@@ -50243,13 +50243,13 @@
         <v>0</v>
       </c>
       <c r="G1679" s="1">
-        <v>191355.02</v>
+        <v>191355.01999999996</v>
       </c>
       <c r="H1679" s="1">
         <v>0</v>
       </c>
       <c r="I1679" s="1">
-        <v>191355.02</v>
+        <v>191355.01999999996</v>
       </c>
     </row>
     <row r="1680" spans="1:9" ht="12.75">
@@ -52119,22 +52119,22 @@
         <v>105</v>
       </c>
       <c r="D1744" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1744" t="s">
-        <v>330</v>
+        <v>344</v>
       </c>
       <c r="F1744" s="1">
         <v>0</v>
       </c>
       <c r="G1744" s="1">
-        <v>31481</v>
+        <v>2017937</v>
       </c>
       <c r="H1744" s="1">
         <v>0</v>
       </c>
       <c r="I1744" s="1">
-        <v>31481</v>
+        <v>2017937</v>
       </c>
     </row>
     <row r="1745" spans="1:9" ht="12.75">
@@ -52151,19 +52151,19 @@
         <v>246</v>
       </c>
       <c r="E1745" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1745" s="1">
         <v>0</v>
       </c>
       <c r="G1745" s="1">
-        <v>6638</v>
+        <v>31481</v>
       </c>
       <c r="H1745" s="1">
         <v>0</v>
       </c>
       <c r="I1745" s="1">
-        <v>6638</v>
+        <v>31481</v>
       </c>
     </row>
     <row r="1746" spans="1:9" ht="12.75">
@@ -52180,19 +52180,19 @@
         <v>246</v>
       </c>
       <c r="E1746" t="s">
-        <v>355</v>
+        <v>331</v>
       </c>
       <c r="F1746" s="1">
         <v>0</v>
       </c>
       <c r="G1746" s="1">
-        <v>7140</v>
+        <v>6638</v>
       </c>
       <c r="H1746" s="1">
         <v>0</v>
       </c>
       <c r="I1746" s="1">
-        <v>7140</v>
+        <v>6638</v>
       </c>
     </row>
     <row r="1747" spans="1:9" ht="12.75">
@@ -52209,19 +52209,19 @@
         <v>246</v>
       </c>
       <c r="E1747" t="s">
-        <v>337</v>
+        <v>355</v>
       </c>
       <c r="F1747" s="1">
         <v>0</v>
       </c>
       <c r="G1747" s="1">
-        <v>41204</v>
+        <v>7140</v>
       </c>
       <c r="H1747" s="1">
         <v>0</v>
       </c>
       <c r="I1747" s="1">
-        <v>41204</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="1748" spans="1:9" ht="12.75">
@@ -52235,22 +52235,22 @@
         <v>105</v>
       </c>
       <c r="D1748" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E1748" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="F1748" s="1">
         <v>0</v>
       </c>
       <c r="G1748" s="1">
-        <v>77571</v>
+        <v>41204</v>
       </c>
       <c r="H1748" s="1">
         <v>0</v>
       </c>
       <c r="I1748" s="1">
-        <v>77571</v>
+        <v>41204</v>
       </c>
     </row>
     <row r="1749" spans="1:9" ht="12.75">
@@ -52267,19 +52267,19 @@
         <v>247</v>
       </c>
       <c r="E1749" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F1749" s="1">
         <v>0</v>
       </c>
       <c r="G1749" s="1">
-        <v>1513824</v>
+        <v>77571</v>
       </c>
       <c r="H1749" s="1">
         <v>0</v>
       </c>
       <c r="I1749" s="1">
-        <v>1513824</v>
+        <v>77571</v>
       </c>
     </row>
     <row r="1750" spans="1:9" ht="12.75">
@@ -52296,19 +52296,19 @@
         <v>247</v>
       </c>
       <c r="E1750" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1750" s="1">
         <v>0</v>
       </c>
       <c r="G1750" s="1">
-        <v>22538</v>
+        <v>1513824</v>
       </c>
       <c r="H1750" s="1">
         <v>0</v>
       </c>
       <c r="I1750" s="1">
-        <v>22538</v>
+        <v>1513824</v>
       </c>
     </row>
     <row r="1751" spans="1:9" ht="12.75">
@@ -52322,22 +52322,22 @@
         <v>105</v>
       </c>
       <c r="D1751" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E1751" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F1751" s="1">
         <v>0</v>
       </c>
       <c r="G1751" s="1">
-        <v>9676</v>
+        <v>22538</v>
       </c>
       <c r="H1751" s="1">
         <v>0</v>
       </c>
       <c r="I1751" s="1">
-        <v>9676</v>
+        <v>22538</v>
       </c>
     </row>
     <row r="1752" spans="1:9" ht="12.75">
@@ -52351,22 +52351,22 @@
         <v>105</v>
       </c>
       <c r="D1752" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E1752" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F1752" s="1">
         <v>0</v>
       </c>
       <c r="G1752" s="1">
-        <v>3353166</v>
+        <v>9676</v>
       </c>
       <c r="H1752" s="1">
         <v>0</v>
       </c>
       <c r="I1752" s="1">
-        <v>3353166</v>
+        <v>9676</v>
       </c>
     </row>
     <row r="1753" spans="1:9" ht="12.75">
@@ -52383,19 +52383,19 @@
         <v>250</v>
       </c>
       <c r="E1753" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F1753" s="1">
         <v>0</v>
       </c>
       <c r="G1753" s="1">
-        <v>662779</v>
+        <v>3353166</v>
       </c>
       <c r="H1753" s="1">
         <v>0</v>
       </c>
       <c r="I1753" s="1">
-        <v>662779</v>
+        <v>3353166</v>
       </c>
     </row>
     <row r="1754" spans="1:9" ht="12.75">
@@ -52412,19 +52412,19 @@
         <v>250</v>
       </c>
       <c r="E1754" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1754" s="1">
         <v>0</v>
       </c>
       <c r="G1754" s="1">
-        <v>31417864</v>
+        <v>662779</v>
       </c>
       <c r="H1754" s="1">
         <v>0</v>
       </c>
       <c r="I1754" s="1">
-        <v>31417864</v>
+        <v>662779</v>
       </c>
     </row>
     <row r="1755" spans="1:9" ht="12.75">
@@ -52441,19 +52441,19 @@
         <v>250</v>
       </c>
       <c r="E1755" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1755" s="1">
         <v>0</v>
       </c>
       <c r="G1755" s="1">
-        <v>2664907</v>
+        <v>31417864</v>
       </c>
       <c r="H1755" s="1">
         <v>0</v>
       </c>
       <c r="I1755" s="1">
-        <v>2664907</v>
+        <v>31417864</v>
       </c>
     </row>
     <row r="1756" spans="1:9" ht="12.75">
@@ -52470,19 +52470,19 @@
         <v>250</v>
       </c>
       <c r="E1756" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1756" s="1">
         <v>0</v>
       </c>
       <c r="G1756" s="1">
-        <v>2021829</v>
+        <v>2664907</v>
       </c>
       <c r="H1756" s="1">
         <v>0</v>
       </c>
       <c r="I1756" s="1">
-        <v>2021829</v>
+        <v>2664907</v>
       </c>
     </row>
     <row r="1757" spans="1:9" ht="12.75">
@@ -52499,19 +52499,19 @@
         <v>250</v>
       </c>
       <c r="E1757" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1757" s="1">
         <v>0</v>
       </c>
       <c r="G1757" s="1">
-        <v>14946353</v>
+        <v>2021829</v>
       </c>
       <c r="H1757" s="1">
         <v>0</v>
       </c>
       <c r="I1757" s="1">
-        <v>14946353</v>
+        <v>2021829</v>
       </c>
     </row>
     <row r="1758" spans="1:9" ht="12.75">
@@ -52528,19 +52528,19 @@
         <v>250</v>
       </c>
       <c r="E1758" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1758" s="1">
         <v>0</v>
       </c>
       <c r="G1758" s="1">
-        <v>5986158</v>
+        <v>14946353</v>
       </c>
       <c r="H1758" s="1">
         <v>0</v>
       </c>
       <c r="I1758" s="1">
-        <v>5986158</v>
+        <v>14946353</v>
       </c>
     </row>
     <row r="1759" spans="1:9" ht="12.75">
@@ -52557,19 +52557,19 @@
         <v>250</v>
       </c>
       <c r="E1759" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1759" s="1">
         <v>0</v>
       </c>
       <c r="G1759" s="1">
-        <v>30819</v>
+        <v>5986158</v>
       </c>
       <c r="H1759" s="1">
         <v>0</v>
       </c>
       <c r="I1759" s="1">
-        <v>30819</v>
+        <v>5986158</v>
       </c>
     </row>
     <row r="1760" spans="1:9" ht="12.75">
@@ -52586,19 +52586,19 @@
         <v>250</v>
       </c>
       <c r="E1760" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F1760" s="1">
         <v>0</v>
       </c>
       <c r="G1760" s="1">
-        <v>1516559</v>
+        <v>30819</v>
       </c>
       <c r="H1760" s="1">
         <v>0</v>
       </c>
       <c r="I1760" s="1">
-        <v>1516559</v>
+        <v>30819</v>
       </c>
     </row>
     <row r="1761" spans="1:9" ht="12.75">
@@ -52615,19 +52615,19 @@
         <v>250</v>
       </c>
       <c r="E1761" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F1761" s="1">
         <v>0</v>
       </c>
       <c r="G1761" s="1">
-        <v>3492740</v>
+        <v>1516559</v>
       </c>
       <c r="H1761" s="1">
         <v>0</v>
       </c>
       <c r="I1761" s="1">
-        <v>3492740</v>
+        <v>1516559</v>
       </c>
     </row>
     <row r="1762" spans="1:9" ht="12.75">
@@ -52644,19 +52644,19 @@
         <v>250</v>
       </c>
       <c r="E1762" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F1762" s="1">
         <v>0</v>
       </c>
       <c r="G1762" s="1">
-        <v>75917498</v>
+        <v>3492740</v>
       </c>
       <c r="H1762" s="1">
-        <v>75931161</v>
+        <v>0</v>
       </c>
       <c r="I1762" s="1">
-        <v>-13663</v>
+        <v>3492740</v>
       </c>
     </row>
     <row r="1763" spans="1:9" ht="12.75">
@@ -52673,19 +52673,19 @@
         <v>250</v>
       </c>
       <c r="E1763" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F1763" s="1">
         <v>0</v>
       </c>
       <c r="G1763" s="1">
-        <v>747484</v>
+        <v>75917498</v>
       </c>
       <c r="H1763" s="1">
-        <v>0</v>
+        <v>75931161</v>
       </c>
       <c r="I1763" s="1">
-        <v>747484</v>
+        <v>-13663</v>
       </c>
     </row>
     <row r="1764" spans="1:9" ht="12.75">
@@ -52702,19 +52702,19 @@
         <v>250</v>
       </c>
       <c r="E1764" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F1764" s="1">
         <v>0</v>
       </c>
       <c r="G1764" s="1">
-        <v>1826516</v>
+        <v>747484</v>
       </c>
       <c r="H1764" s="1">
         <v>0</v>
       </c>
       <c r="I1764" s="1">
-        <v>1826516</v>
+        <v>747484</v>
       </c>
     </row>
     <row r="1765" spans="1:9" ht="12.75">
@@ -52731,19 +52731,19 @@
         <v>250</v>
       </c>
       <c r="E1765" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F1765" s="1">
         <v>0</v>
       </c>
       <c r="G1765" s="1">
-        <v>9827272</v>
+        <v>1826516</v>
       </c>
       <c r="H1765" s="1">
         <v>0</v>
       </c>
       <c r="I1765" s="1">
-        <v>9827272</v>
+        <v>1826516</v>
       </c>
     </row>
     <row r="1766" spans="1:9" ht="12.75">
@@ -52757,22 +52757,22 @@
         <v>105</v>
       </c>
       <c r="D1766" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E1766" t="s">
-        <v>13</v>
+        <v>341</v>
       </c>
       <c r="F1766" s="1">
         <v>0</v>
       </c>
       <c r="G1766" s="1">
-        <v>0.15</v>
+        <v>9827272</v>
       </c>
       <c r="H1766" s="1">
         <v>0</v>
       </c>
       <c r="I1766" s="1">
-        <v>0.15</v>
+        <v>9827272</v>
       </c>
     </row>
     <row r="1767" spans="1:9" ht="12.75">
@@ -52789,19 +52789,19 @@
         <v>253</v>
       </c>
       <c r="E1767" t="s">
-        <v>338</v>
+        <v>13</v>
       </c>
       <c r="F1767" s="1">
         <v>0</v>
       </c>
       <c r="G1767" s="1">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="H1767" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1767" s="1">
-        <v>-1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="1768" spans="1:9" ht="12.75">
@@ -52815,22 +52815,22 @@
         <v>105</v>
       </c>
       <c r="D1768" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E1768" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="F1768" s="1">
         <v>0</v>
       </c>
       <c r="G1768" s="1">
-        <v>148184</v>
+        <v>0</v>
       </c>
       <c r="H1768" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I1768" s="1">
-        <v>148184</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="1769" spans="1:9" ht="12.75">
@@ -52847,19 +52847,19 @@
         <v>257</v>
       </c>
       <c r="E1769" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="F1769" s="1">
         <v>0</v>
       </c>
       <c r="G1769" s="1">
-        <v>74092</v>
+        <v>148184</v>
       </c>
       <c r="H1769" s="1">
         <v>0</v>
       </c>
       <c r="I1769" s="1">
-        <v>74092</v>
+        <v>148184</v>
       </c>
     </row>
     <row r="1770" spans="1:9" ht="12.75">
@@ -52876,19 +52876,19 @@
         <v>257</v>
       </c>
       <c r="E1770" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1770" s="1">
         <v>0</v>
       </c>
       <c r="G1770" s="1">
-        <v>74092.80</v>
+        <v>74092</v>
       </c>
       <c r="H1770" s="1">
         <v>0</v>
       </c>
       <c r="I1770" s="1">
-        <v>74092.80</v>
+        <v>74092</v>
       </c>
     </row>
     <row r="1771" spans="1:9" ht="12.75">
@@ -52902,22 +52902,22 @@
         <v>105</v>
       </c>
       <c r="D1771" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E1771" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="F1771" s="1">
         <v>0</v>
       </c>
       <c r="G1771" s="1">
-        <v>137490</v>
+        <v>74092.80</v>
       </c>
       <c r="H1771" s="1">
         <v>0</v>
       </c>
       <c r="I1771" s="1">
-        <v>137490</v>
+        <v>74092.80</v>
       </c>
     </row>
     <row r="1772" spans="1:9" ht="12.75">
@@ -52934,19 +52934,19 @@
         <v>258</v>
       </c>
       <c r="E1772" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F1772" s="1">
         <v>0</v>
       </c>
       <c r="G1772" s="1">
-        <v>305648</v>
+        <v>137490</v>
       </c>
       <c r="H1772" s="1">
         <v>0</v>
       </c>
       <c r="I1772" s="1">
-        <v>305648</v>
+        <v>137490</v>
       </c>
     </row>
     <row r="1773" spans="1:9" ht="12.75">
@@ -52963,19 +52963,19 @@
         <v>258</v>
       </c>
       <c r="E1773" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1773" s="1">
         <v>0</v>
       </c>
       <c r="G1773" s="1">
-        <v>484</v>
+        <v>305648</v>
       </c>
       <c r="H1773" s="1">
         <v>0</v>
       </c>
       <c r="I1773" s="1">
-        <v>484</v>
+        <v>305648</v>
       </c>
     </row>
     <row r="1774" spans="1:9" ht="12.75">
@@ -52989,22 +52989,22 @@
         <v>105</v>
       </c>
       <c r="D1774" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E1774" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="F1774" s="1">
         <v>0</v>
       </c>
       <c r="G1774" s="1">
-        <v>24000</v>
+        <v>484</v>
       </c>
       <c r="H1774" s="1">
         <v>0</v>
       </c>
       <c r="I1774" s="1">
-        <v>24000</v>
+        <v>484</v>
       </c>
     </row>
     <row r="1775" spans="1:9" ht="12.75">
@@ -53018,22 +53018,22 @@
         <v>105</v>
       </c>
       <c r="D1775" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E1775" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="F1775" s="1">
         <v>0</v>
       </c>
       <c r="G1775" s="1">
-        <v>1125720</v>
+        <v>24000</v>
       </c>
       <c r="H1775" s="1">
         <v>0</v>
       </c>
       <c r="I1775" s="1">
-        <v>1125720</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="1776" spans="1:9" ht="12.75">
@@ -53050,19 +53050,19 @@
         <v>263</v>
       </c>
       <c r="E1776" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="F1776" s="1">
         <v>0</v>
       </c>
       <c r="G1776" s="1">
-        <v>1688580</v>
+        <v>1125720</v>
       </c>
       <c r="H1776" s="1">
         <v>0</v>
       </c>
       <c r="I1776" s="1">
-        <v>1688580</v>
+        <v>1125720</v>
       </c>
     </row>
     <row r="1777" spans="1:9" ht="12.75">
@@ -53070,28 +53070,28 @@
         <v>312</v>
       </c>
       <c r="B1777" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="C1777" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="D1777" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="E1777" t="s">
-        <v>13</v>
+        <v>337</v>
       </c>
       <c r="F1777" s="1">
         <v>0</v>
       </c>
       <c r="G1777" s="1">
-        <v>0</v>
+        <v>1688580</v>
       </c>
       <c r="H1777" s="1">
-        <v>7351276</v>
+        <v>0</v>
       </c>
       <c r="I1777" s="1">
-        <v>-7351276</v>
+        <v>1688580</v>
       </c>
     </row>
     <row r="1778" spans="1:9" ht="12.75">
@@ -53105,7 +53105,7 @@
         <v>264</v>
       </c>
       <c r="D1778" t="s">
-        <v>308</v>
+        <v>267</v>
       </c>
       <c r="E1778" t="s">
         <v>13</v>
@@ -53117,10 +53117,10 @@
         <v>0</v>
       </c>
       <c r="H1778" s="1">
-        <v>0</v>
+        <v>7351276</v>
       </c>
       <c r="I1778" s="1">
-        <v>0</v>
+        <v>-7351276</v>
       </c>
     </row>
     <row r="1779" spans="1:9" ht="12.75">
@@ -53128,28 +53128,28 @@
         <v>312</v>
       </c>
       <c r="B1779" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C1779" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D1779" t="s">
-        <v>269</v>
+        <v>308</v>
       </c>
       <c r="E1779" t="s">
         <v>13</v>
       </c>
       <c r="F1779" s="1">
-        <v>-5418882</v>
+        <v>0</v>
       </c>
       <c r="G1779" s="1">
-        <v>2.8291444627E8</v>
+        <v>0</v>
       </c>
       <c r="H1779" s="1">
-        <v>2.9112331177E8</v>
+        <v>0</v>
       </c>
       <c r="I1779" s="1">
-        <v>-1.36277475E7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1780" spans="1:9" ht="12.75">
@@ -53160,25 +53160,25 @@
         <v>268</v>
       </c>
       <c r="C1780" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D1780" t="s">
-        <v>356</v>
+        <v>269</v>
       </c>
       <c r="E1780" t="s">
         <v>13</v>
       </c>
       <c r="F1780" s="1">
-        <v>0</v>
+        <v>-5418882</v>
       </c>
       <c r="G1780" s="1">
-        <v>2274999</v>
+        <v>2.8291444627E8</v>
       </c>
       <c r="H1780" s="1">
-        <v>5013786</v>
+        <v>2.9453230877E8</v>
       </c>
       <c r="I1780" s="1">
-        <v>-2738787</v>
+        <v>-1.70367445E7</v>
       </c>
     </row>
     <row r="1781" spans="1:9" ht="12.75">
@@ -53192,22 +53192,22 @@
         <v>273</v>
       </c>
       <c r="D1781" t="s">
-        <v>278</v>
+        <v>356</v>
       </c>
       <c r="E1781" t="s">
         <v>13</v>
       </c>
       <c r="F1781" s="1">
-        <v>-22030149</v>
+        <v>0</v>
       </c>
       <c r="G1781" s="1">
-        <v>7656302</v>
+        <v>2274999</v>
       </c>
       <c r="H1781" s="1">
-        <v>9.094276758399999E8</v>
+        <v>5013786</v>
       </c>
       <c r="I1781" s="1">
-        <v>-9.238015228399999E8</v>
+        <v>-2738787</v>
       </c>
     </row>
     <row r="1782" spans="1:9" ht="12.75">
@@ -53221,22 +53221,22 @@
         <v>273</v>
       </c>
       <c r="D1782" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E1782" t="s">
         <v>13</v>
       </c>
       <c r="F1782" s="1">
-        <v>-14989</v>
+        <v>-22030149</v>
       </c>
       <c r="G1782" s="1">
-        <v>5515449</v>
+        <v>7656302</v>
       </c>
       <c r="H1782" s="1">
-        <v>10165830</v>
+        <v>9.094276758399999E8</v>
       </c>
       <c r="I1782" s="1">
-        <v>-4665370</v>
+        <v>-9.238015228399999E8</v>
       </c>
     </row>
     <row r="1783" spans="1:9" ht="12.75">
@@ -53250,22 +53250,22 @@
         <v>273</v>
       </c>
       <c r="D1783" t="s">
-        <v>357</v>
+        <v>282</v>
       </c>
       <c r="E1783" t="s">
         <v>13</v>
       </c>
       <c r="F1783" s="1">
-        <v>0</v>
+        <v>-14989</v>
       </c>
       <c r="G1783" s="1">
-        <v>2659661</v>
+        <v>5515449</v>
       </c>
       <c r="H1783" s="1">
-        <v>2659660</v>
+        <v>10165830</v>
       </c>
       <c r="I1783" s="1">
-        <v>1</v>
+        <v>-4665370</v>
       </c>
     </row>
     <row r="1784" spans="1:9" ht="12.75">
@@ -53279,7 +53279,7 @@
         <v>273</v>
       </c>
       <c r="D1784" t="s">
-        <v>286</v>
+        <v>357</v>
       </c>
       <c r="E1784" t="s">
         <v>13</v>
@@ -53288,13 +53288,13 @@
         <v>0</v>
       </c>
       <c r="G1784" s="1">
-        <v>0</v>
+        <v>2659661</v>
       </c>
       <c r="H1784" s="1">
-        <v>190424</v>
+        <v>2659660</v>
       </c>
       <c r="I1784" s="1">
-        <v>-190424</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1785" spans="1:9" ht="12.75">
@@ -53308,7 +53308,7 @@
         <v>273</v>
       </c>
       <c r="D1785" t="s">
-        <v>358</v>
+        <v>286</v>
       </c>
       <c r="E1785" t="s">
         <v>13</v>
@@ -53317,13 +53317,13 @@
         <v>0</v>
       </c>
       <c r="G1785" s="1">
-        <v>2279773</v>
+        <v>0</v>
       </c>
       <c r="H1785" s="1">
-        <v>2294489</v>
+        <v>190424</v>
       </c>
       <c r="I1785" s="1">
-        <v>-14716</v>
+        <v>-190424</v>
       </c>
     </row>
     <row r="1786" spans="1:9" ht="12.75">
@@ -53337,7 +53337,7 @@
         <v>273</v>
       </c>
       <c r="D1786" t="s">
-        <v>287</v>
+        <v>358</v>
       </c>
       <c r="E1786" t="s">
         <v>13</v>
@@ -53346,13 +53346,13 @@
         <v>0</v>
       </c>
       <c r="G1786" s="1">
-        <v>48730</v>
+        <v>2279773</v>
       </c>
       <c r="H1786" s="1">
-        <v>70730</v>
+        <v>2294489</v>
       </c>
       <c r="I1786" s="1">
-        <v>-22000</v>
+        <v>-14716</v>
       </c>
     </row>
     <row r="1787" spans="1:9" ht="12.75">
@@ -53366,7 +53366,7 @@
         <v>273</v>
       </c>
       <c r="D1787" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E1787" t="s">
         <v>13</v>
@@ -53375,13 +53375,13 @@
         <v>0</v>
       </c>
       <c r="G1787" s="1">
-        <v>840</v>
+        <v>48730</v>
       </c>
       <c r="H1787" s="1">
-        <v>416</v>
+        <v>70730</v>
       </c>
       <c r="I1787" s="1">
-        <v>424</v>
+        <v>-22000</v>
       </c>
     </row>
     <row r="1788" spans="1:9" ht="12.75">
@@ -53395,7 +53395,7 @@
         <v>273</v>
       </c>
       <c r="D1788" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E1788" t="s">
         <v>13</v>
@@ -53404,13 +53404,13 @@
         <v>0</v>
       </c>
       <c r="G1788" s="1">
-        <v>4.89969833E7</v>
+        <v>840</v>
       </c>
       <c r="H1788" s="1">
-        <v>58379674</v>
+        <v>416</v>
       </c>
       <c r="I1788" s="1">
-        <v>-9382690.700000003</v>
+        <v>424</v>
       </c>
     </row>
     <row r="1789" spans="1:9" ht="12.75">
@@ -53424,7 +53424,7 @@
         <v>273</v>
       </c>
       <c r="D1789" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E1789" t="s">
         <v>13</v>
@@ -53433,13 +53433,13 @@
         <v>0</v>
       </c>
       <c r="G1789" s="1">
-        <v>55944</v>
+        <v>4.89969833E7</v>
       </c>
       <c r="H1789" s="1">
-        <v>199075.78999999998</v>
+        <v>58379674</v>
       </c>
       <c r="I1789" s="1">
-        <v>-143131.78999999998</v>
+        <v>-9382690.700000003</v>
       </c>
     </row>
     <row r="1790" spans="1:9" ht="12.75">
@@ -53453,7 +53453,7 @@
         <v>273</v>
       </c>
       <c r="D1790" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E1790" t="s">
         <v>13</v>
@@ -53462,13 +53462,13 @@
         <v>0</v>
       </c>
       <c r="G1790" s="1">
-        <v>105045</v>
+        <v>55944</v>
       </c>
       <c r="H1790" s="1">
-        <v>498838.90</v>
+        <v>199075.78999999998</v>
       </c>
       <c r="I1790" s="1">
-        <v>-393793.90</v>
+        <v>-143131.78999999998</v>
       </c>
     </row>
     <row r="1791" spans="1:9" ht="12.75">
@@ -53482,7 +53482,7 @@
         <v>273</v>
       </c>
       <c r="D1791" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E1791" t="s">
         <v>13</v>
@@ -53491,13 +53491,13 @@
         <v>0</v>
       </c>
       <c r="G1791" s="1">
-        <v>4687449</v>
+        <v>105045</v>
       </c>
       <c r="H1791" s="1">
-        <v>1.422406809E7</v>
+        <v>498838.89999999997</v>
       </c>
       <c r="I1791" s="1">
-        <v>-9536619.09</v>
+        <v>-393793.89999999997</v>
       </c>
     </row>
     <row r="1792" spans="1:9" ht="12.75">
@@ -53511,7 +53511,7 @@
         <v>273</v>
       </c>
       <c r="D1792" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E1792" t="s">
         <v>13</v>
@@ -53520,13 +53520,13 @@
         <v>0</v>
       </c>
       <c r="G1792" s="1">
-        <v>1758542.24</v>
+        <v>4687449</v>
       </c>
       <c r="H1792" s="1">
-        <v>1153027.7400000002</v>
+        <v>1.453971609E7</v>
       </c>
       <c r="I1792" s="1">
-        <v>605514.4999999998</v>
+        <v>-9852267.09</v>
       </c>
     </row>
     <row r="1793" spans="1:9" ht="12.75">
@@ -53540,7 +53540,7 @@
         <v>273</v>
       </c>
       <c r="D1793" t="s">
-        <v>359</v>
+        <v>294</v>
       </c>
       <c r="E1793" t="s">
         <v>13</v>
@@ -53549,13 +53549,13 @@
         <v>0</v>
       </c>
       <c r="G1793" s="1">
-        <v>9251007</v>
+        <v>1758542.24</v>
       </c>
       <c r="H1793" s="1">
-        <v>18902755</v>
+        <v>1153027.74</v>
       </c>
       <c r="I1793" s="1">
-        <v>-9651748</v>
+        <v>605514.50</v>
       </c>
     </row>
     <row r="1794" spans="1:9" ht="12.75">
@@ -53566,10 +53566,10 @@
         <v>268</v>
       </c>
       <c r="C1794" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="D1794" t="s">
-        <v>297</v>
+        <v>359</v>
       </c>
       <c r="E1794" t="s">
         <v>13</v>
@@ -53578,13 +53578,13 @@
         <v>0</v>
       </c>
       <c r="G1794" s="1">
-        <v>2.2518876449E8</v>
+        <v>9251007</v>
       </c>
       <c r="H1794" s="1">
-        <v>2.2518876449E8</v>
+        <v>18902755</v>
       </c>
       <c r="I1794" s="1">
-        <v>0</v>
+        <v>-9651748</v>
       </c>
     </row>
     <row r="1795" spans="1:9" ht="12.75">
@@ -53598,7 +53598,7 @@
         <v>296</v>
       </c>
       <c r="D1795" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E1795" t="s">
         <v>13</v>
@@ -53607,41 +53607,70 @@
         <v>0</v>
       </c>
       <c r="G1795" s="1">
-        <v>0</v>
+        <v>2.2518876449E8</v>
       </c>
       <c r="H1795" s="1">
-        <v>8826219.66</v>
+        <v>2.2518876449E8</v>
       </c>
       <c r="I1795" s="1">
-        <v>-8826219.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1796" spans="1:9" ht="12.75">
       <c r="A1796" t="s">
+        <v>312</v>
+      </c>
+      <c r="B1796" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1796" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1796" t="s">
+        <v>298</v>
+      </c>
+      <c r="E1796" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1796" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1796" s="1">
+        <v>0</v>
+      </c>
+      <c r="H1796" s="1">
+        <v>8826219.66</v>
+      </c>
+      <c r="I1796" s="1">
+        <v>-8826219.66</v>
+      </c>
+    </row>
+    <row r="1797" spans="1:9" ht="12.75">
+      <c r="A1797" t="s">
         <v>360</v>
       </c>
-      <c r="B1796" t="s">
+      <c r="B1797" t="s">
         <v>361</v>
       </c>
-      <c r="C1796" t="s">
+      <c r="C1797" t="s">
         <v>361</v>
       </c>
-      <c r="D1796" t="s">
+      <c r="D1797" t="s">
         <v>361</v>
       </c>
-      <c r="E1796" t="s">
+      <c r="E1797" t="s">
         <v>361</v>
       </c>
-      <c r="F1796" s="1">
+      <c r="F1797" s="1">
         <v>5.9604644775390625E-8</v>
       </c>
-      <c r="G1796" s="1">
-        <v>7.222306260039998E9</v>
-      </c>
-      <c r="H1796" s="1">
-        <v>7.222306260040002E9</v>
-      </c>
-      <c r="I1796" s="1">
+      <c r="G1797" s="1">
+        <v>7.226030905039998E9</v>
+      </c>
+      <c r="H1797" s="1">
+        <v>7.226030905040002E9</v>
+      </c>
+      <c r="I1797" s="1">
         <v>-3.725290298461914E-7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Consol TB report update 2026-03-22
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -1547,7 +1547,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{d3efb514-2c25-46c6-9ab6-fc30dac3ba8f}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9cd9f792-c57b-4212-8117-cad6ba8fe253}">
   <dimension ref="A1:I1797"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -1671,10 +1671,10 @@
         <v>3.9882729998E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.447998005400005E8</v>
+        <v>3.447998005400006E8</v>
       </c>
       <c r="I4" s="1">
-        <v>1.8593025130999953E8</v>
+        <v>1.859302513099994E8</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -3817,10 +3817,10 @@
         <v>4.406711083E7</v>
       </c>
       <c r="H78" s="1">
-        <v>4.346434919999997E7</v>
+        <v>4.346434919999999E7</v>
       </c>
       <c r="I78" s="1">
-        <v>1521467.630000025</v>
+        <v>1521467.6300000101</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="12.75">
@@ -7671,13 +7671,13 @@
         <v>0</v>
       </c>
       <c r="G211" s="1">
-        <v>93200.52</v>
+        <v>93200.51999999999</v>
       </c>
       <c r="H211" s="1">
         <v>0</v>
       </c>
       <c r="I211" s="1">
-        <v>93200.52</v>
+        <v>93200.51999999999</v>
       </c>
     </row>
     <row r="212" spans="1:9" ht="12.75">
@@ -18372,13 +18372,13 @@
         <v>0</v>
       </c>
       <c r="G580" s="1">
-        <v>1064804.01</v>
+        <v>1064804.0100000002</v>
       </c>
       <c r="H580" s="1">
         <v>0</v>
       </c>
       <c r="I580" s="1">
-        <v>1064804.01</v>
+        <v>1064804.0100000002</v>
       </c>
     </row>
     <row r="581" spans="1:9" ht="12.75">
@@ -18575,13 +18575,13 @@
         <v>0</v>
       </c>
       <c r="G587" s="1">
-        <v>2994848.4499999997</v>
+        <v>2994848.45</v>
       </c>
       <c r="H587" s="1">
         <v>14722.75</v>
       </c>
       <c r="I587" s="1">
-        <v>2980125.6999999997</v>
+        <v>2980125.70</v>
       </c>
     </row>
     <row r="588" spans="1:9" ht="12.75">
@@ -18604,13 +18604,13 @@
         <v>0</v>
       </c>
       <c r="G588" s="1">
-        <v>150327.47000000003</v>
+        <v>150327.47</v>
       </c>
       <c r="H588" s="1">
         <v>0</v>
       </c>
       <c r="I588" s="1">
-        <v>150327.47000000003</v>
+        <v>150327.47</v>
       </c>
     </row>
     <row r="589" spans="1:9" ht="12.75">
@@ -18952,13 +18952,13 @@
         <v>0</v>
       </c>
       <c r="G600" s="1">
-        <v>925693.5499999999</v>
+        <v>925693.55</v>
       </c>
       <c r="H600" s="1">
         <v>0</v>
       </c>
       <c r="I600" s="1">
-        <v>925693.5499999999</v>
+        <v>925693.55</v>
       </c>
     </row>
     <row r="601" spans="1:9" ht="12.75">
@@ -19445,13 +19445,13 @@
         <v>0</v>
       </c>
       <c r="G617" s="1">
-        <v>274760.70</v>
+        <v>274760.69999999995</v>
       </c>
       <c r="H617" s="1">
         <v>0</v>
       </c>
       <c r="I617" s="1">
-        <v>274760.70</v>
+        <v>274760.69999999995</v>
       </c>
     </row>
     <row r="618" spans="1:9" ht="12.75">
@@ -19561,13 +19561,13 @@
         <v>0</v>
       </c>
       <c r="G621" s="1">
-        <v>2798165.89</v>
+        <v>2798165.8899999997</v>
       </c>
       <c r="H621" s="1">
         <v>23236.93</v>
       </c>
       <c r="I621" s="1">
-        <v>2774928.96</v>
+        <v>2774928.9599999995</v>
       </c>
     </row>
     <row r="622" spans="1:9" ht="12.75">
@@ -19967,13 +19967,13 @@
         <v>0</v>
       </c>
       <c r="G635" s="1">
-        <v>397731.83</v>
+        <v>397731.82999999996</v>
       </c>
       <c r="H635" s="1">
         <v>0</v>
       </c>
       <c r="I635" s="1">
-        <v>397731.83</v>
+        <v>397731.82999999996</v>
       </c>
     </row>
     <row r="636" spans="1:9" ht="12.75">
@@ -20025,13 +20025,13 @@
         <v>0</v>
       </c>
       <c r="G637" s="1">
-        <v>900877.7399999998</v>
+        <v>900877.74</v>
       </c>
       <c r="H637" s="1">
         <v>0</v>
       </c>
       <c r="I637" s="1">
-        <v>900877.7399999998</v>
+        <v>900877.74</v>
       </c>
     </row>
     <row r="638" spans="1:9" ht="12.75">
@@ -20054,13 +20054,13 @@
         <v>0</v>
       </c>
       <c r="G638" s="1">
-        <v>617359.9500000001</v>
+        <v>617359.95</v>
       </c>
       <c r="H638" s="1">
         <v>0</v>
       </c>
       <c r="I638" s="1">
-        <v>617359.9500000001</v>
+        <v>617359.95</v>
       </c>
     </row>
     <row r="639" spans="1:9" ht="12.75">
@@ -20112,13 +20112,13 @@
         <v>0</v>
       </c>
       <c r="G640" s="1">
-        <v>1595365.7100000002</v>
+        <v>1595365.71</v>
       </c>
       <c r="H640" s="1">
         <v>9049.23</v>
       </c>
       <c r="I640" s="1">
-        <v>1586316.4800000002</v>
+        <v>1586316.48</v>
       </c>
     </row>
     <row r="641" spans="1:9" ht="12.75">
@@ -20141,13 +20141,13 @@
         <v>0</v>
       </c>
       <c r="G641" s="1">
-        <v>703295.7999999999</v>
+        <v>703295.80</v>
       </c>
       <c r="H641" s="1">
         <v>0</v>
       </c>
       <c r="I641" s="1">
-        <v>703295.7999999999</v>
+        <v>703295.80</v>
       </c>
     </row>
     <row r="642" spans="1:9" ht="12.75">
@@ -20170,13 +20170,13 @@
         <v>0</v>
       </c>
       <c r="G642" s="1">
-        <v>516927.00000000006</v>
+        <v>516927</v>
       </c>
       <c r="H642" s="1">
         <v>0</v>
       </c>
       <c r="I642" s="1">
-        <v>516927.00000000006</v>
+        <v>516927</v>
       </c>
     </row>
     <row r="643" spans="1:9" ht="12.75">
@@ -20431,13 +20431,13 @@
         <v>0</v>
       </c>
       <c r="G651" s="1">
-        <v>264343.41000000003</v>
+        <v>264343.41</v>
       </c>
       <c r="H651" s="1">
         <v>0</v>
       </c>
       <c r="I651" s="1">
-        <v>264343.41000000003</v>
+        <v>264343.41</v>
       </c>
     </row>
     <row r="652" spans="1:9" ht="12.75">
@@ -21881,13 +21881,13 @@
         <v>0</v>
       </c>
       <c r="G701" s="1">
-        <v>2907448.8600000003</v>
+        <v>2907448.86</v>
       </c>
       <c r="H701" s="1">
         <v>0</v>
       </c>
       <c r="I701" s="1">
-        <v>2907448.8600000003</v>
+        <v>2907448.86</v>
       </c>
     </row>
     <row r="702" spans="1:9" ht="12.75">
@@ -22026,13 +22026,13 @@
         <v>0</v>
       </c>
       <c r="G706" s="1">
-        <v>5448697.789999999</v>
+        <v>5448697.79</v>
       </c>
       <c r="H706" s="1">
         <v>0</v>
       </c>
       <c r="I706" s="1">
-        <v>5448697.789999999</v>
+        <v>5448697.79</v>
       </c>
     </row>
     <row r="707" spans="1:9" ht="12.75">
@@ -22461,13 +22461,13 @@
         <v>0</v>
       </c>
       <c r="G721" s="1">
-        <v>1220232.6800000002</v>
+        <v>1220232.68</v>
       </c>
       <c r="H721" s="1">
         <v>0</v>
       </c>
       <c r="I721" s="1">
-        <v>1220232.6800000002</v>
+        <v>1220232.68</v>
       </c>
     </row>
     <row r="722" spans="1:9" ht="12.75">
@@ -44820,13 +44820,13 @@
         <v>-1.934719699999994E7</v>
       </c>
       <c r="G1492" s="1">
-        <v>2.1161717229999986E8</v>
+        <v>2.116171722999999E8</v>
       </c>
       <c r="H1492" s="1">
         <v>1.9916543229999998E8</v>
       </c>
       <c r="I1492" s="1">
-        <v>-6895457.00000006</v>
+        <v>-6895457.00000003</v>
       </c>
     </row>
     <row r="1493" spans="1:9" ht="12.75">
@@ -45400,10 +45400,10 @@
         <v>0</v>
       </c>
       <c r="G1512" s="1">
-        <v>556908.05</v>
+        <v>556908.0499999999</v>
       </c>
       <c r="H1512" s="1">
-        <v>588533.4800000001</v>
+        <v>588533.48</v>
       </c>
       <c r="I1512" s="1">
         <v>-31625.43000000005</v>
@@ -45548,10 +45548,10 @@
         <v>1.1068387002800002E9</v>
       </c>
       <c r="H1517" s="1">
-        <v>1.1068387002800004E9</v>
+        <v>1.10683870028E9</v>
       </c>
       <c r="I1517" s="1">
-        <v>-2.384185791015625E-7</v>
+        <v>2.384185791015625E-7</v>
       </c>
     </row>
     <row r="1518" spans="1:9" ht="12.75">
@@ -47085,7 +47085,7 @@
         <v>1243234.22</v>
       </c>
       <c r="H1570" s="1">
-        <v>218466.36000000002</v>
+        <v>218466.36</v>
       </c>
       <c r="I1570" s="1">
         <v>1024767.86</v>
@@ -49373,13 +49373,13 @@
         <v>0</v>
       </c>
       <c r="G1649" s="1">
-        <v>2619977.6799999997</v>
+        <v>2619977.68</v>
       </c>
       <c r="H1649" s="1">
         <v>0</v>
       </c>
       <c r="I1649" s="1">
-        <v>2619977.6799999997</v>
+        <v>2619977.68</v>
       </c>
     </row>
     <row r="1650" spans="1:9" ht="12.75">
@@ -50127,13 +50127,13 @@
         <v>0</v>
       </c>
       <c r="G1675" s="1">
-        <v>218609.22000000003</v>
+        <v>218609.21999999997</v>
       </c>
       <c r="H1675" s="1">
         <v>0</v>
       </c>
       <c r="I1675" s="1">
-        <v>218609.22000000003</v>
+        <v>218609.21999999997</v>
       </c>
     </row>
     <row r="1676" spans="1:9" ht="12.75">
@@ -50156,13 +50156,13 @@
         <v>0</v>
       </c>
       <c r="G1676" s="1">
-        <v>1910663.0799999998</v>
+        <v>1910663.08</v>
       </c>
       <c r="H1676" s="1">
         <v>0</v>
       </c>
       <c r="I1676" s="1">
-        <v>1910663.0799999998</v>
+        <v>1910663.08</v>
       </c>
     </row>
     <row r="1677" spans="1:9" ht="12.75">
@@ -50185,13 +50185,13 @@
         <v>0</v>
       </c>
       <c r="G1677" s="1">
-        <v>685737.61</v>
+        <v>685737.6100000001</v>
       </c>
       <c r="H1677" s="1">
         <v>0</v>
       </c>
       <c r="I1677" s="1">
-        <v>685737.61</v>
+        <v>685737.6100000001</v>
       </c>
     </row>
     <row r="1678" spans="1:9" ht="12.75">
@@ -50243,13 +50243,13 @@
         <v>0</v>
       </c>
       <c r="G1679" s="1">
-        <v>191355.01999999996</v>
+        <v>191355.02</v>
       </c>
       <c r="H1679" s="1">
         <v>0</v>
       </c>
       <c r="I1679" s="1">
-        <v>191355.01999999996</v>
+        <v>191355.02</v>
       </c>
     </row>
     <row r="1680" spans="1:9" ht="12.75">
@@ -50272,13 +50272,13 @@
         <v>0</v>
       </c>
       <c r="G1680" s="1">
-        <v>381348.32</v>
+        <v>381348.31999999995</v>
       </c>
       <c r="H1680" s="1">
         <v>0</v>
       </c>
       <c r="I1680" s="1">
-        <v>381348.32</v>
+        <v>381348.31999999995</v>
       </c>
     </row>
     <row r="1681" spans="1:9" ht="12.75">
@@ -53465,10 +53465,10 @@
         <v>55944</v>
       </c>
       <c r="H1790" s="1">
-        <v>199075.78999999998</v>
+        <v>199075.79</v>
       </c>
       <c r="I1790" s="1">
-        <v>-143131.78999999998</v>
+        <v>-143131.79</v>
       </c>
     </row>
     <row r="1791" spans="1:9" ht="12.75">
@@ -53494,10 +53494,10 @@
         <v>105045</v>
       </c>
       <c r="H1791" s="1">
-        <v>498838.89999999997</v>
+        <v>498838.90</v>
       </c>
       <c r="I1791" s="1">
-        <v>-393793.89999999997</v>
+        <v>-393793.90</v>
       </c>
     </row>
     <row r="1792" spans="1:9" ht="12.75">
@@ -53668,10 +53668,10 @@
         <v>7.226030905039998E9</v>
       </c>
       <c r="H1797" s="1">
-        <v>7.226030905040002E9</v>
+        <v>7.22603090504E9</v>
       </c>
       <c r="I1797" s="1">
-        <v>-3.725290298461914E-7</v>
+        <v>-1.341104507446289E-7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-03-23
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -1547,7 +1547,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9cd9f792-c57b-4212-8117-cad6ba8fe253}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{d83aad5f-9e32-47c2-9e1b-ed0cf053e0ea}">
   <dimension ref="A1:I1797"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -1636,7 +1636,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>-2.9802322387695312E-8</v>
+        <v>0</v>
       </c>
       <c r="G3" s="1">
         <v>3.54</v>
@@ -1645,7 +1645,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>-2.9802321943606103E-8</v>
+        <v>4.440892098500626E-16</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -1671,10 +1671,10 @@
         <v>3.9882729998E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.447998005400006E8</v>
+        <v>3.447998005400005E8</v>
       </c>
       <c r="I4" s="1">
-        <v>1.859302513099994E8</v>
+        <v>1.8593025130999953E8</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -3817,10 +3817,10 @@
         <v>4.406711083E7</v>
       </c>
       <c r="H78" s="1">
-        <v>4.346434919999999E7</v>
+        <v>4.346434919999997E7</v>
       </c>
       <c r="I78" s="1">
-        <v>1521467.6300000101</v>
+        <v>1521467.630000025</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="12.75">
@@ -3898,7 +3898,7 @@
         <v>13</v>
       </c>
       <c r="F81" s="1">
-        <v>0</v>
+        <v>-9.313225746154785E-10</v>
       </c>
       <c r="G81" s="1">
         <v>333614</v>
@@ -3907,7 +3907,7 @@
         <v>333614</v>
       </c>
       <c r="I81" s="1">
-        <v>0</v>
+        <v>-9.313225746154785E-10</v>
       </c>
     </row>
     <row r="82" spans="1:9" ht="12.75">
@@ -7671,13 +7671,13 @@
         <v>0</v>
       </c>
       <c r="G211" s="1">
-        <v>93200.51999999999</v>
+        <v>93200.52</v>
       </c>
       <c r="H211" s="1">
         <v>0</v>
       </c>
       <c r="I211" s="1">
-        <v>93200.51999999999</v>
+        <v>93200.52</v>
       </c>
     </row>
     <row r="212" spans="1:9" ht="12.75">
@@ -18372,13 +18372,13 @@
         <v>0</v>
       </c>
       <c r="G580" s="1">
-        <v>1064804.0100000002</v>
+        <v>1064804.01</v>
       </c>
       <c r="H580" s="1">
         <v>0</v>
       </c>
       <c r="I580" s="1">
-        <v>1064804.0100000002</v>
+        <v>1064804.01</v>
       </c>
     </row>
     <row r="581" spans="1:9" ht="12.75">
@@ -18575,13 +18575,13 @@
         <v>0</v>
       </c>
       <c r="G587" s="1">
-        <v>2994848.45</v>
+        <v>2994848.4499999997</v>
       </c>
       <c r="H587" s="1">
         <v>14722.75</v>
       </c>
       <c r="I587" s="1">
-        <v>2980125.70</v>
+        <v>2980125.6999999997</v>
       </c>
     </row>
     <row r="588" spans="1:9" ht="12.75">
@@ -18604,13 +18604,13 @@
         <v>0</v>
       </c>
       <c r="G588" s="1">
-        <v>150327.47</v>
+        <v>150327.47000000003</v>
       </c>
       <c r="H588" s="1">
         <v>0</v>
       </c>
       <c r="I588" s="1">
-        <v>150327.47</v>
+        <v>150327.47000000003</v>
       </c>
     </row>
     <row r="589" spans="1:9" ht="12.75">
@@ -18952,13 +18952,13 @@
         <v>0</v>
       </c>
       <c r="G600" s="1">
-        <v>925693.55</v>
+        <v>925693.5499999999</v>
       </c>
       <c r="H600" s="1">
         <v>0</v>
       </c>
       <c r="I600" s="1">
-        <v>925693.55</v>
+        <v>925693.5499999999</v>
       </c>
     </row>
     <row r="601" spans="1:9" ht="12.75">
@@ -19445,13 +19445,13 @@
         <v>0</v>
       </c>
       <c r="G617" s="1">
-        <v>274760.69999999995</v>
+        <v>274760.70</v>
       </c>
       <c r="H617" s="1">
         <v>0</v>
       </c>
       <c r="I617" s="1">
-        <v>274760.69999999995</v>
+        <v>274760.70</v>
       </c>
     </row>
     <row r="618" spans="1:9" ht="12.75">
@@ -19561,13 +19561,13 @@
         <v>0</v>
       </c>
       <c r="G621" s="1">
-        <v>2798165.8899999997</v>
+        <v>2798165.89</v>
       </c>
       <c r="H621" s="1">
         <v>23236.93</v>
       </c>
       <c r="I621" s="1">
-        <v>2774928.9599999995</v>
+        <v>2774928.96</v>
       </c>
     </row>
     <row r="622" spans="1:9" ht="12.75">
@@ -19967,13 +19967,13 @@
         <v>0</v>
       </c>
       <c r="G635" s="1">
-        <v>397731.82999999996</v>
+        <v>397731.83</v>
       </c>
       <c r="H635" s="1">
         <v>0</v>
       </c>
       <c r="I635" s="1">
-        <v>397731.82999999996</v>
+        <v>397731.83</v>
       </c>
     </row>
     <row r="636" spans="1:9" ht="12.75">
@@ -20025,13 +20025,13 @@
         <v>0</v>
       </c>
       <c r="G637" s="1">
-        <v>900877.74</v>
+        <v>900877.7399999998</v>
       </c>
       <c r="H637" s="1">
         <v>0</v>
       </c>
       <c r="I637" s="1">
-        <v>900877.74</v>
+        <v>900877.7399999998</v>
       </c>
     </row>
     <row r="638" spans="1:9" ht="12.75">
@@ -20054,13 +20054,13 @@
         <v>0</v>
       </c>
       <c r="G638" s="1">
-        <v>617359.95</v>
+        <v>617359.9500000001</v>
       </c>
       <c r="H638" s="1">
         <v>0</v>
       </c>
       <c r="I638" s="1">
-        <v>617359.95</v>
+        <v>617359.9500000001</v>
       </c>
     </row>
     <row r="639" spans="1:9" ht="12.75">
@@ -20112,13 +20112,13 @@
         <v>0</v>
       </c>
       <c r="G640" s="1">
-        <v>1595365.71</v>
+        <v>1595365.7100000002</v>
       </c>
       <c r="H640" s="1">
         <v>9049.23</v>
       </c>
       <c r="I640" s="1">
-        <v>1586316.48</v>
+        <v>1586316.4800000002</v>
       </c>
     </row>
     <row r="641" spans="1:9" ht="12.75">
@@ -20141,13 +20141,13 @@
         <v>0</v>
       </c>
       <c r="G641" s="1">
-        <v>703295.80</v>
+        <v>703295.7999999999</v>
       </c>
       <c r="H641" s="1">
         <v>0</v>
       </c>
       <c r="I641" s="1">
-        <v>703295.80</v>
+        <v>703295.7999999999</v>
       </c>
     </row>
     <row r="642" spans="1:9" ht="12.75">
@@ -20170,13 +20170,13 @@
         <v>0</v>
       </c>
       <c r="G642" s="1">
-        <v>516927</v>
+        <v>516927.00000000006</v>
       </c>
       <c r="H642" s="1">
         <v>0</v>
       </c>
       <c r="I642" s="1">
-        <v>516927</v>
+        <v>516927.00000000006</v>
       </c>
     </row>
     <row r="643" spans="1:9" ht="12.75">
@@ -20431,13 +20431,13 @@
         <v>0</v>
       </c>
       <c r="G651" s="1">
-        <v>264343.41</v>
+        <v>264343.41000000003</v>
       </c>
       <c r="H651" s="1">
         <v>0</v>
       </c>
       <c r="I651" s="1">
-        <v>264343.41</v>
+        <v>264343.41000000003</v>
       </c>
     </row>
     <row r="652" spans="1:9" ht="12.75">
@@ -21881,13 +21881,13 @@
         <v>0</v>
       </c>
       <c r="G701" s="1">
-        <v>2907448.86</v>
+        <v>2907448.8600000003</v>
       </c>
       <c r="H701" s="1">
         <v>0</v>
       </c>
       <c r="I701" s="1">
-        <v>2907448.86</v>
+        <v>2907448.8600000003</v>
       </c>
     </row>
     <row r="702" spans="1:9" ht="12.75">
@@ -22026,13 +22026,13 @@
         <v>0</v>
       </c>
       <c r="G706" s="1">
-        <v>5448697.79</v>
+        <v>5448697.789999999</v>
       </c>
       <c r="H706" s="1">
         <v>0</v>
       </c>
       <c r="I706" s="1">
-        <v>5448697.79</v>
+        <v>5448697.789999999</v>
       </c>
     </row>
     <row r="707" spans="1:9" ht="12.75">
@@ -22461,13 +22461,13 @@
         <v>0</v>
       </c>
       <c r="G721" s="1">
-        <v>1220232.68</v>
+        <v>1220232.6800000002</v>
       </c>
       <c r="H721" s="1">
         <v>0</v>
       </c>
       <c r="I721" s="1">
-        <v>1220232.68</v>
+        <v>1220232.6800000002</v>
       </c>
     </row>
     <row r="722" spans="1:9" ht="12.75">
@@ -44817,16 +44817,16 @@
         <v>13</v>
       </c>
       <c r="F1492" s="1">
-        <v>-1.934719699999994E7</v>
+        <v>-1.934719699999988E7</v>
       </c>
       <c r="G1492" s="1">
-        <v>2.116171722999999E8</v>
+        <v>2.1161717229999986E8</v>
       </c>
       <c r="H1492" s="1">
         <v>1.9916543229999998E8</v>
       </c>
       <c r="I1492" s="1">
-        <v>-6895457.00000003</v>
+        <v>-6895457</v>
       </c>
     </row>
     <row r="1493" spans="1:9" ht="12.75">
@@ -45400,10 +45400,10 @@
         <v>0</v>
       </c>
       <c r="G1512" s="1">
-        <v>556908.0499999999</v>
+        <v>556908.05</v>
       </c>
       <c r="H1512" s="1">
-        <v>588533.48</v>
+        <v>588533.4800000001</v>
       </c>
       <c r="I1512" s="1">
         <v>-31625.43000000005</v>
@@ -45484,7 +45484,7 @@
         <v>13</v>
       </c>
       <c r="F1515" s="1">
-        <v>-56797.000000003725</v>
+        <v>-56797.000000002794</v>
       </c>
       <c r="G1515" s="1">
         <v>3227421.94</v>
@@ -45493,7 +45493,7 @@
         <v>3631156.939999996</v>
       </c>
       <c r="I1515" s="1">
-        <v>-460532</v>
+        <v>-460531.99999999907</v>
       </c>
     </row>
     <row r="1516" spans="1:9" ht="12.75">
@@ -45548,10 +45548,10 @@
         <v>1.1068387002800002E9</v>
       </c>
       <c r="H1517" s="1">
-        <v>1.10683870028E9</v>
+        <v>1.1068387002800024E9</v>
       </c>
       <c r="I1517" s="1">
-        <v>2.384185791015625E-7</v>
+        <v>-2.1457672119140625E-6</v>
       </c>
     </row>
     <row r="1518" spans="1:9" ht="12.75">
@@ -50127,13 +50127,13 @@
         <v>0</v>
       </c>
       <c r="G1675" s="1">
-        <v>218609.21999999997</v>
+        <v>218609.22</v>
       </c>
       <c r="H1675" s="1">
         <v>0</v>
       </c>
       <c r="I1675" s="1">
-        <v>218609.21999999997</v>
+        <v>218609.22</v>
       </c>
     </row>
     <row r="1676" spans="1:9" ht="12.75">
@@ -50156,13 +50156,13 @@
         <v>0</v>
       </c>
       <c r="G1676" s="1">
-        <v>1910663.08</v>
+        <v>1910663.0799999996</v>
       </c>
       <c r="H1676" s="1">
         <v>0</v>
       </c>
       <c r="I1676" s="1">
-        <v>1910663.08</v>
+        <v>1910663.0799999996</v>
       </c>
     </row>
     <row r="1677" spans="1:9" ht="12.75">
@@ -50185,13 +50185,13 @@
         <v>0</v>
       </c>
       <c r="G1677" s="1">
-        <v>685737.6100000001</v>
+        <v>685737.61</v>
       </c>
       <c r="H1677" s="1">
         <v>0</v>
       </c>
       <c r="I1677" s="1">
-        <v>685737.6100000001</v>
+        <v>685737.61</v>
       </c>
     </row>
     <row r="1678" spans="1:9" ht="12.75">
@@ -53175,10 +53175,10 @@
         <v>2.8291444627E8</v>
       </c>
       <c r="H1780" s="1">
-        <v>2.9453230877E8</v>
+        <v>2.9453230877000004E8</v>
       </c>
       <c r="I1780" s="1">
-        <v>-1.70367445E7</v>
+        <v>-1.703674450000006E7</v>
       </c>
     </row>
     <row r="1781" spans="1:9" ht="12.75">
@@ -53662,16 +53662,16 @@
         <v>361</v>
       </c>
       <c r="F1797" s="1">
-        <v>5.9604644775390625E-8</v>
+        <v>1.1920928955078125E-7</v>
       </c>
       <c r="G1797" s="1">
         <v>7.226030905039998E9</v>
       </c>
       <c r="H1797" s="1">
-        <v>7.22603090504E9</v>
+        <v>7.226030905040004E9</v>
       </c>
       <c r="I1797" s="1">
-        <v>-1.341104507446289E-7</v>
+        <v>-2.2798776626586914E-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-03-24
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8993" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9003" uniqueCount="362">
   <si>
     <t>Book</t>
   </si>
@@ -1052,6 +1052,9 @@
     <t>AIP-0133-Oral Reading-Google Services-Non FCRA</t>
   </si>
   <si>
+    <t>AIP-0106-Early Education-Google IT-Non FCRA</t>
+  </si>
+  <si>
     <t>AIP-0131-Oral Reading-Google IT-Non FCRA</t>
   </si>
   <si>
@@ -1062,9 +1065,6 @@
   </si>
   <si>
     <t>AIP-0106-ECCS IT-Non FCRA</t>
-  </si>
-  <si>
-    <t>AIP-0106-Early Education-Google IT-Non FCRA</t>
   </si>
   <si>
     <t>AIP-0115-Training Infra and MEL-Google Payment-NFC</t>
@@ -1547,8 +1547,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{d83aad5f-9e32-47c2-9e1b-ed0cf053e0ea}">
-  <dimension ref="A1:I1797"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{cddf3534-34d4-4985-89f2-9a1a303a9c2a}">
+  <dimension ref="A1:I1799"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="14.142857142857142" customWidth="1"/>
@@ -1636,7 +1636,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>0</v>
+        <v>5.9604644775390625E-8</v>
       </c>
       <c r="G3" s="1">
         <v>3.54</v>
@@ -1645,7 +1645,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>4.440892098500626E-16</v>
+        <v>5.960464521947983E-8</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -1671,10 +1671,10 @@
         <v>3.9882729998E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.447998005400005E8</v>
+        <v>3.447999505400007E8</v>
       </c>
       <c r="I4" s="1">
-        <v>1.8593025130999953E8</v>
+        <v>1.8593010130999935E8</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -3814,13 +3814,13 @@
         <v>918706</v>
       </c>
       <c r="G78" s="1">
-        <v>4.406711083E7</v>
+        <v>4.406724683E7</v>
       </c>
       <c r="H78" s="1">
-        <v>4.346434919999997E7</v>
+        <v>4.3464485200000025E7</v>
       </c>
       <c r="I78" s="1">
-        <v>1521467.630000025</v>
+        <v>1521467.6299999729</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="12.75">
@@ -6047,13 +6047,13 @@
         <v>0</v>
       </c>
       <c r="G155" s="1">
-        <v>1.9072333009999998E7</v>
+        <v>1.907233301E7</v>
       </c>
       <c r="H155" s="1">
         <v>18680110</v>
       </c>
       <c r="I155" s="1">
-        <v>392223.0099999979</v>
+        <v>392223.01000000164</v>
       </c>
     </row>
     <row r="156" spans="1:9" ht="12.75">
@@ -12804,13 +12804,13 @@
         <v>0</v>
       </c>
       <c r="G388" s="1">
-        <v>1168077</v>
+        <v>1363077</v>
       </c>
       <c r="H388" s="1">
         <v>0</v>
       </c>
       <c r="I388" s="1">
-        <v>1168077</v>
+        <v>1363077</v>
       </c>
     </row>
     <row r="389" spans="1:9" ht="12.75">
@@ -13790,13 +13790,13 @@
         <v>0</v>
       </c>
       <c r="G422" s="1">
-        <v>1153033</v>
+        <v>1166245</v>
       </c>
       <c r="H422" s="1">
         <v>0</v>
       </c>
       <c r="I422" s="1">
-        <v>1153033</v>
+        <v>1166245</v>
       </c>
     </row>
     <row r="423" spans="1:9" ht="12.75">
@@ -14747,13 +14747,13 @@
         <v>0</v>
       </c>
       <c r="G455" s="1">
-        <v>681768.30</v>
+        <v>681768.2999999999</v>
       </c>
       <c r="H455" s="1">
         <v>0</v>
       </c>
       <c r="I455" s="1">
-        <v>681768.30</v>
+        <v>681768.2999999999</v>
       </c>
     </row>
     <row r="456" spans="1:9" ht="12.75">
@@ -15037,13 +15037,13 @@
         <v>0</v>
       </c>
       <c r="G465" s="1">
-        <v>1870416.50</v>
+        <v>1877517.50</v>
       </c>
       <c r="H465" s="1">
         <v>9923</v>
       </c>
       <c r="I465" s="1">
-        <v>1860493.50</v>
+        <v>1867594.50</v>
       </c>
     </row>
     <row r="466" spans="1:9" ht="12.75">
@@ -18372,13 +18372,13 @@
         <v>0</v>
       </c>
       <c r="G580" s="1">
-        <v>1064804.01</v>
+        <v>1064804.0100000002</v>
       </c>
       <c r="H580" s="1">
         <v>0</v>
       </c>
       <c r="I580" s="1">
-        <v>1064804.01</v>
+        <v>1064804.0100000002</v>
       </c>
     </row>
     <row r="581" spans="1:9" ht="12.75">
@@ -18604,13 +18604,13 @@
         <v>0</v>
       </c>
       <c r="G588" s="1">
-        <v>150327.47000000003</v>
+        <v>150327.47</v>
       </c>
       <c r="H588" s="1">
         <v>0</v>
       </c>
       <c r="I588" s="1">
-        <v>150327.47000000003</v>
+        <v>150327.47</v>
       </c>
     </row>
     <row r="589" spans="1:9" ht="12.75">
@@ -18952,13 +18952,13 @@
         <v>0</v>
       </c>
       <c r="G600" s="1">
-        <v>925693.5499999999</v>
+        <v>925693.55</v>
       </c>
       <c r="H600" s="1">
         <v>0</v>
       </c>
       <c r="I600" s="1">
-        <v>925693.5499999999</v>
+        <v>925693.55</v>
       </c>
     </row>
     <row r="601" spans="1:9" ht="12.75">
@@ -19445,13 +19445,13 @@
         <v>0</v>
       </c>
       <c r="G617" s="1">
-        <v>274760.70</v>
+        <v>274760.69999999995</v>
       </c>
       <c r="H617" s="1">
         <v>0</v>
       </c>
       <c r="I617" s="1">
-        <v>274760.70</v>
+        <v>274760.69999999995</v>
       </c>
     </row>
     <row r="618" spans="1:9" ht="12.75">
@@ -19561,13 +19561,13 @@
         <v>0</v>
       </c>
       <c r="G621" s="1">
-        <v>2798165.89</v>
+        <v>2798165.8900000006</v>
       </c>
       <c r="H621" s="1">
         <v>23236.93</v>
       </c>
       <c r="I621" s="1">
-        <v>2774928.96</v>
+        <v>2774928.9600000004</v>
       </c>
     </row>
     <row r="622" spans="1:9" ht="12.75">
@@ -19619,13 +19619,13 @@
         <v>0</v>
       </c>
       <c r="G623" s="1">
-        <v>3046869.40</v>
+        <v>3046869.400000001</v>
       </c>
       <c r="H623" s="1">
         <v>9049.23</v>
       </c>
       <c r="I623" s="1">
-        <v>3037820.17</v>
+        <v>3037820.170000001</v>
       </c>
     </row>
     <row r="624" spans="1:9" ht="12.75">
@@ -20025,13 +20025,13 @@
         <v>0</v>
       </c>
       <c r="G637" s="1">
-        <v>900877.7399999998</v>
+        <v>900877.74</v>
       </c>
       <c r="H637" s="1">
         <v>0</v>
       </c>
       <c r="I637" s="1">
-        <v>900877.7399999998</v>
+        <v>900877.74</v>
       </c>
     </row>
     <row r="638" spans="1:9" ht="12.75">
@@ -20054,13 +20054,13 @@
         <v>0</v>
       </c>
       <c r="G638" s="1">
-        <v>617359.9500000001</v>
+        <v>617359.95</v>
       </c>
       <c r="H638" s="1">
         <v>0</v>
       </c>
       <c r="I638" s="1">
-        <v>617359.9500000001</v>
+        <v>617359.95</v>
       </c>
     </row>
     <row r="639" spans="1:9" ht="12.75">
@@ -20141,13 +20141,13 @@
         <v>0</v>
       </c>
       <c r="G641" s="1">
-        <v>703295.7999999999</v>
+        <v>703295.80</v>
       </c>
       <c r="H641" s="1">
         <v>0</v>
       </c>
       <c r="I641" s="1">
-        <v>703295.7999999999</v>
+        <v>703295.80</v>
       </c>
     </row>
     <row r="642" spans="1:9" ht="12.75">
@@ -20170,13 +20170,13 @@
         <v>0</v>
       </c>
       <c r="G642" s="1">
-        <v>516927.00000000006</v>
+        <v>516927</v>
       </c>
       <c r="H642" s="1">
         <v>0</v>
       </c>
       <c r="I642" s="1">
-        <v>516927.00000000006</v>
+        <v>516927</v>
       </c>
     </row>
     <row r="643" spans="1:9" ht="12.75">
@@ -20344,13 +20344,13 @@
         <v>0</v>
       </c>
       <c r="G648" s="1">
-        <v>1824764.48</v>
+        <v>1824764.4799999997</v>
       </c>
       <c r="H648" s="1">
         <v>13850.19</v>
       </c>
       <c r="I648" s="1">
-        <v>1810914.29</v>
+        <v>1810914.2899999998</v>
       </c>
     </row>
     <row r="649" spans="1:9" ht="12.75">
@@ -22403,13 +22403,13 @@
         <v>0</v>
       </c>
       <c r="G719" s="1">
-        <v>253568.63999999998</v>
+        <v>253568.64</v>
       </c>
       <c r="H719" s="1">
         <v>0</v>
       </c>
       <c r="I719" s="1">
-        <v>253568.63999999998</v>
+        <v>253568.64</v>
       </c>
     </row>
     <row r="720" spans="1:9" ht="12.75">
@@ -28899,13 +28899,13 @@
         <v>0</v>
       </c>
       <c r="G943" s="1">
-        <v>78979</v>
+        <v>78814</v>
       </c>
       <c r="H943" s="1">
         <v>0</v>
       </c>
       <c r="I943" s="1">
-        <v>78979</v>
+        <v>78814</v>
       </c>
     </row>
     <row r="944" spans="1:9" ht="12.75">
@@ -28928,13 +28928,13 @@
         <v>0</v>
       </c>
       <c r="G944" s="1">
-        <v>76560</v>
+        <v>76725</v>
       </c>
       <c r="H944" s="1">
         <v>0</v>
       </c>
       <c r="I944" s="1">
-        <v>76560</v>
+        <v>76725</v>
       </c>
     </row>
     <row r="945" spans="1:9" ht="12.75">
@@ -37773,13 +37773,13 @@
         <v>0</v>
       </c>
       <c r="G1249" s="1">
-        <v>23998.50</v>
+        <v>10786.50</v>
       </c>
       <c r="H1249" s="1">
         <v>0</v>
       </c>
       <c r="I1249" s="1">
-        <v>23998.50</v>
+        <v>10786.50</v>
       </c>
     </row>
     <row r="1250" spans="1:9" ht="12.75">
@@ -39078,13 +39078,13 @@
         <v>0</v>
       </c>
       <c r="G1294" s="1">
-        <v>4252</v>
+        <v>3927</v>
       </c>
       <c r="H1294" s="1">
         <v>0</v>
       </c>
       <c r="I1294" s="1">
-        <v>4252</v>
+        <v>3927</v>
       </c>
     </row>
     <row r="1295" spans="1:9" ht="12.75">
@@ -39107,13 +39107,13 @@
         <v>0</v>
       </c>
       <c r="G1295" s="1">
-        <v>7300</v>
+        <v>7625</v>
       </c>
       <c r="H1295" s="1">
         <v>0</v>
       </c>
       <c r="I1295" s="1">
-        <v>7300</v>
+        <v>7625</v>
       </c>
     </row>
     <row r="1296" spans="1:9" ht="12.75">
@@ -42184,10 +42184,10 @@
         <v>0</v>
       </c>
       <c r="H1401" s="1">
-        <v>3.52</v>
+        <v>139.52</v>
       </c>
       <c r="I1401" s="1">
-        <v>-3.52</v>
+        <v>-139.52</v>
       </c>
     </row>
     <row r="1402" spans="1:9" ht="12.75">
@@ -44817,16 +44817,16 @@
         <v>13</v>
       </c>
       <c r="F1492" s="1">
-        <v>-1.934719699999988E7</v>
+        <v>-19347197</v>
       </c>
       <c r="G1492" s="1">
-        <v>2.1161717229999986E8</v>
+        <v>2.1278430029999983E8</v>
       </c>
       <c r="H1492" s="1">
-        <v>1.9916543229999998E8</v>
+        <v>1.9934816929999986E8</v>
       </c>
       <c r="I1492" s="1">
-        <v>-6895457</v>
+        <v>-5911066.00000003</v>
       </c>
     </row>
     <row r="1493" spans="1:9" ht="12.75">
@@ -45345,10 +45345,10 @@
         <v>2.8008181086E8</v>
       </c>
       <c r="H1510" s="1">
-        <v>278500869</v>
+        <v>279667575</v>
       </c>
       <c r="I1510" s="1">
-        <v>826848.8600000143</v>
+        <v>-339857.1399999857</v>
       </c>
     </row>
     <row r="1511" spans="1:9" ht="12.75">
@@ -45400,13 +45400,13 @@
         <v>0</v>
       </c>
       <c r="G1512" s="1">
-        <v>556908.05</v>
+        <v>556908.0499999999</v>
       </c>
       <c r="H1512" s="1">
-        <v>588533.4800000001</v>
+        <v>588533.4799999999</v>
       </c>
       <c r="I1512" s="1">
-        <v>-31625.43000000005</v>
+        <v>-31625.429999999935</v>
       </c>
     </row>
     <row r="1513" spans="1:9" ht="12.75">
@@ -45461,10 +45461,10 @@
         <v>7533462.2</v>
       </c>
       <c r="H1514" s="1">
-        <v>8545737.919999998</v>
+        <v>8565237.92</v>
       </c>
       <c r="I1514" s="1">
-        <v>-1012275.7199999979</v>
+        <v>-1031775.7199999997</v>
       </c>
     </row>
     <row r="1515" spans="1:9" ht="12.75">
@@ -45484,16 +45484,16 @@
         <v>13</v>
       </c>
       <c r="F1515" s="1">
-        <v>-56797.000000002794</v>
+        <v>-56797.00000000093</v>
       </c>
       <c r="G1515" s="1">
-        <v>3227421.94</v>
+        <v>3227421.9400000004</v>
       </c>
       <c r="H1515" s="1">
-        <v>3631156.939999996</v>
+        <v>3631156.939999997</v>
       </c>
       <c r="I1515" s="1">
-        <v>-460531.99999999907</v>
+        <v>-460531.9999999977</v>
       </c>
     </row>
     <row r="1516" spans="1:9" ht="12.75">
@@ -45542,16 +45542,16 @@
         <v>13</v>
       </c>
       <c r="F1517" s="1">
-        <v>0</v>
+        <v>-5.9604644775390625E-8</v>
       </c>
       <c r="G1517" s="1">
         <v>1.1068387002800002E9</v>
       </c>
       <c r="H1517" s="1">
-        <v>1.1068387002800024E9</v>
+        <v>1.10683870028E9</v>
       </c>
       <c r="I1517" s="1">
-        <v>-2.1457672119140625E-6</v>
+        <v>2.384185791015625E-7</v>
       </c>
     </row>
     <row r="1518" spans="1:9" ht="12.75">
@@ -46444,13 +46444,13 @@
         <v>2.91937089E7</v>
       </c>
       <c r="G1548" s="1">
-        <v>6.515914804E7</v>
+        <v>6.935924803999999E7</v>
       </c>
       <c r="H1548" s="1">
-        <v>6.724710968E7</v>
+        <v>6.898970867999999E7</v>
       </c>
       <c r="I1548" s="1">
-        <v>2.710574725999999E7</v>
+        <v>2.9563248260000005E7</v>
       </c>
     </row>
     <row r="1549" spans="1:9" ht="12.75">
@@ -46534,10 +46534,10 @@
         <v>8.56587629E8</v>
       </c>
       <c r="H1551" s="1">
-        <v>3.856976476E8</v>
+        <v>4.045564786E8</v>
       </c>
       <c r="I1551" s="1">
-        <v>4.708899814E8</v>
+        <v>4.520311504E8</v>
       </c>
     </row>
     <row r="1552" spans="1:9" ht="12.75">
@@ -47053,13 +47053,13 @@
         <v>0</v>
       </c>
       <c r="G1569" s="1">
-        <v>2.121751046E8</v>
+        <v>2.209496436E8</v>
       </c>
       <c r="H1569" s="1">
         <v>1.2661798486E8</v>
       </c>
       <c r="I1569" s="1">
-        <v>8.555711974E7</v>
+        <v>9.433165874E7</v>
       </c>
     </row>
     <row r="1570" spans="1:9" ht="12.75">
@@ -48851,13 +48851,13 @@
         <v>0</v>
       </c>
       <c r="G1631" s="1">
-        <v>7770928.95</v>
+        <v>7868428.95</v>
       </c>
       <c r="H1631" s="1">
         <v>50000</v>
       </c>
       <c r="I1631" s="1">
-        <v>7720928.95</v>
+        <v>7818428.95</v>
       </c>
     </row>
     <row r="1632" spans="1:9" ht="12.75">
@@ -48961,19 +48961,19 @@
         <v>210</v>
       </c>
       <c r="E1635" t="s">
-        <v>334</v>
+        <v>345</v>
       </c>
       <c r="F1635" s="1">
         <v>0</v>
       </c>
       <c r="G1635" s="1">
-        <v>2802830</v>
+        <v>39000</v>
       </c>
       <c r="H1635" s="1">
         <v>0</v>
       </c>
       <c r="I1635" s="1">
-        <v>2802830</v>
+        <v>39000</v>
       </c>
     </row>
     <row r="1636" spans="1:9" ht="12.75">
@@ -48990,19 +48990,19 @@
         <v>210</v>
       </c>
       <c r="E1636" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1636" s="1">
         <v>0</v>
       </c>
       <c r="G1636" s="1">
-        <v>145830</v>
+        <v>2841830</v>
       </c>
       <c r="H1636" s="1">
         <v>0</v>
       </c>
       <c r="I1636" s="1">
-        <v>145830</v>
+        <v>2841830</v>
       </c>
     </row>
     <row r="1637" spans="1:9" ht="12.75">
@@ -49019,19 +49019,19 @@
         <v>210</v>
       </c>
       <c r="E1637" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="F1637" s="1">
         <v>0</v>
       </c>
       <c r="G1637" s="1">
-        <v>271778</v>
+        <v>165330</v>
       </c>
       <c r="H1637" s="1">
         <v>0</v>
       </c>
       <c r="I1637" s="1">
-        <v>271778</v>
+        <v>165330</v>
       </c>
     </row>
     <row r="1638" spans="1:9" ht="12.75">
@@ -49048,19 +49048,19 @@
         <v>210</v>
       </c>
       <c r="E1638" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="F1638" s="1">
         <v>0</v>
       </c>
       <c r="G1638" s="1">
-        <v>442300</v>
+        <v>271778</v>
       </c>
       <c r="H1638" s="1">
         <v>0</v>
       </c>
       <c r="I1638" s="1">
-        <v>442300</v>
+        <v>271778</v>
       </c>
     </row>
     <row r="1639" spans="1:9" ht="12.75">
@@ -49077,19 +49077,19 @@
         <v>210</v>
       </c>
       <c r="E1639" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F1639" s="1">
         <v>0</v>
       </c>
       <c r="G1639" s="1">
-        <v>2881013</v>
+        <v>442300</v>
       </c>
       <c r="H1639" s="1">
         <v>0</v>
       </c>
       <c r="I1639" s="1">
-        <v>2881013</v>
+        <v>442300</v>
       </c>
     </row>
     <row r="1640" spans="1:9" ht="12.75">
@@ -49106,19 +49106,19 @@
         <v>210</v>
       </c>
       <c r="E1640" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F1640" s="1">
         <v>0</v>
       </c>
       <c r="G1640" s="1">
-        <v>47500</v>
+        <v>2881013</v>
       </c>
       <c r="H1640" s="1">
         <v>0</v>
       </c>
       <c r="I1640" s="1">
-        <v>47500</v>
+        <v>2881013</v>
       </c>
     </row>
     <row r="1641" spans="1:9" ht="12.75">
@@ -49135,19 +49135,19 @@
         <v>210</v>
       </c>
       <c r="E1641" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F1641" s="1">
         <v>0</v>
       </c>
       <c r="G1641" s="1">
-        <v>61875</v>
+        <v>47500</v>
       </c>
       <c r="H1641" s="1">
         <v>0</v>
       </c>
       <c r="I1641" s="1">
-        <v>61875</v>
+        <v>47500</v>
       </c>
     </row>
     <row r="1642" spans="1:9" ht="12.75">
@@ -49164,19 +49164,19 @@
         <v>210</v>
       </c>
       <c r="E1642" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F1642" s="1">
         <v>0</v>
       </c>
       <c r="G1642" s="1">
-        <v>1253200</v>
+        <v>61875</v>
       </c>
       <c r="H1642" s="1">
         <v>0</v>
       </c>
       <c r="I1642" s="1">
-        <v>1253200</v>
+        <v>61875</v>
       </c>
     </row>
     <row r="1643" spans="1:9" ht="12.75">
@@ -49193,19 +49193,19 @@
         <v>210</v>
       </c>
       <c r="E1643" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="F1643" s="1">
         <v>0</v>
       </c>
       <c r="G1643" s="1">
-        <v>14465</v>
+        <v>1253200</v>
       </c>
       <c r="H1643" s="1">
         <v>0</v>
       </c>
       <c r="I1643" s="1">
-        <v>14465</v>
+        <v>1253200</v>
       </c>
     </row>
     <row r="1644" spans="1:9" ht="12.75">
@@ -49228,13 +49228,13 @@
         <v>0</v>
       </c>
       <c r="G1644" s="1">
-        <v>2458001</v>
+        <v>14465</v>
       </c>
       <c r="H1644" s="1">
         <v>0</v>
       </c>
       <c r="I1644" s="1">
-        <v>2458001</v>
+        <v>14465</v>
       </c>
     </row>
     <row r="1645" spans="1:9" ht="12.75">
@@ -49248,22 +49248,22 @@
         <v>105</v>
       </c>
       <c r="D1645" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E1645" t="s">
-        <v>13</v>
+        <v>347</v>
       </c>
       <c r="F1645" s="1">
         <v>0</v>
       </c>
       <c r="G1645" s="1">
-        <v>242538</v>
+        <v>2458001</v>
       </c>
       <c r="H1645" s="1">
         <v>0</v>
       </c>
       <c r="I1645" s="1">
-        <v>242538</v>
+        <v>2458001</v>
       </c>
     </row>
     <row r="1646" spans="1:9" ht="12.75">
@@ -49277,7 +49277,7 @@
         <v>105</v>
       </c>
       <c r="D1646" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E1646" t="s">
         <v>13</v>
@@ -49286,13 +49286,13 @@
         <v>0</v>
       </c>
       <c r="G1646" s="1">
-        <v>466917</v>
+        <v>242538</v>
       </c>
       <c r="H1646" s="1">
         <v>0</v>
       </c>
       <c r="I1646" s="1">
-        <v>466917</v>
+        <v>242538</v>
       </c>
     </row>
     <row r="1647" spans="1:9" ht="12.75">
@@ -49309,19 +49309,19 @@
         <v>212</v>
       </c>
       <c r="E1647" t="s">
-        <v>328</v>
+        <v>13</v>
       </c>
       <c r="F1647" s="1">
         <v>0</v>
       </c>
       <c r="G1647" s="1">
-        <v>2133376.20</v>
+        <v>2702</v>
       </c>
       <c r="H1647" s="1">
         <v>0</v>
       </c>
       <c r="I1647" s="1">
-        <v>2133376.20</v>
+        <v>2702</v>
       </c>
     </row>
     <row r="1648" spans="1:9" ht="12.75">
@@ -49338,19 +49338,19 @@
         <v>212</v>
       </c>
       <c r="E1648" t="s">
-        <v>347</v>
+        <v>328</v>
       </c>
       <c r="F1648" s="1">
         <v>0</v>
       </c>
       <c r="G1648" s="1">
-        <v>40134</v>
+        <v>2133376.20</v>
       </c>
       <c r="H1648" s="1">
         <v>0</v>
       </c>
       <c r="I1648" s="1">
-        <v>40134</v>
+        <v>2133376.20</v>
       </c>
     </row>
     <row r="1649" spans="1:9" ht="12.75">
@@ -49367,19 +49367,19 @@
         <v>212</v>
       </c>
       <c r="E1649" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="F1649" s="1">
         <v>0</v>
       </c>
       <c r="G1649" s="1">
-        <v>2619977.68</v>
+        <v>40134</v>
       </c>
       <c r="H1649" s="1">
         <v>0</v>
       </c>
       <c r="I1649" s="1">
-        <v>2619977.68</v>
+        <v>40134</v>
       </c>
     </row>
     <row r="1650" spans="1:9" ht="12.75">
@@ -49396,19 +49396,19 @@
         <v>212</v>
       </c>
       <c r="E1650" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1650" s="1">
         <v>0</v>
       </c>
       <c r="G1650" s="1">
-        <v>2585749.92</v>
+        <v>2619977.68</v>
       </c>
       <c r="H1650" s="1">
         <v>0</v>
       </c>
       <c r="I1650" s="1">
-        <v>2585749.92</v>
+        <v>2619977.68</v>
       </c>
     </row>
     <row r="1651" spans="1:9" ht="12.75">
@@ -49425,19 +49425,19 @@
         <v>212</v>
       </c>
       <c r="E1651" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1651" s="1">
         <v>0</v>
       </c>
       <c r="G1651" s="1">
-        <v>652186</v>
+        <v>2755079.92</v>
       </c>
       <c r="H1651" s="1">
         <v>0</v>
       </c>
       <c r="I1651" s="1">
-        <v>652186</v>
+        <v>2755079.92</v>
       </c>
     </row>
     <row r="1652" spans="1:9" ht="12.75">
@@ -49454,19 +49454,19 @@
         <v>212</v>
       </c>
       <c r="E1652" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1652" s="1">
         <v>0</v>
       </c>
       <c r="G1652" s="1">
-        <v>101989</v>
+        <v>857554</v>
       </c>
       <c r="H1652" s="1">
         <v>0</v>
       </c>
       <c r="I1652" s="1">
-        <v>101989</v>
+        <v>857554</v>
       </c>
     </row>
     <row r="1653" spans="1:9" ht="12.75">
@@ -49483,19 +49483,19 @@
         <v>212</v>
       </c>
       <c r="E1653" t="s">
-        <v>348</v>
+        <v>332</v>
       </c>
       <c r="F1653" s="1">
         <v>0</v>
       </c>
       <c r="G1653" s="1">
-        <v>6559</v>
+        <v>111860</v>
       </c>
       <c r="H1653" s="1">
         <v>0</v>
       </c>
       <c r="I1653" s="1">
-        <v>6559</v>
+        <v>111860</v>
       </c>
     </row>
     <row r="1654" spans="1:9" ht="12.75">
@@ -49512,19 +49512,19 @@
         <v>212</v>
       </c>
       <c r="E1654" t="s">
-        <v>333</v>
+        <v>349</v>
       </c>
       <c r="F1654" s="1">
         <v>0</v>
       </c>
       <c r="G1654" s="1">
-        <v>200632</v>
+        <v>6559</v>
       </c>
       <c r="H1654" s="1">
         <v>0</v>
       </c>
       <c r="I1654" s="1">
-        <v>200632</v>
+        <v>6559</v>
       </c>
     </row>
     <row r="1655" spans="1:9" ht="12.75">
@@ -49541,19 +49541,19 @@
         <v>212</v>
       </c>
       <c r="E1655" t="s">
-        <v>349</v>
+        <v>333</v>
       </c>
       <c r="F1655" s="1">
         <v>0</v>
       </c>
       <c r="G1655" s="1">
-        <v>18505</v>
+        <v>200632</v>
       </c>
       <c r="H1655" s="1">
         <v>0</v>
       </c>
       <c r="I1655" s="1">
-        <v>18505</v>
+        <v>200632</v>
       </c>
     </row>
     <row r="1656" spans="1:9" ht="12.75">
@@ -49570,19 +49570,19 @@
         <v>212</v>
       </c>
       <c r="E1656" t="s">
-        <v>334</v>
+        <v>345</v>
       </c>
       <c r="F1656" s="1">
         <v>0</v>
       </c>
       <c r="G1656" s="1">
-        <v>3436</v>
+        <v>23520</v>
       </c>
       <c r="H1656" s="1">
         <v>0</v>
       </c>
       <c r="I1656" s="1">
-        <v>3436</v>
+        <v>23520</v>
       </c>
     </row>
     <row r="1657" spans="1:9" ht="12.75">
@@ -49599,19 +49599,19 @@
         <v>212</v>
       </c>
       <c r="E1657" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F1657" s="1">
         <v>0</v>
       </c>
       <c r="G1657" s="1">
-        <v>300656</v>
+        <v>13808</v>
       </c>
       <c r="H1657" s="1">
         <v>0</v>
       </c>
       <c r="I1657" s="1">
-        <v>300656</v>
+        <v>13808</v>
       </c>
     </row>
     <row r="1658" spans="1:9" ht="12.75">
@@ -49628,19 +49628,19 @@
         <v>212</v>
       </c>
       <c r="E1658" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="F1658" s="1">
         <v>0</v>
       </c>
       <c r="G1658" s="1">
-        <v>18528</v>
+        <v>300656</v>
       </c>
       <c r="H1658" s="1">
         <v>0</v>
       </c>
       <c r="I1658" s="1">
-        <v>18528</v>
+        <v>300656</v>
       </c>
     </row>
     <row r="1659" spans="1:9" ht="12.75">
@@ -49657,19 +49657,19 @@
         <v>212</v>
       </c>
       <c r="E1659" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="F1659" s="1">
         <v>0</v>
       </c>
       <c r="G1659" s="1">
-        <v>1164147</v>
+        <v>6065</v>
       </c>
       <c r="H1659" s="1">
         <v>0</v>
       </c>
       <c r="I1659" s="1">
-        <v>1164147</v>
+        <v>6065</v>
       </c>
     </row>
     <row r="1660" spans="1:9" ht="12.75">
@@ -49683,22 +49683,22 @@
         <v>105</v>
       </c>
       <c r="D1660" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="E1660" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="F1660" s="1">
         <v>0</v>
       </c>
       <c r="G1660" s="1">
-        <v>1824</v>
+        <v>23471</v>
       </c>
       <c r="H1660" s="1">
         <v>0</v>
       </c>
       <c r="I1660" s="1">
-        <v>1824</v>
+        <v>23471</v>
       </c>
     </row>
     <row r="1661" spans="1:9" ht="12.75">
@@ -49712,22 +49712,22 @@
         <v>105</v>
       </c>
       <c r="D1661" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="E1661" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="F1661" s="1">
         <v>0</v>
       </c>
       <c r="G1661" s="1">
-        <v>223551</v>
+        <v>1330690</v>
       </c>
       <c r="H1661" s="1">
         <v>0</v>
       </c>
       <c r="I1661" s="1">
-        <v>223551</v>
+        <v>1330690</v>
       </c>
     </row>
     <row r="1662" spans="1:9" ht="12.75">
@@ -49741,22 +49741,22 @@
         <v>105</v>
       </c>
       <c r="D1662" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E1662" t="s">
-        <v>328</v>
+        <v>342</v>
       </c>
       <c r="F1662" s="1">
         <v>0</v>
       </c>
       <c r="G1662" s="1">
-        <v>49500</v>
+        <v>1824</v>
       </c>
       <c r="H1662" s="1">
         <v>0</v>
       </c>
       <c r="I1662" s="1">
-        <v>49500</v>
+        <v>1824</v>
       </c>
     </row>
     <row r="1663" spans="1:9" ht="12.75">
@@ -49770,22 +49770,22 @@
         <v>105</v>
       </c>
       <c r="D1663" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E1663" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="F1663" s="1">
         <v>0</v>
       </c>
       <c r="G1663" s="1">
-        <v>2507503</v>
+        <v>223551</v>
       </c>
       <c r="H1663" s="1">
         <v>0</v>
       </c>
       <c r="I1663" s="1">
-        <v>2507503</v>
+        <v>223551</v>
       </c>
     </row>
     <row r="1664" spans="1:9" ht="12.75">
@@ -49802,19 +49802,19 @@
         <v>219</v>
       </c>
       <c r="E1664" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="F1664" s="1">
         <v>0</v>
       </c>
       <c r="G1664" s="1">
-        <v>65932</v>
+        <v>49500</v>
       </c>
       <c r="H1664" s="1">
         <v>0</v>
       </c>
       <c r="I1664" s="1">
-        <v>65932</v>
+        <v>49500</v>
       </c>
     </row>
     <row r="1665" spans="1:9" ht="12.75">
@@ -49831,19 +49831,19 @@
         <v>219</v>
       </c>
       <c r="E1665" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F1665" s="1">
         <v>0</v>
       </c>
       <c r="G1665" s="1">
-        <v>86124</v>
+        <v>2507503</v>
       </c>
       <c r="H1665" s="1">
         <v>0</v>
       </c>
       <c r="I1665" s="1">
-        <v>86124</v>
+        <v>2507503</v>
       </c>
     </row>
     <row r="1666" spans="1:9" ht="12.75">
@@ -49860,19 +49860,19 @@
         <v>219</v>
       </c>
       <c r="E1666" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F1666" s="1">
         <v>0</v>
       </c>
       <c r="G1666" s="1">
-        <v>1021380</v>
+        <v>65932</v>
       </c>
       <c r="H1666" s="1">
         <v>0</v>
       </c>
       <c r="I1666" s="1">
-        <v>1021380</v>
+        <v>65932</v>
       </c>
     </row>
     <row r="1667" spans="1:9" ht="12.75">
@@ -49889,19 +49889,19 @@
         <v>219</v>
       </c>
       <c r="E1667" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F1667" s="1">
         <v>0</v>
       </c>
       <c r="G1667" s="1">
-        <v>138789</v>
+        <v>86124</v>
       </c>
       <c r="H1667" s="1">
         <v>0</v>
       </c>
       <c r="I1667" s="1">
-        <v>138789</v>
+        <v>86124</v>
       </c>
     </row>
     <row r="1668" spans="1:9" ht="12.75">
@@ -49918,19 +49918,19 @@
         <v>219</v>
       </c>
       <c r="E1668" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="F1668" s="1">
         <v>0</v>
       </c>
       <c r="G1668" s="1">
-        <v>8288</v>
+        <v>1021380</v>
       </c>
       <c r="H1668" s="1">
         <v>0</v>
       </c>
       <c r="I1668" s="1">
-        <v>8288</v>
+        <v>1021380</v>
       </c>
     </row>
     <row r="1669" spans="1:9" ht="12.75">
@@ -49947,19 +49947,19 @@
         <v>219</v>
       </c>
       <c r="E1669" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F1669" s="1">
         <v>0</v>
       </c>
       <c r="G1669" s="1">
-        <v>219258</v>
+        <v>138789</v>
       </c>
       <c r="H1669" s="1">
         <v>0</v>
       </c>
       <c r="I1669" s="1">
-        <v>219258</v>
+        <v>138789</v>
       </c>
     </row>
     <row r="1670" spans="1:9" ht="12.75">
@@ -49976,19 +49976,19 @@
         <v>219</v>
       </c>
       <c r="E1670" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="F1670" s="1">
         <v>0</v>
       </c>
       <c r="G1670" s="1">
-        <v>4807583</v>
+        <v>8288</v>
       </c>
       <c r="H1670" s="1">
-        <v>4807583</v>
+        <v>0</v>
       </c>
       <c r="I1670" s="1">
-        <v>0</v>
+        <v>8288</v>
       </c>
     </row>
     <row r="1671" spans="1:9" ht="12.75">
@@ -50005,19 +50005,19 @@
         <v>219</v>
       </c>
       <c r="E1671" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="F1671" s="1">
         <v>0</v>
       </c>
       <c r="G1671" s="1">
-        <v>13811</v>
+        <v>219258</v>
       </c>
       <c r="H1671" s="1">
         <v>0</v>
       </c>
       <c r="I1671" s="1">
-        <v>13811</v>
+        <v>219258</v>
       </c>
     </row>
     <row r="1672" spans="1:9" ht="12.75">
@@ -50034,19 +50034,19 @@
         <v>219</v>
       </c>
       <c r="E1672" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F1672" s="1">
         <v>0</v>
       </c>
       <c r="G1672" s="1">
-        <v>729998</v>
+        <v>4807583</v>
       </c>
       <c r="H1672" s="1">
-        <v>0</v>
+        <v>4807583</v>
       </c>
       <c r="I1672" s="1">
-        <v>729998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1673" spans="1:9" ht="12.75">
@@ -50060,22 +50060,22 @@
         <v>105</v>
       </c>
       <c r="D1673" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E1673" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
       <c r="F1673" s="1">
         <v>0</v>
       </c>
       <c r="G1673" s="1">
-        <v>3734639.2300000004</v>
+        <v>13811</v>
       </c>
       <c r="H1673" s="1">
         <v>0</v>
       </c>
       <c r="I1673" s="1">
-        <v>3734639.2300000004</v>
+        <v>13811</v>
       </c>
     </row>
     <row r="1674" spans="1:9" ht="12.75">
@@ -50089,22 +50089,22 @@
         <v>105</v>
       </c>
       <c r="D1674" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E1674" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="F1674" s="1">
         <v>0</v>
       </c>
       <c r="G1674" s="1">
-        <v>289295.48</v>
+        <v>729998</v>
       </c>
       <c r="H1674" s="1">
         <v>0</v>
       </c>
       <c r="I1674" s="1">
-        <v>289295.48</v>
+        <v>729998</v>
       </c>
     </row>
     <row r="1675" spans="1:9" ht="12.75">
@@ -50121,19 +50121,19 @@
         <v>221</v>
       </c>
       <c r="E1675" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F1675" s="1">
         <v>0</v>
       </c>
       <c r="G1675" s="1">
-        <v>218609.22</v>
+        <v>3734639.2300000004</v>
       </c>
       <c r="H1675" s="1">
         <v>0</v>
       </c>
       <c r="I1675" s="1">
-        <v>218609.22</v>
+        <v>3734639.2300000004</v>
       </c>
     </row>
     <row r="1676" spans="1:9" ht="12.75">
@@ -50150,19 +50150,19 @@
         <v>221</v>
       </c>
       <c r="E1676" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F1676" s="1">
         <v>0</v>
       </c>
       <c r="G1676" s="1">
-        <v>1910663.0799999996</v>
+        <v>289295.48</v>
       </c>
       <c r="H1676" s="1">
         <v>0</v>
       </c>
       <c r="I1676" s="1">
-        <v>1910663.0799999996</v>
+        <v>289295.48</v>
       </c>
     </row>
     <row r="1677" spans="1:9" ht="12.75">
@@ -50179,19 +50179,19 @@
         <v>221</v>
       </c>
       <c r="E1677" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F1677" s="1">
         <v>0</v>
       </c>
       <c r="G1677" s="1">
-        <v>685737.61</v>
+        <v>218609.21999999997</v>
       </c>
       <c r="H1677" s="1">
         <v>0</v>
       </c>
       <c r="I1677" s="1">
-        <v>685737.61</v>
+        <v>218609.21999999997</v>
       </c>
     </row>
     <row r="1678" spans="1:9" ht="12.75">
@@ -50208,19 +50208,19 @@
         <v>221</v>
       </c>
       <c r="E1678" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="F1678" s="1">
         <v>0</v>
       </c>
       <c r="G1678" s="1">
-        <v>4078.70</v>
+        <v>1910663.08</v>
       </c>
       <c r="H1678" s="1">
         <v>0</v>
       </c>
       <c r="I1678" s="1">
-        <v>4078.70</v>
+        <v>1910663.08</v>
       </c>
     </row>
     <row r="1679" spans="1:9" ht="12.75">
@@ -50237,19 +50237,19 @@
         <v>221</v>
       </c>
       <c r="E1679" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="F1679" s="1">
         <v>0</v>
       </c>
       <c r="G1679" s="1">
-        <v>191355.02</v>
+        <v>685737.6100000001</v>
       </c>
       <c r="H1679" s="1">
         <v>0</v>
       </c>
       <c r="I1679" s="1">
-        <v>191355.02</v>
+        <v>685737.6100000001</v>
       </c>
     </row>
     <row r="1680" spans="1:9" ht="12.75">
@@ -50266,19 +50266,19 @@
         <v>221</v>
       </c>
       <c r="E1680" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F1680" s="1">
         <v>0</v>
       </c>
       <c r="G1680" s="1">
-        <v>381348.31999999995</v>
+        <v>4078.70</v>
       </c>
       <c r="H1680" s="1">
         <v>0</v>
       </c>
       <c r="I1680" s="1">
-        <v>381348.31999999995</v>
+        <v>4078.70</v>
       </c>
     </row>
     <row r="1681" spans="1:9" ht="12.75">
@@ -50295,19 +50295,19 @@
         <v>221</v>
       </c>
       <c r="E1681" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F1681" s="1">
         <v>0</v>
       </c>
       <c r="G1681" s="1">
-        <v>93497</v>
+        <v>191355.02</v>
       </c>
       <c r="H1681" s="1">
         <v>0</v>
       </c>
       <c r="I1681" s="1">
-        <v>93497</v>
+        <v>191355.02</v>
       </c>
     </row>
     <row r="1682" spans="1:9" ht="12.75">
@@ -50324,19 +50324,19 @@
         <v>221</v>
       </c>
       <c r="E1682" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="F1682" s="1">
         <v>0</v>
       </c>
       <c r="G1682" s="1">
-        <v>211054</v>
+        <v>381348.31999999995</v>
       </c>
       <c r="H1682" s="1">
         <v>0</v>
       </c>
       <c r="I1682" s="1">
-        <v>211054</v>
+        <v>381348.31999999995</v>
       </c>
     </row>
     <row r="1683" spans="1:9" ht="12.75">
@@ -50353,19 +50353,19 @@
         <v>221</v>
       </c>
       <c r="E1683" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F1683" s="1">
         <v>0</v>
       </c>
       <c r="G1683" s="1">
-        <v>1105942</v>
+        <v>93497</v>
       </c>
       <c r="H1683" s="1">
         <v>0</v>
       </c>
       <c r="I1683" s="1">
-        <v>1105942</v>
+        <v>93497</v>
       </c>
     </row>
     <row r="1684" spans="1:9" ht="12.75">
@@ -50379,22 +50379,22 @@
         <v>105</v>
       </c>
       <c r="D1684" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E1684" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="F1684" s="1">
         <v>0</v>
       </c>
       <c r="G1684" s="1">
-        <v>1711047.58</v>
+        <v>211054</v>
       </c>
       <c r="H1684" s="1">
         <v>0</v>
       </c>
       <c r="I1684" s="1">
-        <v>1711047.58</v>
+        <v>211054</v>
       </c>
     </row>
     <row r="1685" spans="1:9" ht="12.75">
@@ -50408,22 +50408,22 @@
         <v>105</v>
       </c>
       <c r="D1685" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E1685" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="F1685" s="1">
         <v>0</v>
       </c>
       <c r="G1685" s="1">
-        <v>1338867.5899999999</v>
+        <v>1105942</v>
       </c>
       <c r="H1685" s="1">
         <v>0</v>
       </c>
       <c r="I1685" s="1">
-        <v>1338867.5899999999</v>
+        <v>1105942</v>
       </c>
     </row>
     <row r="1686" spans="1:9" ht="12.75">
@@ -50440,19 +50440,19 @@
         <v>222</v>
       </c>
       <c r="E1686" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F1686" s="1">
         <v>0</v>
       </c>
       <c r="G1686" s="1">
-        <v>6084145</v>
+        <v>1711047.58</v>
       </c>
       <c r="H1686" s="1">
         <v>0</v>
       </c>
       <c r="I1686" s="1">
-        <v>6084145</v>
+        <v>1711047.58</v>
       </c>
     </row>
     <row r="1687" spans="1:9" ht="12.75">
@@ -50469,19 +50469,19 @@
         <v>222</v>
       </c>
       <c r="E1687" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1687" s="1">
         <v>0</v>
       </c>
       <c r="G1687" s="1">
-        <v>492996</v>
+        <v>1338867.5899999999</v>
       </c>
       <c r="H1687" s="1">
         <v>0</v>
       </c>
       <c r="I1687" s="1">
-        <v>492996</v>
+        <v>1338867.5899999999</v>
       </c>
     </row>
     <row r="1688" spans="1:9" ht="12.75">
@@ -50498,19 +50498,19 @@
         <v>222</v>
       </c>
       <c r="E1688" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F1688" s="1">
         <v>0</v>
       </c>
       <c r="G1688" s="1">
-        <v>351533</v>
+        <v>6084145</v>
       </c>
       <c r="H1688" s="1">
         <v>0</v>
       </c>
       <c r="I1688" s="1">
-        <v>351533</v>
+        <v>6084145</v>
       </c>
     </row>
     <row r="1689" spans="1:9" ht="12.75">
@@ -50527,19 +50527,19 @@
         <v>222</v>
       </c>
       <c r="E1689" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F1689" s="1">
         <v>0</v>
       </c>
       <c r="G1689" s="1">
-        <v>10682502</v>
+        <v>492996</v>
       </c>
       <c r="H1689" s="1">
         <v>0</v>
       </c>
       <c r="I1689" s="1">
-        <v>10682502</v>
+        <v>492996</v>
       </c>
     </row>
     <row r="1690" spans="1:9" ht="12.75">
@@ -50556,19 +50556,19 @@
         <v>222</v>
       </c>
       <c r="E1690" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F1690" s="1">
         <v>0</v>
       </c>
       <c r="G1690" s="1">
-        <v>992656</v>
+        <v>351533</v>
       </c>
       <c r="H1690" s="1">
         <v>0</v>
       </c>
       <c r="I1690" s="1">
-        <v>992656</v>
+        <v>351533</v>
       </c>
     </row>
     <row r="1691" spans="1:9" ht="12.75">
@@ -50585,19 +50585,19 @@
         <v>222</v>
       </c>
       <c r="E1691" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="F1691" s="1">
         <v>0</v>
       </c>
       <c r="G1691" s="1">
-        <v>12048</v>
+        <v>10682502</v>
       </c>
       <c r="H1691" s="1">
         <v>0</v>
       </c>
       <c r="I1691" s="1">
-        <v>12048</v>
+        <v>10682502</v>
       </c>
     </row>
     <row r="1692" spans="1:9" ht="12.75">
@@ -50614,19 +50614,19 @@
         <v>222</v>
       </c>
       <c r="E1692" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="F1692" s="1">
         <v>0</v>
       </c>
       <c r="G1692" s="1">
-        <v>25244</v>
+        <v>992656</v>
       </c>
       <c r="H1692" s="1">
         <v>0</v>
       </c>
       <c r="I1692" s="1">
-        <v>25244</v>
+        <v>992656</v>
       </c>
     </row>
     <row r="1693" spans="1:9" ht="12.75">
@@ -50643,19 +50643,19 @@
         <v>222</v>
       </c>
       <c r="E1693" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F1693" s="1">
         <v>0</v>
       </c>
       <c r="G1693" s="1">
-        <v>288601</v>
+        <v>12048</v>
       </c>
       <c r="H1693" s="1">
         <v>0</v>
       </c>
       <c r="I1693" s="1">
-        <v>288601</v>
+        <v>12048</v>
       </c>
     </row>
     <row r="1694" spans="1:9" ht="12.75">
@@ -50672,19 +50672,19 @@
         <v>222</v>
       </c>
       <c r="E1694" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="F1694" s="1">
         <v>0</v>
       </c>
       <c r="G1694" s="1">
-        <v>1595017</v>
+        <v>25244</v>
       </c>
       <c r="H1694" s="1">
         <v>0</v>
       </c>
       <c r="I1694" s="1">
-        <v>1595017</v>
+        <v>25244</v>
       </c>
     </row>
     <row r="1695" spans="1:9" ht="12.75">
@@ -50701,19 +50701,19 @@
         <v>222</v>
       </c>
       <c r="E1695" t="s">
-        <v>350</v>
+        <v>336</v>
       </c>
       <c r="F1695" s="1">
         <v>0</v>
       </c>
       <c r="G1695" s="1">
-        <v>100146</v>
+        <v>288601</v>
       </c>
       <c r="H1695" s="1">
         <v>0</v>
       </c>
       <c r="I1695" s="1">
-        <v>100146</v>
+        <v>288601</v>
       </c>
     </row>
     <row r="1696" spans="1:9" ht="12.75">
@@ -50730,19 +50730,19 @@
         <v>222</v>
       </c>
       <c r="E1696" t="s">
-        <v>351</v>
+        <v>337</v>
       </c>
       <c r="F1696" s="1">
         <v>0</v>
       </c>
       <c r="G1696" s="1">
-        <v>279211</v>
+        <v>1595017</v>
       </c>
       <c r="H1696" s="1">
         <v>0</v>
       </c>
       <c r="I1696" s="1">
-        <v>279211</v>
+        <v>1595017</v>
       </c>
     </row>
     <row r="1697" spans="1:9" ht="12.75">
@@ -50759,19 +50759,19 @@
         <v>222</v>
       </c>
       <c r="E1697" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="F1697" s="1">
         <v>0</v>
       </c>
       <c r="G1697" s="1">
-        <v>227931</v>
+        <v>100146</v>
       </c>
       <c r="H1697" s="1">
         <v>0</v>
       </c>
       <c r="I1697" s="1">
-        <v>227931</v>
+        <v>100146</v>
       </c>
     </row>
     <row r="1698" spans="1:9" ht="12.75">
@@ -50788,19 +50788,19 @@
         <v>222</v>
       </c>
       <c r="E1698" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F1698" s="1">
         <v>0</v>
       </c>
       <c r="G1698" s="1">
-        <v>53925</v>
+        <v>279211</v>
       </c>
       <c r="H1698" s="1">
         <v>0</v>
       </c>
       <c r="I1698" s="1">
-        <v>53925</v>
+        <v>279211</v>
       </c>
     </row>
     <row r="1699" spans="1:9" ht="12.75">
@@ -50814,22 +50814,22 @@
         <v>105</v>
       </c>
       <c r="D1699" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E1699" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="F1699" s="1">
         <v>0</v>
       </c>
       <c r="G1699" s="1">
-        <v>0</v>
+        <v>227931</v>
       </c>
       <c r="H1699" s="1">
-        <v>2.423587017E7</v>
+        <v>0</v>
       </c>
       <c r="I1699" s="1">
-        <v>-2.423587017E7</v>
+        <v>227931</v>
       </c>
     </row>
     <row r="1700" spans="1:9" ht="12.75">
@@ -50843,22 +50843,22 @@
         <v>105</v>
       </c>
       <c r="D1700" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E1700" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="F1700" s="1">
         <v>0</v>
       </c>
       <c r="G1700" s="1">
-        <v>119165</v>
+        <v>53925</v>
       </c>
       <c r="H1700" s="1">
         <v>0</v>
       </c>
       <c r="I1700" s="1">
-        <v>119165</v>
+        <v>53925</v>
       </c>
     </row>
     <row r="1701" spans="1:9" ht="12.75">
@@ -50872,22 +50872,22 @@
         <v>105</v>
       </c>
       <c r="D1701" t="s">
-        <v>307</v>
+        <v>224</v>
       </c>
       <c r="E1701" t="s">
-        <v>328</v>
+        <v>348</v>
       </c>
       <c r="F1701" s="1">
         <v>0</v>
       </c>
       <c r="G1701" s="1">
-        <v>10532</v>
+        <v>0</v>
       </c>
       <c r="H1701" s="1">
-        <v>0</v>
+        <v>2.423587017E7</v>
       </c>
       <c r="I1701" s="1">
-        <v>10532</v>
+        <v>-2.423587017E7</v>
       </c>
     </row>
     <row r="1702" spans="1:9" ht="12.75">
@@ -50901,22 +50901,22 @@
         <v>105</v>
       </c>
       <c r="D1702" t="s">
-        <v>307</v>
+        <v>225</v>
       </c>
       <c r="E1702" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="F1702" s="1">
         <v>0</v>
       </c>
       <c r="G1702" s="1">
-        <v>1417</v>
+        <v>119165</v>
       </c>
       <c r="H1702" s="1">
         <v>0</v>
       </c>
       <c r="I1702" s="1">
-        <v>1417</v>
+        <v>119165</v>
       </c>
     </row>
     <row r="1703" spans="1:9" ht="12.75">
@@ -50933,19 +50933,19 @@
         <v>307</v>
       </c>
       <c r="E1703" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F1703" s="1">
         <v>0</v>
       </c>
       <c r="G1703" s="1">
-        <v>88200</v>
+        <v>10532</v>
       </c>
       <c r="H1703" s="1">
         <v>0</v>
       </c>
       <c r="I1703" s="1">
-        <v>88200</v>
+        <v>10532</v>
       </c>
     </row>
     <row r="1704" spans="1:9" ht="12.75">
@@ -50962,19 +50962,19 @@
         <v>307</v>
       </c>
       <c r="E1704" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1704" s="1">
         <v>0</v>
       </c>
       <c r="G1704" s="1">
-        <v>3374</v>
+        <v>1417</v>
       </c>
       <c r="H1704" s="1">
         <v>0</v>
       </c>
       <c r="I1704" s="1">
-        <v>3374</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="1705" spans="1:9" ht="12.75">
@@ -50991,19 +50991,19 @@
         <v>307</v>
       </c>
       <c r="E1705" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F1705" s="1">
         <v>0</v>
       </c>
       <c r="G1705" s="1">
-        <v>5996</v>
+        <v>88200</v>
       </c>
       <c r="H1705" s="1">
         <v>0</v>
       </c>
       <c r="I1705" s="1">
-        <v>5996</v>
+        <v>88200</v>
       </c>
     </row>
     <row r="1706" spans="1:9" ht="12.75">
@@ -51020,19 +51020,19 @@
         <v>307</v>
       </c>
       <c r="E1706" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F1706" s="1">
         <v>0</v>
       </c>
       <c r="G1706" s="1">
-        <v>22800</v>
+        <v>3374</v>
       </c>
       <c r="H1706" s="1">
         <v>0</v>
       </c>
       <c r="I1706" s="1">
-        <v>22800</v>
+        <v>3374</v>
       </c>
     </row>
     <row r="1707" spans="1:9" ht="12.75">
@@ -51049,19 +51049,19 @@
         <v>307</v>
       </c>
       <c r="E1707" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F1707" s="1">
         <v>0</v>
       </c>
       <c r="G1707" s="1">
-        <v>12631</v>
+        <v>5996</v>
       </c>
       <c r="H1707" s="1">
         <v>0</v>
       </c>
       <c r="I1707" s="1">
-        <v>12631</v>
+        <v>5996</v>
       </c>
     </row>
     <row r="1708" spans="1:9" ht="12.75">
@@ -51078,19 +51078,19 @@
         <v>307</v>
       </c>
       <c r="E1708" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="F1708" s="1">
         <v>0</v>
       </c>
       <c r="G1708" s="1">
-        <v>179</v>
+        <v>22800</v>
       </c>
       <c r="H1708" s="1">
         <v>0</v>
       </c>
       <c r="I1708" s="1">
-        <v>179</v>
+        <v>22800</v>
       </c>
     </row>
     <row r="1709" spans="1:9" ht="12.75">
@@ -51107,19 +51107,19 @@
         <v>307</v>
       </c>
       <c r="E1709" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="F1709" s="1">
         <v>0</v>
       </c>
       <c r="G1709" s="1">
-        <v>1584</v>
+        <v>12631</v>
       </c>
       <c r="H1709" s="1">
         <v>0</v>
       </c>
       <c r="I1709" s="1">
-        <v>1584</v>
+        <v>12631</v>
       </c>
     </row>
     <row r="1710" spans="1:9" ht="12.75">
@@ -51136,19 +51136,19 @@
         <v>307</v>
       </c>
       <c r="E1710" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F1710" s="1">
         <v>0</v>
       </c>
       <c r="G1710" s="1">
-        <v>10660</v>
+        <v>179</v>
       </c>
       <c r="H1710" s="1">
         <v>0</v>
       </c>
       <c r="I1710" s="1">
-        <v>10660</v>
+        <v>179</v>
       </c>
     </row>
     <row r="1711" spans="1:9" ht="12.75">
@@ -51165,19 +51165,19 @@
         <v>307</v>
       </c>
       <c r="E1711" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F1711" s="1">
         <v>0</v>
       </c>
       <c r="G1711" s="1">
-        <v>154499</v>
+        <v>1584</v>
       </c>
       <c r="H1711" s="1">
-        <v>154499</v>
+        <v>0</v>
       </c>
       <c r="I1711" s="1">
-        <v>0</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="1712" spans="1:9" ht="12.75">
@@ -51194,19 +51194,19 @@
         <v>307</v>
       </c>
       <c r="E1712" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="F1712" s="1">
         <v>0</v>
       </c>
       <c r="G1712" s="1">
-        <v>249</v>
+        <v>10660</v>
       </c>
       <c r="H1712" s="1">
         <v>0</v>
       </c>
       <c r="I1712" s="1">
-        <v>249</v>
+        <v>10660</v>
       </c>
     </row>
     <row r="1713" spans="1:9" ht="12.75">
@@ -51223,19 +51223,19 @@
         <v>307</v>
       </c>
       <c r="E1713" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F1713" s="1">
         <v>0</v>
       </c>
       <c r="G1713" s="1">
-        <v>375</v>
+        <v>154499</v>
       </c>
       <c r="H1713" s="1">
-        <v>0</v>
+        <v>154499</v>
       </c>
       <c r="I1713" s="1">
-        <v>375</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1714" spans="1:9" ht="12.75">
@@ -51252,19 +51252,19 @@
         <v>307</v>
       </c>
       <c r="E1714" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F1714" s="1">
         <v>0</v>
       </c>
       <c r="G1714" s="1">
-        <v>667</v>
+        <v>249</v>
       </c>
       <c r="H1714" s="1">
         <v>0</v>
       </c>
       <c r="I1714" s="1">
-        <v>667</v>
+        <v>249</v>
       </c>
     </row>
     <row r="1715" spans="1:9" ht="12.75">
@@ -51278,22 +51278,22 @@
         <v>105</v>
       </c>
       <c r="D1715" t="s">
-        <v>228</v>
+        <v>307</v>
       </c>
       <c r="E1715" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="F1715" s="1">
         <v>0</v>
       </c>
       <c r="G1715" s="1">
-        <v>121502</v>
+        <v>375</v>
       </c>
       <c r="H1715" s="1">
         <v>0</v>
       </c>
       <c r="I1715" s="1">
-        <v>121502</v>
+        <v>375</v>
       </c>
     </row>
     <row r="1716" spans="1:9" ht="12.75">
@@ -51307,22 +51307,22 @@
         <v>105</v>
       </c>
       <c r="D1716" t="s">
-        <v>233</v>
+        <v>307</v>
       </c>
       <c r="E1716" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="F1716" s="1">
         <v>0</v>
       </c>
       <c r="G1716" s="1">
-        <v>3500</v>
+        <v>667</v>
       </c>
       <c r="H1716" s="1">
         <v>0</v>
       </c>
       <c r="I1716" s="1">
-        <v>3500</v>
+        <v>667</v>
       </c>
     </row>
     <row r="1717" spans="1:9" ht="12.75">
@@ -51336,22 +51336,22 @@
         <v>105</v>
       </c>
       <c r="D1717" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="E1717" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="F1717" s="1">
         <v>0</v>
       </c>
       <c r="G1717" s="1">
-        <v>9000</v>
+        <v>121502</v>
       </c>
       <c r="H1717" s="1">
         <v>0</v>
       </c>
       <c r="I1717" s="1">
-        <v>9000</v>
+        <v>121502</v>
       </c>
     </row>
     <row r="1718" spans="1:9" ht="12.75">
@@ -51365,22 +51365,22 @@
         <v>105</v>
       </c>
       <c r="D1718" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E1718" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
       <c r="F1718" s="1">
         <v>0</v>
       </c>
       <c r="G1718" s="1">
-        <v>516448</v>
+        <v>3500</v>
       </c>
       <c r="H1718" s="1">
         <v>0</v>
       </c>
       <c r="I1718" s="1">
-        <v>516448</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="1719" spans="1:9" ht="12.75">
@@ -51394,22 +51394,22 @@
         <v>105</v>
       </c>
       <c r="D1719" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E1719" t="s">
-        <v>244</v>
+        <v>342</v>
       </c>
       <c r="F1719" s="1">
         <v>0</v>
       </c>
       <c r="G1719" s="1">
-        <v>853156</v>
+        <v>9000</v>
       </c>
       <c r="H1719" s="1">
         <v>0</v>
       </c>
       <c r="I1719" s="1">
-        <v>853156</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="1720" spans="1:9" ht="12.75">
@@ -51423,22 +51423,22 @@
         <v>105</v>
       </c>
       <c r="D1720" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E1720" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="F1720" s="1">
         <v>0</v>
       </c>
       <c r="G1720" s="1">
-        <v>1317706</v>
+        <v>516448</v>
       </c>
       <c r="H1720" s="1">
         <v>0</v>
       </c>
       <c r="I1720" s="1">
-        <v>1317706</v>
+        <v>516448</v>
       </c>
     </row>
     <row r="1721" spans="1:9" ht="12.75">
@@ -51455,19 +51455,19 @@
         <v>235</v>
       </c>
       <c r="E1721" t="s">
-        <v>351</v>
+        <v>244</v>
       </c>
       <c r="F1721" s="1">
         <v>0</v>
       </c>
       <c r="G1721" s="1">
-        <v>3665552</v>
+        <v>853156</v>
       </c>
       <c r="H1721" s="1">
         <v>0</v>
       </c>
       <c r="I1721" s="1">
-        <v>3665552</v>
+        <v>853156</v>
       </c>
     </row>
     <row r="1722" spans="1:9" ht="12.75">
@@ -51484,19 +51484,19 @@
         <v>235</v>
       </c>
       <c r="E1722" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="F1722" s="1">
         <v>0</v>
       </c>
       <c r="G1722" s="1">
-        <v>2999088</v>
+        <v>1317706</v>
       </c>
       <c r="H1722" s="1">
         <v>0</v>
       </c>
       <c r="I1722" s="1">
-        <v>2999088</v>
+        <v>1317706</v>
       </c>
     </row>
     <row r="1723" spans="1:9" ht="12.75">
@@ -51513,19 +51513,19 @@
         <v>235</v>
       </c>
       <c r="E1723" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F1723" s="1">
         <v>0</v>
       </c>
       <c r="G1723" s="1">
-        <v>709534</v>
+        <v>3665552</v>
       </c>
       <c r="H1723" s="1">
         <v>0</v>
       </c>
       <c r="I1723" s="1">
-        <v>709534</v>
+        <v>3665552</v>
       </c>
     </row>
     <row r="1724" spans="1:9" ht="12.75">
@@ -51539,22 +51539,22 @@
         <v>105</v>
       </c>
       <c r="D1724" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E1724" t="s">
-        <v>329</v>
+        <v>352</v>
       </c>
       <c r="F1724" s="1">
         <v>0</v>
       </c>
       <c r="G1724" s="1">
-        <v>32840</v>
+        <v>2999088</v>
       </c>
       <c r="H1724" s="1">
         <v>0</v>
       </c>
       <c r="I1724" s="1">
-        <v>32840</v>
+        <v>2999088</v>
       </c>
     </row>
     <row r="1725" spans="1:9" ht="12.75">
@@ -51568,22 +51568,22 @@
         <v>105</v>
       </c>
       <c r="D1725" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E1725" t="s">
-        <v>328</v>
+        <v>353</v>
       </c>
       <c r="F1725" s="1">
         <v>0</v>
       </c>
       <c r="G1725" s="1">
-        <v>212400</v>
+        <v>709534</v>
       </c>
       <c r="H1725" s="1">
         <v>0</v>
       </c>
       <c r="I1725" s="1">
-        <v>212400</v>
+        <v>709534</v>
       </c>
     </row>
     <row r="1726" spans="1:9" ht="12.75">
@@ -51597,7 +51597,7 @@
         <v>105</v>
       </c>
       <c r="D1726" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E1726" t="s">
         <v>329</v>
@@ -51606,13 +51606,13 @@
         <v>0</v>
       </c>
       <c r="G1726" s="1">
-        <v>577360</v>
+        <v>32840</v>
       </c>
       <c r="H1726" s="1">
         <v>0</v>
       </c>
       <c r="I1726" s="1">
-        <v>577360</v>
+        <v>32840</v>
       </c>
     </row>
     <row r="1727" spans="1:9" ht="12.75">
@@ -51629,19 +51629,19 @@
         <v>238</v>
       </c>
       <c r="E1727" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F1727" s="1">
         <v>0</v>
       </c>
       <c r="G1727" s="1">
-        <v>518969</v>
+        <v>212400</v>
       </c>
       <c r="H1727" s="1">
         <v>0</v>
       </c>
       <c r="I1727" s="1">
-        <v>518969</v>
+        <v>212400</v>
       </c>
     </row>
     <row r="1728" spans="1:9" ht="12.75">
@@ -51658,19 +51658,19 @@
         <v>238</v>
       </c>
       <c r="E1728" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="F1728" s="1">
         <v>0</v>
       </c>
       <c r="G1728" s="1">
-        <v>271070</v>
+        <v>577360</v>
       </c>
       <c r="H1728" s="1">
         <v>0</v>
       </c>
       <c r="I1728" s="1">
-        <v>271070</v>
+        <v>577360</v>
       </c>
     </row>
     <row r="1729" spans="1:9" ht="12.75">
@@ -51687,19 +51687,19 @@
         <v>238</v>
       </c>
       <c r="E1729" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="F1729" s="1">
         <v>0</v>
       </c>
       <c r="G1729" s="1">
-        <v>137184</v>
+        <v>518969</v>
       </c>
       <c r="H1729" s="1">
         <v>0</v>
       </c>
       <c r="I1729" s="1">
-        <v>137184</v>
+        <v>518969</v>
       </c>
     </row>
     <row r="1730" spans="1:9" ht="12.75">
@@ -51716,19 +51716,19 @@
         <v>238</v>
       </c>
       <c r="E1730" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="F1730" s="1">
         <v>0</v>
       </c>
       <c r="G1730" s="1">
-        <v>91456</v>
+        <v>271070</v>
       </c>
       <c r="H1730" s="1">
         <v>0</v>
       </c>
       <c r="I1730" s="1">
-        <v>91456</v>
+        <v>271070</v>
       </c>
     </row>
     <row r="1731" spans="1:9" ht="12.75">
@@ -51745,19 +51745,19 @@
         <v>238</v>
       </c>
       <c r="E1731" t="s">
-        <v>351</v>
+        <v>334</v>
       </c>
       <c r="F1731" s="1">
         <v>0</v>
       </c>
       <c r="G1731" s="1">
-        <v>8275</v>
+        <v>137184</v>
       </c>
       <c r="H1731" s="1">
         <v>0</v>
       </c>
       <c r="I1731" s="1">
-        <v>8275</v>
+        <v>137184</v>
       </c>
     </row>
     <row r="1732" spans="1:9" ht="12.75">
@@ -51774,19 +51774,19 @@
         <v>238</v>
       </c>
       <c r="E1732" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="F1732" s="1">
         <v>0</v>
       </c>
       <c r="G1732" s="1">
-        <v>104725</v>
+        <v>91456</v>
       </c>
       <c r="H1732" s="1">
         <v>0</v>
       </c>
       <c r="I1732" s="1">
-        <v>104725</v>
+        <v>91456</v>
       </c>
     </row>
     <row r="1733" spans="1:9" ht="12.75">
@@ -51800,22 +51800,22 @@
         <v>105</v>
       </c>
       <c r="D1733" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E1733" t="s">
-        <v>329</v>
+        <v>351</v>
       </c>
       <c r="F1733" s="1">
         <v>0</v>
       </c>
       <c r="G1733" s="1">
-        <v>8770</v>
+        <v>8275</v>
       </c>
       <c r="H1733" s="1">
         <v>0</v>
       </c>
       <c r="I1733" s="1">
-        <v>8770</v>
+        <v>8275</v>
       </c>
     </row>
     <row r="1734" spans="1:9" ht="12.75">
@@ -51829,22 +51829,22 @@
         <v>105</v>
       </c>
       <c r="D1734" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E1734" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="F1734" s="1">
         <v>0</v>
       </c>
       <c r="G1734" s="1">
-        <v>77798.34</v>
+        <v>104725</v>
       </c>
       <c r="H1734" s="1">
         <v>0</v>
       </c>
       <c r="I1734" s="1">
-        <v>77798.34</v>
+        <v>104725</v>
       </c>
     </row>
     <row r="1735" spans="1:9" ht="12.75">
@@ -51858,22 +51858,22 @@
         <v>105</v>
       </c>
       <c r="D1735" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E1735" t="s">
-        <v>13</v>
+        <v>329</v>
       </c>
       <c r="F1735" s="1">
         <v>0</v>
       </c>
       <c r="G1735" s="1">
-        <v>0.90</v>
+        <v>8770</v>
       </c>
       <c r="H1735" s="1">
-        <v>12.20</v>
+        <v>0</v>
       </c>
       <c r="I1735" s="1">
-        <v>-11.30</v>
+        <v>8770</v>
       </c>
     </row>
     <row r="1736" spans="1:9" ht="12.75">
@@ -51887,22 +51887,22 @@
         <v>105</v>
       </c>
       <c r="D1736" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="E1736" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F1736" s="1">
         <v>0</v>
       </c>
       <c r="G1736" s="1">
-        <v>8760</v>
+        <v>77798.34</v>
       </c>
       <c r="H1736" s="1">
         <v>0</v>
       </c>
       <c r="I1736" s="1">
-        <v>8760</v>
+        <v>77798.34</v>
       </c>
     </row>
     <row r="1737" spans="1:9" ht="12.75">
@@ -51916,22 +51916,22 @@
         <v>105</v>
       </c>
       <c r="D1737" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E1737" t="s">
-        <v>330</v>
+        <v>13</v>
       </c>
       <c r="F1737" s="1">
         <v>0</v>
       </c>
       <c r="G1737" s="1">
-        <v>3533773</v>
+        <v>0.90</v>
       </c>
       <c r="H1737" s="1">
-        <v>0</v>
+        <v>12.20</v>
       </c>
       <c r="I1737" s="1">
-        <v>3533773</v>
+        <v>-11.30</v>
       </c>
     </row>
     <row r="1738" spans="1:9" ht="12.75">
@@ -51948,19 +51948,19 @@
         <v>243</v>
       </c>
       <c r="E1738" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="F1738" s="1">
         <v>0</v>
       </c>
       <c r="G1738" s="1">
-        <v>117363390</v>
+        <v>8760</v>
       </c>
       <c r="H1738" s="1">
         <v>0</v>
       </c>
       <c r="I1738" s="1">
-        <v>117363390</v>
+        <v>8760</v>
       </c>
     </row>
     <row r="1739" spans="1:9" ht="12.75">
@@ -51977,19 +51977,19 @@
         <v>243</v>
       </c>
       <c r="E1739" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="F1739" s="1">
         <v>0</v>
       </c>
       <c r="G1739" s="1">
-        <v>16245060</v>
+        <v>3533773</v>
       </c>
       <c r="H1739" s="1">
         <v>0</v>
       </c>
       <c r="I1739" s="1">
-        <v>16245060</v>
+        <v>3533773</v>
       </c>
     </row>
     <row r="1740" spans="1:9" ht="12.75">
@@ -52006,19 +52006,19 @@
         <v>243</v>
       </c>
       <c r="E1740" t="s">
-        <v>354</v>
+        <v>333</v>
       </c>
       <c r="F1740" s="1">
         <v>0</v>
       </c>
       <c r="G1740" s="1">
-        <v>6372000</v>
+        <v>117363390</v>
       </c>
       <c r="H1740" s="1">
         <v>0</v>
       </c>
       <c r="I1740" s="1">
-        <v>6372000</v>
+        <v>117363390</v>
       </c>
     </row>
     <row r="1741" spans="1:9" ht="12.75">
@@ -52035,19 +52035,19 @@
         <v>243</v>
       </c>
       <c r="E1741" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F1741" s="1">
         <v>0</v>
       </c>
       <c r="G1741" s="1">
-        <v>12266100</v>
+        <v>16245060</v>
       </c>
       <c r="H1741" s="1">
         <v>0</v>
       </c>
       <c r="I1741" s="1">
-        <v>12266100</v>
+        <v>16245060</v>
       </c>
     </row>
     <row r="1742" spans="1:9" ht="12.75">
@@ -52064,19 +52064,19 @@
         <v>243</v>
       </c>
       <c r="E1742" t="s">
-        <v>340</v>
+        <v>354</v>
       </c>
       <c r="F1742" s="1">
         <v>0</v>
       </c>
       <c r="G1742" s="1">
-        <v>41158322</v>
+        <v>6372000</v>
       </c>
       <c r="H1742" s="1">
         <v>0</v>
       </c>
       <c r="I1742" s="1">
-        <v>41158322</v>
+        <v>6372000</v>
       </c>
     </row>
     <row r="1743" spans="1:9" ht="12.75">
@@ -52093,19 +52093,19 @@
         <v>243</v>
       </c>
       <c r="E1743" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="F1743" s="1">
         <v>0</v>
       </c>
       <c r="G1743" s="1">
-        <v>1194533</v>
+        <v>12266100</v>
       </c>
       <c r="H1743" s="1">
         <v>0</v>
       </c>
       <c r="I1743" s="1">
-        <v>1194533</v>
+        <v>12266100</v>
       </c>
     </row>
     <row r="1744" spans="1:9" ht="12.75">
@@ -52122,19 +52122,19 @@
         <v>243</v>
       </c>
       <c r="E1744" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="F1744" s="1">
         <v>0</v>
       </c>
       <c r="G1744" s="1">
-        <v>2017937</v>
+        <v>41158322</v>
       </c>
       <c r="H1744" s="1">
         <v>0</v>
       </c>
       <c r="I1744" s="1">
-        <v>2017937</v>
+        <v>41158322</v>
       </c>
     </row>
     <row r="1745" spans="1:9" ht="12.75">
@@ -52148,22 +52148,22 @@
         <v>105</v>
       </c>
       <c r="D1745" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1745" t="s">
-        <v>330</v>
+        <v>346</v>
       </c>
       <c r="F1745" s="1">
         <v>0</v>
       </c>
       <c r="G1745" s="1">
-        <v>31481</v>
+        <v>1194533</v>
       </c>
       <c r="H1745" s="1">
         <v>0</v>
       </c>
       <c r="I1745" s="1">
-        <v>31481</v>
+        <v>1194533</v>
       </c>
     </row>
     <row r="1746" spans="1:9" ht="12.75">
@@ -52177,22 +52177,22 @@
         <v>105</v>
       </c>
       <c r="D1746" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1746" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
       <c r="F1746" s="1">
         <v>0</v>
       </c>
       <c r="G1746" s="1">
-        <v>6638</v>
+        <v>2017937</v>
       </c>
       <c r="H1746" s="1">
         <v>0</v>
       </c>
       <c r="I1746" s="1">
-        <v>6638</v>
+        <v>2017937</v>
       </c>
     </row>
     <row r="1747" spans="1:9" ht="12.75">
@@ -52209,19 +52209,19 @@
         <v>246</v>
       </c>
       <c r="E1747" t="s">
-        <v>355</v>
+        <v>330</v>
       </c>
       <c r="F1747" s="1">
         <v>0</v>
       </c>
       <c r="G1747" s="1">
-        <v>7140</v>
+        <v>31481</v>
       </c>
       <c r="H1747" s="1">
         <v>0</v>
       </c>
       <c r="I1747" s="1">
-        <v>7140</v>
+        <v>31481</v>
       </c>
     </row>
     <row r="1748" spans="1:9" ht="12.75">
@@ -52238,19 +52238,19 @@
         <v>246</v>
       </c>
       <c r="E1748" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="F1748" s="1">
         <v>0</v>
       </c>
       <c r="G1748" s="1">
-        <v>41204</v>
+        <v>6638</v>
       </c>
       <c r="H1748" s="1">
         <v>0</v>
       </c>
       <c r="I1748" s="1">
-        <v>41204</v>
+        <v>6638</v>
       </c>
     </row>
     <row r="1749" spans="1:9" ht="12.75">
@@ -52264,22 +52264,22 @@
         <v>105</v>
       </c>
       <c r="D1749" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E1749" t="s">
-        <v>328</v>
+        <v>355</v>
       </c>
       <c r="F1749" s="1">
         <v>0</v>
       </c>
       <c r="G1749" s="1">
-        <v>77571</v>
+        <v>7140</v>
       </c>
       <c r="H1749" s="1">
         <v>0</v>
       </c>
       <c r="I1749" s="1">
-        <v>77571</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="1750" spans="1:9" ht="12.75">
@@ -52293,22 +52293,22 @@
         <v>105</v>
       </c>
       <c r="D1750" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E1750" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="F1750" s="1">
         <v>0</v>
       </c>
       <c r="G1750" s="1">
-        <v>1513824</v>
+        <v>41204</v>
       </c>
       <c r="H1750" s="1">
         <v>0</v>
       </c>
       <c r="I1750" s="1">
-        <v>1513824</v>
+        <v>41204</v>
       </c>
     </row>
     <row r="1751" spans="1:9" ht="12.75">
@@ -52325,19 +52325,19 @@
         <v>247</v>
       </c>
       <c r="E1751" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="F1751" s="1">
         <v>0</v>
       </c>
       <c r="G1751" s="1">
-        <v>22538</v>
+        <v>77571</v>
       </c>
       <c r="H1751" s="1">
         <v>0</v>
       </c>
       <c r="I1751" s="1">
-        <v>22538</v>
+        <v>77571</v>
       </c>
     </row>
     <row r="1752" spans="1:9" ht="12.75">
@@ -52351,22 +52351,22 @@
         <v>105</v>
       </c>
       <c r="D1752" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E1752" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1752" s="1">
         <v>0</v>
       </c>
       <c r="G1752" s="1">
-        <v>9676</v>
+        <v>1513824</v>
       </c>
       <c r="H1752" s="1">
         <v>0</v>
       </c>
       <c r="I1752" s="1">
-        <v>9676</v>
+        <v>1513824</v>
       </c>
     </row>
     <row r="1753" spans="1:9" ht="12.75">
@@ -52380,22 +52380,22 @@
         <v>105</v>
       </c>
       <c r="D1753" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E1753" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="F1753" s="1">
         <v>0</v>
       </c>
       <c r="G1753" s="1">
-        <v>3353166</v>
+        <v>22538</v>
       </c>
       <c r="H1753" s="1">
         <v>0</v>
       </c>
       <c r="I1753" s="1">
-        <v>3353166</v>
+        <v>22538</v>
       </c>
     </row>
     <row r="1754" spans="1:9" ht="12.75">
@@ -52409,22 +52409,22 @@
         <v>105</v>
       </c>
       <c r="D1754" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E1754" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F1754" s="1">
         <v>0</v>
       </c>
       <c r="G1754" s="1">
-        <v>662779</v>
+        <v>9676</v>
       </c>
       <c r="H1754" s="1">
         <v>0</v>
       </c>
       <c r="I1754" s="1">
-        <v>662779</v>
+        <v>9676</v>
       </c>
     </row>
     <row r="1755" spans="1:9" ht="12.75">
@@ -52441,19 +52441,19 @@
         <v>250</v>
       </c>
       <c r="E1755" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F1755" s="1">
         <v>0</v>
       </c>
       <c r="G1755" s="1">
-        <v>31417864</v>
+        <v>3353166</v>
       </c>
       <c r="H1755" s="1">
         <v>0</v>
       </c>
       <c r="I1755" s="1">
-        <v>31417864</v>
+        <v>3353166</v>
       </c>
     </row>
     <row r="1756" spans="1:9" ht="12.75">
@@ -52470,19 +52470,19 @@
         <v>250</v>
       </c>
       <c r="E1756" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1756" s="1">
         <v>0</v>
       </c>
       <c r="G1756" s="1">
-        <v>2664907</v>
+        <v>662779</v>
       </c>
       <c r="H1756" s="1">
         <v>0</v>
       </c>
       <c r="I1756" s="1">
-        <v>2664907</v>
+        <v>662779</v>
       </c>
     </row>
     <row r="1757" spans="1:9" ht="12.75">
@@ -52499,19 +52499,19 @@
         <v>250</v>
       </c>
       <c r="E1757" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F1757" s="1">
         <v>0</v>
       </c>
       <c r="G1757" s="1">
-        <v>2021829</v>
+        <v>31417864</v>
       </c>
       <c r="H1757" s="1">
         <v>0</v>
       </c>
       <c r="I1757" s="1">
-        <v>2021829</v>
+        <v>31417864</v>
       </c>
     </row>
     <row r="1758" spans="1:9" ht="12.75">
@@ -52528,19 +52528,19 @@
         <v>250</v>
       </c>
       <c r="E1758" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="F1758" s="1">
         <v>0</v>
       </c>
       <c r="G1758" s="1">
-        <v>14946353</v>
+        <v>2664907</v>
       </c>
       <c r="H1758" s="1">
         <v>0</v>
       </c>
       <c r="I1758" s="1">
-        <v>14946353</v>
+        <v>2664907</v>
       </c>
     </row>
     <row r="1759" spans="1:9" ht="12.75">
@@ -52557,19 +52557,19 @@
         <v>250</v>
       </c>
       <c r="E1759" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F1759" s="1">
         <v>0</v>
       </c>
       <c r="G1759" s="1">
-        <v>5986158</v>
+        <v>2021829</v>
       </c>
       <c r="H1759" s="1">
         <v>0</v>
       </c>
       <c r="I1759" s="1">
-        <v>5986158</v>
+        <v>2021829</v>
       </c>
     </row>
     <row r="1760" spans="1:9" ht="12.75">
@@ -52586,19 +52586,19 @@
         <v>250</v>
       </c>
       <c r="E1760" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="F1760" s="1">
         <v>0</v>
       </c>
       <c r="G1760" s="1">
-        <v>30819</v>
+        <v>14946353</v>
       </c>
       <c r="H1760" s="1">
         <v>0</v>
       </c>
       <c r="I1760" s="1">
-        <v>30819</v>
+        <v>14946353</v>
       </c>
     </row>
     <row r="1761" spans="1:9" ht="12.75">
@@ -52615,19 +52615,19 @@
         <v>250</v>
       </c>
       <c r="E1761" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="F1761" s="1">
         <v>0</v>
       </c>
       <c r="G1761" s="1">
-        <v>1516559</v>
+        <v>5986158</v>
       </c>
       <c r="H1761" s="1">
         <v>0</v>
       </c>
       <c r="I1761" s="1">
-        <v>1516559</v>
+        <v>5986158</v>
       </c>
     </row>
     <row r="1762" spans="1:9" ht="12.75">
@@ -52644,19 +52644,19 @@
         <v>250</v>
       </c>
       <c r="E1762" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F1762" s="1">
         <v>0</v>
       </c>
       <c r="G1762" s="1">
-        <v>3492740</v>
+        <v>30819</v>
       </c>
       <c r="H1762" s="1">
         <v>0</v>
       </c>
       <c r="I1762" s="1">
-        <v>3492740</v>
+        <v>30819</v>
       </c>
     </row>
     <row r="1763" spans="1:9" ht="12.75">
@@ -52673,19 +52673,19 @@
         <v>250</v>
       </c>
       <c r="E1763" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F1763" s="1">
         <v>0</v>
       </c>
       <c r="G1763" s="1">
-        <v>75917498</v>
+        <v>1516559</v>
       </c>
       <c r="H1763" s="1">
-        <v>75931161</v>
+        <v>0</v>
       </c>
       <c r="I1763" s="1">
-        <v>-13663</v>
+        <v>1516559</v>
       </c>
     </row>
     <row r="1764" spans="1:9" ht="12.75">
@@ -52702,19 +52702,19 @@
         <v>250</v>
       </c>
       <c r="E1764" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="F1764" s="1">
         <v>0</v>
       </c>
       <c r="G1764" s="1">
-        <v>747484</v>
+        <v>3492740</v>
       </c>
       <c r="H1764" s="1">
         <v>0</v>
       </c>
       <c r="I1764" s="1">
-        <v>747484</v>
+        <v>3492740</v>
       </c>
     </row>
     <row r="1765" spans="1:9" ht="12.75">
@@ -52731,19 +52731,19 @@
         <v>250</v>
       </c>
       <c r="E1765" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F1765" s="1">
         <v>0</v>
       </c>
       <c r="G1765" s="1">
-        <v>1826516</v>
+        <v>75917498</v>
       </c>
       <c r="H1765" s="1">
-        <v>0</v>
+        <v>75931161</v>
       </c>
       <c r="I1765" s="1">
-        <v>1826516</v>
+        <v>-13663</v>
       </c>
     </row>
     <row r="1766" spans="1:9" ht="12.75">
@@ -52760,19 +52760,19 @@
         <v>250</v>
       </c>
       <c r="E1766" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F1766" s="1">
         <v>0</v>
       </c>
       <c r="G1766" s="1">
-        <v>9827272</v>
+        <v>747484</v>
       </c>
       <c r="H1766" s="1">
         <v>0</v>
       </c>
       <c r="I1766" s="1">
-        <v>9827272</v>
+        <v>747484</v>
       </c>
     </row>
     <row r="1767" spans="1:9" ht="12.75">
@@ -52786,22 +52786,22 @@
         <v>105</v>
       </c>
       <c r="D1767" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E1767" t="s">
-        <v>13</v>
+        <v>340</v>
       </c>
       <c r="F1767" s="1">
         <v>0</v>
       </c>
       <c r="G1767" s="1">
-        <v>0.15</v>
+        <v>1826516</v>
       </c>
       <c r="H1767" s="1">
         <v>0</v>
       </c>
       <c r="I1767" s="1">
-        <v>0.15</v>
+        <v>1826516</v>
       </c>
     </row>
     <row r="1768" spans="1:9" ht="12.75">
@@ -52815,22 +52815,22 @@
         <v>105</v>
       </c>
       <c r="D1768" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E1768" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F1768" s="1">
         <v>0</v>
       </c>
       <c r="G1768" s="1">
-        <v>0</v>
+        <v>9827272</v>
       </c>
       <c r="H1768" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1768" s="1">
-        <v>-1</v>
+        <v>9827272</v>
       </c>
     </row>
     <row r="1769" spans="1:9" ht="12.75">
@@ -52844,22 +52844,22 @@
         <v>105</v>
       </c>
       <c r="D1769" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E1769" t="s">
-        <v>330</v>
+        <v>13</v>
       </c>
       <c r="F1769" s="1">
         <v>0</v>
       </c>
       <c r="G1769" s="1">
-        <v>148184</v>
+        <v>0.15</v>
       </c>
       <c r="H1769" s="1">
         <v>0</v>
       </c>
       <c r="I1769" s="1">
-        <v>148184</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="1770" spans="1:9" ht="12.75">
@@ -52873,22 +52873,22 @@
         <v>105</v>
       </c>
       <c r="D1770" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E1770" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="F1770" s="1">
         <v>0</v>
       </c>
       <c r="G1770" s="1">
-        <v>74092</v>
+        <v>0</v>
       </c>
       <c r="H1770" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I1770" s="1">
-        <v>74092</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="1771" spans="1:9" ht="12.75">
@@ -52905,19 +52905,19 @@
         <v>257</v>
       </c>
       <c r="E1771" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="F1771" s="1">
         <v>0</v>
       </c>
       <c r="G1771" s="1">
-        <v>74092.80</v>
+        <v>148184</v>
       </c>
       <c r="H1771" s="1">
         <v>0</v>
       </c>
       <c r="I1771" s="1">
-        <v>74092.80</v>
+        <v>148184</v>
       </c>
     </row>
     <row r="1772" spans="1:9" ht="12.75">
@@ -52931,22 +52931,22 @@
         <v>105</v>
       </c>
       <c r="D1772" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E1772" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="F1772" s="1">
         <v>0</v>
       </c>
       <c r="G1772" s="1">
-        <v>137490</v>
+        <v>74092</v>
       </c>
       <c r="H1772" s="1">
         <v>0</v>
       </c>
       <c r="I1772" s="1">
-        <v>137490</v>
+        <v>74092</v>
       </c>
     </row>
     <row r="1773" spans="1:9" ht="12.75">
@@ -52960,22 +52960,22 @@
         <v>105</v>
       </c>
       <c r="D1773" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E1773" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="F1773" s="1">
         <v>0</v>
       </c>
       <c r="G1773" s="1">
-        <v>305648</v>
+        <v>74092.80</v>
       </c>
       <c r="H1773" s="1">
         <v>0</v>
       </c>
       <c r="I1773" s="1">
-        <v>305648</v>
+        <v>74092.80</v>
       </c>
     </row>
     <row r="1774" spans="1:9" ht="12.75">
@@ -52992,19 +52992,19 @@
         <v>258</v>
       </c>
       <c r="E1774" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="F1774" s="1">
         <v>0</v>
       </c>
       <c r="G1774" s="1">
-        <v>484</v>
+        <v>137490</v>
       </c>
       <c r="H1774" s="1">
         <v>0</v>
       </c>
       <c r="I1774" s="1">
-        <v>484</v>
+        <v>137490</v>
       </c>
     </row>
     <row r="1775" spans="1:9" ht="12.75">
@@ -53018,22 +53018,22 @@
         <v>105</v>
       </c>
       <c r="D1775" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E1775" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
       <c r="F1775" s="1">
         <v>0</v>
       </c>
       <c r="G1775" s="1">
-        <v>24000</v>
+        <v>305648</v>
       </c>
       <c r="H1775" s="1">
         <v>0</v>
       </c>
       <c r="I1775" s="1">
-        <v>24000</v>
+        <v>305648</v>
       </c>
     </row>
     <row r="1776" spans="1:9" ht="12.75">
@@ -53047,7 +53047,7 @@
         <v>105</v>
       </c>
       <c r="D1776" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="E1776" t="s">
         <v>330</v>
@@ -53056,13 +53056,13 @@
         <v>0</v>
       </c>
       <c r="G1776" s="1">
-        <v>1125720</v>
+        <v>484</v>
       </c>
       <c r="H1776" s="1">
         <v>0</v>
       </c>
       <c r="I1776" s="1">
-        <v>1125720</v>
+        <v>484</v>
       </c>
     </row>
     <row r="1777" spans="1:9" ht="12.75">
@@ -53076,22 +53076,22 @@
         <v>105</v>
       </c>
       <c r="D1777" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E1777" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F1777" s="1">
         <v>0</v>
       </c>
       <c r="G1777" s="1">
-        <v>1688580</v>
+        <v>24000</v>
       </c>
       <c r="H1777" s="1">
         <v>0</v>
       </c>
       <c r="I1777" s="1">
-        <v>1688580</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="1778" spans="1:9" ht="12.75">
@@ -53099,28 +53099,28 @@
         <v>312</v>
       </c>
       <c r="B1778" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="C1778" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="D1778" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="E1778" t="s">
-        <v>13</v>
+        <v>330</v>
       </c>
       <c r="F1778" s="1">
         <v>0</v>
       </c>
       <c r="G1778" s="1">
-        <v>0</v>
+        <v>1125720</v>
       </c>
       <c r="H1778" s="1">
-        <v>7351276</v>
+        <v>0</v>
       </c>
       <c r="I1778" s="1">
-        <v>-7351276</v>
+        <v>1125720</v>
       </c>
     </row>
     <row r="1779" spans="1:9" ht="12.75">
@@ -53128,28 +53128,28 @@
         <v>312</v>
       </c>
       <c r="B1779" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="C1779" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="D1779" t="s">
-        <v>308</v>
+        <v>263</v>
       </c>
       <c r="E1779" t="s">
-        <v>13</v>
+        <v>337</v>
       </c>
       <c r="F1779" s="1">
         <v>0</v>
       </c>
       <c r="G1779" s="1">
-        <v>0</v>
+        <v>1688580</v>
       </c>
       <c r="H1779" s="1">
         <v>0</v>
       </c>
       <c r="I1779" s="1">
-        <v>0</v>
+        <v>1688580</v>
       </c>
     </row>
     <row r="1780" spans="1:9" ht="12.75">
@@ -53157,28 +53157,28 @@
         <v>312</v>
       </c>
       <c r="B1780" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C1780" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D1780" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E1780" t="s">
         <v>13</v>
       </c>
       <c r="F1780" s="1">
-        <v>-5418882</v>
+        <v>0</v>
       </c>
       <c r="G1780" s="1">
-        <v>2.8291444627E8</v>
+        <v>0</v>
       </c>
       <c r="H1780" s="1">
-        <v>2.9453230877000004E8</v>
+        <v>7351276</v>
       </c>
       <c r="I1780" s="1">
-        <v>-1.703674450000006E7</v>
+        <v>-7351276</v>
       </c>
     </row>
     <row r="1781" spans="1:9" ht="12.75">
@@ -53186,13 +53186,13 @@
         <v>312</v>
       </c>
       <c r="B1781" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C1781" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="D1781" t="s">
-        <v>356</v>
+        <v>308</v>
       </c>
       <c r="E1781" t="s">
         <v>13</v>
@@ -53201,13 +53201,13 @@
         <v>0</v>
       </c>
       <c r="G1781" s="1">
-        <v>2274999</v>
+        <v>0</v>
       </c>
       <c r="H1781" s="1">
-        <v>5013786</v>
+        <v>0</v>
       </c>
       <c r="I1781" s="1">
-        <v>-2738787</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1782" spans="1:9" ht="12.75">
@@ -53218,25 +53218,25 @@
         <v>268</v>
       </c>
       <c r="C1782" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D1782" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="E1782" t="s">
         <v>13</v>
       </c>
       <c r="F1782" s="1">
-        <v>-22030149</v>
+        <v>-5418882</v>
       </c>
       <c r="G1782" s="1">
-        <v>7656302</v>
+        <v>2.9474133727E8</v>
       </c>
       <c r="H1782" s="1">
-        <v>9.094276758399999E8</v>
+        <v>2.9482110077E8</v>
       </c>
       <c r="I1782" s="1">
-        <v>-9.238015228399999E8</v>
+        <v>-5498645.5</v>
       </c>
     </row>
     <row r="1783" spans="1:9" ht="12.75">
@@ -53250,22 +53250,22 @@
         <v>273</v>
       </c>
       <c r="D1783" t="s">
-        <v>282</v>
+        <v>356</v>
       </c>
       <c r="E1783" t="s">
         <v>13</v>
       </c>
       <c r="F1783" s="1">
-        <v>-14989</v>
+        <v>0</v>
       </c>
       <c r="G1783" s="1">
-        <v>5515449</v>
+        <v>2274999</v>
       </c>
       <c r="H1783" s="1">
-        <v>10165830</v>
+        <v>5013786</v>
       </c>
       <c r="I1783" s="1">
-        <v>-4665370</v>
+        <v>-2738787</v>
       </c>
     </row>
     <row r="1784" spans="1:9" ht="12.75">
@@ -53279,22 +53279,22 @@
         <v>273</v>
       </c>
       <c r="D1784" t="s">
-        <v>357</v>
+        <v>278</v>
       </c>
       <c r="E1784" t="s">
         <v>13</v>
       </c>
       <c r="F1784" s="1">
-        <v>0</v>
+        <v>-22030149</v>
       </c>
       <c r="G1784" s="1">
-        <v>2659661</v>
+        <v>7656302</v>
       </c>
       <c r="H1784" s="1">
-        <v>2659660</v>
+        <v>9.136277758399999E8</v>
       </c>
       <c r="I1784" s="1">
-        <v>1</v>
+        <v>-9.280016228399999E8</v>
       </c>
     </row>
     <row r="1785" spans="1:9" ht="12.75">
@@ -53308,22 +53308,22 @@
         <v>273</v>
       </c>
       <c r="D1785" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="E1785" t="s">
         <v>13</v>
       </c>
       <c r="F1785" s="1">
-        <v>0</v>
+        <v>-14989</v>
       </c>
       <c r="G1785" s="1">
-        <v>0</v>
+        <v>5515449</v>
       </c>
       <c r="H1785" s="1">
-        <v>190424</v>
+        <v>10165830</v>
       </c>
       <c r="I1785" s="1">
-        <v>-190424</v>
+        <v>-4665370</v>
       </c>
     </row>
     <row r="1786" spans="1:9" ht="12.75">
@@ -53337,7 +53337,7 @@
         <v>273</v>
       </c>
       <c r="D1786" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E1786" t="s">
         <v>13</v>
@@ -53346,13 +53346,13 @@
         <v>0</v>
       </c>
       <c r="G1786" s="1">
-        <v>2279773</v>
+        <v>2659661</v>
       </c>
       <c r="H1786" s="1">
-        <v>2294489</v>
+        <v>2659660</v>
       </c>
       <c r="I1786" s="1">
-        <v>-14716</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1787" spans="1:9" ht="12.75">
@@ -53366,7 +53366,7 @@
         <v>273</v>
       </c>
       <c r="D1787" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E1787" t="s">
         <v>13</v>
@@ -53375,13 +53375,13 @@
         <v>0</v>
       </c>
       <c r="G1787" s="1">
-        <v>48730</v>
+        <v>0</v>
       </c>
       <c r="H1787" s="1">
-        <v>70730</v>
+        <v>190424</v>
       </c>
       <c r="I1787" s="1">
-        <v>-22000</v>
+        <v>-190424</v>
       </c>
     </row>
     <row r="1788" spans="1:9" ht="12.75">
@@ -53395,7 +53395,7 @@
         <v>273</v>
       </c>
       <c r="D1788" t="s">
-        <v>288</v>
+        <v>358</v>
       </c>
       <c r="E1788" t="s">
         <v>13</v>
@@ -53404,13 +53404,13 @@
         <v>0</v>
       </c>
       <c r="G1788" s="1">
-        <v>840</v>
+        <v>2279773</v>
       </c>
       <c r="H1788" s="1">
-        <v>416</v>
+        <v>2294489</v>
       </c>
       <c r="I1788" s="1">
-        <v>424</v>
+        <v>-14716</v>
       </c>
     </row>
     <row r="1789" spans="1:9" ht="12.75">
@@ -53424,7 +53424,7 @@
         <v>273</v>
       </c>
       <c r="D1789" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E1789" t="s">
         <v>13</v>
@@ -53433,13 +53433,13 @@
         <v>0</v>
       </c>
       <c r="G1789" s="1">
-        <v>4.89969833E7</v>
+        <v>48730</v>
       </c>
       <c r="H1789" s="1">
-        <v>58379674</v>
+        <v>70730</v>
       </c>
       <c r="I1789" s="1">
-        <v>-9382690.700000003</v>
+        <v>-22000</v>
       </c>
     </row>
     <row r="1790" spans="1:9" ht="12.75">
@@ -53453,7 +53453,7 @@
         <v>273</v>
       </c>
       <c r="D1790" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E1790" t="s">
         <v>13</v>
@@ -53462,13 +53462,13 @@
         <v>0</v>
       </c>
       <c r="G1790" s="1">
-        <v>55944</v>
+        <v>840</v>
       </c>
       <c r="H1790" s="1">
-        <v>199075.79</v>
+        <v>416</v>
       </c>
       <c r="I1790" s="1">
-        <v>-143131.79</v>
+        <v>424</v>
       </c>
     </row>
     <row r="1791" spans="1:9" ht="12.75">
@@ -53482,7 +53482,7 @@
         <v>273</v>
       </c>
       <c r="D1791" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="E1791" t="s">
         <v>13</v>
@@ -53491,13 +53491,13 @@
         <v>0</v>
       </c>
       <c r="G1791" s="1">
-        <v>105045</v>
+        <v>4.89969833E7</v>
       </c>
       <c r="H1791" s="1">
-        <v>498838.90</v>
+        <v>58379674</v>
       </c>
       <c r="I1791" s="1">
-        <v>-393793.90</v>
+        <v>-9382690.700000003</v>
       </c>
     </row>
     <row r="1792" spans="1:9" ht="12.75">
@@ -53511,7 +53511,7 @@
         <v>273</v>
       </c>
       <c r="D1792" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="E1792" t="s">
         <v>13</v>
@@ -53520,13 +53520,13 @@
         <v>0</v>
       </c>
       <c r="G1792" s="1">
-        <v>4687449</v>
+        <v>55944</v>
       </c>
       <c r="H1792" s="1">
-        <v>1.453971609E7</v>
+        <v>199075.79</v>
       </c>
       <c r="I1792" s="1">
-        <v>-9852267.09</v>
+        <v>-143131.79</v>
       </c>
     </row>
     <row r="1793" spans="1:9" ht="12.75">
@@ -53540,7 +53540,7 @@
         <v>273</v>
       </c>
       <c r="D1793" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="E1793" t="s">
         <v>13</v>
@@ -53549,13 +53549,13 @@
         <v>0</v>
       </c>
       <c r="G1793" s="1">
-        <v>1758542.24</v>
+        <v>105045</v>
       </c>
       <c r="H1793" s="1">
-        <v>1153027.74</v>
+        <v>498838.90</v>
       </c>
       <c r="I1793" s="1">
-        <v>605514.50</v>
+        <v>-393793.90</v>
       </c>
     </row>
     <row r="1794" spans="1:9" ht="12.75">
@@ -53569,7 +53569,7 @@
         <v>273</v>
       </c>
       <c r="D1794" t="s">
-        <v>359</v>
+        <v>293</v>
       </c>
       <c r="E1794" t="s">
         <v>13</v>
@@ -53578,13 +53578,13 @@
         <v>0</v>
       </c>
       <c r="G1794" s="1">
-        <v>9251007</v>
+        <v>4687449</v>
       </c>
       <c r="H1794" s="1">
-        <v>18902755</v>
+        <v>1.455921609E7</v>
       </c>
       <c r="I1794" s="1">
-        <v>-9651748</v>
+        <v>-9871767.09</v>
       </c>
     </row>
     <row r="1795" spans="1:9" ht="12.75">
@@ -53595,10 +53595,10 @@
         <v>268</v>
       </c>
       <c r="C1795" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="D1795" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="E1795" t="s">
         <v>13</v>
@@ -53607,13 +53607,13 @@
         <v>0</v>
       </c>
       <c r="G1795" s="1">
-        <v>2.2518876449E8</v>
+        <v>1758542.24</v>
       </c>
       <c r="H1795" s="1">
-        <v>2.2518876449E8</v>
+        <v>1153027.74</v>
       </c>
       <c r="I1795" s="1">
-        <v>0</v>
+        <v>605514.50</v>
       </c>
     </row>
     <row r="1796" spans="1:9" ht="12.75">
@@ -53624,10 +53624,10 @@
         <v>268</v>
       </c>
       <c r="C1796" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="D1796" t="s">
-        <v>298</v>
+        <v>359</v>
       </c>
       <c r="E1796" t="s">
         <v>13</v>
@@ -53636,42 +53636,100 @@
         <v>0</v>
       </c>
       <c r="G1796" s="1">
-        <v>0</v>
+        <v>9251007</v>
       </c>
       <c r="H1796" s="1">
-        <v>8826219.66</v>
+        <v>18902755</v>
       </c>
       <c r="I1796" s="1">
-        <v>-8826219.66</v>
+        <v>-9651748</v>
       </c>
     </row>
     <row r="1797" spans="1:9" ht="12.75">
       <c r="A1797" t="s">
+        <v>312</v>
+      </c>
+      <c r="B1797" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1797" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1797" t="s">
+        <v>297</v>
+      </c>
+      <c r="E1797" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1797" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1797" s="1">
+        <v>2.2518876449E8</v>
+      </c>
+      <c r="H1797" s="1">
+        <v>2.2518876449E8</v>
+      </c>
+      <c r="I1797" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1798" spans="1:9" ht="12.75">
+      <c r="A1798" t="s">
+        <v>312</v>
+      </c>
+      <c r="B1798" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1798" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1798" t="s">
+        <v>298</v>
+      </c>
+      <c r="E1798" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1798" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1798" s="1">
+        <v>0</v>
+      </c>
+      <c r="H1798" s="1">
+        <v>8826219.66</v>
+      </c>
+      <c r="I1798" s="1">
+        <v>-8826219.66</v>
+      </c>
+    </row>
+    <row r="1799" spans="1:9" ht="12.75">
+      <c r="A1799" t="s">
         <v>360</v>
       </c>
-      <c r="B1797" t="s">
+      <c r="B1799" t="s">
         <v>361</v>
       </c>
-      <c r="C1797" t="s">
+      <c r="C1799" t="s">
         <v>361</v>
       </c>
-      <c r="D1797" t="s">
+      <c r="D1799" t="s">
         <v>361</v>
       </c>
-      <c r="E1797" t="s">
+      <c r="E1799" t="s">
         <v>361</v>
       </c>
-      <c r="F1797" s="1">
-        <v>1.1920928955078125E-7</v>
-      </c>
-      <c r="G1797" s="1">
-        <v>7.226030905039998E9</v>
-      </c>
-      <c r="H1797" s="1">
-        <v>7.226030905040004E9</v>
-      </c>
-      <c r="I1797" s="1">
-        <v>-2.2798776626586914E-6</v>
+      <c r="F1799" s="1">
+        <v>5.9604644775390625E-8</v>
+      </c>
+      <c r="G1799" s="1">
+        <v>7.252510092039998E9</v>
+      </c>
+      <c r="H1799" s="1">
+        <v>7.25251009204E9</v>
+      </c>
+      <c r="I1799" s="1">
+        <v>-1.341104507446289E-7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-03-27
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9103" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9108" uniqueCount="364">
   <si>
     <t>Book</t>
   </si>
@@ -1082,10 +1082,10 @@
     <t>AIP-0120-Training Infra and MEL-Waymo-NFC</t>
   </si>
   <si>
-    <t>AIP-0109-Education Innovation-Google Cloud</t>
+    <t>AIP-0103-Administration-RFR-NFC</t>
   </si>
   <si>
-    <t>AIP-0103-Administration-RFR-NFC</t>
+    <t>AIP-0109-Education Innovation-Google Cloud</t>
   </si>
   <si>
     <t>AIP-0118-Training Infra and MEL-Google Digital-NFC</t>
@@ -1553,8 +1553,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2da46727-7291-423f-a96e-a82d53a172d6}">
-  <dimension ref="A1:I1819"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{d0c3e953-58ae-42c3-978d-4ac5e32bf239}">
+  <dimension ref="A1:I1820"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="14.142857142857142" customWidth="1"/>
@@ -1674,13 +1674,13 @@
         <v>1.3190275187E8</v>
       </c>
       <c r="G4" s="1">
-        <v>3.9882729998E8</v>
+        <v>3.9887229998E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.4504202754000014E8</v>
+        <v>3.4664425354000056E8</v>
       </c>
       <c r="I4" s="1">
-        <v>1.8568802430999988E8</v>
+        <v>1.8413079830999947E8</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -1793,10 +1793,10 @@
         <v>5.43186561E8</v>
       </c>
       <c r="H8" s="1">
-        <v>2.717296269799999E8</v>
+        <v>2.7487199097999996E8</v>
       </c>
       <c r="I8" s="1">
-        <v>2.714569340200001E8</v>
+        <v>2.6831457002000004E8</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="12.75">
@@ -3820,13 +3820,13 @@
         <v>918706</v>
       </c>
       <c r="G78" s="1">
-        <v>4.426599483000001E7</v>
+        <v>4.805299582999999E7</v>
       </c>
       <c r="H78" s="1">
-        <v>4.398579120000001E7</v>
+        <v>4.781173219999998E7</v>
       </c>
       <c r="I78" s="1">
-        <v>1198909.6300000027</v>
+        <v>1159969.6300000101</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="12.75">
@@ -3904,7 +3904,7 @@
         <v>13</v>
       </c>
       <c r="F81" s="1">
-        <v>0</v>
+        <v>-9.313225746154785E-10</v>
       </c>
       <c r="G81" s="1">
         <v>333614</v>
@@ -3913,7 +3913,7 @@
         <v>333614</v>
       </c>
       <c r="I81" s="1">
-        <v>0</v>
+        <v>-9.313225746154785E-10</v>
       </c>
     </row>
     <row r="82" spans="1:9" ht="12.75">
@@ -15826,13 +15826,13 @@
         <v>0</v>
       </c>
       <c r="G492" s="1">
-        <v>581512</v>
+        <v>648581</v>
       </c>
       <c r="H492" s="1">
         <v>0</v>
       </c>
       <c r="I492" s="1">
-        <v>581512</v>
+        <v>648581</v>
       </c>
     </row>
     <row r="493" spans="1:9" ht="12.75">
@@ -16000,13 +16000,13 @@
         <v>0</v>
       </c>
       <c r="G498" s="1">
-        <v>594595</v>
+        <v>642481</v>
       </c>
       <c r="H498" s="1">
         <v>0</v>
       </c>
       <c r="I498" s="1">
-        <v>594595</v>
+        <v>642481</v>
       </c>
     </row>
     <row r="499" spans="1:9" ht="12.75">
@@ -16029,13 +16029,13 @@
         <v>0</v>
       </c>
       <c r="G499" s="1">
-        <v>702904</v>
+        <v>756352</v>
       </c>
       <c r="H499" s="1">
         <v>0</v>
       </c>
       <c r="I499" s="1">
-        <v>702904</v>
+        <v>756352</v>
       </c>
     </row>
     <row r="500" spans="1:9" ht="12.75">
@@ -16232,13 +16232,13 @@
         <v>0</v>
       </c>
       <c r="G506" s="1">
-        <v>2094659</v>
+        <v>2297773</v>
       </c>
       <c r="H506" s="1">
         <v>0</v>
       </c>
       <c r="I506" s="1">
-        <v>2094659</v>
+        <v>2297773</v>
       </c>
     </row>
     <row r="507" spans="1:9" ht="12.75">
@@ -16609,13 +16609,13 @@
         <v>0</v>
       </c>
       <c r="G519" s="1">
-        <v>478757</v>
+        <v>506881</v>
       </c>
       <c r="H519" s="1">
         <v>0</v>
       </c>
       <c r="I519" s="1">
-        <v>478757</v>
+        <v>506881</v>
       </c>
     </row>
     <row r="520" spans="1:9" ht="12.75">
@@ -17102,13 +17102,13 @@
         <v>0</v>
       </c>
       <c r="G536" s="1">
-        <v>150793</v>
+        <v>158293</v>
       </c>
       <c r="H536" s="1">
         <v>0</v>
       </c>
       <c r="I536" s="1">
-        <v>150793</v>
+        <v>158293</v>
       </c>
     </row>
     <row r="537" spans="1:9" ht="12.75">
@@ -17247,13 +17247,13 @@
         <v>0</v>
       </c>
       <c r="G541" s="1">
-        <v>1798316</v>
+        <v>1988088</v>
       </c>
       <c r="H541" s="1">
         <v>0</v>
       </c>
       <c r="I541" s="1">
-        <v>1798316</v>
+        <v>1988088</v>
       </c>
     </row>
     <row r="542" spans="1:9" ht="12.75">
@@ -17276,13 +17276,13 @@
         <v>0</v>
       </c>
       <c r="G542" s="1">
-        <v>830426</v>
+        <v>851888</v>
       </c>
       <c r="H542" s="1">
         <v>0</v>
       </c>
       <c r="I542" s="1">
-        <v>830426</v>
+        <v>851888</v>
       </c>
     </row>
     <row r="543" spans="1:9" ht="12.75">
@@ -17305,13 +17305,13 @@
         <v>0</v>
       </c>
       <c r="G543" s="1">
-        <v>1795673</v>
+        <v>1954235</v>
       </c>
       <c r="H543" s="1">
         <v>0</v>
       </c>
       <c r="I543" s="1">
-        <v>1795673</v>
+        <v>1954235</v>
       </c>
     </row>
     <row r="544" spans="1:9" ht="12.75">
@@ -17537,13 +17537,13 @@
         <v>0</v>
       </c>
       <c r="G551" s="1">
-        <v>338383</v>
+        <v>349733</v>
       </c>
       <c r="H551" s="1">
         <v>0</v>
       </c>
       <c r="I551" s="1">
-        <v>338383</v>
+        <v>349733</v>
       </c>
     </row>
     <row r="552" spans="1:9" ht="12.75">
@@ -17566,13 +17566,13 @@
         <v>0</v>
       </c>
       <c r="G552" s="1">
-        <v>139808</v>
+        <v>147008</v>
       </c>
       <c r="H552" s="1">
         <v>0</v>
       </c>
       <c r="I552" s="1">
-        <v>139808</v>
+        <v>147008</v>
       </c>
     </row>
     <row r="553" spans="1:9" ht="12.75">
@@ -17595,13 +17595,13 @@
         <v>0</v>
       </c>
       <c r="G553" s="1">
-        <v>267189</v>
+        <v>284968</v>
       </c>
       <c r="H553" s="1">
         <v>0</v>
       </c>
       <c r="I553" s="1">
-        <v>267189</v>
+        <v>284968</v>
       </c>
     </row>
     <row r="554" spans="1:9" ht="12.75">
@@ -17624,13 +17624,13 @@
         <v>0</v>
       </c>
       <c r="G554" s="1">
-        <v>19081519</v>
+        <v>19105775</v>
       </c>
       <c r="H554" s="1">
-        <v>18756242</v>
+        <v>20106655</v>
       </c>
       <c r="I554" s="1">
-        <v>325277</v>
+        <v>-1000880</v>
       </c>
     </row>
     <row r="555" spans="1:9" ht="12.75">
@@ -17653,13 +17653,13 @@
         <v>0</v>
       </c>
       <c r="G555" s="1">
-        <v>217070</v>
+        <v>228870</v>
       </c>
       <c r="H555" s="1">
         <v>0</v>
       </c>
       <c r="I555" s="1">
-        <v>217070</v>
+        <v>228870</v>
       </c>
     </row>
     <row r="556" spans="1:9" ht="12.75">
@@ -17711,13 +17711,13 @@
         <v>0</v>
       </c>
       <c r="G557" s="1">
-        <v>527058</v>
+        <v>553064</v>
       </c>
       <c r="H557" s="1">
         <v>0</v>
       </c>
       <c r="I557" s="1">
-        <v>527058</v>
+        <v>553064</v>
       </c>
     </row>
     <row r="558" spans="1:9" ht="12.75">
@@ -17740,13 +17740,13 @@
         <v>0</v>
       </c>
       <c r="G558" s="1">
-        <v>324918</v>
+        <v>339720</v>
       </c>
       <c r="H558" s="1">
         <v>0</v>
       </c>
       <c r="I558" s="1">
-        <v>324918</v>
+        <v>339720</v>
       </c>
     </row>
     <row r="559" spans="1:9" ht="12.75">
@@ -17798,13 +17798,13 @@
         <v>0</v>
       </c>
       <c r="G560" s="1">
-        <v>1194825</v>
+        <v>1339946</v>
       </c>
       <c r="H560" s="1">
         <v>0</v>
       </c>
       <c r="I560" s="1">
-        <v>1194825</v>
+        <v>1339946</v>
       </c>
     </row>
     <row r="561" spans="1:9" ht="12.75">
@@ -17827,13 +17827,13 @@
         <v>0</v>
       </c>
       <c r="G561" s="1">
-        <v>441747</v>
+        <v>469009</v>
       </c>
       <c r="H561" s="1">
         <v>0</v>
       </c>
       <c r="I561" s="1">
-        <v>441747</v>
+        <v>469009</v>
       </c>
     </row>
     <row r="562" spans="1:9" ht="12.75">
@@ -17914,13 +17914,13 @@
         <v>0</v>
       </c>
       <c r="G564" s="1">
-        <v>192869</v>
+        <v>197074</v>
       </c>
       <c r="H564" s="1">
         <v>0</v>
       </c>
       <c r="I564" s="1">
-        <v>192869</v>
+        <v>197074</v>
       </c>
     </row>
     <row r="565" spans="1:9" ht="12.75">
@@ -18001,13 +18001,13 @@
         <v>0</v>
       </c>
       <c r="G567" s="1">
-        <v>1122012</v>
+        <v>1351407</v>
       </c>
       <c r="H567" s="1">
         <v>0</v>
       </c>
       <c r="I567" s="1">
-        <v>1122012</v>
+        <v>1351407</v>
       </c>
     </row>
     <row r="568" spans="1:9" ht="12.75">
@@ -18030,13 +18030,13 @@
         <v>0</v>
       </c>
       <c r="G568" s="1">
-        <v>114769</v>
+        <v>139635</v>
       </c>
       <c r="H568" s="1">
         <v>0</v>
       </c>
       <c r="I568" s="1">
-        <v>114769</v>
+        <v>139635</v>
       </c>
     </row>
     <row r="569" spans="1:9" ht="12.75">
@@ -18059,13 +18059,13 @@
         <v>0</v>
       </c>
       <c r="G569" s="1">
-        <v>7286</v>
+        <v>11035</v>
       </c>
       <c r="H569" s="1">
         <v>0</v>
       </c>
       <c r="I569" s="1">
-        <v>7286</v>
+        <v>11035</v>
       </c>
     </row>
     <row r="570" spans="1:9" ht="12.75">
@@ -18088,13 +18088,13 @@
         <v>0</v>
       </c>
       <c r="G570" s="1">
-        <v>70898</v>
+        <v>96583</v>
       </c>
       <c r="H570" s="1">
         <v>0</v>
       </c>
       <c r="I570" s="1">
-        <v>70898</v>
+        <v>96583</v>
       </c>
     </row>
     <row r="571" spans="1:9" ht="12.75">
@@ -18262,13 +18262,13 @@
         <v>0</v>
       </c>
       <c r="G576" s="1">
-        <v>816861.20</v>
+        <v>893548.20</v>
       </c>
       <c r="H576" s="1">
         <v>3527.18</v>
       </c>
       <c r="I576" s="1">
-        <v>813334.0199999999</v>
+        <v>890021.0199999999</v>
       </c>
     </row>
     <row r="577" spans="1:9" ht="12.75">
@@ -18436,13 +18436,13 @@
         <v>0</v>
       </c>
       <c r="G582" s="1">
-        <v>892804.57</v>
+        <v>959829.5700000001</v>
       </c>
       <c r="H582" s="1">
         <v>0</v>
       </c>
       <c r="I582" s="1">
-        <v>892804.57</v>
+        <v>959829.5700000001</v>
       </c>
     </row>
     <row r="583" spans="1:9" ht="12.75">
@@ -18465,13 +18465,13 @@
         <v>0</v>
       </c>
       <c r="G583" s="1">
-        <v>1064804.0099999998</v>
+        <v>1134248.01</v>
       </c>
       <c r="H583" s="1">
         <v>0</v>
       </c>
       <c r="I583" s="1">
-        <v>1064804.0099999998</v>
+        <v>1134248.01</v>
       </c>
     </row>
     <row r="584" spans="1:9" ht="12.75">
@@ -18668,13 +18668,13 @@
         <v>0</v>
       </c>
       <c r="G590" s="1">
-        <v>2994848.4499999997</v>
+        <v>3206769.4499999997</v>
       </c>
       <c r="H590" s="1">
         <v>14722.75</v>
       </c>
       <c r="I590" s="1">
-        <v>2980125.6999999997</v>
+        <v>3192046.6999999997</v>
       </c>
     </row>
     <row r="591" spans="1:9" ht="12.75">
@@ -18697,13 +18697,13 @@
         <v>0</v>
       </c>
       <c r="G591" s="1">
-        <v>150327.47</v>
+        <v>154978.47000000003</v>
       </c>
       <c r="H591" s="1">
         <v>0</v>
       </c>
       <c r="I591" s="1">
-        <v>150327.47</v>
+        <v>154978.47000000003</v>
       </c>
     </row>
     <row r="592" spans="1:9" ht="12.75">
@@ -19045,13 +19045,13 @@
         <v>0</v>
       </c>
       <c r="G603" s="1">
-        <v>925693.5499999999</v>
+        <v>1022249.5499999999</v>
       </c>
       <c r="H603" s="1">
         <v>0</v>
       </c>
       <c r="I603" s="1">
-        <v>925693.5499999999</v>
+        <v>1022249.5499999999</v>
       </c>
     </row>
     <row r="604" spans="1:9" ht="12.75">
@@ -19538,13 +19538,13 @@
         <v>0</v>
       </c>
       <c r="G620" s="1">
-        <v>274760.70</v>
+        <v>310627.70</v>
       </c>
       <c r="H620" s="1">
         <v>0</v>
       </c>
       <c r="I620" s="1">
-        <v>274760.70</v>
+        <v>310627.70</v>
       </c>
     </row>
     <row r="621" spans="1:9" ht="12.75">
@@ -19625,13 +19625,13 @@
         <v>0</v>
       </c>
       <c r="G623" s="1">
-        <v>582585.4599999998</v>
+        <v>584250.46</v>
       </c>
       <c r="H623" s="1">
         <v>0</v>
       </c>
       <c r="I623" s="1">
-        <v>582585.4599999998</v>
+        <v>584250.46</v>
       </c>
     </row>
     <row r="624" spans="1:9" ht="12.75">
@@ -19654,13 +19654,13 @@
         <v>0</v>
       </c>
       <c r="G624" s="1">
-        <v>2798165.889999999</v>
+        <v>3041021.89</v>
       </c>
       <c r="H624" s="1">
         <v>23236.93</v>
       </c>
       <c r="I624" s="1">
-        <v>2774928.959999999</v>
+        <v>3017784.96</v>
       </c>
     </row>
     <row r="625" spans="1:9" ht="12.75">
@@ -19683,13 +19683,13 @@
         <v>0</v>
       </c>
       <c r="G625" s="1">
-        <v>1374964.32</v>
+        <v>1404331.3199999998</v>
       </c>
       <c r="H625" s="1">
         <v>0</v>
       </c>
       <c r="I625" s="1">
-        <v>1374964.32</v>
+        <v>1404331.3199999998</v>
       </c>
     </row>
     <row r="626" spans="1:9" ht="12.75">
@@ -19712,13 +19712,13 @@
         <v>0</v>
       </c>
       <c r="G626" s="1">
-        <v>3046869.3999999994</v>
+        <v>3337176.3999999994</v>
       </c>
       <c r="H626" s="1">
         <v>9049.23</v>
       </c>
       <c r="I626" s="1">
-        <v>3037820.1699999995</v>
+        <v>3328127.1699999995</v>
       </c>
     </row>
     <row r="627" spans="1:9" ht="12.75">
@@ -19944,13 +19944,13 @@
         <v>0</v>
       </c>
       <c r="G634" s="1">
-        <v>620559.99</v>
+        <v>652271.99</v>
       </c>
       <c r="H634" s="1">
         <v>2836.72</v>
       </c>
       <c r="I634" s="1">
-        <v>617723.27</v>
+        <v>649435.27</v>
       </c>
     </row>
     <row r="635" spans="1:9" ht="12.75">
@@ -19973,13 +19973,13 @@
         <v>0</v>
       </c>
       <c r="G635" s="1">
-        <v>268446.66</v>
+        <v>287725.66000000003</v>
       </c>
       <c r="H635" s="1">
         <v>0</v>
       </c>
       <c r="I635" s="1">
-        <v>268446.66</v>
+        <v>287725.66000000003</v>
       </c>
     </row>
     <row r="636" spans="1:9" ht="12.75">
@@ -20002,13 +20002,13 @@
         <v>0</v>
       </c>
       <c r="G636" s="1">
-        <v>997754.49</v>
+        <v>1052593.49</v>
       </c>
       <c r="H636" s="1">
         <v>0</v>
       </c>
       <c r="I636" s="1">
-        <v>997754.49</v>
+        <v>1052593.49</v>
       </c>
     </row>
     <row r="637" spans="1:9" ht="12.75">
@@ -20031,13 +20031,13 @@
         <v>0</v>
       </c>
       <c r="G637" s="1">
-        <v>536750.2400000001</v>
+        <v>555001.24</v>
       </c>
       <c r="H637" s="1">
         <v>0</v>
       </c>
       <c r="I637" s="1">
-        <v>536750.2400000001</v>
+        <v>555001.24</v>
       </c>
     </row>
     <row r="638" spans="1:9" ht="12.75">
@@ -20060,13 +20060,13 @@
         <v>0</v>
       </c>
       <c r="G638" s="1">
-        <v>397731.83</v>
+        <v>457844.83</v>
       </c>
       <c r="H638" s="1">
         <v>0</v>
       </c>
       <c r="I638" s="1">
-        <v>397731.83</v>
+        <v>457844.83</v>
       </c>
     </row>
     <row r="639" spans="1:9" ht="12.75">
@@ -20118,13 +20118,13 @@
         <v>0</v>
       </c>
       <c r="G640" s="1">
-        <v>900877.7399999998</v>
+        <v>964873.7399999998</v>
       </c>
       <c r="H640" s="1">
         <v>0</v>
       </c>
       <c r="I640" s="1">
-        <v>900877.7399999998</v>
+        <v>964873.7399999998</v>
       </c>
     </row>
     <row r="641" spans="1:9" ht="12.75">
@@ -20147,13 +20147,13 @@
         <v>0</v>
       </c>
       <c r="G641" s="1">
-        <v>617359.95</v>
+        <v>641168.95</v>
       </c>
       <c r="H641" s="1">
         <v>0</v>
       </c>
       <c r="I641" s="1">
-        <v>617359.95</v>
+        <v>641168.95</v>
       </c>
     </row>
     <row r="642" spans="1:9" ht="12.75">
@@ -20205,13 +20205,13 @@
         <v>0</v>
       </c>
       <c r="G643" s="1">
-        <v>1595365.71</v>
+        <v>1757794.71</v>
       </c>
       <c r="H643" s="1">
         <v>9049.23</v>
       </c>
       <c r="I643" s="1">
-        <v>1586316.48</v>
+        <v>1748745.48</v>
       </c>
     </row>
     <row r="644" spans="1:9" ht="12.75">
@@ -20234,13 +20234,13 @@
         <v>0</v>
       </c>
       <c r="G644" s="1">
-        <v>703295.80</v>
+        <v>744682.7999999999</v>
       </c>
       <c r="H644" s="1">
         <v>0</v>
       </c>
       <c r="I644" s="1">
-        <v>703295.80</v>
+        <v>744682.7999999999</v>
       </c>
     </row>
     <row r="645" spans="1:9" ht="12.75">
@@ -20263,13 +20263,13 @@
         <v>0</v>
       </c>
       <c r="G645" s="1">
-        <v>516927.00000000006</v>
+        <v>544076</v>
       </c>
       <c r="H645" s="1">
         <v>0</v>
       </c>
       <c r="I645" s="1">
-        <v>516927.00000000006</v>
+        <v>544076</v>
       </c>
     </row>
     <row r="646" spans="1:9" ht="12.75">
@@ -20292,13 +20292,13 @@
         <v>0</v>
       </c>
       <c r="G646" s="1">
-        <v>123946.87</v>
+        <v>130673.87</v>
       </c>
       <c r="H646" s="1">
         <v>0</v>
       </c>
       <c r="I646" s="1">
-        <v>123946.87</v>
+        <v>130673.87</v>
       </c>
     </row>
     <row r="647" spans="1:9" ht="12.75">
@@ -20321,13 +20321,13 @@
         <v>0</v>
       </c>
       <c r="G647" s="1">
-        <v>393958.93999999994</v>
+        <v>416845.94000000006</v>
       </c>
       <c r="H647" s="1">
         <v>0</v>
       </c>
       <c r="I647" s="1">
-        <v>393958.93999999994</v>
+        <v>416845.94000000006</v>
       </c>
     </row>
     <row r="648" spans="1:9" ht="12.75">
@@ -20437,13 +20437,13 @@
         <v>0</v>
       </c>
       <c r="G651" s="1">
-        <v>1824764.48</v>
+        <v>2189217.48</v>
       </c>
       <c r="H651" s="1">
         <v>13850.19</v>
       </c>
       <c r="I651" s="1">
-        <v>1810914.29</v>
+        <v>2175367.29</v>
       </c>
     </row>
     <row r="652" spans="1:9" ht="12.75">
@@ -20466,13 +20466,13 @@
         <v>0</v>
       </c>
       <c r="G652" s="1">
-        <v>289510.8900000001</v>
+        <v>346941.89</v>
       </c>
       <c r="H652" s="1">
         <v>0</v>
       </c>
       <c r="I652" s="1">
-        <v>289510.8900000001</v>
+        <v>346941.89</v>
       </c>
     </row>
     <row r="653" spans="1:9" ht="12.75">
@@ -20495,13 +20495,13 @@
         <v>0</v>
       </c>
       <c r="G653" s="1">
-        <v>19451</v>
+        <v>26855</v>
       </c>
       <c r="H653" s="1">
         <v>0</v>
       </c>
       <c r="I653" s="1">
-        <v>19451</v>
+        <v>26855</v>
       </c>
     </row>
     <row r="654" spans="1:9" ht="12.75">
@@ -20524,13 +20524,13 @@
         <v>0</v>
       </c>
       <c r="G654" s="1">
-        <v>264343.41000000003</v>
+        <v>341636.41000000003</v>
       </c>
       <c r="H654" s="1">
         <v>0</v>
       </c>
       <c r="I654" s="1">
-        <v>264343.41000000003</v>
+        <v>341636.41000000003</v>
       </c>
     </row>
     <row r="655" spans="1:9" ht="12.75">
@@ -20553,13 +20553,13 @@
         <v>0</v>
       </c>
       <c r="G655" s="1">
-        <v>211110</v>
+        <v>308971</v>
       </c>
       <c r="H655" s="1">
         <v>0</v>
       </c>
       <c r="I655" s="1">
-        <v>211110</v>
+        <v>308971</v>
       </c>
     </row>
     <row r="656" spans="1:9" ht="12.75">
@@ -20669,13 +20669,13 @@
         <v>0</v>
       </c>
       <c r="G659" s="1">
-        <v>2292091.5599999996</v>
+        <v>2292091.56</v>
       </c>
       <c r="H659" s="1">
         <v>0</v>
       </c>
       <c r="I659" s="1">
-        <v>2292091.5599999996</v>
+        <v>2292091.56</v>
       </c>
     </row>
     <row r="660" spans="1:9" ht="12.75">
@@ -20814,13 +20814,13 @@
         <v>0</v>
       </c>
       <c r="G664" s="1">
-        <v>171980.19999999998</v>
+        <v>171980.20</v>
       </c>
       <c r="H664" s="1">
         <v>0</v>
       </c>
       <c r="I664" s="1">
-        <v>171980.19999999998</v>
+        <v>171980.20</v>
       </c>
     </row>
     <row r="665" spans="1:9" ht="12.75">
@@ -20988,13 +20988,13 @@
         <v>0</v>
       </c>
       <c r="G670" s="1">
-        <v>780446.0900000001</v>
+        <v>780446.09</v>
       </c>
       <c r="H670" s="1">
         <v>0</v>
       </c>
       <c r="I670" s="1">
-        <v>780446.0900000001</v>
+        <v>780446.09</v>
       </c>
     </row>
     <row r="671" spans="1:9" ht="12.75">
@@ -21046,13 +21046,13 @@
         <v>0</v>
       </c>
       <c r="G672" s="1">
-        <v>617404.2000000001</v>
+        <v>617404.20</v>
       </c>
       <c r="H672" s="1">
         <v>0</v>
       </c>
       <c r="I672" s="1">
-        <v>617404.2000000001</v>
+        <v>617404.20</v>
       </c>
     </row>
     <row r="673" spans="1:9" ht="12.75">
@@ -21945,13 +21945,13 @@
         <v>0</v>
       </c>
       <c r="G703" s="1">
-        <v>2568009.0999999996</v>
+        <v>2568009.10</v>
       </c>
       <c r="H703" s="1">
         <v>0</v>
       </c>
       <c r="I703" s="1">
-        <v>2568009.0999999996</v>
+        <v>2568009.10</v>
       </c>
     </row>
     <row r="704" spans="1:9" ht="12.75">
@@ -22032,13 +22032,13 @@
         <v>0</v>
       </c>
       <c r="G706" s="1">
-        <v>906485.9900000001</v>
+        <v>906485.99</v>
       </c>
       <c r="H706" s="1">
         <v>0</v>
       </c>
       <c r="I706" s="1">
-        <v>906485.9900000001</v>
+        <v>906485.99</v>
       </c>
     </row>
     <row r="707" spans="1:9" ht="12.75">
@@ -22090,13 +22090,13 @@
         <v>0</v>
       </c>
       <c r="G708" s="1">
-        <v>4420392.420000001</v>
+        <v>4420392.42</v>
       </c>
       <c r="H708" s="1">
         <v>0</v>
       </c>
       <c r="I708" s="1">
-        <v>4420392.420000001</v>
+        <v>4420392.42</v>
       </c>
     </row>
     <row r="709" spans="1:9" ht="12.75">
@@ -22119,13 +22119,13 @@
         <v>0</v>
       </c>
       <c r="G709" s="1">
-        <v>5448697.79</v>
+        <v>5448697.789999999</v>
       </c>
       <c r="H709" s="1">
         <v>0</v>
       </c>
       <c r="I709" s="1">
-        <v>5448697.79</v>
+        <v>5448697.789999999</v>
       </c>
     </row>
     <row r="710" spans="1:9" ht="12.75">
@@ -22206,13 +22206,13 @@
         <v>0</v>
       </c>
       <c r="G712" s="1">
-        <v>699050.80</v>
+        <v>699050.7999999999</v>
       </c>
       <c r="H712" s="1">
         <v>0</v>
       </c>
       <c r="I712" s="1">
-        <v>699050.80</v>
+        <v>699050.7999999999</v>
       </c>
     </row>
     <row r="713" spans="1:9" ht="12.75">
@@ -22496,13 +22496,13 @@
         <v>0</v>
       </c>
       <c r="G722" s="1">
-        <v>253568.64</v>
+        <v>253568.63999999998</v>
       </c>
       <c r="H722" s="1">
         <v>0</v>
       </c>
       <c r="I722" s="1">
-        <v>253568.64</v>
+        <v>253568.63999999998</v>
       </c>
     </row>
     <row r="723" spans="1:9" ht="12.75">
@@ -22583,13 +22583,13 @@
         <v>0</v>
       </c>
       <c r="G725" s="1">
-        <v>742650.70</v>
+        <v>742650.7000000001</v>
       </c>
       <c r="H725" s="1">
         <v>0</v>
       </c>
       <c r="I725" s="1">
-        <v>742650.70</v>
+        <v>742650.7000000001</v>
       </c>
     </row>
     <row r="726" spans="1:9" ht="12.75">
@@ -22612,13 +22612,13 @@
         <v>0</v>
       </c>
       <c r="G726" s="1">
-        <v>180148.38999999998</v>
+        <v>180148.39</v>
       </c>
       <c r="H726" s="1">
         <v>0</v>
       </c>
       <c r="I726" s="1">
-        <v>180148.38999999998</v>
+        <v>180148.39</v>
       </c>
     </row>
     <row r="727" spans="1:9" ht="12.75">
@@ -22963,10 +22963,10 @@
         <v>0</v>
       </c>
       <c r="H738" s="1">
-        <v>7.258656367999999E7</v>
+        <v>7.258656368E7</v>
       </c>
       <c r="I738" s="1">
-        <v>-7.258656367999999E7</v>
+        <v>-7.258656368E7</v>
       </c>
     </row>
     <row r="739" spans="1:9" ht="12.75">
@@ -39896,13 +39896,13 @@
         <v>0</v>
       </c>
       <c r="G1322" s="1">
-        <v>8924065</v>
+        <v>9791056</v>
       </c>
       <c r="H1322" s="1">
         <v>42962</v>
       </c>
       <c r="I1322" s="1">
-        <v>8881103</v>
+        <v>9748094</v>
       </c>
     </row>
     <row r="1323" spans="1:9" ht="12.75">
@@ -40070,13 +40070,13 @@
         <v>0</v>
       </c>
       <c r="G1328" s="1">
-        <v>9735144</v>
+        <v>1.05036353E7</v>
       </c>
       <c r="H1328" s="1">
         <v>0</v>
       </c>
       <c r="I1328" s="1">
-        <v>9735144</v>
+        <v>1.05036353E7</v>
       </c>
     </row>
     <row r="1329" spans="1:9" ht="12.75">
@@ -40099,13 +40099,13 @@
         <v>0</v>
       </c>
       <c r="G1329" s="1">
-        <v>11579115</v>
+        <v>1.23715218E7</v>
       </c>
       <c r="H1329" s="1">
         <v>0</v>
       </c>
       <c r="I1329" s="1">
-        <v>11579115</v>
+        <v>1.23715218E7</v>
       </c>
     </row>
     <row r="1330" spans="1:9" ht="12.75">
@@ -40302,13 +40302,13 @@
         <v>0</v>
       </c>
       <c r="G1336" s="1">
-        <v>3.10352075E7</v>
+        <v>3.3413358649999995E7</v>
       </c>
       <c r="H1336" s="1">
         <v>179327</v>
       </c>
       <c r="I1336" s="1">
-        <v>3.08558805E7</v>
+        <v>3.3234031649999995E7</v>
       </c>
     </row>
     <row r="1337" spans="1:9" ht="12.75">
@@ -40331,13 +40331,13 @@
         <v>0</v>
       </c>
       <c r="G1337" s="1">
-        <v>1606330</v>
+        <v>1662977.08</v>
       </c>
       <c r="H1337" s="1">
         <v>0</v>
       </c>
       <c r="I1337" s="1">
-        <v>1606330</v>
+        <v>1662977.08</v>
       </c>
     </row>
     <row r="1338" spans="1:9" ht="12.75">
@@ -40679,13 +40679,13 @@
         <v>0</v>
       </c>
       <c r="G1349" s="1">
-        <v>10394483</v>
+        <v>1.154246725E7</v>
       </c>
       <c r="H1349" s="1">
         <v>0</v>
       </c>
       <c r="I1349" s="1">
-        <v>10394483</v>
+        <v>1.154246725E7</v>
       </c>
     </row>
     <row r="1350" spans="1:9" ht="12.75">
@@ -41172,13 +41172,13 @@
         <v>0</v>
       </c>
       <c r="G1366" s="1">
-        <v>2389566</v>
+        <v>2818928.45</v>
       </c>
       <c r="H1366" s="1">
         <v>0</v>
       </c>
       <c r="I1366" s="1">
-        <v>2389566</v>
+        <v>2818928.45</v>
       </c>
     </row>
     <row r="1367" spans="1:9" ht="12.75">
@@ -41259,13 +41259,13 @@
         <v>0</v>
       </c>
       <c r="G1369" s="1">
-        <v>6136325.75</v>
+        <v>6156604.55</v>
       </c>
       <c r="H1369" s="1">
         <v>0</v>
       </c>
       <c r="I1369" s="1">
-        <v>6136325.75</v>
+        <v>6156604.55</v>
       </c>
     </row>
     <row r="1370" spans="1:9" ht="12.75">
@@ -41317,13 +41317,13 @@
         <v>0</v>
       </c>
       <c r="G1371" s="1">
-        <v>29335095</v>
+        <v>3.2103355849999998E7</v>
       </c>
       <c r="H1371" s="1">
         <v>283032</v>
       </c>
       <c r="I1371" s="1">
-        <v>29052063</v>
+        <v>3.1820323849999998E7</v>
       </c>
     </row>
     <row r="1372" spans="1:9" ht="12.75">
@@ -41346,13 +41346,13 @@
         <v>0</v>
       </c>
       <c r="G1372" s="1">
-        <v>11579754</v>
+        <v>11915993</v>
       </c>
       <c r="H1372" s="1">
         <v>0</v>
       </c>
       <c r="I1372" s="1">
-        <v>11579754</v>
+        <v>11915993</v>
       </c>
     </row>
     <row r="1373" spans="1:9" ht="12.75">
@@ -41375,13 +41375,13 @@
         <v>0</v>
       </c>
       <c r="G1373" s="1">
-        <v>32093655</v>
+        <v>3.547111165E7</v>
       </c>
       <c r="H1373" s="1">
         <v>110222</v>
       </c>
       <c r="I1373" s="1">
-        <v>31983433</v>
+        <v>3.536088965E7</v>
       </c>
     </row>
     <row r="1374" spans="1:9" ht="12.75">
@@ -41607,13 +41607,13 @@
         <v>0</v>
       </c>
       <c r="G1381" s="1">
-        <v>6314857</v>
+        <v>6689781.3</v>
       </c>
       <c r="H1381" s="1">
         <v>34552</v>
       </c>
       <c r="I1381" s="1">
-        <v>6280305</v>
+        <v>6655229.3</v>
       </c>
     </row>
     <row r="1382" spans="1:9" ht="12.75">
@@ -41636,13 +41636,13 @@
         <v>0</v>
       </c>
       <c r="G1382" s="1">
-        <v>2982081</v>
+        <v>3209702</v>
       </c>
       <c r="H1382" s="1">
         <v>0</v>
       </c>
       <c r="I1382" s="1">
-        <v>2982081</v>
+        <v>3209702</v>
       </c>
     </row>
     <row r="1383" spans="1:9" ht="12.75">
@@ -41665,13 +41665,13 @@
         <v>0</v>
       </c>
       <c r="G1383" s="1">
-        <v>10318565</v>
+        <v>1.096874375E7</v>
       </c>
       <c r="H1383" s="1">
         <v>0</v>
       </c>
       <c r="I1383" s="1">
-        <v>10318565</v>
+        <v>1.096874375E7</v>
       </c>
     </row>
     <row r="1384" spans="1:9" ht="12.75">
@@ -41694,13 +41694,13 @@
         <v>0</v>
       </c>
       <c r="G1384" s="1">
-        <v>342536167</v>
+        <v>3.4273422562E8</v>
       </c>
       <c r="H1384" s="1">
-        <v>336929317</v>
+        <v>3.6262405171000004E8</v>
       </c>
       <c r="I1384" s="1">
-        <v>5606850</v>
+        <v>-1.9889826090000033E7</v>
       </c>
     </row>
     <row r="1385" spans="1:9" ht="12.75">
@@ -41723,13 +41723,13 @@
         <v>0</v>
       </c>
       <c r="G1385" s="1">
-        <v>4331900</v>
+        <v>5052296.40</v>
       </c>
       <c r="H1385" s="1">
         <v>0</v>
       </c>
       <c r="I1385" s="1">
-        <v>4331900</v>
+        <v>5052296.40</v>
       </c>
     </row>
     <row r="1386" spans="1:9" ht="12.75">
@@ -41781,13 +41781,13 @@
         <v>0</v>
       </c>
       <c r="G1387" s="1">
-        <v>10283936</v>
+        <v>1.10374221E7</v>
       </c>
       <c r="H1387" s="1">
         <v>0</v>
       </c>
       <c r="I1387" s="1">
-        <v>10283936</v>
+        <v>1.10374221E7</v>
       </c>
     </row>
     <row r="1388" spans="1:9" ht="12.75">
@@ -41810,13 +41810,13 @@
         <v>0</v>
       </c>
       <c r="G1388" s="1">
-        <v>7195666</v>
+        <v>7470866.4</v>
       </c>
       <c r="H1388" s="1">
         <v>0</v>
       </c>
       <c r="I1388" s="1">
-        <v>7195666</v>
+        <v>7470866.4</v>
       </c>
     </row>
     <row r="1389" spans="1:9" ht="12.75">
@@ -41868,13 +41868,13 @@
         <v>0</v>
       </c>
       <c r="G1390" s="1">
-        <v>1.701113675E7</v>
+        <v>1.8844467549999997E7</v>
       </c>
       <c r="H1390" s="1">
         <v>110222</v>
       </c>
       <c r="I1390" s="1">
-        <v>1.690091475E7</v>
+        <v>1.8734245549999997E7</v>
       </c>
     </row>
     <row r="1391" spans="1:9" ht="12.75">
@@ -41897,13 +41897,13 @@
         <v>0</v>
       </c>
       <c r="G1391" s="1">
-        <v>7541429</v>
+        <v>8018272.12</v>
       </c>
       <c r="H1391" s="1">
         <v>0</v>
       </c>
       <c r="I1391" s="1">
-        <v>7541429</v>
+        <v>8018272.12</v>
       </c>
     </row>
     <row r="1392" spans="1:9" ht="12.75">
@@ -41926,13 +41926,13 @@
         <v>0</v>
       </c>
       <c r="G1392" s="1">
-        <v>5548066</v>
+        <v>5878752</v>
       </c>
       <c r="H1392" s="1">
         <v>0</v>
       </c>
       <c r="I1392" s="1">
-        <v>5548066</v>
+        <v>5878752</v>
       </c>
     </row>
     <row r="1393" spans="1:9" ht="12.75">
@@ -41955,13 +41955,13 @@
         <v>0</v>
       </c>
       <c r="G1393" s="1">
-        <v>1357106</v>
+        <v>1439035.55</v>
       </c>
       <c r="H1393" s="1">
         <v>0</v>
       </c>
       <c r="I1393" s="1">
-        <v>1357106</v>
+        <v>1439035.55</v>
       </c>
     </row>
     <row r="1394" spans="1:9" ht="12.75">
@@ -41984,13 +41984,13 @@
         <v>0</v>
       </c>
       <c r="G1394" s="1">
-        <v>4232925</v>
+        <v>4507476.449999999</v>
       </c>
       <c r="H1394" s="1">
         <v>0</v>
       </c>
       <c r="I1394" s="1">
-        <v>4232925</v>
+        <v>4507476.449999999</v>
       </c>
     </row>
     <row r="1395" spans="1:9" ht="12.75">
@@ -42100,13 +42100,13 @@
         <v>0</v>
       </c>
       <c r="G1398" s="1">
-        <v>20221609</v>
+        <v>2.443130324E7</v>
       </c>
       <c r="H1398" s="1">
         <v>168699</v>
       </c>
       <c r="I1398" s="1">
-        <v>20052910</v>
+        <v>2.426260424E7</v>
       </c>
     </row>
     <row r="1399" spans="1:9" ht="12.75">
@@ -42129,13 +42129,13 @@
         <v>0</v>
       </c>
       <c r="G1399" s="1">
-        <v>2693220</v>
+        <v>3242649.65</v>
       </c>
       <c r="H1399" s="1">
         <v>0</v>
       </c>
       <c r="I1399" s="1">
-        <v>2693220</v>
+        <v>3242649.65</v>
       </c>
     </row>
     <row r="1400" spans="1:9" ht="12.75">
@@ -42158,13 +42158,13 @@
         <v>0</v>
       </c>
       <c r="G1400" s="1">
-        <v>187224</v>
+        <v>257508</v>
       </c>
       <c r="H1400" s="1">
         <v>0</v>
       </c>
       <c r="I1400" s="1">
-        <v>187224</v>
+        <v>257508</v>
       </c>
     </row>
     <row r="1401" spans="1:9" ht="12.75">
@@ -42187,13 +42187,13 @@
         <v>0</v>
       </c>
       <c r="G1401" s="1">
-        <v>2340270</v>
+        <v>3087516.70</v>
       </c>
       <c r="H1401" s="1">
         <v>0</v>
       </c>
       <c r="I1401" s="1">
-        <v>2340270</v>
+        <v>3087516.70</v>
       </c>
     </row>
     <row r="1402" spans="1:9" ht="12.75">
@@ -42216,13 +42216,13 @@
         <v>0</v>
       </c>
       <c r="G1402" s="1">
-        <v>2109421</v>
+        <v>3088025.30</v>
       </c>
       <c r="H1402" s="1">
         <v>0</v>
       </c>
       <c r="I1402" s="1">
-        <v>2109421</v>
+        <v>3088025.30</v>
       </c>
     </row>
     <row r="1403" spans="1:9" ht="12.75">
@@ -43782,13 +43782,13 @@
         <v>0</v>
       </c>
       <c r="G1456" s="1">
-        <v>1894601.3199999998</v>
+        <v>1894601.32</v>
       </c>
       <c r="H1456" s="1">
         <v>0</v>
       </c>
       <c r="I1456" s="1">
-        <v>1894601.3199999998</v>
+        <v>1894601.32</v>
       </c>
     </row>
     <row r="1457" spans="1:9" ht="12.75">
@@ -44968,16 +44968,16 @@
         <v>13</v>
       </c>
       <c r="F1497" s="1">
-        <v>-1.934719699999994E7</v>
+        <v>-1.934719699999988E7</v>
       </c>
       <c r="G1497" s="1">
-        <v>2.1356943530000022E8</v>
+        <v>2.1835296529999974E8</v>
       </c>
       <c r="H1497" s="1">
-        <v>2.0463859630000007E8</v>
+        <v>2.0468359629999986E8</v>
       </c>
       <c r="I1497" s="1">
-        <v>-1.0416357999999791E7</v>
+        <v>-5677828</v>
       </c>
     </row>
     <row r="1498" spans="1:9" ht="12.75">
@@ -45061,10 +45061,10 @@
         <v>2.288005138E7</v>
       </c>
       <c r="H1500" s="1">
-        <v>1.7524591380000003E7</v>
+        <v>1.752459138E7</v>
       </c>
       <c r="I1500" s="1">
-        <v>-3.725290298461914E-9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1501" spans="1:9" ht="12.75">
@@ -45551,13 +45551,13 @@
         <v>0</v>
       </c>
       <c r="G1517" s="1">
-        <v>557550.9299999999</v>
+        <v>557550.9300000002</v>
       </c>
       <c r="H1517" s="1">
-        <v>605654.3599999998</v>
+        <v>605654.3600000001</v>
       </c>
       <c r="I1517" s="1">
-        <v>-48103.42999999982</v>
+        <v>-48103.429999999935</v>
       </c>
     </row>
     <row r="1518" spans="1:9" ht="12.75">
@@ -45609,13 +45609,13 @@
         <v>0</v>
       </c>
       <c r="G1519" s="1">
-        <v>7533462.2</v>
+        <v>7533462.200000001</v>
       </c>
       <c r="H1519" s="1">
         <v>8946451.92</v>
       </c>
       <c r="I1519" s="1">
-        <v>-1412989.7199999997</v>
+        <v>-1412989.7199999988</v>
       </c>
     </row>
     <row r="1520" spans="1:9" ht="12.75">
@@ -45635,16 +45635,16 @@
         <v>13</v>
       </c>
       <c r="F1520" s="1">
-        <v>-56797.000000002794</v>
+        <v>-56797.00000000186</v>
       </c>
       <c r="G1520" s="1">
-        <v>3227421.9400000004</v>
+        <v>3227421.94</v>
       </c>
       <c r="H1520" s="1">
-        <v>3631156.9399999976</v>
+        <v>3631156.939999996</v>
       </c>
       <c r="I1520" s="1">
-        <v>-460532</v>
+        <v>-460531.99999999814</v>
       </c>
     </row>
     <row r="1521" spans="1:9" ht="12.75">
@@ -45693,16 +45693,16 @@
         <v>13</v>
       </c>
       <c r="F1522" s="1">
-        <v>-5.9604644775390625E-8</v>
+        <v>0</v>
       </c>
       <c r="G1522" s="1">
-        <v>1.1103225841799998E9</v>
+        <v>1.13963109789E9</v>
       </c>
       <c r="H1522" s="1">
-        <v>1.1103225841800017E9</v>
+        <v>1.139631097890001E9</v>
       </c>
       <c r="I1522" s="1">
-        <v>-1.9073486328125E-6</v>
+        <v>-9.5367431640625E-7</v>
       </c>
     </row>
     <row r="1523" spans="1:9" ht="12.75">
@@ -45728,10 +45728,10 @@
         <v>12492016</v>
       </c>
       <c r="H1523" s="1">
-        <v>3.1714416150000002E7</v>
+        <v>3.3977782150000006E7</v>
       </c>
       <c r="I1523" s="1">
-        <v>-2.0927816150000002E7</v>
+        <v>-2.3191182150000006E7</v>
       </c>
     </row>
     <row r="1524" spans="1:9" ht="12.75">
@@ -46624,13 +46624,13 @@
         <v>2.91937089E7</v>
       </c>
       <c r="G1554" s="1">
-        <v>6.935924803999999E7</v>
+        <v>6.935924804E7</v>
       </c>
       <c r="H1554" s="1">
-        <v>7.726492467999999E7</v>
+        <v>8.109376578E7</v>
       </c>
       <c r="I1554" s="1">
-        <v>2.1288032260000005E7</v>
+        <v>1.7459191159999996E7</v>
       </c>
     </row>
     <row r="1555" spans="1:9" ht="12.75">
@@ -46714,10 +46714,10 @@
         <v>8.56587629E8</v>
       </c>
       <c r="H1557" s="1">
-        <v>4.044345516E8</v>
+        <v>4.129673205999999E8</v>
       </c>
       <c r="I1557" s="1">
-        <v>4.521530774E8</v>
+        <v>4.436203084000001E8</v>
       </c>
     </row>
     <row r="1558" spans="1:9" ht="12.75">
@@ -47233,13 +47233,13 @@
         <v>0</v>
       </c>
       <c r="G1575" s="1">
-        <v>2.214539456E8</v>
+        <v>2.296955347E8</v>
       </c>
       <c r="H1575" s="1">
-        <v>1.3139281886000001E8</v>
+        <v>1.3963439582E8</v>
       </c>
       <c r="I1575" s="1">
-        <v>9.006112673999998E7</v>
+        <v>9.006113888E7</v>
       </c>
     </row>
     <row r="1576" spans="1:9" ht="12.75">
@@ -49785,13 +49785,13 @@
         <v>0</v>
       </c>
       <c r="G1663" s="1">
-        <v>2650789.6799999997</v>
+        <v>2650789.68</v>
       </c>
       <c r="H1663" s="1">
         <v>0</v>
       </c>
       <c r="I1663" s="1">
-        <v>2650789.6799999997</v>
+        <v>2650789.68</v>
       </c>
     </row>
     <row r="1664" spans="1:9" ht="12.75">
@@ -49843,13 +49843,13 @@
         <v>0</v>
       </c>
       <c r="G1665" s="1">
-        <v>1044931</v>
+        <v>1064956</v>
       </c>
       <c r="H1665" s="1">
         <v>0</v>
       </c>
       <c r="I1665" s="1">
-        <v>1044931</v>
+        <v>1064956</v>
       </c>
     </row>
     <row r="1666" spans="1:9" ht="12.75">
@@ -49872,13 +49872,13 @@
         <v>0</v>
       </c>
       <c r="G1666" s="1">
-        <v>194293</v>
+        <v>204303</v>
       </c>
       <c r="H1666" s="1">
         <v>0</v>
       </c>
       <c r="I1666" s="1">
-        <v>194293</v>
+        <v>204303</v>
       </c>
     </row>
     <row r="1667" spans="1:9" ht="12.75">
@@ -50104,13 +50104,13 @@
         <v>0</v>
       </c>
       <c r="G1674" s="1">
-        <v>2462526</v>
+        <v>2471021</v>
       </c>
       <c r="H1674" s="1">
         <v>0</v>
       </c>
       <c r="I1674" s="1">
-        <v>2462526</v>
+        <v>2471021</v>
       </c>
     </row>
     <row r="1675" spans="1:9" ht="12.75">
@@ -50278,13 +50278,13 @@
         <v>0</v>
       </c>
       <c r="G1680" s="1">
-        <v>65932</v>
+        <v>87682</v>
       </c>
       <c r="H1680" s="1">
         <v>0</v>
       </c>
       <c r="I1680" s="1">
-        <v>65932</v>
+        <v>87682</v>
       </c>
     </row>
     <row r="1681" spans="1:9" ht="12.75">
@@ -50307,13 +50307,13 @@
         <v>0</v>
       </c>
       <c r="G1681" s="1">
-        <v>86124</v>
+        <v>138888</v>
       </c>
       <c r="H1681" s="1">
         <v>0</v>
       </c>
       <c r="I1681" s="1">
-        <v>86124</v>
+        <v>138888</v>
       </c>
     </row>
     <row r="1682" spans="1:9" ht="12.75">
@@ -50336,13 +50336,13 @@
         <v>0</v>
       </c>
       <c r="G1682" s="1">
-        <v>1021380</v>
+        <v>1364844</v>
       </c>
       <c r="H1682" s="1">
         <v>0</v>
       </c>
       <c r="I1682" s="1">
-        <v>1021380</v>
+        <v>1364844</v>
       </c>
     </row>
     <row r="1683" spans="1:9" ht="12.75">
@@ -50423,13 +50423,13 @@
         <v>0</v>
       </c>
       <c r="G1685" s="1">
-        <v>219258</v>
+        <v>268442</v>
       </c>
       <c r="H1685" s="1">
         <v>0</v>
       </c>
       <c r="I1685" s="1">
-        <v>219258</v>
+        <v>268442</v>
       </c>
     </row>
     <row r="1686" spans="1:9" ht="12.75">
@@ -50455,10 +50455,10 @@
         <v>4807583</v>
       </c>
       <c r="H1686" s="1">
-        <v>4807583</v>
+        <v>6154176</v>
       </c>
       <c r="I1686" s="1">
-        <v>0</v>
+        <v>-1346593</v>
       </c>
     </row>
     <row r="1687" spans="1:9" ht="12.75">
@@ -50481,13 +50481,13 @@
         <v>0</v>
       </c>
       <c r="G1687" s="1">
-        <v>152600</v>
+        <v>187978</v>
       </c>
       <c r="H1687" s="1">
         <v>0</v>
       </c>
       <c r="I1687" s="1">
-        <v>152600</v>
+        <v>187978</v>
       </c>
     </row>
     <row r="1688" spans="1:9" ht="12.75">
@@ -50510,13 +50510,13 @@
         <v>0</v>
       </c>
       <c r="G1688" s="1">
-        <v>1414429</v>
+        <v>2258482</v>
       </c>
       <c r="H1688" s="1">
         <v>0</v>
       </c>
       <c r="I1688" s="1">
-        <v>1414429</v>
+        <v>2258482</v>
       </c>
     </row>
     <row r="1689" spans="1:9" ht="12.75">
@@ -50597,13 +50597,13 @@
         <v>0</v>
       </c>
       <c r="G1691" s="1">
-        <v>289295.48</v>
+        <v>438832.48</v>
       </c>
       <c r="H1691" s="1">
         <v>0</v>
       </c>
       <c r="I1691" s="1">
-        <v>289295.48</v>
+        <v>438832.48</v>
       </c>
     </row>
     <row r="1692" spans="1:9" ht="12.75">
@@ -50626,13 +50626,13 @@
         <v>0</v>
       </c>
       <c r="G1692" s="1">
-        <v>218609.21999999997</v>
+        <v>307784.22</v>
       </c>
       <c r="H1692" s="1">
         <v>0</v>
       </c>
       <c r="I1692" s="1">
-        <v>218609.21999999997</v>
+        <v>307784.22</v>
       </c>
     </row>
     <row r="1693" spans="1:9" ht="12.75">
@@ -50655,13 +50655,13 @@
         <v>0</v>
       </c>
       <c r="G1693" s="1">
-        <v>1910663.08</v>
+        <v>2335546.08</v>
       </c>
       <c r="H1693" s="1">
         <v>0</v>
       </c>
       <c r="I1693" s="1">
-        <v>1910663.08</v>
+        <v>2335546.08</v>
       </c>
     </row>
     <row r="1694" spans="1:9" ht="12.75">
@@ -50684,13 +50684,13 @@
         <v>0</v>
       </c>
       <c r="G1694" s="1">
+        <v>685737.6100000001</v>
+      </c>
+      <c r="H1694" s="1">
         <v>685737.61</v>
       </c>
-      <c r="H1694" s="1">
-        <v>685737.6100000001</v>
-      </c>
       <c r="I1694" s="1">
-        <v>-1.1641532182693481E-10</v>
+        <v>1.1641532182693481E-10</v>
       </c>
     </row>
     <row r="1695" spans="1:9" ht="12.75">
@@ -50742,13 +50742,13 @@
         <v>0</v>
       </c>
       <c r="G1696" s="1">
-        <v>191355.02</v>
+        <v>191355.02000000002</v>
       </c>
       <c r="H1696" s="1">
         <v>93523</v>
       </c>
       <c r="I1696" s="1">
-        <v>97832.01999999999</v>
+        <v>97832.02000000002</v>
       </c>
     </row>
     <row r="1697" spans="1:9" ht="12.75">
@@ -50771,13 +50771,13 @@
         <v>0</v>
       </c>
       <c r="G1697" s="1">
-        <v>381348.31999999995</v>
+        <v>456691.32</v>
       </c>
       <c r="H1697" s="1">
         <v>0</v>
       </c>
       <c r="I1697" s="1">
-        <v>381348.31999999995</v>
+        <v>456691.32</v>
       </c>
     </row>
     <row r="1698" spans="1:9" ht="12.75">
@@ -50800,13 +50800,13 @@
         <v>0</v>
       </c>
       <c r="G1698" s="1">
-        <v>280517</v>
+        <v>410088</v>
       </c>
       <c r="H1698" s="1">
         <v>93497</v>
       </c>
       <c r="I1698" s="1">
-        <v>187020</v>
+        <v>316591</v>
       </c>
     </row>
     <row r="1699" spans="1:9" ht="12.75">
@@ -50829,13 +50829,13 @@
         <v>0</v>
       </c>
       <c r="G1699" s="1">
-        <v>1107845.6099999999</v>
+        <v>1406462.6099999999</v>
       </c>
       <c r="H1699" s="1">
         <v>211054</v>
       </c>
       <c r="I1699" s="1">
-        <v>896791.6099999999</v>
+        <v>1195408.6099999999</v>
       </c>
     </row>
     <row r="1700" spans="1:9" ht="12.75">
@@ -50858,13 +50858,13 @@
         <v>0</v>
       </c>
       <c r="G1700" s="1">
-        <v>2193609</v>
+        <v>3389832</v>
       </c>
       <c r="H1700" s="1">
         <v>0</v>
       </c>
       <c r="I1700" s="1">
-        <v>2193609</v>
+        <v>3389832</v>
       </c>
     </row>
     <row r="1701" spans="1:9" ht="12.75">
@@ -52163,13 +52163,13 @@
         <v>0</v>
       </c>
       <c r="G1745" s="1">
-        <v>577360</v>
+        <v>595360</v>
       </c>
       <c r="H1745" s="1">
         <v>0</v>
       </c>
       <c r="I1745" s="1">
-        <v>577360</v>
+        <v>595360</v>
       </c>
     </row>
     <row r="1746" spans="1:9" ht="12.75">
@@ -52215,19 +52215,19 @@
         <v>238</v>
       </c>
       <c r="E1747" t="s">
-        <v>334</v>
+        <v>355</v>
       </c>
       <c r="F1747" s="1">
         <v>0</v>
       </c>
       <c r="G1747" s="1">
-        <v>279345</v>
+        <v>42000</v>
       </c>
       <c r="H1747" s="1">
         <v>0</v>
       </c>
       <c r="I1747" s="1">
-        <v>279345</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="1748" spans="1:9" ht="12.75">
@@ -52244,19 +52244,19 @@
         <v>238</v>
       </c>
       <c r="E1748" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1748" s="1">
         <v>0</v>
       </c>
       <c r="G1748" s="1">
-        <v>137184</v>
+        <v>279345</v>
       </c>
       <c r="H1748" s="1">
         <v>0</v>
       </c>
       <c r="I1748" s="1">
-        <v>137184</v>
+        <v>279345</v>
       </c>
     </row>
     <row r="1749" spans="1:9" ht="12.75">
@@ -52273,19 +52273,19 @@
         <v>238</v>
       </c>
       <c r="E1749" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F1749" s="1">
         <v>0</v>
       </c>
       <c r="G1749" s="1">
-        <v>91456</v>
+        <v>137184</v>
       </c>
       <c r="H1749" s="1">
         <v>0</v>
       </c>
       <c r="I1749" s="1">
-        <v>91456</v>
+        <v>137184</v>
       </c>
     </row>
     <row r="1750" spans="1:9" ht="12.75">
@@ -52302,19 +52302,19 @@
         <v>238</v>
       </c>
       <c r="E1750" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="F1750" s="1">
         <v>0</v>
       </c>
       <c r="G1750" s="1">
-        <v>104725</v>
+        <v>91456</v>
       </c>
       <c r="H1750" s="1">
         <v>0</v>
       </c>
       <c r="I1750" s="1">
-        <v>104725</v>
+        <v>91456</v>
       </c>
     </row>
     <row r="1751" spans="1:9" ht="12.75">
@@ -52331,19 +52331,19 @@
         <v>238</v>
       </c>
       <c r="E1751" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F1751" s="1">
         <v>0</v>
       </c>
       <c r="G1751" s="1">
-        <v>209450</v>
+        <v>104725</v>
       </c>
       <c r="H1751" s="1">
         <v>0</v>
       </c>
       <c r="I1751" s="1">
-        <v>209450</v>
+        <v>104725</v>
       </c>
     </row>
     <row r="1752" spans="1:9" ht="12.75">
@@ -52357,22 +52357,22 @@
         <v>105</v>
       </c>
       <c r="D1752" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E1752" t="s">
-        <v>330</v>
+        <v>346</v>
       </c>
       <c r="F1752" s="1">
         <v>0</v>
       </c>
       <c r="G1752" s="1">
-        <v>8770</v>
+        <v>209450</v>
       </c>
       <c r="H1752" s="1">
         <v>0</v>
       </c>
       <c r="I1752" s="1">
-        <v>8770</v>
+        <v>209450</v>
       </c>
     </row>
     <row r="1753" spans="1:9" ht="12.75">
@@ -52386,7 +52386,7 @@
         <v>105</v>
       </c>
       <c r="D1753" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E1753" t="s">
         <v>330</v>
@@ -52395,13 +52395,13 @@
         <v>0</v>
       </c>
       <c r="G1753" s="1">
-        <v>77798.34</v>
+        <v>8770</v>
       </c>
       <c r="H1753" s="1">
         <v>0</v>
       </c>
       <c r="I1753" s="1">
-        <v>77798.34</v>
+        <v>8770</v>
       </c>
     </row>
     <row r="1754" spans="1:9" ht="12.75">
@@ -52415,22 +52415,22 @@
         <v>105</v>
       </c>
       <c r="D1754" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E1754" t="s">
-        <v>13</v>
+        <v>330</v>
       </c>
       <c r="F1754" s="1">
         <v>0</v>
       </c>
       <c r="G1754" s="1">
-        <v>0.9000000000000001</v>
+        <v>84726.34</v>
       </c>
       <c r="H1754" s="1">
-        <v>12.20</v>
+        <v>0</v>
       </c>
       <c r="I1754" s="1">
-        <v>-11.30</v>
+        <v>84726.34</v>
       </c>
     </row>
     <row r="1755" spans="1:9" ht="12.75">
@@ -52444,22 +52444,22 @@
         <v>105</v>
       </c>
       <c r="D1755" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E1755" t="s">
-        <v>329</v>
+        <v>13</v>
       </c>
       <c r="F1755" s="1">
         <v>0</v>
       </c>
       <c r="G1755" s="1">
-        <v>8760</v>
+        <v>0.9000000000000001</v>
       </c>
       <c r="H1755" s="1">
-        <v>0</v>
+        <v>12.20</v>
       </c>
       <c r="I1755" s="1">
-        <v>8760</v>
+        <v>-11.30</v>
       </c>
     </row>
     <row r="1756" spans="1:9" ht="12.75">
@@ -52476,19 +52476,19 @@
         <v>243</v>
       </c>
       <c r="E1756" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1756" s="1">
         <v>0</v>
       </c>
       <c r="G1756" s="1">
-        <v>10453827</v>
+        <v>8760</v>
       </c>
       <c r="H1756" s="1">
         <v>0</v>
       </c>
       <c r="I1756" s="1">
-        <v>10453827</v>
+        <v>8760</v>
       </c>
     </row>
     <row r="1757" spans="1:9" ht="12.75">
@@ -52505,19 +52505,19 @@
         <v>243</v>
       </c>
       <c r="E1757" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1757" s="1">
         <v>0</v>
       </c>
       <c r="G1757" s="1">
-        <v>7800000</v>
+        <v>10453827</v>
       </c>
       <c r="H1757" s="1">
         <v>0</v>
       </c>
       <c r="I1757" s="1">
-        <v>7800000</v>
+        <v>10453827</v>
       </c>
     </row>
     <row r="1758" spans="1:9" ht="12.75">
@@ -52534,19 +52534,19 @@
         <v>243</v>
       </c>
       <c r="E1758" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F1758" s="1">
         <v>0</v>
       </c>
       <c r="G1758" s="1">
-        <v>117363390</v>
+        <v>7800000</v>
       </c>
       <c r="H1758" s="1">
         <v>0</v>
       </c>
       <c r="I1758" s="1">
-        <v>117363390</v>
+        <v>7800000</v>
       </c>
     </row>
     <row r="1759" spans="1:9" ht="12.75">
@@ -52563,19 +52563,19 @@
         <v>243</v>
       </c>
       <c r="E1759" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1759" s="1">
         <v>0</v>
       </c>
       <c r="G1759" s="1">
-        <v>5415020</v>
+        <v>117363390</v>
       </c>
       <c r="H1759" s="1">
         <v>0</v>
       </c>
       <c r="I1759" s="1">
-        <v>5415020</v>
+        <v>117363390</v>
       </c>
     </row>
     <row r="1760" spans="1:9" ht="12.75">
@@ -52592,19 +52592,19 @@
         <v>243</v>
       </c>
       <c r="E1760" t="s">
-        <v>355</v>
+        <v>335</v>
       </c>
       <c r="F1760" s="1">
         <v>0</v>
       </c>
       <c r="G1760" s="1">
-        <v>6372000</v>
+        <v>5415020</v>
       </c>
       <c r="H1760" s="1">
         <v>0</v>
       </c>
       <c r="I1760" s="1">
-        <v>6372000</v>
+        <v>5415020</v>
       </c>
     </row>
     <row r="1761" spans="1:9" ht="12.75">
@@ -52621,19 +52621,19 @@
         <v>243</v>
       </c>
       <c r="E1761" t="s">
-        <v>338</v>
+        <v>356</v>
       </c>
       <c r="F1761" s="1">
         <v>0</v>
       </c>
       <c r="G1761" s="1">
-        <v>12480860</v>
+        <v>6372000</v>
       </c>
       <c r="H1761" s="1">
         <v>0</v>
       </c>
       <c r="I1761" s="1">
-        <v>12480860</v>
+        <v>6372000</v>
       </c>
     </row>
     <row r="1762" spans="1:9" ht="12.75">
@@ -52650,19 +52650,19 @@
         <v>243</v>
       </c>
       <c r="E1762" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F1762" s="1">
         <v>0</v>
       </c>
       <c r="G1762" s="1">
-        <v>51988362</v>
+        <v>12480860</v>
       </c>
       <c r="H1762" s="1">
         <v>0</v>
       </c>
       <c r="I1762" s="1">
-        <v>51988362</v>
+        <v>12480860</v>
       </c>
     </row>
     <row r="1763" spans="1:9" ht="12.75">
@@ -52679,19 +52679,19 @@
         <v>243</v>
       </c>
       <c r="E1763" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="F1763" s="1">
         <v>0</v>
       </c>
       <c r="G1763" s="1">
-        <v>1194533</v>
+        <v>51988362</v>
       </c>
       <c r="H1763" s="1">
         <v>0</v>
       </c>
       <c r="I1763" s="1">
-        <v>1194533</v>
+        <v>51988362</v>
       </c>
     </row>
     <row r="1764" spans="1:9" ht="12.75">
@@ -52708,19 +52708,19 @@
         <v>243</v>
       </c>
       <c r="E1764" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="F1764" s="1">
         <v>0</v>
       </c>
       <c r="G1764" s="1">
-        <v>3212470</v>
+        <v>1194533</v>
       </c>
       <c r="H1764" s="1">
         <v>0</v>
       </c>
       <c r="I1764" s="1">
-        <v>3212470</v>
+        <v>1194533</v>
       </c>
     </row>
     <row r="1765" spans="1:9" ht="12.75">
@@ -52737,19 +52737,19 @@
         <v>243</v>
       </c>
       <c r="E1765" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F1765" s="1">
         <v>0</v>
       </c>
       <c r="G1765" s="1">
-        <v>1194533</v>
+        <v>3212470</v>
       </c>
       <c r="H1765" s="1">
         <v>0</v>
       </c>
       <c r="I1765" s="1">
-        <v>1194533</v>
+        <v>3212470</v>
       </c>
     </row>
     <row r="1766" spans="1:9" ht="12.75">
@@ -52763,22 +52763,22 @@
         <v>105</v>
       </c>
       <c r="D1766" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1766" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="F1766" s="1">
         <v>0</v>
       </c>
       <c r="G1766" s="1">
-        <v>31481</v>
+        <v>1194533</v>
       </c>
       <c r="H1766" s="1">
         <v>0</v>
       </c>
       <c r="I1766" s="1">
-        <v>31481</v>
+        <v>1194533</v>
       </c>
     </row>
     <row r="1767" spans="1:9" ht="12.75">
@@ -52795,19 +52795,19 @@
         <v>246</v>
       </c>
       <c r="E1767" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1767" s="1">
         <v>0</v>
       </c>
       <c r="G1767" s="1">
-        <v>6638</v>
+        <v>31481</v>
       </c>
       <c r="H1767" s="1">
         <v>0</v>
       </c>
       <c r="I1767" s="1">
-        <v>6638</v>
+        <v>31481</v>
       </c>
     </row>
     <row r="1768" spans="1:9" ht="12.75">
@@ -52824,19 +52824,19 @@
         <v>246</v>
       </c>
       <c r="E1768" t="s">
-        <v>356</v>
+        <v>332</v>
       </c>
       <c r="F1768" s="1">
         <v>0</v>
       </c>
       <c r="G1768" s="1">
-        <v>7140</v>
+        <v>6638</v>
       </c>
       <c r="H1768" s="1">
         <v>0</v>
       </c>
       <c r="I1768" s="1">
-        <v>7140</v>
+        <v>6638</v>
       </c>
     </row>
     <row r="1769" spans="1:9" ht="12.75">
@@ -52853,19 +52853,19 @@
         <v>246</v>
       </c>
       <c r="E1769" t="s">
-        <v>338</v>
+        <v>355</v>
       </c>
       <c r="F1769" s="1">
         <v>0</v>
       </c>
       <c r="G1769" s="1">
-        <v>41204</v>
+        <v>7140</v>
       </c>
       <c r="H1769" s="1">
         <v>0</v>
       </c>
       <c r="I1769" s="1">
-        <v>41204</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="1770" spans="1:9" ht="12.75">
@@ -52879,22 +52879,22 @@
         <v>105</v>
       </c>
       <c r="D1770" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E1770" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="F1770" s="1">
         <v>0</v>
       </c>
       <c r="G1770" s="1">
-        <v>77571</v>
+        <v>41204</v>
       </c>
       <c r="H1770" s="1">
         <v>0</v>
       </c>
       <c r="I1770" s="1">
-        <v>77571</v>
+        <v>41204</v>
       </c>
     </row>
     <row r="1771" spans="1:9" ht="12.75">
@@ -52911,19 +52911,19 @@
         <v>247</v>
       </c>
       <c r="E1771" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1771" s="1">
         <v>0</v>
       </c>
       <c r="G1771" s="1">
-        <v>1513824</v>
+        <v>77571</v>
       </c>
       <c r="H1771" s="1">
         <v>0</v>
       </c>
       <c r="I1771" s="1">
-        <v>1513824</v>
+        <v>77571</v>
       </c>
     </row>
     <row r="1772" spans="1:9" ht="12.75">
@@ -52940,19 +52940,19 @@
         <v>247</v>
       </c>
       <c r="E1772" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F1772" s="1">
         <v>0</v>
       </c>
       <c r="G1772" s="1">
-        <v>22538</v>
+        <v>1513824</v>
       </c>
       <c r="H1772" s="1">
         <v>0</v>
       </c>
       <c r="I1772" s="1">
-        <v>22538</v>
+        <v>1513824</v>
       </c>
     </row>
     <row r="1773" spans="1:9" ht="12.75">
@@ -52966,22 +52966,22 @@
         <v>105</v>
       </c>
       <c r="D1773" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E1773" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F1773" s="1">
         <v>0</v>
       </c>
       <c r="G1773" s="1">
-        <v>9676</v>
+        <v>22538</v>
       </c>
       <c r="H1773" s="1">
         <v>0</v>
       </c>
       <c r="I1773" s="1">
-        <v>9676</v>
+        <v>22538</v>
       </c>
     </row>
     <row r="1774" spans="1:9" ht="12.75">
@@ -52995,22 +52995,22 @@
         <v>105</v>
       </c>
       <c r="D1774" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E1774" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F1774" s="1">
         <v>0</v>
       </c>
       <c r="G1774" s="1">
-        <v>3353166</v>
+        <v>9676</v>
       </c>
       <c r="H1774" s="1">
         <v>0</v>
       </c>
       <c r="I1774" s="1">
-        <v>3353166</v>
+        <v>9676</v>
       </c>
     </row>
     <row r="1775" spans="1:9" ht="12.75">
@@ -53027,19 +53027,19 @@
         <v>250</v>
       </c>
       <c r="E1775" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1775" s="1">
         <v>0</v>
       </c>
       <c r="G1775" s="1">
-        <v>662779</v>
+        <v>3556925.1799999997</v>
       </c>
       <c r="H1775" s="1">
         <v>0</v>
       </c>
       <c r="I1775" s="1">
-        <v>662779</v>
+        <v>3556925.1799999997</v>
       </c>
     </row>
     <row r="1776" spans="1:9" ht="12.75">
@@ -53056,19 +53056,19 @@
         <v>250</v>
       </c>
       <c r="E1776" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1776" s="1">
         <v>0</v>
       </c>
       <c r="G1776" s="1">
-        <v>31417864</v>
+        <v>734237.45</v>
       </c>
       <c r="H1776" s="1">
-        <v>31417864</v>
+        <v>0</v>
       </c>
       <c r="I1776" s="1">
-        <v>0</v>
+        <v>734237.45</v>
       </c>
     </row>
     <row r="1777" spans="1:9" ht="12.75">
@@ -53085,19 +53085,19 @@
         <v>250</v>
       </c>
       <c r="E1777" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1777" s="1">
         <v>0</v>
       </c>
       <c r="G1777" s="1">
-        <v>2664907</v>
+        <v>31417864</v>
       </c>
       <c r="H1777" s="1">
-        <v>0</v>
+        <v>31417864</v>
       </c>
       <c r="I1777" s="1">
-        <v>2664907</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1778" spans="1:9" ht="12.75">
@@ -53114,19 +53114,19 @@
         <v>250</v>
       </c>
       <c r="E1778" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1778" s="1">
         <v>0</v>
       </c>
       <c r="G1778" s="1">
-        <v>2021829</v>
+        <v>4138525.55</v>
       </c>
       <c r="H1778" s="1">
         <v>0</v>
       </c>
       <c r="I1778" s="1">
-        <v>2021829</v>
+        <v>4138525.55</v>
       </c>
     </row>
     <row r="1779" spans="1:9" ht="12.75">
@@ -53143,19 +53143,19 @@
         <v>250</v>
       </c>
       <c r="E1779" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F1779" s="1">
         <v>0</v>
       </c>
       <c r="G1779" s="1">
-        <v>14946353</v>
+        <v>2860819.35</v>
       </c>
       <c r="H1779" s="1">
         <v>0</v>
       </c>
       <c r="I1779" s="1">
-        <v>14946353</v>
+        <v>2860819.35</v>
       </c>
     </row>
     <row r="1780" spans="1:9" ht="12.75">
@@ -53172,19 +53172,19 @@
         <v>250</v>
       </c>
       <c r="E1780" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1780" s="1">
         <v>0</v>
       </c>
       <c r="G1780" s="1">
-        <v>5986158</v>
+        <v>1.88516954E7</v>
       </c>
       <c r="H1780" s="1">
-        <v>5986158</v>
+        <v>0</v>
       </c>
       <c r="I1780" s="1">
-        <v>0</v>
+        <v>1.88516954E7</v>
       </c>
     </row>
     <row r="1781" spans="1:9" ht="12.75">
@@ -53201,19 +53201,19 @@
         <v>250</v>
       </c>
       <c r="E1781" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F1781" s="1">
         <v>0</v>
       </c>
       <c r="G1781" s="1">
-        <v>30819</v>
+        <v>5986158</v>
       </c>
       <c r="H1781" s="1">
-        <v>0</v>
+        <v>5986158</v>
       </c>
       <c r="I1781" s="1">
-        <v>30819</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1782" spans="1:9" ht="12.75">
@@ -53230,19 +53230,19 @@
         <v>250</v>
       </c>
       <c r="E1782" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F1782" s="1">
         <v>0</v>
       </c>
       <c r="G1782" s="1">
-        <v>1516559</v>
+        <v>30819</v>
       </c>
       <c r="H1782" s="1">
-        <v>747735</v>
+        <v>0</v>
       </c>
       <c r="I1782" s="1">
-        <v>768824</v>
+        <v>30819</v>
       </c>
     </row>
     <row r="1783" spans="1:9" ht="12.75">
@@ -53259,19 +53259,19 @@
         <v>250</v>
       </c>
       <c r="E1783" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F1783" s="1">
         <v>0</v>
       </c>
       <c r="G1783" s="1">
-        <v>3492740</v>
+        <v>1516559</v>
       </c>
       <c r="H1783" s="1">
-        <v>0</v>
+        <v>747735</v>
       </c>
       <c r="I1783" s="1">
-        <v>3492740</v>
+        <v>768824</v>
       </c>
     </row>
     <row r="1784" spans="1:9" ht="12.75">
@@ -53288,19 +53288,19 @@
         <v>250</v>
       </c>
       <c r="E1784" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F1784" s="1">
         <v>0</v>
       </c>
       <c r="G1784" s="1">
-        <v>75917498</v>
+        <v>4196982</v>
       </c>
       <c r="H1784" s="1">
-        <v>75931161</v>
+        <v>0</v>
       </c>
       <c r="I1784" s="1">
-        <v>-13663</v>
+        <v>4196982</v>
       </c>
     </row>
     <row r="1785" spans="1:9" ht="12.75">
@@ -53317,19 +53317,19 @@
         <v>250</v>
       </c>
       <c r="E1785" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F1785" s="1">
         <v>0</v>
       </c>
       <c r="G1785" s="1">
-        <v>1495219</v>
+        <v>75917498</v>
       </c>
       <c r="H1785" s="1">
-        <v>0</v>
+        <v>9.849326033E7</v>
       </c>
       <c r="I1785" s="1">
-        <v>1495219</v>
+        <v>-2.257576233E7</v>
       </c>
     </row>
     <row r="1786" spans="1:9" ht="12.75">
@@ -53346,19 +53346,19 @@
         <v>250</v>
       </c>
       <c r="E1786" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F1786" s="1">
         <v>0</v>
       </c>
       <c r="G1786" s="1">
-        <v>7812674</v>
+        <v>2790926.0999999996</v>
       </c>
       <c r="H1786" s="1">
         <v>0</v>
       </c>
       <c r="I1786" s="1">
-        <v>7812674</v>
+        <v>2790926.0999999996</v>
       </c>
     </row>
     <row r="1787" spans="1:9" ht="12.75">
@@ -53375,19 +53375,19 @@
         <v>250</v>
       </c>
       <c r="E1787" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F1787" s="1">
         <v>0</v>
       </c>
       <c r="G1787" s="1">
-        <v>19540359</v>
+        <v>1.07634571E7</v>
       </c>
       <c r="H1787" s="1">
         <v>0</v>
       </c>
       <c r="I1787" s="1">
-        <v>19540359</v>
+        <v>1.07634571E7</v>
       </c>
     </row>
     <row r="1788" spans="1:9" ht="12.75">
@@ -53404,19 +53404,19 @@
         <v>250</v>
       </c>
       <c r="E1788" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F1788" s="1">
         <v>0</v>
       </c>
       <c r="G1788" s="1">
-        <v>21704777</v>
+        <v>3.0658557200000003E7</v>
       </c>
       <c r="H1788" s="1">
         <v>0</v>
       </c>
       <c r="I1788" s="1">
-        <v>21704777</v>
+        <v>3.0658557200000003E7</v>
       </c>
     </row>
     <row r="1789" spans="1:9" ht="12.75">
@@ -53430,22 +53430,22 @@
         <v>105</v>
       </c>
       <c r="D1789" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E1789" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="F1789" s="1">
         <v>0</v>
       </c>
       <c r="G1789" s="1">
-        <v>0.15</v>
+        <v>21704777</v>
       </c>
       <c r="H1789" s="1">
         <v>0</v>
       </c>
       <c r="I1789" s="1">
-        <v>0.15</v>
+        <v>21704777</v>
       </c>
     </row>
     <row r="1790" spans="1:9" ht="12.75">
@@ -53462,19 +53462,19 @@
         <v>253</v>
       </c>
       <c r="E1790" t="s">
-        <v>339</v>
+        <v>349</v>
       </c>
       <c r="F1790" s="1">
         <v>0</v>
       </c>
       <c r="G1790" s="1">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="H1790" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I1790" s="1">
-        <v>-1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="1791" spans="1:9" ht="12.75">
@@ -53488,22 +53488,22 @@
         <v>105</v>
       </c>
       <c r="D1791" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E1791" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="F1791" s="1">
         <v>0</v>
       </c>
       <c r="G1791" s="1">
-        <v>148184</v>
+        <v>0</v>
       </c>
       <c r="H1791" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I1791" s="1">
-        <v>148184</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="1792" spans="1:9" ht="12.75">
@@ -53520,19 +53520,19 @@
         <v>257</v>
       </c>
       <c r="E1792" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F1792" s="1">
         <v>0</v>
       </c>
       <c r="G1792" s="1">
-        <v>74092</v>
+        <v>148184</v>
       </c>
       <c r="H1792" s="1">
         <v>0</v>
       </c>
       <c r="I1792" s="1">
-        <v>74092</v>
+        <v>148184</v>
       </c>
     </row>
     <row r="1793" spans="1:9" ht="12.75">
@@ -53549,19 +53549,19 @@
         <v>257</v>
       </c>
       <c r="E1793" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1793" s="1">
         <v>0</v>
       </c>
       <c r="G1793" s="1">
-        <v>74092.80</v>
+        <v>74092</v>
       </c>
       <c r="H1793" s="1">
         <v>0</v>
       </c>
       <c r="I1793" s="1">
-        <v>74092.80</v>
+        <v>74092</v>
       </c>
     </row>
     <row r="1794" spans="1:9" ht="12.75">
@@ -53578,19 +53578,19 @@
         <v>257</v>
       </c>
       <c r="E1794" t="s">
-        <v>357</v>
+        <v>335</v>
       </c>
       <c r="F1794" s="1">
         <v>0</v>
       </c>
       <c r="G1794" s="1">
-        <v>163430</v>
+        <v>74092.80</v>
       </c>
       <c r="H1794" s="1">
         <v>0</v>
       </c>
       <c r="I1794" s="1">
-        <v>163430</v>
+        <v>74092.80</v>
       </c>
     </row>
     <row r="1795" spans="1:9" ht="12.75">
@@ -53604,22 +53604,22 @@
         <v>105</v>
       </c>
       <c r="D1795" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E1795" t="s">
-        <v>329</v>
+        <v>357</v>
       </c>
       <c r="F1795" s="1">
         <v>0</v>
       </c>
       <c r="G1795" s="1">
-        <v>137490</v>
+        <v>163430</v>
       </c>
       <c r="H1795" s="1">
         <v>0</v>
       </c>
       <c r="I1795" s="1">
-        <v>137490</v>
+        <v>163430</v>
       </c>
     </row>
     <row r="1796" spans="1:9" ht="12.75">
@@ -53636,19 +53636,19 @@
         <v>258</v>
       </c>
       <c r="E1796" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F1796" s="1">
         <v>0</v>
       </c>
       <c r="G1796" s="1">
-        <v>305648</v>
+        <v>137490</v>
       </c>
       <c r="H1796" s="1">
         <v>0</v>
       </c>
       <c r="I1796" s="1">
-        <v>305648</v>
+        <v>137490</v>
       </c>
     </row>
     <row r="1797" spans="1:9" ht="12.75">
@@ -53665,19 +53665,19 @@
         <v>258</v>
       </c>
       <c r="E1797" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F1797" s="1">
         <v>0</v>
       </c>
       <c r="G1797" s="1">
-        <v>484</v>
+        <v>305648</v>
       </c>
       <c r="H1797" s="1">
         <v>0</v>
       </c>
       <c r="I1797" s="1">
-        <v>484</v>
+        <v>305648</v>
       </c>
     </row>
     <row r="1798" spans="1:9" ht="12.75">
@@ -53691,22 +53691,22 @@
         <v>105</v>
       </c>
       <c r="D1798" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E1798" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="F1798" s="1">
         <v>0</v>
       </c>
       <c r="G1798" s="1">
-        <v>24000</v>
+        <v>484</v>
       </c>
       <c r="H1798" s="1">
         <v>0</v>
       </c>
       <c r="I1798" s="1">
-        <v>24000</v>
+        <v>484</v>
       </c>
     </row>
     <row r="1799" spans="1:9" ht="12.75">
@@ -53720,22 +53720,22 @@
         <v>105</v>
       </c>
       <c r="D1799" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E1799" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F1799" s="1">
         <v>0</v>
       </c>
       <c r="G1799" s="1">
-        <v>2814300</v>
+        <v>24000</v>
       </c>
       <c r="H1799" s="1">
         <v>0</v>
       </c>
       <c r="I1799" s="1">
-        <v>2814300</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="1800" spans="1:9" ht="12.75">
@@ -53743,28 +53743,28 @@
         <v>313</v>
       </c>
       <c r="B1800" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="C1800" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="D1800" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="E1800" t="s">
-        <v>13</v>
+        <v>338</v>
       </c>
       <c r="F1800" s="1">
         <v>0</v>
       </c>
       <c r="G1800" s="1">
-        <v>0</v>
+        <v>2814300</v>
       </c>
       <c r="H1800" s="1">
-        <v>7351276</v>
+        <v>0</v>
       </c>
       <c r="I1800" s="1">
-        <v>-7351276</v>
+        <v>2814300</v>
       </c>
     </row>
     <row r="1801" spans="1:9" ht="12.75">
@@ -53778,7 +53778,7 @@
         <v>264</v>
       </c>
       <c r="D1801" t="s">
-        <v>309</v>
+        <v>267</v>
       </c>
       <c r="E1801" t="s">
         <v>13</v>
@@ -53790,10 +53790,10 @@
         <v>0</v>
       </c>
       <c r="H1801" s="1">
-        <v>0</v>
+        <v>7351276</v>
       </c>
       <c r="I1801" s="1">
-        <v>0</v>
+        <v>-7351276</v>
       </c>
     </row>
     <row r="1802" spans="1:9" ht="12.75">
@@ -53801,28 +53801,28 @@
         <v>313</v>
       </c>
       <c r="B1802" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C1802" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D1802" t="s">
-        <v>269</v>
+        <v>309</v>
       </c>
       <c r="E1802" t="s">
         <v>13</v>
       </c>
       <c r="F1802" s="1">
-        <v>-5418882</v>
+        <v>0</v>
       </c>
       <c r="G1802" s="1">
-        <v>3.071942442699999E8</v>
+        <v>0</v>
       </c>
       <c r="H1802" s="1">
-        <v>3.236654322299999E8</v>
+        <v>0</v>
       </c>
       <c r="I1802" s="1">
-        <v>-2.189006995999998E7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1803" spans="1:9" ht="12.75">
@@ -53833,25 +53833,25 @@
         <v>268</v>
       </c>
       <c r="C1803" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D1803" t="s">
-        <v>358</v>
+        <v>269</v>
       </c>
       <c r="E1803" t="s">
         <v>13</v>
       </c>
       <c r="F1803" s="1">
-        <v>0</v>
+        <v>-5418882</v>
       </c>
       <c r="G1803" s="1">
-        <v>5013786</v>
+        <v>3.195558422299999E8</v>
       </c>
       <c r="H1803" s="1">
-        <v>5013786</v>
+        <v>3.2376489022999996E8</v>
       </c>
       <c r="I1803" s="1">
-        <v>0</v>
+        <v>-9627930.00000006</v>
       </c>
     </row>
     <row r="1804" spans="1:9" ht="12.75">
@@ -53865,22 +53865,22 @@
         <v>273</v>
       </c>
       <c r="D1804" t="s">
-        <v>278</v>
+        <v>358</v>
       </c>
       <c r="E1804" t="s">
         <v>13</v>
       </c>
       <c r="F1804" s="1">
-        <v>-22030149</v>
+        <v>0</v>
       </c>
       <c r="G1804" s="1">
-        <v>7656302</v>
+        <v>5013786</v>
       </c>
       <c r="H1804" s="1">
-        <v>9.136277758399999E8</v>
+        <v>5013786</v>
       </c>
       <c r="I1804" s="1">
-        <v>-9.280016228399999E8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1805" spans="1:9" ht="12.75">
@@ -53894,22 +53894,22 @@
         <v>273</v>
       </c>
       <c r="D1805" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="E1805" t="s">
         <v>13</v>
       </c>
       <c r="F1805" s="1">
-        <v>-14989</v>
+        <v>-22030149</v>
       </c>
       <c r="G1805" s="1">
-        <v>5515449</v>
+        <v>7656302</v>
       </c>
       <c r="H1805" s="1">
-        <v>10165830</v>
+        <v>9.136277758399999E8</v>
       </c>
       <c r="I1805" s="1">
-        <v>-4665370</v>
+        <v>-9.280016228399999E8</v>
       </c>
     </row>
     <row r="1806" spans="1:9" ht="12.75">
@@ -53923,22 +53923,22 @@
         <v>273</v>
       </c>
       <c r="D1806" t="s">
-        <v>359</v>
+        <v>282</v>
       </c>
       <c r="E1806" t="s">
         <v>13</v>
       </c>
       <c r="F1806" s="1">
-        <v>0</v>
+        <v>-14989</v>
       </c>
       <c r="G1806" s="1">
-        <v>2659661</v>
+        <v>5515449</v>
       </c>
       <c r="H1806" s="1">
-        <v>2659660</v>
+        <v>10165830</v>
       </c>
       <c r="I1806" s="1">
-        <v>1</v>
+        <v>-4665370</v>
       </c>
     </row>
     <row r="1807" spans="1:9" ht="12.75">
@@ -53952,7 +53952,7 @@
         <v>273</v>
       </c>
       <c r="D1807" t="s">
-        <v>286</v>
+        <v>359</v>
       </c>
       <c r="E1807" t="s">
         <v>13</v>
@@ -53961,13 +53961,13 @@
         <v>0</v>
       </c>
       <c r="G1807" s="1">
-        <v>0</v>
+        <v>2659661</v>
       </c>
       <c r="H1807" s="1">
-        <v>190424</v>
+        <v>2659660</v>
       </c>
       <c r="I1807" s="1">
-        <v>-190424</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1808" spans="1:9" ht="12.75">
@@ -53981,7 +53981,7 @@
         <v>273</v>
       </c>
       <c r="D1808" t="s">
-        <v>360</v>
+        <v>286</v>
       </c>
       <c r="E1808" t="s">
         <v>13</v>
@@ -53990,13 +53990,13 @@
         <v>0</v>
       </c>
       <c r="G1808" s="1">
-        <v>2230780</v>
+        <v>0</v>
       </c>
       <c r="H1808" s="1">
-        <v>2294489</v>
+        <v>190424</v>
       </c>
       <c r="I1808" s="1">
-        <v>-63709</v>
+        <v>-190424</v>
       </c>
     </row>
     <row r="1809" spans="1:9" ht="12.75">
@@ -54010,7 +54010,7 @@
         <v>273</v>
       </c>
       <c r="D1809" t="s">
-        <v>287</v>
+        <v>360</v>
       </c>
       <c r="E1809" t="s">
         <v>13</v>
@@ -54019,13 +54019,13 @@
         <v>0</v>
       </c>
       <c r="G1809" s="1">
-        <v>48730</v>
+        <v>2230780</v>
       </c>
       <c r="H1809" s="1">
-        <v>70730</v>
+        <v>2294489</v>
       </c>
       <c r="I1809" s="1">
-        <v>-22000</v>
+        <v>-63709</v>
       </c>
     </row>
     <row r="1810" spans="1:9" ht="12.75">
@@ -54039,7 +54039,7 @@
         <v>273</v>
       </c>
       <c r="D1810" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E1810" t="s">
         <v>13</v>
@@ -54048,13 +54048,13 @@
         <v>0</v>
       </c>
       <c r="G1810" s="1">
-        <v>840</v>
+        <v>48730</v>
       </c>
       <c r="H1810" s="1">
-        <v>416</v>
+        <v>70730</v>
       </c>
       <c r="I1810" s="1">
-        <v>424</v>
+        <v>-22000</v>
       </c>
     </row>
     <row r="1811" spans="1:9" ht="12.75">
@@ -54068,7 +54068,7 @@
         <v>273</v>
       </c>
       <c r="D1811" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E1811" t="s">
         <v>13</v>
@@ -54077,13 +54077,13 @@
         <v>0</v>
       </c>
       <c r="G1811" s="1">
-        <v>4.89969833E7</v>
+        <v>840</v>
       </c>
       <c r="H1811" s="1">
-        <v>58379674</v>
+        <v>416</v>
       </c>
       <c r="I1811" s="1">
-        <v>-9382690.700000003</v>
+        <v>424</v>
       </c>
     </row>
     <row r="1812" spans="1:9" ht="12.75">
@@ -54097,7 +54097,7 @@
         <v>273</v>
       </c>
       <c r="D1812" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E1812" t="s">
         <v>13</v>
@@ -54106,13 +54106,13 @@
         <v>0</v>
       </c>
       <c r="G1812" s="1">
-        <v>55944</v>
+        <v>4.89969833E7</v>
       </c>
       <c r="H1812" s="1">
-        <v>232407.78999999998</v>
+        <v>58379674</v>
       </c>
       <c r="I1812" s="1">
-        <v>-176463.78999999998</v>
+        <v>-9382690.700000003</v>
       </c>
     </row>
     <row r="1813" spans="1:9" ht="12.75">
@@ -54126,7 +54126,7 @@
         <v>273</v>
       </c>
       <c r="D1813" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E1813" t="s">
         <v>13</v>
@@ -54135,13 +54135,13 @@
         <v>0</v>
       </c>
       <c r="G1813" s="1">
-        <v>105045</v>
+        <v>55944</v>
       </c>
       <c r="H1813" s="1">
-        <v>498838.90</v>
+        <v>232407.78999999998</v>
       </c>
       <c r="I1813" s="1">
-        <v>-393793.90</v>
+        <v>-176463.78999999998</v>
       </c>
     </row>
     <row r="1814" spans="1:9" ht="12.75">
@@ -54155,7 +54155,7 @@
         <v>273</v>
       </c>
       <c r="D1814" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E1814" t="s">
         <v>13</v>
@@ -54164,13 +54164,13 @@
         <v>0</v>
       </c>
       <c r="G1814" s="1">
-        <v>4687449</v>
+        <v>105045</v>
       </c>
       <c r="H1814" s="1">
-        <v>1.623181255E7</v>
+        <v>504838.90</v>
       </c>
       <c r="I1814" s="1">
-        <v>-1.154436355E7</v>
+        <v>-399793.90</v>
       </c>
     </row>
     <row r="1815" spans="1:9" ht="12.75">
@@ -54184,7 +54184,7 @@
         <v>273</v>
       </c>
       <c r="D1815" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E1815" t="s">
         <v>13</v>
@@ -54193,13 +54193,13 @@
         <v>0</v>
       </c>
       <c r="G1815" s="1">
-        <v>1758542.24</v>
+        <v>4687449</v>
       </c>
       <c r="H1815" s="1">
-        <v>1164129.74</v>
+        <v>1.623181255E7</v>
       </c>
       <c r="I1815" s="1">
-        <v>594412.50</v>
+        <v>-1.154436355E7</v>
       </c>
     </row>
     <row r="1816" spans="1:9" ht="12.75">
@@ -54213,7 +54213,7 @@
         <v>273</v>
       </c>
       <c r="D1816" t="s">
-        <v>361</v>
+        <v>294</v>
       </c>
       <c r="E1816" t="s">
         <v>13</v>
@@ -54222,13 +54222,13 @@
         <v>0</v>
       </c>
       <c r="G1816" s="1">
-        <v>9251007</v>
+        <v>1758542.24</v>
       </c>
       <c r="H1816" s="1">
-        <v>18931841</v>
+        <v>1164129.74</v>
       </c>
       <c r="I1816" s="1">
-        <v>-9680834</v>
+        <v>594412.50</v>
       </c>
     </row>
     <row r="1817" spans="1:9" ht="12.75">
@@ -54239,10 +54239,10 @@
         <v>268</v>
       </c>
       <c r="C1817" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="D1817" t="s">
-        <v>297</v>
+        <v>361</v>
       </c>
       <c r="E1817" t="s">
         <v>13</v>
@@ -54251,13 +54251,13 @@
         <v>0</v>
       </c>
       <c r="G1817" s="1">
-        <v>2.8078775699E8</v>
+        <v>9251007</v>
       </c>
       <c r="H1817" s="1">
-        <v>2.8078775699E8</v>
+        <v>18931841</v>
       </c>
       <c r="I1817" s="1">
-        <v>0</v>
+        <v>-9680834</v>
       </c>
     </row>
     <row r="1818" spans="1:9" ht="12.75">
@@ -54271,7 +54271,7 @@
         <v>296</v>
       </c>
       <c r="D1818" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E1818" t="s">
         <v>13</v>
@@ -54280,41 +54280,70 @@
         <v>0</v>
       </c>
       <c r="G1818" s="1">
-        <v>0</v>
+        <v>3.0705979832000005E8</v>
       </c>
       <c r="H1818" s="1">
-        <v>8826219.66</v>
+        <v>3.0705979832000005E8</v>
       </c>
       <c r="I1818" s="1">
-        <v>-8826219.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1819" spans="1:9" ht="12.75">
       <c r="A1819" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1819" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1819" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1819" t="s">
+        <v>298</v>
+      </c>
+      <c r="E1819" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1819" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1819" s="1">
+        <v>0</v>
+      </c>
+      <c r="H1819" s="1">
+        <v>1.118956866E7</v>
+      </c>
+      <c r="I1819" s="1">
+        <v>-1.118956866E7</v>
+      </c>
+    </row>
+    <row r="1820" spans="1:9" ht="12.75">
+      <c r="A1820" t="s">
         <v>362</v>
       </c>
-      <c r="B1819" t="s">
+      <c r="B1820" t="s">
         <v>363</v>
       </c>
-      <c r="C1819" t="s">
+      <c r="C1820" t="s">
         <v>363</v>
       </c>
-      <c r="D1819" t="s">
+      <c r="D1820" t="s">
         <v>363</v>
       </c>
-      <c r="E1819" t="s">
+      <c r="E1820" t="s">
         <v>363</v>
       </c>
-      <c r="F1819" s="1">
-        <v>0</v>
-      </c>
-      <c r="G1819" s="1">
-        <v>7.426324492279996E9</v>
-      </c>
-      <c r="H1819" s="1">
-        <v>7.426324492280001E9</v>
-      </c>
-      <c r="I1819" s="1">
+      <c r="F1820" s="1">
+        <v>1.1920928955078125E-7</v>
+      </c>
+      <c r="G1820" s="1">
+        <v>7.566809778419996E9</v>
+      </c>
+      <c r="H1820" s="1">
+        <v>7.566809778419999E9</v>
+      </c>
+      <c r="I1820" s="1">
         <v>-1.7657876014709473E-6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Consol TB report update 2026-03-28
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -1553,7 +1553,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34b63e51-f875-4947-8146-bb01bafa9d99}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ef35d8f-ae2c-4227-bc0f-1f2096d804a7}">
   <dimension ref="A1:I1823"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -1642,7 +1642,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>-2.9802322387695312E-8</v>
+        <v>-8.940696716308594E-8</v>
       </c>
       <c r="G3" s="1">
         <v>3.54</v>
@@ -1651,7 +1651,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>-2.9802321943606103E-8</v>
+        <v>-8.940696671899673E-8</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -1677,10 +1677,10 @@
         <v>3.9887229998E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.4664425354000056E8</v>
+        <v>3.4664425354000014E8</v>
       </c>
       <c r="I4" s="1">
-        <v>1.8413079830999947E8</v>
+        <v>1.8413079830999988E8</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -1793,10 +1793,10 @@
         <v>5.83186561E8</v>
       </c>
       <c r="H8" s="1">
-        <v>2.7487199097999996E8</v>
+        <v>2.748719909799999E8</v>
       </c>
       <c r="I8" s="1">
-        <v>3.0831457002000004E8</v>
+        <v>3.083145700200001E8</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="12.75">
@@ -3820,13 +3820,13 @@
         <v>918706</v>
       </c>
       <c r="G78" s="1">
-        <v>4.805299583E7</v>
+        <v>4.805299583000001E7</v>
       </c>
       <c r="H78" s="1">
-        <v>4.781173219999998E7</v>
+        <v>4.781173220000003E7</v>
       </c>
       <c r="I78" s="1">
-        <v>1159969.6300000176</v>
+        <v>1159969.6299999803</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="12.75">
@@ -18436,13 +18436,13 @@
         <v>0</v>
       </c>
       <c r="G582" s="1">
-        <v>959829.5700000001</v>
+        <v>959829.57</v>
       </c>
       <c r="H582" s="1">
         <v>0</v>
       </c>
       <c r="I582" s="1">
-        <v>959829.5700000001</v>
+        <v>959829.57</v>
       </c>
     </row>
     <row r="583" spans="1:9" ht="12.75">
@@ -18465,13 +18465,13 @@
         <v>0</v>
       </c>
       <c r="G583" s="1">
-        <v>1134248.01</v>
+        <v>1134248.0099999998</v>
       </c>
       <c r="H583" s="1">
         <v>0</v>
       </c>
       <c r="I583" s="1">
-        <v>1134248.01</v>
+        <v>1134248.0099999998</v>
       </c>
     </row>
     <row r="584" spans="1:9" ht="12.75">
@@ -18697,13 +18697,13 @@
         <v>0</v>
       </c>
       <c r="G591" s="1">
-        <v>154978.47000000003</v>
+        <v>154978.47</v>
       </c>
       <c r="H591" s="1">
         <v>0</v>
       </c>
       <c r="I591" s="1">
-        <v>154978.47000000003</v>
+        <v>154978.47</v>
       </c>
     </row>
     <row r="592" spans="1:9" ht="12.75">
@@ -19625,13 +19625,13 @@
         <v>0</v>
       </c>
       <c r="G623" s="1">
-        <v>584250.46</v>
+        <v>584250.4599999998</v>
       </c>
       <c r="H623" s="1">
         <v>0</v>
       </c>
       <c r="I623" s="1">
-        <v>584250.46</v>
+        <v>584250.4599999998</v>
       </c>
     </row>
     <row r="624" spans="1:9" ht="12.75">
@@ -19683,13 +19683,13 @@
         <v>0</v>
       </c>
       <c r="G625" s="1">
-        <v>1404331.3199999998</v>
+        <v>1404331.32</v>
       </c>
       <c r="H625" s="1">
         <v>0</v>
       </c>
       <c r="I625" s="1">
-        <v>1404331.3199999998</v>
+        <v>1404331.32</v>
       </c>
     </row>
     <row r="626" spans="1:9" ht="12.75">
@@ -20031,13 +20031,13 @@
         <v>0</v>
       </c>
       <c r="G637" s="1">
-        <v>555001.24</v>
+        <v>555001.2400000001</v>
       </c>
       <c r="H637" s="1">
         <v>0</v>
       </c>
       <c r="I637" s="1">
-        <v>555001.24</v>
+        <v>555001.2400000001</v>
       </c>
     </row>
     <row r="638" spans="1:9" ht="12.75">
@@ -20205,13 +20205,13 @@
         <v>0</v>
       </c>
       <c r="G643" s="1">
-        <v>1757794.71</v>
+        <v>1757794.7100000002</v>
       </c>
       <c r="H643" s="1">
         <v>9049.23</v>
       </c>
       <c r="I643" s="1">
-        <v>1748745.48</v>
+        <v>1748745.4800000002</v>
       </c>
     </row>
     <row r="644" spans="1:9" ht="12.75">
@@ -20234,13 +20234,13 @@
         <v>0</v>
       </c>
       <c r="G644" s="1">
-        <v>744682.7999999999</v>
+        <v>744682.80</v>
       </c>
       <c r="H644" s="1">
         <v>0</v>
       </c>
       <c r="I644" s="1">
-        <v>744682.7999999999</v>
+        <v>744682.80</v>
       </c>
     </row>
     <row r="645" spans="1:9" ht="12.75">
@@ -20263,13 +20263,13 @@
         <v>0</v>
       </c>
       <c r="G645" s="1">
-        <v>544076</v>
+        <v>544075.9999999998</v>
       </c>
       <c r="H645" s="1">
         <v>0</v>
       </c>
       <c r="I645" s="1">
-        <v>544076</v>
+        <v>544075.9999999998</v>
       </c>
     </row>
     <row r="646" spans="1:9" ht="12.75">
@@ -20524,13 +20524,13 @@
         <v>0</v>
       </c>
       <c r="G654" s="1">
-        <v>341636.41000000003</v>
+        <v>341636.4099999999</v>
       </c>
       <c r="H654" s="1">
         <v>0</v>
       </c>
       <c r="I654" s="1">
-        <v>341636.41000000003</v>
+        <v>341636.4099999999</v>
       </c>
     </row>
     <row r="655" spans="1:9" ht="12.75">
@@ -20669,13 +20669,13 @@
         <v>0</v>
       </c>
       <c r="G659" s="1">
-        <v>2292091.56</v>
+        <v>2292091.5599999996</v>
       </c>
       <c r="H659" s="1">
         <v>0</v>
       </c>
       <c r="I659" s="1">
-        <v>2292091.56</v>
+        <v>2292091.5599999996</v>
       </c>
     </row>
     <row r="660" spans="1:9" ht="12.75">
@@ -20814,13 +20814,13 @@
         <v>0</v>
       </c>
       <c r="G664" s="1">
-        <v>171980.20</v>
+        <v>171980.19999999998</v>
       </c>
       <c r="H664" s="1">
         <v>0</v>
       </c>
       <c r="I664" s="1">
-        <v>171980.20</v>
+        <v>171980.19999999998</v>
       </c>
     </row>
     <row r="665" spans="1:9" ht="12.75">
@@ -20988,13 +20988,13 @@
         <v>0</v>
       </c>
       <c r="G670" s="1">
-        <v>780446.09</v>
+        <v>780446.0900000001</v>
       </c>
       <c r="H670" s="1">
         <v>0</v>
       </c>
       <c r="I670" s="1">
-        <v>780446.09</v>
+        <v>780446.0900000001</v>
       </c>
     </row>
     <row r="671" spans="1:9" ht="12.75">
@@ -21046,13 +21046,13 @@
         <v>0</v>
       </c>
       <c r="G672" s="1">
-        <v>617404.20</v>
+        <v>617404.2000000001</v>
       </c>
       <c r="H672" s="1">
         <v>0</v>
       </c>
       <c r="I672" s="1">
-        <v>617404.20</v>
+        <v>617404.2000000001</v>
       </c>
     </row>
     <row r="673" spans="1:9" ht="12.75">
@@ -21945,13 +21945,13 @@
         <v>0</v>
       </c>
       <c r="G703" s="1">
-        <v>2568009.10</v>
+        <v>2568009.0999999996</v>
       </c>
       <c r="H703" s="1">
         <v>0</v>
       </c>
       <c r="I703" s="1">
-        <v>2568009.10</v>
+        <v>2568009.0999999996</v>
       </c>
     </row>
     <row r="704" spans="1:9" ht="12.75">
@@ -22032,13 +22032,13 @@
         <v>0</v>
       </c>
       <c r="G706" s="1">
-        <v>906485.99</v>
+        <v>906485.9900000001</v>
       </c>
       <c r="H706" s="1">
         <v>0</v>
       </c>
       <c r="I706" s="1">
-        <v>906485.99</v>
+        <v>906485.9900000001</v>
       </c>
     </row>
     <row r="707" spans="1:9" ht="12.75">
@@ -22090,13 +22090,13 @@
         <v>0</v>
       </c>
       <c r="G708" s="1">
-        <v>4420392.42</v>
+        <v>4420392.420000001</v>
       </c>
       <c r="H708" s="1">
         <v>0</v>
       </c>
       <c r="I708" s="1">
-        <v>4420392.42</v>
+        <v>4420392.420000001</v>
       </c>
     </row>
     <row r="709" spans="1:9" ht="12.75">
@@ -22119,13 +22119,13 @@
         <v>0</v>
       </c>
       <c r="G709" s="1">
-        <v>5448697.789999999</v>
+        <v>5448697.79</v>
       </c>
       <c r="H709" s="1">
         <v>0</v>
       </c>
       <c r="I709" s="1">
-        <v>5448697.789999999</v>
+        <v>5448697.79</v>
       </c>
     </row>
     <row r="710" spans="1:9" ht="12.75">
@@ -22206,13 +22206,13 @@
         <v>0</v>
       </c>
       <c r="G712" s="1">
-        <v>699050.7999999999</v>
+        <v>699050.80</v>
       </c>
       <c r="H712" s="1">
         <v>0</v>
       </c>
       <c r="I712" s="1">
-        <v>699050.7999999999</v>
+        <v>699050.80</v>
       </c>
     </row>
     <row r="713" spans="1:9" ht="12.75">
@@ -22496,13 +22496,13 @@
         <v>0</v>
       </c>
       <c r="G722" s="1">
-        <v>253568.63999999998</v>
+        <v>253568.64</v>
       </c>
       <c r="H722" s="1">
         <v>0</v>
       </c>
       <c r="I722" s="1">
-        <v>253568.63999999998</v>
+        <v>253568.64</v>
       </c>
     </row>
     <row r="723" spans="1:9" ht="12.75">
@@ -22583,13 +22583,13 @@
         <v>0</v>
       </c>
       <c r="G725" s="1">
-        <v>742650.7000000001</v>
+        <v>742650.70</v>
       </c>
       <c r="H725" s="1">
         <v>0</v>
       </c>
       <c r="I725" s="1">
-        <v>742650.7000000001</v>
+        <v>742650.70</v>
       </c>
     </row>
     <row r="726" spans="1:9" ht="12.75">
@@ -22612,13 +22612,13 @@
         <v>0</v>
       </c>
       <c r="G726" s="1">
-        <v>180148.39</v>
+        <v>180148.38999999998</v>
       </c>
       <c r="H726" s="1">
         <v>0</v>
       </c>
       <c r="I726" s="1">
-        <v>180148.39</v>
+        <v>180148.38999999998</v>
       </c>
     </row>
     <row r="727" spans="1:9" ht="12.75">
@@ -22963,10 +22963,10 @@
         <v>0</v>
       </c>
       <c r="H738" s="1">
-        <v>7.258656368E7</v>
+        <v>7.258656367999999E7</v>
       </c>
       <c r="I738" s="1">
-        <v>-7.258656368E7</v>
+        <v>-7.258656367999999E7</v>
       </c>
     </row>
     <row r="739" spans="1:9" ht="12.75">
@@ -40302,13 +40302,13 @@
         <v>0</v>
       </c>
       <c r="G1336" s="1">
-        <v>3.341335865E7</v>
+        <v>3.3413358649999995E7</v>
       </c>
       <c r="H1336" s="1">
         <v>179327</v>
       </c>
       <c r="I1336" s="1">
-        <v>3.323403165E7</v>
+        <v>3.3234031649999995E7</v>
       </c>
     </row>
     <row r="1337" spans="1:9" ht="12.75">
@@ -41317,13 +41317,13 @@
         <v>0</v>
       </c>
       <c r="G1371" s="1">
-        <v>3.210335585E7</v>
+        <v>3.2103355849999998E7</v>
       </c>
       <c r="H1371" s="1">
         <v>283032</v>
       </c>
       <c r="I1371" s="1">
-        <v>3.182032385E7</v>
+        <v>3.1820323849999998E7</v>
       </c>
     </row>
     <row r="1372" spans="1:9" ht="12.75">
@@ -41607,13 +41607,13 @@
         <v>0</v>
       </c>
       <c r="G1381" s="1">
-        <v>6689781.300000001</v>
+        <v>6689781.3</v>
       </c>
       <c r="H1381" s="1">
         <v>34552</v>
       </c>
       <c r="I1381" s="1">
-        <v>6655229.300000001</v>
+        <v>6655229.3</v>
       </c>
     </row>
     <row r="1382" spans="1:9" ht="12.75">
@@ -41697,10 +41697,10 @@
         <v>3.6842895962E8</v>
       </c>
       <c r="H1384" s="1">
-        <v>3.6262405171000004E8</v>
+        <v>3.6262405171E8</v>
       </c>
       <c r="I1384" s="1">
-        <v>5804907.909999967</v>
+        <v>5804907.910000026</v>
       </c>
     </row>
     <row r="1385" spans="1:9" ht="12.75">
@@ -41868,13 +41868,13 @@
         <v>0</v>
       </c>
       <c r="G1390" s="1">
-        <v>1.884446755E7</v>
+        <v>1.8844467549999997E7</v>
       </c>
       <c r="H1390" s="1">
         <v>110222</v>
       </c>
       <c r="I1390" s="1">
-        <v>1.873424555E7</v>
+        <v>1.8734245549999997E7</v>
       </c>
     </row>
     <row r="1391" spans="1:9" ht="12.75">
@@ -41897,13 +41897,13 @@
         <v>0</v>
       </c>
       <c r="G1391" s="1">
-        <v>8018272.119999999</v>
+        <v>8018272.12</v>
       </c>
       <c r="H1391" s="1">
         <v>0</v>
       </c>
       <c r="I1391" s="1">
-        <v>8018272.119999999</v>
+        <v>8018272.12</v>
       </c>
     </row>
     <row r="1392" spans="1:9" ht="12.75">
@@ -41984,13 +41984,13 @@
         <v>0</v>
       </c>
       <c r="G1394" s="1">
-        <v>4507476.45</v>
+        <v>4507476.449999999</v>
       </c>
       <c r="H1394" s="1">
         <v>0</v>
       </c>
       <c r="I1394" s="1">
-        <v>4507476.45</v>
+        <v>4507476.449999999</v>
       </c>
     </row>
     <row r="1395" spans="1:9" ht="12.75">
@@ -43782,13 +43782,13 @@
         <v>0</v>
       </c>
       <c r="G1456" s="1">
-        <v>1894601.32</v>
+        <v>1894601.3199999998</v>
       </c>
       <c r="H1456" s="1">
         <v>0</v>
       </c>
       <c r="I1456" s="1">
-        <v>1894601.32</v>
+        <v>1894601.3199999998</v>
       </c>
     </row>
     <row r="1457" spans="1:9" ht="12.75">
@@ -44968,16 +44968,16 @@
         <v>13</v>
       </c>
       <c r="F1497" s="1">
-        <v>-1.934719699999994E7</v>
+        <v>-1.934719700000018E7</v>
       </c>
       <c r="G1497" s="1">
-        <v>2.1835296529999974E8</v>
+        <v>2.183529653000001E8</v>
       </c>
       <c r="H1497" s="1">
-        <v>2.0468359629999986E8</v>
+        <v>2.046835963000001E8</v>
       </c>
       <c r="I1497" s="1">
-        <v>-5677828.00000006</v>
+        <v>-5677828.000000179</v>
       </c>
     </row>
     <row r="1498" spans="1:9" ht="12.75">
@@ -45061,10 +45061,10 @@
         <v>2.288005138E7</v>
       </c>
       <c r="H1500" s="1">
-        <v>1.752459138E7</v>
+        <v>1.7524591380000003E7</v>
       </c>
       <c r="I1500" s="1">
-        <v>0</v>
+        <v>-3.725290298461914E-9</v>
       </c>
     </row>
     <row r="1501" spans="1:9" ht="12.75">
@@ -45551,13 +45551,13 @@
         <v>0</v>
       </c>
       <c r="G1517" s="1">
-        <v>557550.9300000002</v>
+        <v>557550.9299999999</v>
       </c>
       <c r="H1517" s="1">
-        <v>605654.3600000001</v>
+        <v>605654.3599999998</v>
       </c>
       <c r="I1517" s="1">
-        <v>-48103.429999999935</v>
+        <v>-48103.42999999982</v>
       </c>
     </row>
     <row r="1518" spans="1:9" ht="12.75">
@@ -45609,13 +45609,13 @@
         <v>0</v>
       </c>
       <c r="G1519" s="1">
-        <v>7533462.200000001</v>
+        <v>7533462.2</v>
       </c>
       <c r="H1519" s="1">
         <v>8946451.92</v>
       </c>
       <c r="I1519" s="1">
-        <v>-1412989.7199999988</v>
+        <v>-1412989.7199999997</v>
       </c>
     </row>
     <row r="1520" spans="1:9" ht="12.75">
@@ -45635,16 +45635,16 @@
         <v>13</v>
       </c>
       <c r="F1520" s="1">
-        <v>-56797.00000000186</v>
+        <v>-56797.00000000559</v>
       </c>
       <c r="G1520" s="1">
-        <v>3227421.94</v>
+        <v>3227421.9400000004</v>
       </c>
       <c r="H1520" s="1">
-        <v>3631156.939999996</v>
+        <v>3631156.9399999976</v>
       </c>
       <c r="I1520" s="1">
-        <v>-460531.99999999814</v>
+        <v>-460532.0000000028</v>
       </c>
     </row>
     <row r="1521" spans="1:9" ht="12.75">
@@ -45693,16 +45693,16 @@
         <v>13</v>
       </c>
       <c r="F1522" s="1">
-        <v>-5.9604644775390625E-8</v>
+        <v>0</v>
       </c>
       <c r="G1522" s="1">
-        <v>1.1669682698900006E9</v>
+        <v>1.16696826989E9</v>
       </c>
       <c r="H1522" s="1">
-        <v>1.1669682698900025E9</v>
+        <v>1.1669682698900018E9</v>
       </c>
       <c r="I1522" s="1">
-        <v>-1.9073486328125E-6</v>
+        <v>-1.6689300537109375E-6</v>
       </c>
     </row>
     <row r="1523" spans="1:9" ht="12.75">
@@ -45728,10 +45728,10 @@
         <v>12492016</v>
       </c>
       <c r="H1523" s="1">
-        <v>3.3977782150000006E7</v>
+        <v>3.397778215E7</v>
       </c>
       <c r="I1523" s="1">
-        <v>-2.3191182150000006E7</v>
+        <v>-2.319118215E7</v>
       </c>
     </row>
     <row r="1524" spans="1:9" ht="12.75">
@@ -46627,10 +46627,10 @@
         <v>6.935924804E7</v>
       </c>
       <c r="H1554" s="1">
-        <v>8.109376578E7</v>
+        <v>8.324784969999999E7</v>
       </c>
       <c r="I1554" s="1">
-        <v>1.7459191159999996E7</v>
+        <v>1.530510724000001E7</v>
       </c>
     </row>
     <row r="1555" spans="1:9" ht="12.75">
@@ -46714,10 +46714,10 @@
         <v>8.56587629E8</v>
       </c>
       <c r="H1557" s="1">
-        <v>4.129673205999999E8</v>
+        <v>4.3765868599E8</v>
       </c>
       <c r="I1557" s="1">
-        <v>4.436203084000001E8</v>
+        <v>4.1892894301E8</v>
       </c>
     </row>
     <row r="1558" spans="1:9" ht="12.75">
@@ -48683,13 +48683,13 @@
         <v>0</v>
       </c>
       <c r="G1625" s="1">
-        <v>307964.57</v>
+        <v>307964.56999999995</v>
       </c>
       <c r="H1625" s="1">
         <v>0</v>
       </c>
       <c r="I1625" s="1">
-        <v>307964.57</v>
+        <v>307964.56999999995</v>
       </c>
     </row>
     <row r="1626" spans="1:9" ht="12.75">
@@ -50771,13 +50771,13 @@
         <v>0</v>
       </c>
       <c r="G1697" s="1">
+        <v>685737.61</v>
+      </c>
+      <c r="H1697" s="1">
         <v>685737.6100000001</v>
       </c>
-      <c r="H1697" s="1">
-        <v>685737.61</v>
-      </c>
       <c r="I1697" s="1">
-        <v>1.1641532182693481E-10</v>
+        <v>-1.1641532182693481E-10</v>
       </c>
     </row>
     <row r="1698" spans="1:9" ht="12.75">
@@ -50829,13 +50829,13 @@
         <v>0</v>
       </c>
       <c r="G1699" s="1">
-        <v>191355.02000000002</v>
+        <v>191355.02</v>
       </c>
       <c r="H1699" s="1">
         <v>93523</v>
       </c>
       <c r="I1699" s="1">
-        <v>97832.02000000002</v>
+        <v>97832.01999999999</v>
       </c>
     </row>
     <row r="1700" spans="1:9" ht="12.75">
@@ -50974,13 +50974,13 @@
         <v>0</v>
       </c>
       <c r="G1704" s="1">
-        <v>2646972.23</v>
+        <v>2646972.2299999995</v>
       </c>
       <c r="H1704" s="1">
         <v>0</v>
       </c>
       <c r="I1704" s="1">
-        <v>2646972.23</v>
+        <v>2646972.2299999995</v>
       </c>
     </row>
     <row r="1705" spans="1:9" ht="12.75">
@@ -53439,13 +53439,13 @@
         <v>0</v>
       </c>
       <c r="G1789" s="1">
-        <v>2790926.10</v>
+        <v>2790926.0999999996</v>
       </c>
       <c r="H1789" s="1">
         <v>0</v>
       </c>
       <c r="I1789" s="1">
-        <v>2790926.10</v>
+        <v>2790926.0999999996</v>
       </c>
     </row>
     <row r="1790" spans="1:9" ht="12.75">
@@ -53468,13 +53468,13 @@
         <v>0</v>
       </c>
       <c r="G1790" s="1">
-        <v>1.07634571E7</v>
+        <v>1.0763457100000001E7</v>
       </c>
       <c r="H1790" s="1">
         <v>0</v>
       </c>
       <c r="I1790" s="1">
-        <v>1.07634571E7</v>
+        <v>1.0763457100000001E7</v>
       </c>
     </row>
     <row r="1791" spans="1:9" ht="12.75">
@@ -53497,13 +53497,13 @@
         <v>0</v>
       </c>
       <c r="G1791" s="1">
-        <v>3.06585572E7</v>
+        <v>3.0658557200000003E7</v>
       </c>
       <c r="H1791" s="1">
         <v>0</v>
       </c>
       <c r="I1791" s="1">
-        <v>3.06585572E7</v>
+        <v>3.0658557200000003E7</v>
       </c>
     </row>
     <row r="1792" spans="1:9" ht="12.75">
@@ -53932,13 +53932,13 @@
         <v>-5418882</v>
       </c>
       <c r="G1806" s="1">
-        <v>3.195558422299999E8</v>
+        <v>3.2086133222999984E8</v>
       </c>
       <c r="H1806" s="1">
         <v>3.305558458299999E8</v>
       </c>
       <c r="I1806" s="1">
-        <v>-1.6418885600000024E7</v>
+        <v>-1.5113395600000083E7</v>
       </c>
     </row>
     <row r="1807" spans="1:9" ht="12.75">
@@ -54193,13 +54193,13 @@
         <v>0</v>
       </c>
       <c r="G1815" s="1">
-        <v>4.89969833E7</v>
+        <v>7.453694261E7</v>
       </c>
       <c r="H1815" s="1">
         <v>7.480879472E7</v>
       </c>
       <c r="I1815" s="1">
-        <v>-2.581181142E7</v>
+        <v>-271852.1099999994</v>
       </c>
     </row>
     <row r="1816" spans="1:9" ht="12.75">
@@ -54283,10 +54283,10 @@
         <v>4687449</v>
       </c>
       <c r="H1818" s="1">
-        <v>1.6562694950000001E7</v>
+        <v>1.6562694950000005E7</v>
       </c>
       <c r="I1818" s="1">
-        <v>-1.1875245950000001E7</v>
+        <v>-1.1875245950000005E7</v>
       </c>
     </row>
     <row r="1819" spans="1:9" ht="12.75">
@@ -54312,10 +54312,10 @@
         <v>1758542.24</v>
       </c>
       <c r="H1819" s="1">
-        <v>1164129.74</v>
+        <v>1164129.7400000002</v>
       </c>
       <c r="I1819" s="1">
-        <v>594412.50</v>
+        <v>594412.4999999998</v>
       </c>
     </row>
     <row r="1820" spans="1:9" ht="12.75">
@@ -54367,10 +54367,10 @@
         <v>0</v>
       </c>
       <c r="G1821" s="1">
-        <v>3.311609546500001E8</v>
+        <v>3.3116095465000004E8</v>
       </c>
       <c r="H1821" s="1">
-        <v>3.3116095465000004E8</v>
+        <v>3.3116095465E8</v>
       </c>
       <c r="I1821" s="1">
         <v>5.9604644775390625E-8</v>
@@ -54422,16 +54422,16 @@
         <v>363</v>
       </c>
       <c r="F1823" s="1">
-        <v>0</v>
+        <v>-1.862645149230957E-7</v>
       </c>
       <c r="G1823" s="1">
-        <v>7.716808789079996E9</v>
+        <v>7.743654238389995E9</v>
       </c>
       <c r="H1823" s="1">
-        <v>7.716808789080001E9</v>
+        <v>7.743654238389999E9</v>
       </c>
       <c r="I1823" s="1">
-        <v>-2.641230821609497E-6</v>
+        <v>-1.866370439529419E-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-03-30
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9193" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9223" uniqueCount="372">
   <si>
     <t>Book</t>
   </si>
@@ -1085,7 +1085,7 @@
     <t>AIP-0112-Training Infra and MEL-Google Cloud-NFC</t>
   </si>
   <si>
-    <t>AIP-0117-Training Infra and MEL-Google IT-NFC</t>
+    <t>AIP-0141-Training Infra and MEL-Google-NFC</t>
   </si>
   <si>
     <t>AIP-0103-Administration-RFR-NFC</t>
@@ -1098,6 +1098,18 @@
   </si>
   <si>
     <t>AIP-0137-SEAP-Google Digital-Non FCRA</t>
+  </si>
+  <si>
+    <t>AIP-0138-SEAP-Google Cloud-Non FCRA</t>
+  </si>
+  <si>
+    <t>AIP-0139-SEAP-GOC-Non FCRA</t>
+  </si>
+  <si>
+    <t>AIP-0140-SEAP-Google Connect-Non FCRA</t>
+  </si>
+  <si>
+    <t>AIP-0142-Ecosystem Building-Google India-Non FCRA</t>
   </si>
   <si>
     <t>AIP-0118-Training Infra and MEL-Google Digital-NFC</t>
@@ -1565,8 +1577,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3c8f77cf-00d0-4347-8ab3-07952200a4be}">
-  <dimension ref="A1:I1837"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24ef6e39-1797-4eb8-8e32-ce387745437a}">
+  <dimension ref="A1:I1843"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="14.142857142857142" customWidth="1"/>
@@ -1654,7 +1666,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>-8.940696716308594E-8</v>
+        <v>-2.9802322387695312E-8</v>
       </c>
       <c r="G3" s="1">
         <v>3.54</v>
@@ -1663,7 +1675,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>-8.940696671899673E-8</v>
+        <v>-2.9802321943606103E-8</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -3916,7 +3928,7 @@
         <v>13</v>
       </c>
       <c r="F81" s="1">
-        <v>-9.313225746154785E-10</v>
+        <v>0</v>
       </c>
       <c r="G81" s="1">
         <v>333614</v>
@@ -3925,7 +3937,7 @@
         <v>333614</v>
       </c>
       <c r="I81" s="1">
-        <v>-9.313225746154785E-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:9" ht="12.75">
@@ -40401,13 +40413,13 @@
         <v>0</v>
       </c>
       <c r="G1339" s="1">
-        <v>3.341335865E7</v>
+        <v>3.3413358650000002E7</v>
       </c>
       <c r="H1339" s="1">
         <v>179327</v>
       </c>
       <c r="I1339" s="1">
-        <v>3.323403165E7</v>
+        <v>3.3234031650000002E7</v>
       </c>
     </row>
     <row r="1340" spans="1:9" ht="12.75">
@@ -41706,13 +41718,13 @@
         <v>0</v>
       </c>
       <c r="G1384" s="1">
-        <v>6689781.300000001</v>
+        <v>6689781.3</v>
       </c>
       <c r="H1384" s="1">
         <v>34552</v>
       </c>
       <c r="I1384" s="1">
-        <v>6655229.300000001</v>
+        <v>6655229.3</v>
       </c>
     </row>
     <row r="1385" spans="1:9" ht="12.75">
@@ -41996,13 +42008,13 @@
         <v>0</v>
       </c>
       <c r="G1394" s="1">
-        <v>8018272.119999999</v>
+        <v>8018272.12</v>
       </c>
       <c r="H1394" s="1">
         <v>0</v>
       </c>
       <c r="I1394" s="1">
-        <v>8018272.119999999</v>
+        <v>8018272.12</v>
       </c>
     </row>
     <row r="1395" spans="1:9" ht="12.75">
@@ -42199,13 +42211,13 @@
         <v>0</v>
       </c>
       <c r="G1401" s="1">
-        <v>2.4431303240000002E7</v>
+        <v>2.443130324E7</v>
       </c>
       <c r="H1401" s="1">
         <v>168699</v>
       </c>
       <c r="I1401" s="1">
-        <v>2.4262604240000002E7</v>
+        <v>2.426260424E7</v>
       </c>
     </row>
     <row r="1402" spans="1:9" ht="12.75">
@@ -45067,16 +45079,16 @@
         <v>13</v>
       </c>
       <c r="F1500" s="1">
-        <v>-1.934719700000012E7</v>
+        <v>-1.934719699999994E7</v>
       </c>
       <c r="G1500" s="1">
-        <v>2.1835296529999968E8</v>
+        <v>2.1835296529999974E8</v>
       </c>
       <c r="H1500" s="1">
-        <v>2.078658930799998E8</v>
+        <v>2.0786589307999983E8</v>
       </c>
       <c r="I1500" s="1">
-        <v>-8860124.78000024</v>
+        <v>-8860124.780000031</v>
       </c>
     </row>
     <row r="1501" spans="1:9" ht="12.75">
@@ -45653,10 +45665,10 @@
         <v>557840.1600000001</v>
       </c>
       <c r="H1520" s="1">
-        <v>620679.3400000002</v>
+        <v>620679.3400000001</v>
       </c>
       <c r="I1520" s="1">
-        <v>-62839.18000000005</v>
+        <v>-62839.179999999935</v>
       </c>
     </row>
     <row r="1521" spans="1:9" ht="12.75">
@@ -45734,7 +45746,7 @@
         <v>13</v>
       </c>
       <c r="F1523" s="1">
-        <v>-56797.00000000559</v>
+        <v>-56797.000000002794</v>
       </c>
       <c r="G1523" s="1">
         <v>3227421.94</v>
@@ -45743,7 +45755,7 @@
         <v>3631156.939999996</v>
       </c>
       <c r="I1523" s="1">
-        <v>-460532.00000000186</v>
+        <v>-460531.99999999907</v>
       </c>
     </row>
     <row r="1524" spans="1:9" ht="12.75">
@@ -45795,10 +45807,10 @@
         <v>0</v>
       </c>
       <c r="G1525" s="1">
-        <v>1.1669682698900006E9</v>
+        <v>1.1669682698900003E9</v>
       </c>
       <c r="H1525" s="1">
-        <v>1.1669682698900025E9</v>
+        <v>1.1669682698900023E9</v>
       </c>
       <c r="I1525" s="1">
         <v>-1.9073486328125E-6</v>
@@ -46726,10 +46738,10 @@
         <v>6.935924803999999E7</v>
       </c>
       <c r="H1557" s="1">
-        <v>8.273642369999999E7</v>
+        <v>8.27364237E7</v>
       </c>
       <c r="I1557" s="1">
-        <v>1.581653324000001E7</v>
+        <v>1.5816533239999995E7</v>
       </c>
     </row>
     <row r="1558" spans="1:9" ht="12.75">
@@ -46813,10 +46825,10 @@
         <v>8.56587629E8</v>
       </c>
       <c r="H1560" s="1">
-        <v>4.564666996899999E8</v>
+        <v>4.5646669968999994E8</v>
       </c>
       <c r="I1560" s="1">
-        <v>4.001209293100001E8</v>
+        <v>4.0012092931000006E8</v>
       </c>
     </row>
     <row r="1561" spans="1:9" ht="12.75">
@@ -47303,10 +47315,10 @@
         <v>0</v>
       </c>
       <c r="G1577" s="1">
-        <v>2.297129868E8</v>
+        <v>2.2971298679999998E8</v>
       </c>
       <c r="H1577" s="1">
-        <v>1.9410629792000005E8</v>
+        <v>1.9410629792000002E8</v>
       </c>
       <c r="I1577" s="1">
         <v>3.5606688879999965E7</v>
@@ -48782,13 +48794,13 @@
         <v>0</v>
       </c>
       <c r="G1628" s="1">
-        <v>307964.57</v>
+        <v>307964.56999999995</v>
       </c>
       <c r="H1628" s="1">
         <v>0</v>
       </c>
       <c r="I1628" s="1">
-        <v>307964.57</v>
+        <v>307964.56999999995</v>
       </c>
     </row>
     <row r="1629" spans="1:9" ht="12.75">
@@ -49971,13 +49983,13 @@
         <v>0</v>
       </c>
       <c r="G1669" s="1">
-        <v>2650789.68</v>
+        <v>2650789.6799999997</v>
       </c>
       <c r="H1669" s="1">
         <v>0</v>
       </c>
       <c r="I1669" s="1">
-        <v>2650789.68</v>
+        <v>2650789.6799999997</v>
       </c>
     </row>
     <row r="1670" spans="1:9" ht="12.75">
@@ -50754,13 +50766,13 @@
         <v>0</v>
       </c>
       <c r="G1696" s="1">
+        <v>3734639.2299999995</v>
+      </c>
+      <c r="H1696" s="1">
         <v>3734639.23</v>
       </c>
-      <c r="H1696" s="1">
-        <v>3734639.2299999995</v>
-      </c>
       <c r="I1696" s="1">
-        <v>4.6566128730773926E-10</v>
+        <v>-4.6566128730773926E-10</v>
       </c>
     </row>
     <row r="1697" spans="1:9" ht="12.75">
@@ -50841,13 +50853,13 @@
         <v>0</v>
       </c>
       <c r="G1699" s="1">
-        <v>2335546.0799999996</v>
+        <v>2335546.08</v>
       </c>
       <c r="H1699" s="1">
         <v>0</v>
       </c>
       <c r="I1699" s="1">
-        <v>2335546.0799999996</v>
+        <v>2335546.08</v>
       </c>
     </row>
     <row r="1700" spans="1:9" ht="12.75">
@@ -50957,13 +50969,13 @@
         <v>0</v>
       </c>
       <c r="G1703" s="1">
-        <v>456691.31999999995</v>
+        <v>456691.32</v>
       </c>
       <c r="H1703" s="1">
         <v>0</v>
       </c>
       <c r="I1703" s="1">
-        <v>456691.31999999995</v>
+        <v>456691.32</v>
       </c>
     </row>
     <row r="1704" spans="1:9" ht="12.75">
@@ -51015,13 +51027,13 @@
         <v>0</v>
       </c>
       <c r="G1705" s="1">
-        <v>1406462.61</v>
+        <v>1406462.6099999999</v>
       </c>
       <c r="H1705" s="1">
         <v>211054</v>
       </c>
       <c r="I1705" s="1">
-        <v>1195408.61</v>
+        <v>1195408.6099999999</v>
       </c>
     </row>
     <row r="1706" spans="1:9" ht="12.75">
@@ -52256,19 +52268,19 @@
         <v>235</v>
       </c>
       <c r="E1748" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="F1748" s="1">
         <v>0</v>
       </c>
       <c r="G1748" s="1">
-        <v>16956271</v>
+        <v>2999088</v>
       </c>
       <c r="H1748" s="1">
         <v>0</v>
       </c>
       <c r="I1748" s="1">
-        <v>16956271</v>
+        <v>2999088</v>
       </c>
     </row>
     <row r="1749" spans="1:9" ht="12.75">
@@ -52285,19 +52297,19 @@
         <v>235</v>
       </c>
       <c r="E1749" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F1749" s="1">
         <v>0</v>
       </c>
       <c r="G1749" s="1">
-        <v>2999088</v>
+        <v>743494</v>
       </c>
       <c r="H1749" s="1">
         <v>0</v>
       </c>
       <c r="I1749" s="1">
-        <v>2999088</v>
+        <v>743494</v>
       </c>
     </row>
     <row r="1750" spans="1:9" ht="12.75">
@@ -52314,19 +52326,19 @@
         <v>235</v>
       </c>
       <c r="E1750" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="F1750" s="1">
         <v>0</v>
       </c>
       <c r="G1750" s="1">
-        <v>743494</v>
+        <v>16956271</v>
       </c>
       <c r="H1750" s="1">
         <v>0</v>
       </c>
       <c r="I1750" s="1">
-        <v>743494</v>
+        <v>16956271</v>
       </c>
     </row>
     <row r="1751" spans="1:9" ht="12.75">
@@ -52720,19 +52732,19 @@
         <v>243</v>
       </c>
       <c r="E1764" t="s">
-        <v>329</v>
+        <v>13</v>
       </c>
       <c r="F1764" s="1">
         <v>0</v>
       </c>
       <c r="G1764" s="1">
-        <v>8760</v>
+        <v>1295677.1400000001</v>
       </c>
       <c r="H1764" s="1">
         <v>0</v>
       </c>
       <c r="I1764" s="1">
-        <v>8760</v>
+        <v>1295677.1400000001</v>
       </c>
     </row>
     <row r="1765" spans="1:9" ht="12.75">
@@ -52749,19 +52761,19 @@
         <v>243</v>
       </c>
       <c r="E1765" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1765" s="1">
         <v>0</v>
       </c>
       <c r="G1765" s="1">
-        <v>12718517</v>
+        <v>8760</v>
       </c>
       <c r="H1765" s="1">
         <v>0</v>
       </c>
       <c r="I1765" s="1">
-        <v>12718517</v>
+        <v>8760</v>
       </c>
     </row>
     <row r="1766" spans="1:9" ht="12.75">
@@ -52778,19 +52790,19 @@
         <v>243</v>
       </c>
       <c r="E1766" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1766" s="1">
         <v>0</v>
       </c>
       <c r="G1766" s="1">
-        <v>7800000</v>
+        <v>12718517</v>
       </c>
       <c r="H1766" s="1">
         <v>0</v>
       </c>
       <c r="I1766" s="1">
-        <v>7800000</v>
+        <v>12718517</v>
       </c>
     </row>
     <row r="1767" spans="1:9" ht="12.75">
@@ -52807,19 +52819,19 @@
         <v>243</v>
       </c>
       <c r="E1767" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="F1767" s="1">
         <v>0</v>
       </c>
       <c r="G1767" s="1">
-        <v>176000000</v>
+        <v>7800000</v>
       </c>
       <c r="H1767" s="1">
         <v>0</v>
       </c>
       <c r="I1767" s="1">
-        <v>176000000</v>
+        <v>7800000</v>
       </c>
     </row>
     <row r="1768" spans="1:9" ht="12.75">
@@ -52836,19 +52848,19 @@
         <v>243</v>
       </c>
       <c r="E1768" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1768" s="1">
         <v>0</v>
       </c>
       <c r="G1768" s="1">
-        <v>8041700</v>
+        <v>176000000</v>
       </c>
       <c r="H1768" s="1">
         <v>0</v>
       </c>
       <c r="I1768" s="1">
-        <v>8041700</v>
+        <v>176000000</v>
       </c>
     </row>
     <row r="1769" spans="1:9" ht="12.75">
@@ -52865,19 +52877,19 @@
         <v>243</v>
       </c>
       <c r="E1769" t="s">
-        <v>358</v>
+        <v>335</v>
       </c>
       <c r="F1769" s="1">
         <v>0</v>
       </c>
       <c r="G1769" s="1">
-        <v>6372000</v>
+        <v>43981641</v>
       </c>
       <c r="H1769" s="1">
         <v>0</v>
       </c>
       <c r="I1769" s="1">
-        <v>6372000</v>
+        <v>43981641</v>
       </c>
     </row>
     <row r="1770" spans="1:9" ht="12.75">
@@ -52894,19 +52906,19 @@
         <v>243</v>
       </c>
       <c r="E1770" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F1770" s="1">
         <v>0</v>
       </c>
       <c r="G1770" s="1">
-        <v>18337200</v>
+        <v>2340942</v>
       </c>
       <c r="H1770" s="1">
         <v>0</v>
       </c>
       <c r="I1770" s="1">
-        <v>18337200</v>
+        <v>2340942</v>
       </c>
     </row>
     <row r="1771" spans="1:9" ht="12.75">
@@ -52923,19 +52935,19 @@
         <v>243</v>
       </c>
       <c r="E1771" t="s">
-        <v>340</v>
+        <v>358</v>
       </c>
       <c r="F1771" s="1">
         <v>0</v>
       </c>
       <c r="G1771" s="1">
-        <v>872630</v>
+        <v>6372000</v>
       </c>
       <c r="H1771" s="1">
         <v>0</v>
       </c>
       <c r="I1771" s="1">
-        <v>872630</v>
+        <v>6372000</v>
       </c>
     </row>
     <row r="1772" spans="1:9" ht="12.75">
@@ -52952,19 +52964,19 @@
         <v>243</v>
       </c>
       <c r="E1772" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F1772" s="1">
         <v>0</v>
       </c>
       <c r="G1772" s="1">
-        <v>52038512</v>
+        <v>9772778</v>
       </c>
       <c r="H1772" s="1">
         <v>0</v>
       </c>
       <c r="I1772" s="1">
-        <v>52038512</v>
+        <v>9772778</v>
       </c>
     </row>
     <row r="1773" spans="1:9" ht="12.75">
@@ -52981,19 +52993,19 @@
         <v>243</v>
       </c>
       <c r="E1773" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="F1773" s="1">
         <v>0</v>
       </c>
       <c r="G1773" s="1">
-        <v>70210</v>
+        <v>872630</v>
       </c>
       <c r="H1773" s="1">
         <v>0</v>
       </c>
       <c r="I1773" s="1">
-        <v>70210</v>
+        <v>872630</v>
       </c>
     </row>
     <row r="1774" spans="1:9" ht="12.75">
@@ -53010,19 +53022,19 @@
         <v>243</v>
       </c>
       <c r="E1774" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="F1774" s="1">
         <v>0</v>
       </c>
       <c r="G1774" s="1">
-        <v>17744958</v>
+        <v>50150</v>
       </c>
       <c r="H1774" s="1">
         <v>0</v>
       </c>
       <c r="I1774" s="1">
-        <v>17744958</v>
+        <v>50150</v>
       </c>
     </row>
     <row r="1775" spans="1:9" ht="12.75">
@@ -53039,19 +53051,19 @@
         <v>243</v>
       </c>
       <c r="E1775" t="s">
-        <v>359</v>
+        <v>342</v>
       </c>
       <c r="F1775" s="1">
         <v>0</v>
       </c>
       <c r="G1775" s="1">
-        <v>13652305</v>
+        <v>70210</v>
       </c>
       <c r="H1775" s="1">
         <v>0</v>
       </c>
       <c r="I1775" s="1">
-        <v>13652305</v>
+        <v>70210</v>
       </c>
     </row>
     <row r="1776" spans="1:9" ht="12.75">
@@ -53068,19 +53080,19 @@
         <v>243</v>
       </c>
       <c r="E1776" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="F1776" s="1">
         <v>0</v>
       </c>
       <c r="G1776" s="1">
-        <v>4310342</v>
+        <v>17744958</v>
       </c>
       <c r="H1776" s="1">
         <v>0</v>
       </c>
       <c r="I1776" s="1">
-        <v>4310342</v>
+        <v>17744958</v>
       </c>
     </row>
     <row r="1777" spans="1:9" ht="12.75">
@@ -53097,19 +53109,19 @@
         <v>243</v>
       </c>
       <c r="E1777" t="s">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="F1777" s="1">
         <v>0</v>
       </c>
       <c r="G1777" s="1">
-        <v>2002986</v>
+        <v>11311363</v>
       </c>
       <c r="H1777" s="1">
         <v>0</v>
       </c>
       <c r="I1777" s="1">
-        <v>2002986</v>
+        <v>11311363</v>
       </c>
     </row>
     <row r="1778" spans="1:9" ht="12.75">
@@ -53126,19 +53138,19 @@
         <v>243</v>
       </c>
       <c r="E1778" t="s">
-        <v>360</v>
+        <v>348</v>
       </c>
       <c r="F1778" s="1">
         <v>0</v>
       </c>
       <c r="G1778" s="1">
-        <v>10830040</v>
+        <v>4310342</v>
       </c>
       <c r="H1778" s="1">
         <v>0</v>
       </c>
       <c r="I1778" s="1">
-        <v>10830040</v>
+        <v>4310342</v>
       </c>
     </row>
     <row r="1779" spans="1:9" ht="12.75">
@@ -53152,22 +53164,22 @@
         <v>105</v>
       </c>
       <c r="D1779" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1779" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
       <c r="F1779" s="1">
         <v>0</v>
       </c>
       <c r="G1779" s="1">
-        <v>31481</v>
+        <v>2002986</v>
       </c>
       <c r="H1779" s="1">
         <v>0</v>
       </c>
       <c r="I1779" s="1">
-        <v>31481</v>
+        <v>2002986</v>
       </c>
     </row>
     <row r="1780" spans="1:9" ht="12.75">
@@ -53181,22 +53193,22 @@
         <v>105</v>
       </c>
       <c r="D1780" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1780" t="s">
-        <v>332</v>
+        <v>360</v>
       </c>
       <c r="F1780" s="1">
         <v>0</v>
       </c>
       <c r="G1780" s="1">
-        <v>6638</v>
+        <v>10830040</v>
       </c>
       <c r="H1780" s="1">
         <v>0</v>
       </c>
       <c r="I1780" s="1">
-        <v>6638</v>
+        <v>10830040</v>
       </c>
     </row>
     <row r="1781" spans="1:9" ht="12.75">
@@ -53210,22 +53222,22 @@
         <v>105</v>
       </c>
       <c r="D1781" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1781" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="F1781" s="1">
         <v>0</v>
       </c>
       <c r="G1781" s="1">
-        <v>7140</v>
+        <v>3949794</v>
       </c>
       <c r="H1781" s="1">
         <v>0</v>
       </c>
       <c r="I1781" s="1">
-        <v>7140</v>
+        <v>3949794</v>
       </c>
     </row>
     <row r="1782" spans="1:9" ht="12.75">
@@ -53239,22 +53251,22 @@
         <v>105</v>
       </c>
       <c r="D1782" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E1782" t="s">
-        <v>338</v>
+        <v>362</v>
       </c>
       <c r="F1782" s="1">
         <v>0</v>
       </c>
       <c r="G1782" s="1">
-        <v>41204</v>
+        <v>7554538</v>
       </c>
       <c r="H1782" s="1">
         <v>0</v>
       </c>
       <c r="I1782" s="1">
-        <v>41204</v>
+        <v>7554538</v>
       </c>
     </row>
     <row r="1783" spans="1:9" ht="12.75">
@@ -53268,22 +53280,22 @@
         <v>105</v>
       </c>
       <c r="D1783" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="E1783" t="s">
-        <v>329</v>
+        <v>363</v>
       </c>
       <c r="F1783" s="1">
         <v>0</v>
       </c>
       <c r="G1783" s="1">
-        <v>77571</v>
+        <v>3248411.86</v>
       </c>
       <c r="H1783" s="1">
         <v>0</v>
       </c>
       <c r="I1783" s="1">
-        <v>77571</v>
+        <v>3248411.86</v>
       </c>
     </row>
     <row r="1784" spans="1:9" ht="12.75">
@@ -53297,22 +53309,22 @@
         <v>105</v>
       </c>
       <c r="D1784" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="E1784" t="s">
-        <v>330</v>
+        <v>364</v>
       </c>
       <c r="F1784" s="1">
         <v>0</v>
       </c>
       <c r="G1784" s="1">
-        <v>1513824</v>
+        <v>8564422</v>
       </c>
       <c r="H1784" s="1">
         <v>0</v>
       </c>
       <c r="I1784" s="1">
-        <v>1513824</v>
+        <v>8564422</v>
       </c>
     </row>
     <row r="1785" spans="1:9" ht="12.75">
@@ -53326,22 +53338,22 @@
         <v>105</v>
       </c>
       <c r="D1785" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E1785" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F1785" s="1">
         <v>0</v>
       </c>
       <c r="G1785" s="1">
-        <v>22538</v>
+        <v>31481</v>
       </c>
       <c r="H1785" s="1">
         <v>0</v>
       </c>
       <c r="I1785" s="1">
-        <v>22538</v>
+        <v>31481</v>
       </c>
     </row>
     <row r="1786" spans="1:9" ht="12.75">
@@ -53355,22 +53367,22 @@
         <v>105</v>
       </c>
       <c r="D1786" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E1786" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F1786" s="1">
         <v>0</v>
       </c>
       <c r="G1786" s="1">
-        <v>9676</v>
+        <v>6638</v>
       </c>
       <c r="H1786" s="1">
         <v>0</v>
       </c>
       <c r="I1786" s="1">
-        <v>9676</v>
+        <v>6638</v>
       </c>
     </row>
     <row r="1787" spans="1:9" ht="12.75">
@@ -53384,22 +53396,22 @@
         <v>105</v>
       </c>
       <c r="D1787" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E1787" t="s">
-        <v>329</v>
+        <v>357</v>
       </c>
       <c r="F1787" s="1">
         <v>0</v>
       </c>
       <c r="G1787" s="1">
-        <v>3556925.1799999997</v>
+        <v>7140</v>
       </c>
       <c r="H1787" s="1">
         <v>0</v>
       </c>
       <c r="I1787" s="1">
-        <v>3556925.1799999997</v>
+        <v>7140</v>
       </c>
     </row>
     <row r="1788" spans="1:9" ht="12.75">
@@ -53413,22 +53425,22 @@
         <v>105</v>
       </c>
       <c r="D1788" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E1788" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="F1788" s="1">
         <v>0</v>
       </c>
       <c r="G1788" s="1">
-        <v>734237.45</v>
+        <v>41204</v>
       </c>
       <c r="H1788" s="1">
         <v>0</v>
       </c>
       <c r="I1788" s="1">
-        <v>734237.45</v>
+        <v>41204</v>
       </c>
     </row>
     <row r="1789" spans="1:9" ht="12.75">
@@ -53442,22 +53454,22 @@
         <v>105</v>
       </c>
       <c r="D1789" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E1789" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F1789" s="1">
         <v>0</v>
       </c>
       <c r="G1789" s="1">
-        <v>31417864</v>
+        <v>77571</v>
       </c>
       <c r="H1789" s="1">
-        <v>31417864</v>
+        <v>0</v>
       </c>
       <c r="I1789" s="1">
-        <v>0</v>
+        <v>77571</v>
       </c>
     </row>
     <row r="1790" spans="1:9" ht="12.75">
@@ -53471,22 +53483,22 @@
         <v>105</v>
       </c>
       <c r="D1790" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E1790" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="F1790" s="1">
         <v>0</v>
       </c>
       <c r="G1790" s="1">
-        <v>4138525.55</v>
+        <v>1513824</v>
       </c>
       <c r="H1790" s="1">
         <v>0</v>
       </c>
       <c r="I1790" s="1">
-        <v>4138525.55</v>
+        <v>1513824</v>
       </c>
     </row>
     <row r="1791" spans="1:9" ht="12.75">
@@ -53500,22 +53512,22 @@
         <v>105</v>
       </c>
       <c r="D1791" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E1791" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F1791" s="1">
         <v>0</v>
       </c>
       <c r="G1791" s="1">
-        <v>2860819.3499999996</v>
+        <v>22538</v>
       </c>
       <c r="H1791" s="1">
         <v>0</v>
       </c>
       <c r="I1791" s="1">
-        <v>2860819.3499999996</v>
+        <v>22538</v>
       </c>
     </row>
     <row r="1792" spans="1:9" ht="12.75">
@@ -53529,22 +53541,22 @@
         <v>105</v>
       </c>
       <c r="D1792" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E1792" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F1792" s="1">
         <v>0</v>
       </c>
       <c r="G1792" s="1">
-        <v>1.8851695400000002E7</v>
+        <v>9676</v>
       </c>
       <c r="H1792" s="1">
         <v>0</v>
       </c>
       <c r="I1792" s="1">
-        <v>1.8851695400000002E7</v>
+        <v>9676</v>
       </c>
     </row>
     <row r="1793" spans="1:9" ht="12.75">
@@ -53561,19 +53573,19 @@
         <v>250</v>
       </c>
       <c r="E1793" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="F1793" s="1">
         <v>0</v>
       </c>
       <c r="G1793" s="1">
-        <v>5986158</v>
+        <v>3556925.18</v>
       </c>
       <c r="H1793" s="1">
-        <v>5986158</v>
+        <v>0</v>
       </c>
       <c r="I1793" s="1">
-        <v>0</v>
+        <v>3556925.18</v>
       </c>
     </row>
     <row r="1794" spans="1:9" ht="12.75">
@@ -53590,19 +53602,19 @@
         <v>250</v>
       </c>
       <c r="E1794" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="F1794" s="1">
         <v>0</v>
       </c>
       <c r="G1794" s="1">
-        <v>30819</v>
+        <v>734237.45</v>
       </c>
       <c r="H1794" s="1">
         <v>0</v>
       </c>
       <c r="I1794" s="1">
-        <v>30819</v>
+        <v>734237.45</v>
       </c>
     </row>
     <row r="1795" spans="1:9" ht="12.75">
@@ -53619,19 +53631,19 @@
         <v>250</v>
       </c>
       <c r="E1795" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="F1795" s="1">
         <v>0</v>
       </c>
       <c r="G1795" s="1">
-        <v>1516559</v>
+        <v>31417864</v>
       </c>
       <c r="H1795" s="1">
-        <v>747735</v>
+        <v>31417864</v>
       </c>
       <c r="I1795" s="1">
-        <v>768824</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1796" spans="1:9" ht="12.75">
@@ -53648,19 +53660,19 @@
         <v>250</v>
       </c>
       <c r="E1796" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="F1796" s="1">
         <v>0</v>
       </c>
       <c r="G1796" s="1">
-        <v>4196982</v>
+        <v>4138525.55</v>
       </c>
       <c r="H1796" s="1">
         <v>0</v>
       </c>
       <c r="I1796" s="1">
-        <v>4196982</v>
+        <v>4138525.55</v>
       </c>
     </row>
     <row r="1797" spans="1:9" ht="12.75">
@@ -53677,19 +53689,19 @@
         <v>250</v>
       </c>
       <c r="E1797" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="F1797" s="1">
         <v>0</v>
       </c>
       <c r="G1797" s="1">
-        <v>9.847959733E7</v>
+        <v>2860819.35</v>
       </c>
       <c r="H1797" s="1">
-        <v>9.849326033E7</v>
+        <v>0</v>
       </c>
       <c r="I1797" s="1">
-        <v>-13663</v>
+        <v>2860819.35</v>
       </c>
     </row>
     <row r="1798" spans="1:9" ht="12.75">
@@ -53706,19 +53718,19 @@
         <v>250</v>
       </c>
       <c r="E1798" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="F1798" s="1">
         <v>0</v>
       </c>
       <c r="G1798" s="1">
-        <v>2790926.10</v>
+        <v>1.8851695400000002E7</v>
       </c>
       <c r="H1798" s="1">
         <v>0</v>
       </c>
       <c r="I1798" s="1">
-        <v>2790926.10</v>
+        <v>1.8851695400000002E7</v>
       </c>
     </row>
     <row r="1799" spans="1:9" ht="12.75">
@@ -53735,19 +53747,19 @@
         <v>250</v>
       </c>
       <c r="E1799" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="F1799" s="1">
         <v>0</v>
       </c>
       <c r="G1799" s="1">
-        <v>1.0763457100000001E7</v>
+        <v>5986158</v>
       </c>
       <c r="H1799" s="1">
-        <v>0</v>
+        <v>5986158</v>
       </c>
       <c r="I1799" s="1">
-        <v>1.0763457100000001E7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1800" spans="1:9" ht="12.75">
@@ -53764,19 +53776,19 @@
         <v>250</v>
       </c>
       <c r="E1800" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="F1800" s="1">
         <v>0</v>
       </c>
       <c r="G1800" s="1">
-        <v>3.0658557199999996E7</v>
+        <v>30819</v>
       </c>
       <c r="H1800" s="1">
         <v>0</v>
       </c>
       <c r="I1800" s="1">
-        <v>3.0658557199999996E7</v>
+        <v>30819</v>
       </c>
     </row>
     <row r="1801" spans="1:9" ht="12.75">
@@ -53793,19 +53805,19 @@
         <v>250</v>
       </c>
       <c r="E1801" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="F1801" s="1">
         <v>0</v>
       </c>
       <c r="G1801" s="1">
-        <v>21704777</v>
+        <v>1516559</v>
       </c>
       <c r="H1801" s="1">
-        <v>0</v>
+        <v>747735</v>
       </c>
       <c r="I1801" s="1">
-        <v>21704777</v>
+        <v>768824</v>
       </c>
     </row>
     <row r="1802" spans="1:9" ht="12.75">
@@ -53819,22 +53831,22 @@
         <v>105</v>
       </c>
       <c r="D1802" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E1802" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="F1802" s="1">
         <v>0</v>
       </c>
       <c r="G1802" s="1">
-        <v>0.25</v>
+        <v>4196982</v>
       </c>
       <c r="H1802" s="1">
         <v>0</v>
       </c>
       <c r="I1802" s="1">
-        <v>0.25</v>
+        <v>4196982</v>
       </c>
     </row>
     <row r="1803" spans="1:9" ht="12.75">
@@ -53848,7 +53860,7 @@
         <v>105</v>
       </c>
       <c r="D1803" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E1803" t="s">
         <v>339</v>
@@ -53857,13 +53869,13 @@
         <v>0</v>
       </c>
       <c r="G1803" s="1">
-        <v>0</v>
+        <v>9.847959733E7</v>
       </c>
       <c r="H1803" s="1">
-        <v>1</v>
+        <v>9.849326033E7</v>
       </c>
       <c r="I1803" s="1">
-        <v>-1</v>
+        <v>-13663</v>
       </c>
     </row>
     <row r="1804" spans="1:9" ht="12.75">
@@ -53877,22 +53889,22 @@
         <v>105</v>
       </c>
       <c r="D1804" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="E1804" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="F1804" s="1">
         <v>0</v>
       </c>
       <c r="G1804" s="1">
-        <v>411206</v>
+        <v>2790926.10</v>
       </c>
       <c r="H1804" s="1">
         <v>0</v>
       </c>
       <c r="I1804" s="1">
-        <v>411206</v>
+        <v>2790926.10</v>
       </c>
     </row>
     <row r="1805" spans="1:9" ht="12.75">
@@ -53906,22 +53918,22 @@
         <v>105</v>
       </c>
       <c r="D1805" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="E1805" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="F1805" s="1">
         <v>0</v>
       </c>
       <c r="G1805" s="1">
-        <v>137069</v>
+        <v>1.0763457100000001E7</v>
       </c>
       <c r="H1805" s="1">
         <v>0</v>
       </c>
       <c r="I1805" s="1">
-        <v>137069</v>
+        <v>1.0763457100000001E7</v>
       </c>
     </row>
     <row r="1806" spans="1:9" ht="12.75">
@@ -53935,22 +53947,22 @@
         <v>105</v>
       </c>
       <c r="D1806" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="E1806" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="F1806" s="1">
         <v>0</v>
       </c>
       <c r="G1806" s="1">
-        <v>68534</v>
+        <v>3.0658557199999996E7</v>
       </c>
       <c r="H1806" s="1">
         <v>0</v>
       </c>
       <c r="I1806" s="1">
-        <v>68534</v>
+        <v>3.0658557199999996E7</v>
       </c>
     </row>
     <row r="1807" spans="1:9" ht="12.75">
@@ -53964,22 +53976,22 @@
         <v>105</v>
       </c>
       <c r="D1807" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="E1807" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="F1807" s="1">
         <v>0</v>
       </c>
       <c r="G1807" s="1">
-        <v>68534</v>
+        <v>21704777</v>
       </c>
       <c r="H1807" s="1">
         <v>0</v>
       </c>
       <c r="I1807" s="1">
-        <v>68534</v>
+        <v>21704777</v>
       </c>
     </row>
     <row r="1808" spans="1:9" ht="12.75">
@@ -53993,22 +54005,22 @@
         <v>105</v>
       </c>
       <c r="D1808" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E1808" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="F1808" s="1">
         <v>0</v>
       </c>
       <c r="G1808" s="1">
-        <v>835419</v>
+        <v>0.25</v>
       </c>
       <c r="H1808" s="1">
         <v>0</v>
       </c>
       <c r="I1808" s="1">
-        <v>835419</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="1809" spans="1:9" ht="12.75">
@@ -54022,22 +54034,22 @@
         <v>105</v>
       </c>
       <c r="D1809" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="E1809" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="F1809" s="1">
         <v>0</v>
       </c>
       <c r="G1809" s="1">
-        <v>148184</v>
+        <v>0</v>
       </c>
       <c r="H1809" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I1809" s="1">
-        <v>148184</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="1810" spans="1:9" ht="12.75">
@@ -54051,22 +54063,22 @@
         <v>105</v>
       </c>
       <c r="D1810" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E1810" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F1810" s="1">
         <v>0</v>
       </c>
       <c r="G1810" s="1">
-        <v>74092</v>
+        <v>411206</v>
       </c>
       <c r="H1810" s="1">
         <v>0</v>
       </c>
       <c r="I1810" s="1">
-        <v>74092</v>
+        <v>411206</v>
       </c>
     </row>
     <row r="1811" spans="1:9" ht="12.75">
@@ -54080,22 +54092,22 @@
         <v>105</v>
       </c>
       <c r="D1811" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E1811" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F1811" s="1">
         <v>0</v>
       </c>
       <c r="G1811" s="1">
-        <v>74092.80</v>
+        <v>137069</v>
       </c>
       <c r="H1811" s="1">
         <v>0</v>
       </c>
       <c r="I1811" s="1">
-        <v>74092.80</v>
+        <v>137069</v>
       </c>
     </row>
     <row r="1812" spans="1:9" ht="12.75">
@@ -54109,22 +54121,22 @@
         <v>105</v>
       </c>
       <c r="D1812" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E1812" t="s">
-        <v>361</v>
+        <v>335</v>
       </c>
       <c r="F1812" s="1">
         <v>0</v>
       </c>
       <c r="G1812" s="1">
-        <v>163430</v>
+        <v>68534</v>
       </c>
       <c r="H1812" s="1">
         <v>0</v>
       </c>
       <c r="I1812" s="1">
-        <v>163430</v>
+        <v>68534</v>
       </c>
     </row>
     <row r="1813" spans="1:9" ht="12.75">
@@ -54138,22 +54150,22 @@
         <v>105</v>
       </c>
       <c r="D1813" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E1813" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="F1813" s="1">
         <v>0</v>
       </c>
       <c r="G1813" s="1">
-        <v>137490</v>
+        <v>68534</v>
       </c>
       <c r="H1813" s="1">
         <v>0</v>
       </c>
       <c r="I1813" s="1">
-        <v>137490</v>
+        <v>68534</v>
       </c>
     </row>
     <row r="1814" spans="1:9" ht="12.75">
@@ -54167,22 +54179,22 @@
         <v>105</v>
       </c>
       <c r="D1814" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="E1814" t="s">
-        <v>330</v>
+        <v>355</v>
       </c>
       <c r="F1814" s="1">
         <v>0</v>
       </c>
       <c r="G1814" s="1">
-        <v>305648</v>
+        <v>835419</v>
       </c>
       <c r="H1814" s="1">
         <v>0</v>
       </c>
       <c r="I1814" s="1">
-        <v>305648</v>
+        <v>835419</v>
       </c>
     </row>
     <row r="1815" spans="1:9" ht="12.75">
@@ -54196,7 +54208,7 @@
         <v>105</v>
       </c>
       <c r="D1815" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E1815" t="s">
         <v>331</v>
@@ -54205,13 +54217,13 @@
         <v>0</v>
       </c>
       <c r="G1815" s="1">
-        <v>484</v>
+        <v>148184</v>
       </c>
       <c r="H1815" s="1">
         <v>0</v>
       </c>
       <c r="I1815" s="1">
-        <v>484</v>
+        <v>148184</v>
       </c>
     </row>
     <row r="1816" spans="1:9" ht="12.75">
@@ -54225,22 +54237,22 @@
         <v>105</v>
       </c>
       <c r="D1816" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E1816" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="F1816" s="1">
         <v>0</v>
       </c>
       <c r="G1816" s="1">
-        <v>32000</v>
+        <v>74092</v>
       </c>
       <c r="H1816" s="1">
         <v>0</v>
       </c>
       <c r="I1816" s="1">
-        <v>32000</v>
+        <v>74092</v>
       </c>
     </row>
     <row r="1817" spans="1:9" ht="12.75">
@@ -54254,22 +54266,22 @@
         <v>105</v>
       </c>
       <c r="D1817" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="E1817" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="F1817" s="1">
         <v>0</v>
       </c>
       <c r="G1817" s="1">
-        <v>2814300</v>
+        <v>74092.80</v>
       </c>
       <c r="H1817" s="1">
         <v>0</v>
       </c>
       <c r="I1817" s="1">
-        <v>2814300</v>
+        <v>74092.80</v>
       </c>
     </row>
     <row r="1818" spans="1:9" ht="12.75">
@@ -54277,28 +54289,28 @@
         <v>313</v>
       </c>
       <c r="B1818" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="C1818" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="D1818" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="E1818" t="s">
-        <v>13</v>
+        <v>365</v>
       </c>
       <c r="F1818" s="1">
         <v>0</v>
       </c>
       <c r="G1818" s="1">
-        <v>0</v>
+        <v>163430</v>
       </c>
       <c r="H1818" s="1">
-        <v>7351276</v>
+        <v>0</v>
       </c>
       <c r="I1818" s="1">
-        <v>-7351276</v>
+        <v>163430</v>
       </c>
     </row>
     <row r="1819" spans="1:9" ht="12.75">
@@ -54306,28 +54318,28 @@
         <v>313</v>
       </c>
       <c r="B1819" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="C1819" t="s">
-        <v>264</v>
+        <v>105</v>
       </c>
       <c r="D1819" t="s">
-        <v>309</v>
+        <v>258</v>
       </c>
       <c r="E1819" t="s">
-        <v>13</v>
+        <v>329</v>
       </c>
       <c r="F1819" s="1">
         <v>0</v>
       </c>
       <c r="G1819" s="1">
-        <v>0</v>
+        <v>137490</v>
       </c>
       <c r="H1819" s="1">
         <v>0</v>
       </c>
       <c r="I1819" s="1">
-        <v>0</v>
+        <v>137490</v>
       </c>
     </row>
     <row r="1820" spans="1:9" ht="12.75">
@@ -54335,28 +54347,28 @@
         <v>313</v>
       </c>
       <c r="B1820" t="s">
-        <v>268</v>
+        <v>105</v>
       </c>
       <c r="C1820" t="s">
-        <v>269</v>
+        <v>105</v>
       </c>
       <c r="D1820" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="E1820" t="s">
-        <v>13</v>
+        <v>330</v>
       </c>
       <c r="F1820" s="1">
-        <v>-5418882</v>
+        <v>0</v>
       </c>
       <c r="G1820" s="1">
-        <v>3.7604722833000004E8</v>
+        <v>305648</v>
       </c>
       <c r="H1820" s="1">
-        <v>4.556299534799999E8</v>
+        <v>0</v>
       </c>
       <c r="I1820" s="1">
-        <v>-8.500160714999986E7</v>
+        <v>305648</v>
       </c>
     </row>
     <row r="1821" spans="1:9" ht="12.75">
@@ -54364,28 +54376,28 @@
         <v>313</v>
       </c>
       <c r="B1821" t="s">
-        <v>268</v>
+        <v>105</v>
       </c>
       <c r="C1821" t="s">
-        <v>273</v>
+        <v>105</v>
       </c>
       <c r="D1821" t="s">
-        <v>362</v>
+        <v>258</v>
       </c>
       <c r="E1821" t="s">
-        <v>13</v>
+        <v>331</v>
       </c>
       <c r="F1821" s="1">
         <v>0</v>
       </c>
       <c r="G1821" s="1">
-        <v>5013786</v>
+        <v>484</v>
       </c>
       <c r="H1821" s="1">
-        <v>5013786</v>
+        <v>0</v>
       </c>
       <c r="I1821" s="1">
-        <v>0</v>
+        <v>484</v>
       </c>
     </row>
     <row r="1822" spans="1:9" ht="12.75">
@@ -54393,28 +54405,28 @@
         <v>313</v>
       </c>
       <c r="B1822" t="s">
-        <v>268</v>
+        <v>105</v>
       </c>
       <c r="C1822" t="s">
-        <v>273</v>
+        <v>105</v>
       </c>
       <c r="D1822" t="s">
-        <v>278</v>
+        <v>259</v>
       </c>
       <c r="E1822" t="s">
-        <v>13</v>
+        <v>339</v>
       </c>
       <c r="F1822" s="1">
-        <v>-22030149</v>
+        <v>0</v>
       </c>
       <c r="G1822" s="1">
-        <v>7656302</v>
+        <v>32000</v>
       </c>
       <c r="H1822" s="1">
-        <v>9.136277758399999E8</v>
+        <v>0</v>
       </c>
       <c r="I1822" s="1">
-        <v>-9.280016228399999E8</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="1823" spans="1:9" ht="12.75">
@@ -54422,28 +54434,28 @@
         <v>313</v>
       </c>
       <c r="B1823" t="s">
-        <v>268</v>
+        <v>105</v>
       </c>
       <c r="C1823" t="s">
-        <v>273</v>
+        <v>105</v>
       </c>
       <c r="D1823" t="s">
-        <v>282</v>
+        <v>263</v>
       </c>
       <c r="E1823" t="s">
-        <v>13</v>
+        <v>338</v>
       </c>
       <c r="F1823" s="1">
-        <v>-14989</v>
+        <v>0</v>
       </c>
       <c r="G1823" s="1">
-        <v>10075535</v>
+        <v>2814300</v>
       </c>
       <c r="H1823" s="1">
-        <v>12988627</v>
+        <v>0</v>
       </c>
       <c r="I1823" s="1">
-        <v>-2928081</v>
+        <v>2814300</v>
       </c>
     </row>
     <row r="1824" spans="1:9" ht="12.75">
@@ -54451,13 +54463,13 @@
         <v>313</v>
       </c>
       <c r="B1824" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C1824" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="D1824" t="s">
-        <v>363</v>
+        <v>267</v>
       </c>
       <c r="E1824" t="s">
         <v>13</v>
@@ -54466,13 +54478,13 @@
         <v>0</v>
       </c>
       <c r="G1824" s="1">
-        <v>2659661</v>
+        <v>0</v>
       </c>
       <c r="H1824" s="1">
-        <v>2659660</v>
+        <v>7351276</v>
       </c>
       <c r="I1824" s="1">
-        <v>1</v>
+        <v>-7351276</v>
       </c>
     </row>
     <row r="1825" spans="1:9" ht="12.75">
@@ -54480,13 +54492,13 @@
         <v>313</v>
       </c>
       <c r="B1825" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C1825" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="D1825" t="s">
-        <v>286</v>
+        <v>309</v>
       </c>
       <c r="E1825" t="s">
         <v>13</v>
@@ -54498,10 +54510,10 @@
         <v>0</v>
       </c>
       <c r="H1825" s="1">
-        <v>190424</v>
+        <v>0</v>
       </c>
       <c r="I1825" s="1">
-        <v>-190424</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1826" spans="1:9" ht="12.75">
@@ -54512,25 +54524,25 @@
         <v>268</v>
       </c>
       <c r="C1826" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D1826" t="s">
-        <v>364</v>
+        <v>269</v>
       </c>
       <c r="E1826" t="s">
         <v>13</v>
       </c>
       <c r="F1826" s="1">
-        <v>0</v>
+        <v>-5418882</v>
       </c>
       <c r="G1826" s="1">
-        <v>2230780</v>
+        <v>3.7604722833000004E8</v>
       </c>
       <c r="H1826" s="1">
-        <v>2294489</v>
+        <v>4.5562995347999996E8</v>
       </c>
       <c r="I1826" s="1">
-        <v>-63709</v>
+        <v>-8.500160714999992E7</v>
       </c>
     </row>
     <row r="1827" spans="1:9" ht="12.75">
@@ -54544,7 +54556,7 @@
         <v>273</v>
       </c>
       <c r="D1827" t="s">
-        <v>287</v>
+        <v>366</v>
       </c>
       <c r="E1827" t="s">
         <v>13</v>
@@ -54553,13 +54565,13 @@
         <v>0</v>
       </c>
       <c r="G1827" s="1">
-        <v>70730</v>
+        <v>5013786</v>
       </c>
       <c r="H1827" s="1">
-        <v>81950</v>
+        <v>5013786</v>
       </c>
       <c r="I1827" s="1">
-        <v>-11220</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1828" spans="1:9" ht="12.75">
@@ -54573,22 +54585,22 @@
         <v>273</v>
       </c>
       <c r="D1828" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="E1828" t="s">
         <v>13</v>
       </c>
       <c r="F1828" s="1">
-        <v>0</v>
+        <v>-22030149</v>
       </c>
       <c r="G1828" s="1">
-        <v>840</v>
+        <v>7656302</v>
       </c>
       <c r="H1828" s="1">
-        <v>416</v>
+        <v>9.136277758399999E8</v>
       </c>
       <c r="I1828" s="1">
-        <v>424</v>
+        <v>-9.280016228399999E8</v>
       </c>
     </row>
     <row r="1829" spans="1:9" ht="12.75">
@@ -54602,22 +54614,22 @@
         <v>273</v>
       </c>
       <c r="D1829" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="E1829" t="s">
         <v>13</v>
       </c>
       <c r="F1829" s="1">
-        <v>0</v>
+        <v>-14989</v>
       </c>
       <c r="G1829" s="1">
-        <v>7.462776786E7</v>
+        <v>10075535</v>
       </c>
       <c r="H1829" s="1">
-        <v>7.480879472E7</v>
+        <v>12988627</v>
       </c>
       <c r="I1829" s="1">
-        <v>-181026.8599999994</v>
+        <v>-2928081</v>
       </c>
     </row>
     <row r="1830" spans="1:9" ht="12.75">
@@ -54631,7 +54643,7 @@
         <v>273</v>
       </c>
       <c r="D1830" t="s">
-        <v>291</v>
+        <v>367</v>
       </c>
       <c r="E1830" t="s">
         <v>13</v>
@@ -54640,13 +54652,13 @@
         <v>0</v>
       </c>
       <c r="G1830" s="1">
-        <v>167905.90</v>
+        <v>2659661</v>
       </c>
       <c r="H1830" s="1">
-        <v>243277.03999999998</v>
+        <v>2659660</v>
       </c>
       <c r="I1830" s="1">
-        <v>-75371.13999999998</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1831" spans="1:9" ht="12.75">
@@ -54660,7 +54672,7 @@
         <v>273</v>
       </c>
       <c r="D1831" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="E1831" t="s">
         <v>13</v>
@@ -54669,13 +54681,13 @@
         <v>0</v>
       </c>
       <c r="G1831" s="1">
-        <v>475515</v>
+        <v>0</v>
       </c>
       <c r="H1831" s="1">
-        <v>504838.90</v>
+        <v>190424</v>
       </c>
       <c r="I1831" s="1">
-        <v>-29323.900000000023</v>
+        <v>-190424</v>
       </c>
     </row>
     <row r="1832" spans="1:9" ht="12.75">
@@ -54689,7 +54701,7 @@
         <v>273</v>
       </c>
       <c r="D1832" t="s">
-        <v>293</v>
+        <v>368</v>
       </c>
       <c r="E1832" t="s">
         <v>13</v>
@@ -54698,13 +54710,13 @@
         <v>0</v>
       </c>
       <c r="G1832" s="1">
-        <v>8376122</v>
+        <v>2230780</v>
       </c>
       <c r="H1832" s="1">
-        <v>1.9194978950000003E7</v>
+        <v>2294489</v>
       </c>
       <c r="I1832" s="1">
-        <v>-1.0818856950000003E7</v>
+        <v>-63709</v>
       </c>
     </row>
     <row r="1833" spans="1:9" ht="12.75">
@@ -54718,7 +54730,7 @@
         <v>273</v>
       </c>
       <c r="D1833" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="E1833" t="s">
         <v>13</v>
@@ -54727,13 +54739,13 @@
         <v>0</v>
       </c>
       <c r="G1833" s="1">
-        <v>1758542.24</v>
+        <v>70730</v>
       </c>
       <c r="H1833" s="1">
-        <v>1164129.7399999998</v>
+        <v>81950</v>
       </c>
       <c r="I1833" s="1">
-        <v>594412.5000000002</v>
+        <v>-11220</v>
       </c>
     </row>
     <row r="1834" spans="1:9" ht="12.75">
@@ -54747,7 +54759,7 @@
         <v>273</v>
       </c>
       <c r="D1834" t="s">
-        <v>365</v>
+        <v>288</v>
       </c>
       <c r="E1834" t="s">
         <v>13</v>
@@ -54756,13 +54768,13 @@
         <v>0</v>
       </c>
       <c r="G1834" s="1">
-        <v>18462722</v>
+        <v>840</v>
       </c>
       <c r="H1834" s="1">
-        <v>2.376985961E7</v>
+        <v>416</v>
       </c>
       <c r="I1834" s="1">
-        <v>-5307137.609999999</v>
+        <v>424</v>
       </c>
     </row>
     <row r="1835" spans="1:9" ht="12.75">
@@ -54773,10 +54785,10 @@
         <v>268</v>
       </c>
       <c r="C1835" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="D1835" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="E1835" t="s">
         <v>13</v>
@@ -54785,13 +54797,13 @@
         <v>0</v>
       </c>
       <c r="G1835" s="1">
-        <v>3.311609599000001E8</v>
+        <v>7.462776786E7</v>
       </c>
       <c r="H1835" s="1">
-        <v>3.3116095990000004E8</v>
+        <v>7.480879472E7</v>
       </c>
       <c r="I1835" s="1">
-        <v>5.9604644775390625E-8</v>
+        <v>-181026.8599999994</v>
       </c>
     </row>
     <row r="1836" spans="1:9" ht="12.75">
@@ -54802,10 +54814,10 @@
         <v>268</v>
       </c>
       <c r="C1836" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="D1836" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="E1836" t="s">
         <v>13</v>
@@ -54814,42 +54826,216 @@
         <v>0</v>
       </c>
       <c r="G1836" s="1">
-        <v>0</v>
+        <v>167905.90</v>
       </c>
       <c r="H1836" s="1">
-        <v>1.118956866E7</v>
+        <v>243277.04</v>
       </c>
       <c r="I1836" s="1">
-        <v>-1.118956866E7</v>
+        <v>-75371.14000000001</v>
       </c>
     </row>
     <row r="1837" spans="1:9" ht="12.75">
       <c r="A1837" t="s">
-        <v>366</v>
+        <v>313</v>
       </c>
       <c r="B1837" t="s">
-        <v>367</v>
+        <v>268</v>
       </c>
       <c r="C1837" t="s">
-        <v>367</v>
+        <v>273</v>
       </c>
       <c r="D1837" t="s">
-        <v>367</v>
+        <v>292</v>
       </c>
       <c r="E1837" t="s">
-        <v>367</v>
+        <v>13</v>
       </c>
       <c r="F1837" s="1">
-        <v>-1.2665987014770508E-7</v>
+        <v>0</v>
       </c>
       <c r="G1837" s="1">
-        <v>7.948051563499996E9</v>
+        <v>475515</v>
       </c>
       <c r="H1837" s="1">
+        <v>504838.90</v>
+      </c>
+      <c r="I1837" s="1">
+        <v>-29323.900000000023</v>
+      </c>
+    </row>
+    <row r="1838" spans="1:9" ht="12.75">
+      <c r="A1838" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1838" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1838" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1838" t="s">
+        <v>293</v>
+      </c>
+      <c r="E1838" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1838" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1838" s="1">
+        <v>8376122</v>
+      </c>
+      <c r="H1838" s="1">
+        <v>1.919497895E7</v>
+      </c>
+      <c r="I1838" s="1">
+        <v>-1.081885695E7</v>
+      </c>
+    </row>
+    <row r="1839" spans="1:9" ht="12.75">
+      <c r="A1839" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1839" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1839" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1839" t="s">
+        <v>294</v>
+      </c>
+      <c r="E1839" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1839" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1839" s="1">
+        <v>1758542.24</v>
+      </c>
+      <c r="H1839" s="1">
+        <v>1164129.74</v>
+      </c>
+      <c r="I1839" s="1">
+        <v>594412.50</v>
+      </c>
+    </row>
+    <row r="1840" spans="1:9" ht="12.75">
+      <c r="A1840" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1840" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1840" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1840" t="s">
+        <v>369</v>
+      </c>
+      <c r="E1840" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1840" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1840" s="1">
+        <v>18462722</v>
+      </c>
+      <c r="H1840" s="1">
+        <v>2.376985961E7</v>
+      </c>
+      <c r="I1840" s="1">
+        <v>-5307137.609999999</v>
+      </c>
+    </row>
+    <row r="1841" spans="1:9" ht="12.75">
+      <c r="A1841" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1841" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1841" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1841" t="s">
+        <v>297</v>
+      </c>
+      <c r="E1841" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1841" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1841" s="1">
+        <v>3.3116095990000004E8</v>
+      </c>
+      <c r="H1841" s="1">
+        <v>3.311609599E8</v>
+      </c>
+      <c r="I1841" s="1">
+        <v>5.9604644775390625E-8</v>
+      </c>
+    </row>
+    <row r="1842" spans="1:9" ht="12.75">
+      <c r="A1842" t="s">
+        <v>313</v>
+      </c>
+      <c r="B1842" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1842" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1842" t="s">
+        <v>298</v>
+      </c>
+      <c r="E1842" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1842" s="1">
+        <v>0</v>
+      </c>
+      <c r="G1842" s="1">
+        <v>0</v>
+      </c>
+      <c r="H1842" s="1">
+        <v>1.118956866E7</v>
+      </c>
+      <c r="I1842" s="1">
+        <v>-1.118956866E7</v>
+      </c>
+    </row>
+    <row r="1843" spans="1:9" ht="12.75">
+      <c r="A1843" t="s">
+        <v>370</v>
+      </c>
+      <c r="B1843" t="s">
+        <v>371</v>
+      </c>
+      <c r="C1843" t="s">
+        <v>371</v>
+      </c>
+      <c r="D1843" t="s">
+        <v>371</v>
+      </c>
+      <c r="E1843" t="s">
+        <v>371</v>
+      </c>
+      <c r="F1843" s="1">
+        <v>5.9604644775390625E-8</v>
+      </c>
+      <c r="G1843" s="1">
+        <v>7.948051563499995E9</v>
+      </c>
+      <c r="H1843" s="1">
         <v>7.948051563500001E9</v>
       </c>
-      <c r="I1837" s="1">
-        <v>-3.155320882797241E-6</v>
+      <c r="I1843" s="1">
+        <v>-2.913177013397217E-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-04-01
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -1601,7 +1601,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7caa9224-b425-455c-8cee-a9b9aec4a241}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{560220c1-3116-4852-aa27-8e4edb1967e0}">
   <dimension ref="A1:I1859"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -1690,7 +1690,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>5.9604644775390625E-8</v>
+        <v>1.4901161193847656E-7</v>
       </c>
       <c r="G3" s="1">
         <v>3.54</v>
@@ -1699,7 +1699,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>5.960464521947983E-8</v>
+        <v>1.4901161238256577E-7</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -1725,10 +1725,10 @@
         <v>3.9890307998E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.611305209900004E8</v>
+        <v>3.6113052099000067E8</v>
       </c>
       <c r="I4" s="1">
-        <v>1.696753108599996E8</v>
+        <v>1.6967531085999936E8</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -1841,10 +1841,10 @@
         <v>5.83186561E8</v>
       </c>
       <c r="H8" s="1">
-        <v>2.947547559799999E8</v>
+        <v>2.9475475598E8</v>
       </c>
       <c r="I8" s="1">
-        <v>2.884318050200001E8</v>
+        <v>2.8843180502E8</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="12.75">
@@ -3871,10 +3871,10 @@
         <v>4.8207301830000006E7</v>
       </c>
       <c r="H78" s="1">
-        <v>4.8063201199999996E7</v>
+        <v>4.806320120000003E7</v>
       </c>
       <c r="I78" s="1">
-        <v>1062806.6300000101</v>
+        <v>1062806.6299999729</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="12.75">
@@ -6130,13 +6130,13 @@
         <v>0</v>
       </c>
       <c r="G156" s="1">
-        <v>1.9072333009999998E7</v>
+        <v>1.907233301E7</v>
       </c>
       <c r="H156" s="1">
         <v>18680110</v>
       </c>
       <c r="I156" s="1">
-        <v>392223.0099999979</v>
+        <v>392223.01000000164</v>
       </c>
     </row>
     <row r="157" spans="1:9" ht="12.75">
@@ -18600,13 +18600,13 @@
         <v>0</v>
       </c>
       <c r="G586" s="1">
-        <v>1134248.0099999998</v>
+        <v>1134248.01</v>
       </c>
       <c r="H586" s="1">
         <v>0</v>
       </c>
       <c r="I586" s="1">
-        <v>1134248.0099999998</v>
+        <v>1134248.01</v>
       </c>
     </row>
     <row r="587" spans="1:9" ht="12.75">
@@ -18832,13 +18832,13 @@
         <v>0</v>
       </c>
       <c r="G594" s="1">
-        <v>154978.47</v>
+        <v>154978.47000000003</v>
       </c>
       <c r="H594" s="1">
         <v>0</v>
       </c>
       <c r="I594" s="1">
-        <v>154978.47</v>
+        <v>154978.47000000003</v>
       </c>
     </row>
     <row r="595" spans="1:9" ht="12.75">
@@ -19180,13 +19180,13 @@
         <v>0</v>
       </c>
       <c r="G606" s="1">
-        <v>1022249.5499999999</v>
+        <v>1022249.55</v>
       </c>
       <c r="H606" s="1">
         <v>0</v>
       </c>
       <c r="I606" s="1">
-        <v>1022249.5499999999</v>
+        <v>1022249.55</v>
       </c>
     </row>
     <row r="607" spans="1:9" ht="12.75">
@@ -19731,13 +19731,13 @@
         <v>0</v>
       </c>
       <c r="G625" s="1">
-        <v>635480.0199999999</v>
+        <v>635480.02</v>
       </c>
       <c r="H625" s="1">
         <v>0</v>
       </c>
       <c r="I625" s="1">
-        <v>635480.0199999999</v>
+        <v>635480.02</v>
       </c>
     </row>
     <row r="626" spans="1:9" ht="12.75">
@@ -19760,13 +19760,13 @@
         <v>0</v>
       </c>
       <c r="G626" s="1">
-        <v>584250.4599999998</v>
+        <v>584250.46</v>
       </c>
       <c r="H626" s="1">
         <v>0</v>
       </c>
       <c r="I626" s="1">
-        <v>584250.4599999998</v>
+        <v>584250.46</v>
       </c>
     </row>
     <row r="627" spans="1:9" ht="12.75">
@@ -19789,13 +19789,13 @@
         <v>0</v>
       </c>
       <c r="G627" s="1">
-        <v>3041021.889999999</v>
+        <v>3041021.8900000006</v>
       </c>
       <c r="H627" s="1">
         <v>23236.93</v>
       </c>
       <c r="I627" s="1">
-        <v>3017784.959999999</v>
+        <v>3017784.9600000004</v>
       </c>
     </row>
     <row r="628" spans="1:9" ht="12.75">
@@ -19818,13 +19818,13 @@
         <v>0</v>
       </c>
       <c r="G628" s="1">
-        <v>1404331.32</v>
+        <v>1404331.3199999998</v>
       </c>
       <c r="H628" s="1">
         <v>0</v>
       </c>
       <c r="I628" s="1">
-        <v>1404331.32</v>
+        <v>1404331.3199999998</v>
       </c>
     </row>
     <row r="629" spans="1:9" ht="12.75">
@@ -19847,13 +19847,13 @@
         <v>0</v>
       </c>
       <c r="G629" s="1">
-        <v>3337176.3999999994</v>
+        <v>3337176.400000001</v>
       </c>
       <c r="H629" s="1">
         <v>9049.23</v>
       </c>
       <c r="I629" s="1">
-        <v>3328127.1699999995</v>
+        <v>3328127.170000001</v>
       </c>
     </row>
     <row r="630" spans="1:9" ht="12.75">
@@ -20108,13 +20108,13 @@
         <v>0</v>
       </c>
       <c r="G638" s="1">
-        <v>287725.66</v>
+        <v>287725.66000000003</v>
       </c>
       <c r="H638" s="1">
         <v>0</v>
       </c>
       <c r="I638" s="1">
-        <v>287725.66</v>
+        <v>287725.66000000003</v>
       </c>
     </row>
     <row r="639" spans="1:9" ht="12.75">
@@ -20166,13 +20166,13 @@
         <v>0</v>
       </c>
       <c r="G640" s="1">
-        <v>555001.2400000001</v>
+        <v>555001.24</v>
       </c>
       <c r="H640" s="1">
         <v>0</v>
       </c>
       <c r="I640" s="1">
-        <v>555001.2400000001</v>
+        <v>555001.24</v>
       </c>
     </row>
     <row r="641" spans="1:9" ht="12.75">
@@ -20253,13 +20253,13 @@
         <v>0</v>
       </c>
       <c r="G643" s="1">
-        <v>964873.7399999998</v>
+        <v>964873.74</v>
       </c>
       <c r="H643" s="1">
         <v>0</v>
       </c>
       <c r="I643" s="1">
-        <v>964873.7399999998</v>
+        <v>964873.74</v>
       </c>
     </row>
     <row r="644" spans="1:9" ht="12.75">
@@ -20369,13 +20369,13 @@
         <v>0</v>
       </c>
       <c r="G647" s="1">
-        <v>744682.80</v>
+        <v>744682.7999999999</v>
       </c>
       <c r="H647" s="1">
         <v>0</v>
       </c>
       <c r="I647" s="1">
-        <v>744682.80</v>
+        <v>744682.7999999999</v>
       </c>
     </row>
     <row r="648" spans="1:9" ht="12.75">
@@ -20398,13 +20398,13 @@
         <v>0</v>
       </c>
       <c r="G648" s="1">
-        <v>544075.9999999998</v>
+        <v>544076</v>
       </c>
       <c r="H648" s="1">
         <v>0</v>
       </c>
       <c r="I648" s="1">
-        <v>544075.9999999998</v>
+        <v>544076</v>
       </c>
     </row>
     <row r="649" spans="1:9" ht="12.75">
@@ -20456,13 +20456,13 @@
         <v>0</v>
       </c>
       <c r="G650" s="1">
-        <v>416845.93999999994</v>
+        <v>416845.94000000006</v>
       </c>
       <c r="H650" s="1">
         <v>0</v>
       </c>
       <c r="I650" s="1">
-        <v>416845.93999999994</v>
+        <v>416845.94000000006</v>
       </c>
     </row>
     <row r="651" spans="1:9" ht="12.75">
@@ -20659,13 +20659,13 @@
         <v>0</v>
       </c>
       <c r="G657" s="1">
-        <v>341636.4099999999</v>
+        <v>341636.41</v>
       </c>
       <c r="H657" s="1">
         <v>0</v>
       </c>
       <c r="I657" s="1">
-        <v>341636.4099999999</v>
+        <v>341636.41</v>
       </c>
     </row>
     <row r="658" spans="1:9" ht="12.75">
@@ -20833,13 +20833,13 @@
         <v>0</v>
       </c>
       <c r="G663" s="1">
-        <v>2292091.5599999996</v>
+        <v>2292091.56</v>
       </c>
       <c r="H663" s="1">
         <v>0</v>
       </c>
       <c r="I663" s="1">
-        <v>2292091.5599999996</v>
+        <v>2292091.56</v>
       </c>
     </row>
     <row r="664" spans="1:9" ht="12.75">
@@ -22109,13 +22109,13 @@
         <v>0</v>
       </c>
       <c r="G707" s="1">
-        <v>2568009.0999999996</v>
+        <v>2568009.10</v>
       </c>
       <c r="H707" s="1">
         <v>0</v>
       </c>
       <c r="I707" s="1">
-        <v>2568009.0999999996</v>
+        <v>2568009.10</v>
       </c>
     </row>
     <row r="708" spans="1:9" ht="12.75">
@@ -22254,13 +22254,13 @@
         <v>0</v>
       </c>
       <c r="G712" s="1">
-        <v>4420392.420000001</v>
+        <v>4420392.42</v>
       </c>
       <c r="H712" s="1">
         <v>0</v>
       </c>
       <c r="I712" s="1">
-        <v>4420392.420000001</v>
+        <v>4420392.42</v>
       </c>
     </row>
     <row r="713" spans="1:9" ht="12.75">
@@ -23127,10 +23127,10 @@
         <v>0</v>
       </c>
       <c r="H742" s="1">
-        <v>7.258656367999999E7</v>
+        <v>7.258656368E7</v>
       </c>
       <c r="I742" s="1">
-        <v>-7.258656367999999E7</v>
+        <v>-7.258656368E7</v>
       </c>
     </row>
     <row r="743" spans="1:9" ht="12.75">
@@ -40727,13 +40727,13 @@
         <v>0</v>
       </c>
       <c r="G1349" s="1">
-        <v>3.3413358650000002E7</v>
+        <v>3.341335865E7</v>
       </c>
       <c r="H1349" s="1">
         <v>179327</v>
       </c>
       <c r="I1349" s="1">
-        <v>3.3234031650000002E7</v>
+        <v>3.323403165E7</v>
       </c>
     </row>
     <row r="1350" spans="1:9" ht="12.75">
@@ -41742,13 +41742,13 @@
         <v>0</v>
       </c>
       <c r="G1384" s="1">
-        <v>3.210335585E7</v>
+        <v>3.2103355849999998E7</v>
       </c>
       <c r="H1384" s="1">
         <v>283032</v>
       </c>
       <c r="I1384" s="1">
-        <v>3.182032385E7</v>
+        <v>3.1820323849999998E7</v>
       </c>
     </row>
     <row r="1385" spans="1:9" ht="12.75">
@@ -42032,13 +42032,13 @@
         <v>0</v>
       </c>
       <c r="G1394" s="1">
-        <v>6689781.3</v>
+        <v>6689781.300000001</v>
       </c>
       <c r="H1394" s="1">
         <v>34552</v>
       </c>
       <c r="I1394" s="1">
-        <v>6655229.3</v>
+        <v>6655229.300000001</v>
       </c>
     </row>
     <row r="1395" spans="1:9" ht="12.75">
@@ -42293,13 +42293,13 @@
         <v>0</v>
       </c>
       <c r="G1403" s="1">
-        <v>1.884446755E7</v>
+        <v>1.8844467549999997E7</v>
       </c>
       <c r="H1403" s="1">
         <v>110222</v>
       </c>
       <c r="I1403" s="1">
-        <v>1.873424555E7</v>
+        <v>1.8734245549999997E7</v>
       </c>
     </row>
     <row r="1404" spans="1:9" ht="12.75">
@@ -42409,13 +42409,13 @@
         <v>0</v>
       </c>
       <c r="G1407" s="1">
-        <v>4507476.45</v>
+        <v>4507476.449999999</v>
       </c>
       <c r="H1407" s="1">
         <v>0</v>
       </c>
       <c r="I1407" s="1">
-        <v>4507476.45</v>
+        <v>4507476.449999999</v>
       </c>
     </row>
     <row r="1408" spans="1:9" ht="12.75">
@@ -44207,13 +44207,13 @@
         <v>0</v>
       </c>
       <c r="G1469" s="1">
-        <v>2104980.3200000003</v>
+        <v>2104980.32</v>
       </c>
       <c r="H1469" s="1">
         <v>0</v>
       </c>
       <c r="I1469" s="1">
-        <v>2104980.3200000003</v>
+        <v>2104980.32</v>
       </c>
     </row>
     <row r="1470" spans="1:9" ht="12.75">
@@ -45393,16 +45393,16 @@
         <v>13</v>
       </c>
       <c r="F1510" s="1">
-        <v>-19347197</v>
+        <v>-1.934719700000024E7</v>
       </c>
       <c r="G1510" s="1">
-        <v>2.3300178275000003E8</v>
+        <v>2.3300178274999985E8</v>
       </c>
       <c r="H1510" s="1">
-        <v>2.2633682455000007E8</v>
+        <v>2.2633682454999992E8</v>
       </c>
       <c r="I1510" s="1">
-        <v>-1.2682238800000042E7</v>
+        <v>-1.268223880000031E7</v>
       </c>
     </row>
     <row r="1511" spans="1:9" ht="12.75">
@@ -45486,10 +45486,10 @@
         <v>2.288005138E7</v>
       </c>
       <c r="H1513" s="1">
-        <v>1.752459138E7</v>
+        <v>1.7524591380000003E7</v>
       </c>
       <c r="I1513" s="1">
-        <v>0</v>
+        <v>-3.725290298461914E-9</v>
       </c>
     </row>
     <row r="1514" spans="1:9" ht="12.75">
@@ -45979,10 +45979,10 @@
         <v>596729.46</v>
       </c>
       <c r="H1530" s="1">
-        <v>710966.37</v>
+        <v>710966.3699999999</v>
       </c>
       <c r="I1530" s="1">
-        <v>-114236.91000000003</v>
+        <v>-114236.90999999992</v>
       </c>
     </row>
     <row r="1531" spans="1:9" ht="12.75">
@@ -46037,10 +46037,10 @@
         <v>7496556.2</v>
       </c>
       <c r="H1532" s="1">
-        <v>9693394.120000001</v>
+        <v>9693394.120000012</v>
       </c>
       <c r="I1532" s="1">
-        <v>-2196837.920000001</v>
+        <v>-2196837.920000012</v>
       </c>
     </row>
     <row r="1533" spans="1:9" ht="12.75">
@@ -46060,16 +46060,16 @@
         <v>13</v>
       </c>
       <c r="F1533" s="1">
-        <v>-56797.00000000093</v>
+        <v>-56797.00000000186</v>
       </c>
       <c r="G1533" s="1">
-        <v>3227421.94</v>
+        <v>3227421.9400000004</v>
       </c>
       <c r="H1533" s="1">
-        <v>3624656.939999996</v>
+        <v>3624656.9399999976</v>
       </c>
       <c r="I1533" s="1">
-        <v>-454031.9999999972</v>
+        <v>-454031.99999999907</v>
       </c>
     </row>
     <row r="1534" spans="1:9" ht="12.75">
@@ -46121,13 +46121,13 @@
         <v>0</v>
       </c>
       <c r="G1535" s="1">
-        <v>1.2159178278899999E9</v>
+        <v>1.21591782789E9</v>
       </c>
       <c r="H1535" s="1">
-        <v>1.2159178278900023E9</v>
+        <v>1.2159178278899996E9</v>
       </c>
       <c r="I1535" s="1">
-        <v>-2.384185791015625E-6</v>
+        <v>4.76837158203125E-7</v>
       </c>
     </row>
     <row r="1536" spans="1:9" ht="12.75">
@@ -46153,10 +46153,10 @@
         <v>34390731</v>
       </c>
       <c r="H1536" s="1">
-        <v>3.397778215E7</v>
+        <v>3.3977782150000006E7</v>
       </c>
       <c r="I1536" s="1">
-        <v>-1292467.1499999985</v>
+        <v>-1292467.150000006</v>
       </c>
     </row>
     <row r="1537" spans="1:9" ht="12.75">
@@ -47052,10 +47052,10 @@
         <v>9.562248610000001E7</v>
       </c>
       <c r="H1567" s="1">
-        <v>8.89163377E7</v>
+        <v>8.891633769999999E7</v>
       </c>
       <c r="I1567" s="1">
-        <v>3.58998573E7</v>
+        <v>3.589985730000001E7</v>
       </c>
     </row>
     <row r="1568" spans="1:9" ht="12.75">
@@ -47139,10 +47139,10 @@
         <v>8.56662631E8</v>
       </c>
       <c r="H1570" s="1">
-        <v>8.56662631E8</v>
+        <v>8.566626309999999E8</v>
       </c>
       <c r="I1570" s="1">
-        <v>0</v>
+        <v>1.1920928955078125E-7</v>
       </c>
     </row>
     <row r="1571" spans="1:9" ht="12.75">
@@ -49137,13 +49137,13 @@
         <v>0</v>
       </c>
       <c r="G1639" s="1">
-        <v>1957807.57</v>
+        <v>1957807.5700000003</v>
       </c>
       <c r="H1639" s="1">
         <v>0</v>
       </c>
       <c r="I1639" s="1">
-        <v>1957807.57</v>
+        <v>1957807.5700000003</v>
       </c>
     </row>
     <row r="1640" spans="1:9" ht="12.75">
@@ -51199,10 +51199,10 @@
         <v>3734639.2299999995</v>
       </c>
       <c r="H1710" s="1">
-        <v>3776932.53</v>
+        <v>3776932.5300000003</v>
       </c>
       <c r="I1710" s="1">
-        <v>-42293.30000000028</v>
+        <v>-42293.300000000745</v>
       </c>
     </row>
     <row r="1711" spans="1:9" ht="12.75">
@@ -51254,13 +51254,13 @@
         <v>0</v>
       </c>
       <c r="G1712" s="1">
-        <v>307784.22000000003</v>
+        <v>307784.22</v>
       </c>
       <c r="H1712" s="1">
         <v>0</v>
       </c>
       <c r="I1712" s="1">
-        <v>307784.22000000003</v>
+        <v>307784.22</v>
       </c>
     </row>
     <row r="1713" spans="1:9" ht="12.75">
@@ -51312,10 +51312,10 @@
         <v>0</v>
       </c>
       <c r="G1714" s="1">
-        <v>685737.6099999999</v>
+        <v>685737.61</v>
       </c>
       <c r="H1714" s="1">
-        <v>709966.5099999999</v>
+        <v>709966.51</v>
       </c>
       <c r="I1714" s="1">
         <v>-24228.900000000023</v>
@@ -51370,13 +51370,13 @@
         <v>0</v>
       </c>
       <c r="G1716" s="1">
-        <v>191355.02000000002</v>
+        <v>191355.02</v>
       </c>
       <c r="H1716" s="1">
         <v>110022.99999999999</v>
       </c>
       <c r="I1716" s="1">
-        <v>81332.02000000003</v>
+        <v>81332.02</v>
       </c>
     </row>
     <row r="1717" spans="1:9" ht="12.75">
@@ -51399,13 +51399,13 @@
         <v>0</v>
       </c>
       <c r="G1717" s="1">
-        <v>456691.31999999995</v>
+        <v>456691.32</v>
       </c>
       <c r="H1717" s="1">
         <v>0</v>
       </c>
       <c r="I1717" s="1">
-        <v>456691.31999999995</v>
+        <v>456691.32</v>
       </c>
     </row>
     <row r="1718" spans="1:9" ht="12.75">
@@ -54096,13 +54096,13 @@
         <v>0</v>
       </c>
       <c r="G1810" s="1">
-        <v>4138525.55</v>
+        <v>4138525.5500000003</v>
       </c>
       <c r="H1810" s="1">
         <v>0</v>
       </c>
       <c r="I1810" s="1">
-        <v>4138525.55</v>
+        <v>4138525.5500000003</v>
       </c>
     </row>
     <row r="1811" spans="1:9" ht="12.75">
@@ -54386,13 +54386,13 @@
         <v>0</v>
       </c>
       <c r="G1820" s="1">
-        <v>3.06585572E7</v>
+        <v>3.0658557200000003E7</v>
       </c>
       <c r="H1820" s="1">
         <v>0</v>
       </c>
       <c r="I1820" s="1">
-        <v>3.06585572E7</v>
+        <v>3.0658557200000003E7</v>
       </c>
     </row>
     <row r="1821" spans="1:9" ht="12.75">
@@ -54995,13 +54995,13 @@
         <v>-5418882</v>
       </c>
       <c r="G1841" s="1">
-        <v>4.6276280172E8</v>
+        <v>4.6276280171999997E8</v>
       </c>
       <c r="H1841" s="1">
         <v>4.6301141603E8</v>
       </c>
       <c r="I1841" s="1">
-        <v>-5667496.309999943</v>
+        <v>-5667496.310000002</v>
       </c>
     </row>
     <row r="1842" spans="1:9" ht="12.75">
@@ -55346,10 +55346,10 @@
         <v>505065</v>
       </c>
       <c r="H1853" s="1">
-        <v>504838.89999999997</v>
+        <v>504838.90</v>
       </c>
       <c r="I1853" s="1">
-        <v>226.10000000003492</v>
+        <v>226.09999999997672</v>
       </c>
     </row>
     <row r="1854" spans="1:9" ht="12.75">
@@ -55404,10 +55404,10 @@
         <v>1758542.24</v>
       </c>
       <c r="H1855" s="1">
-        <v>1164129.6900000002</v>
+        <v>1164129.69</v>
       </c>
       <c r="I1855" s="1">
-        <v>594412.5499999998</v>
+        <v>594412.55</v>
       </c>
     </row>
     <row r="1856" spans="1:9" ht="12.75">
@@ -55462,10 +55462,10 @@
         <v>3.313550968999999E8</v>
       </c>
       <c r="H1857" s="1">
-        <v>3.3135509690000004E8</v>
+        <v>3.313550969000001E8</v>
       </c>
       <c r="I1857" s="1">
-        <v>-1.1920928955078125E-7</v>
+        <v>-1.7881393432617188E-7</v>
       </c>
     </row>
     <row r="1858" spans="1:9" ht="12.75">
@@ -55514,16 +55514,16 @@
         <v>379</v>
       </c>
       <c r="F1859" s="1">
-        <v>1.1920928955078125E-7</v>
+        <v>0</v>
       </c>
       <c r="G1859" s="1">
         <v>8.5176262581799965E9</v>
       </c>
       <c r="H1859" s="1">
-        <v>8.517626258180002E9</v>
+        <v>8.51762625818E9</v>
       </c>
       <c r="I1859" s="1">
-        <v>-3.38628888130188E-6</v>
+        <v>-1.1790543794631958E-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-04-04
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -1607,7 +1607,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{c18e03f5-082a-4d37-9b5e-5b89521089d7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{fb6a5285-21ed-4910-81b7-8b1ba85be485}">
   <dimension ref="A1:I1864"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -1696,7 +1696,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>8.940696716308594E-8</v>
+        <v>1.1920928955078125E-7</v>
       </c>
       <c r="G3" s="1">
         <v>3.54</v>
@@ -1705,7 +1705,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>8.940696760717515E-8</v>
+        <v>1.1920928999487046E-7</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -1731,10 +1731,10 @@
         <v>3.9937306298E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.828903106500006E8</v>
+        <v>3.828903106500005E8</v>
       </c>
       <c r="I4" s="1">
-        <v>1.4838550419999945E8</v>
+        <v>1.483855041999995E8</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -1847,10 +1847,10 @@
         <v>5.856383294E8</v>
       </c>
       <c r="H8" s="1">
-        <v>2.958804599799999E8</v>
+        <v>2.9588045998E8</v>
       </c>
       <c r="I8" s="1">
-        <v>2.897578694200001E8</v>
+        <v>2.8975786941999996E8</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="12.75">
@@ -3906,10 +3906,10 @@
         <v>4.841186783000001E7</v>
       </c>
       <c r="H79" s="1">
-        <v>4.80975932E7</v>
+        <v>4.809759320000002E7</v>
       </c>
       <c r="I79" s="1">
-        <v>1232980.6300000101</v>
+        <v>1232980.6299999952</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="12.75">
@@ -6165,13 +6165,13 @@
         <v>0</v>
       </c>
       <c r="G157" s="1">
-        <v>1.9072333009999998E7</v>
+        <v>1.907233301E7</v>
       </c>
       <c r="H157" s="1">
         <v>18680110</v>
       </c>
       <c r="I157" s="1">
-        <v>392223.0099999979</v>
+        <v>392223.01000000164</v>
       </c>
     </row>
     <row r="158" spans="1:9" ht="12.75">
@@ -18635,13 +18635,13 @@
         <v>0</v>
       </c>
       <c r="G587" s="1">
-        <v>1134248.01</v>
+        <v>1134248.0099999998</v>
       </c>
       <c r="H587" s="1">
         <v>0</v>
       </c>
       <c r="I587" s="1">
-        <v>1134248.01</v>
+        <v>1134248.0099999998</v>
       </c>
     </row>
     <row r="588" spans="1:9" ht="12.75">
@@ -19766,13 +19766,13 @@
         <v>0</v>
       </c>
       <c r="G626" s="1">
-        <v>635480.0199999999</v>
+        <v>635480.02</v>
       </c>
       <c r="H626" s="1">
         <v>0</v>
       </c>
       <c r="I626" s="1">
-        <v>635480.0199999999</v>
+        <v>635480.02</v>
       </c>
     </row>
     <row r="627" spans="1:9" ht="12.75">
@@ -19824,13 +19824,13 @@
         <v>0</v>
       </c>
       <c r="G628" s="1">
-        <v>3041021.889999999</v>
+        <v>3041021.8899999997</v>
       </c>
       <c r="H628" s="1">
         <v>23236.93</v>
       </c>
       <c r="I628" s="1">
-        <v>3017784.959999999</v>
+        <v>3017784.9599999995</v>
       </c>
     </row>
     <row r="629" spans="1:9" ht="12.75">
@@ -20607,13 +20607,13 @@
         <v>0</v>
       </c>
       <c r="G655" s="1">
-        <v>2189217.48</v>
+        <v>2189217.4799999995</v>
       </c>
       <c r="H655" s="1">
         <v>13850.19</v>
       </c>
       <c r="I655" s="1">
-        <v>2175367.29</v>
+        <v>2175367.2899999996</v>
       </c>
     </row>
     <row r="656" spans="1:9" ht="12.75">
@@ -40588,13 +40588,13 @@
         <v>0</v>
       </c>
       <c r="G1344" s="1">
-        <v>1.23715218E7</v>
+        <v>1.2371521799999999E7</v>
       </c>
       <c r="H1344" s="1">
         <v>0</v>
       </c>
       <c r="I1344" s="1">
-        <v>1.23715218E7</v>
+        <v>1.2371521799999999E7</v>
       </c>
     </row>
     <row r="1345" spans="1:9" ht="12.75">
@@ -40791,13 +40791,13 @@
         <v>0</v>
       </c>
       <c r="G1351" s="1">
-        <v>3.341335865E7</v>
+        <v>3.3413358650000002E7</v>
       </c>
       <c r="H1351" s="1">
         <v>179327</v>
       </c>
       <c r="I1351" s="1">
-        <v>3.323403165E7</v>
+        <v>3.3234031650000002E7</v>
       </c>
     </row>
     <row r="1352" spans="1:9" ht="12.75">
@@ -41806,13 +41806,13 @@
         <v>0</v>
       </c>
       <c r="G1386" s="1">
-        <v>3.210335585E7</v>
+        <v>3.2103355849999998E7</v>
       </c>
       <c r="H1386" s="1">
         <v>283032</v>
       </c>
       <c r="I1386" s="1">
-        <v>3.182032385E7</v>
+        <v>3.1820323849999998E7</v>
       </c>
     </row>
     <row r="1387" spans="1:9" ht="12.75">
@@ -42096,13 +42096,13 @@
         <v>0</v>
       </c>
       <c r="G1396" s="1">
-        <v>6689781.300000001</v>
+        <v>6689781.3</v>
       </c>
       <c r="H1396" s="1">
         <v>34552</v>
       </c>
       <c r="I1396" s="1">
-        <v>6655229.300000001</v>
+        <v>6655229.3</v>
       </c>
     </row>
     <row r="1397" spans="1:9" ht="12.75">
@@ -42357,13 +42357,13 @@
         <v>0</v>
       </c>
       <c r="G1405" s="1">
-        <v>1.884446755E7</v>
+        <v>1.8844467549999997E7</v>
       </c>
       <c r="H1405" s="1">
         <v>110222</v>
       </c>
       <c r="I1405" s="1">
-        <v>1.873424555E7</v>
+        <v>1.8734245549999997E7</v>
       </c>
     </row>
     <row r="1406" spans="1:9" ht="12.75">
@@ -42589,13 +42589,13 @@
         <v>0</v>
       </c>
       <c r="G1413" s="1">
-        <v>2.443130324E7</v>
+        <v>2.4431303240000002E7</v>
       </c>
       <c r="H1413" s="1">
         <v>168699</v>
       </c>
       <c r="I1413" s="1">
-        <v>2.426260424E7</v>
+        <v>2.4262604240000002E7</v>
       </c>
     </row>
     <row r="1414" spans="1:9" ht="12.75">
@@ -42618,13 +42618,13 @@
         <v>0</v>
       </c>
       <c r="G1414" s="1">
-        <v>3242649.65</v>
+        <v>3242649.6500000004</v>
       </c>
       <c r="H1414" s="1">
         <v>0</v>
       </c>
       <c r="I1414" s="1">
-        <v>3242649.65</v>
+        <v>3242649.6500000004</v>
       </c>
     </row>
     <row r="1415" spans="1:9" ht="12.75">
@@ -42705,13 +42705,13 @@
         <v>0</v>
       </c>
       <c r="G1417" s="1">
-        <v>3088025.3000000003</v>
+        <v>3088025.30</v>
       </c>
       <c r="H1417" s="1">
         <v>0</v>
       </c>
       <c r="I1417" s="1">
-        <v>3088025.3000000003</v>
+        <v>3088025.30</v>
       </c>
     </row>
     <row r="1418" spans="1:9" ht="12.75">
@@ -45457,16 +45457,16 @@
         <v>13</v>
       </c>
       <c r="F1512" s="1">
-        <v>-19347197</v>
+        <v>-1.934719700000006E7</v>
       </c>
       <c r="G1512" s="1">
-        <v>2.3813537074999997E8</v>
+        <v>2.3813537075000006E8</v>
       </c>
       <c r="H1512" s="1">
         <v>2.263767387500001E8</v>
       </c>
       <c r="I1512" s="1">
-        <v>-7588565.000000119</v>
+        <v>-7588565.000000089</v>
       </c>
     </row>
     <row r="1513" spans="1:9" ht="12.75">
@@ -46043,10 +46043,10 @@
         <v>768503.4599999998</v>
       </c>
       <c r="H1532" s="1">
-        <v>710966.3700000002</v>
+        <v>710966.3699999999</v>
       </c>
       <c r="I1532" s="1">
-        <v>57537.08999999962</v>
+        <v>57537.08999999997</v>
       </c>
     </row>
     <row r="1533" spans="1:9" ht="12.75">
@@ -46124,7 +46124,7 @@
         <v>13</v>
       </c>
       <c r="F1535" s="1">
-        <v>-56797.00000000186</v>
+        <v>-56797.000000002794</v>
       </c>
       <c r="G1535" s="1">
         <v>3227421.94</v>
@@ -46133,7 +46133,7 @@
         <v>3624656.9399999967</v>
       </c>
       <c r="I1535" s="1">
-        <v>-454031.9999999986</v>
+        <v>-454031.99999999953</v>
       </c>
     </row>
     <row r="1536" spans="1:9" ht="12.75">
@@ -46185,13 +46185,13 @@
         <v>0</v>
       </c>
       <c r="G1537" s="1">
-        <v>1.2159178315499997E9</v>
+        <v>1.21591783155E9</v>
       </c>
       <c r="H1537" s="1">
-        <v>1.215917831550002E9</v>
+        <v>1.2159178315500016E9</v>
       </c>
       <c r="I1537" s="1">
-        <v>-2.384185791015625E-6</v>
+        <v>-1.6689300537109375E-6</v>
       </c>
     </row>
     <row r="1538" spans="1:9" ht="12.75">
@@ -46217,10 +46217,10 @@
         <v>34390731</v>
       </c>
       <c r="H1538" s="1">
-        <v>3.397778215E7</v>
+        <v>3.3977782150000006E7</v>
       </c>
       <c r="I1538" s="1">
-        <v>-1292467.1499999985</v>
+        <v>-1292467.150000006</v>
       </c>
     </row>
     <row r="1539" spans="1:9" ht="12.75">
@@ -47116,10 +47116,10 @@
         <v>9.666654010000001E7</v>
       </c>
       <c r="H1569" s="1">
-        <v>8.634201063999999E7</v>
+        <v>8.634201064E7</v>
       </c>
       <c r="I1569" s="1">
-        <v>3.9518238360000014E7</v>
+        <v>3.951823836E7</v>
       </c>
     </row>
     <row r="1570" spans="1:9" ht="12.75">
@@ -47754,10 +47754,10 @@
         <v>2.3235801356E8</v>
       </c>
       <c r="H1591" s="1">
-        <v>2.0116685636E8</v>
+        <v>2.0116685635999998E8</v>
       </c>
       <c r="I1591" s="1">
-        <v>3.1191157199999988E7</v>
+        <v>3.1191157200000018E7</v>
       </c>
     </row>
     <row r="1592" spans="1:9" ht="12.75">
@@ -51263,10 +51263,10 @@
         <v>3734639.2300000004</v>
       </c>
       <c r="H1712" s="1">
-        <v>3776932.5300000003</v>
+        <v>3776932.5300000007</v>
       </c>
       <c r="I1712" s="1">
-        <v>-42293.299999999814</v>
+        <v>-42293.30000000028</v>
       </c>
     </row>
     <row r="1713" spans="1:9" ht="12.75">
@@ -51521,13 +51521,13 @@
         <v>0</v>
       </c>
       <c r="G1721" s="1">
-        <v>1406462.61</v>
+        <v>1406462.6099999999</v>
       </c>
       <c r="H1721" s="1">
         <v>234699.50</v>
       </c>
       <c r="I1721" s="1">
-        <v>1171763.11</v>
+        <v>1171763.1099999999</v>
       </c>
     </row>
     <row r="1722" spans="1:9" ht="12.75">
@@ -51553,7 +51553,7 @@
         <v>3389832</v>
       </c>
       <c r="H1722" s="1">
-        <v>44210.100000000006</v>
+        <v>44210.10</v>
       </c>
       <c r="I1722" s="1">
         <v>3345621.90</v>
@@ -55665,7 +55665,7 @@
         <v>381</v>
       </c>
       <c r="F1864" s="1">
-        <v>1.1920928955078125E-7</v>
+        <v>5.9604644775390625E-8</v>
       </c>
       <c r="G1864" s="1">
         <v>8.546960143279996E9</v>
@@ -55674,7 +55674,7 @@
         <v>8.546960143280002E9</v>
       </c>
       <c r="I1864" s="1">
-        <v>-4.0102750062942505E-6</v>
+        <v>-3.0566006898880005E-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Consol TB report update 2026-04-05
</commit_message>
<xml_diff>
--- a/Consol_TB_FY25-26.xlsx
+++ b/Consol_TB_FY25-26.xlsx
@@ -1607,7 +1607,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{fb6a5285-21ed-4910-81b7-8b1ba85be485}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{c8157c8e-9918-4935-bc4a-5bf3c0619830}">
   <dimension ref="A1:I1864"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -1696,7 +1696,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1">
-        <v>1.1920928955078125E-7</v>
+        <v>8.940696716308594E-8</v>
       </c>
       <c r="G3" s="1">
         <v>3.54</v>
@@ -1705,7 +1705,7 @@
         <v>3.5399999999999996</v>
       </c>
       <c r="I3" s="1">
-        <v>1.1920928999487046E-7</v>
+        <v>8.940696760717515E-8</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="12.75">
@@ -1731,10 +1731,10 @@
         <v>3.9937306298E8</v>
       </c>
       <c r="H4" s="1">
-        <v>3.828903106500005E8</v>
+        <v>3.828903106500006E8</v>
       </c>
       <c r="I4" s="1">
-        <v>1.483855041999995E8</v>
+        <v>1.4838550419999945E8</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="12.75">
@@ -3906,10 +3906,10 @@
         <v>4.841186783000001E7</v>
       </c>
       <c r="H79" s="1">
-        <v>4.809759320000002E7</v>
+        <v>4.80975932E7</v>
       </c>
       <c r="I79" s="1">
-        <v>1232980.6299999952</v>
+        <v>1232980.6300000101</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="12.75">
@@ -40588,13 +40588,13 @@
         <v>0</v>
       </c>
       <c r="G1344" s="1">
-        <v>1.2371521799999999E7</v>
+        <v>1.23715218E7</v>
       </c>
       <c r="H1344" s="1">
         <v>0</v>
       </c>
       <c r="I1344" s="1">
-        <v>1.2371521799999999E7</v>
+        <v>1.23715218E7</v>
       </c>
     </row>
     <row r="1345" spans="1:9" ht="12.75">
@@ -40791,13 +40791,13 @@
         <v>0</v>
       </c>
       <c r="G1351" s="1">
-        <v>3.3413358650000002E7</v>
+        <v>3.341335865E7</v>
       </c>
       <c r="H1351" s="1">
         <v>179327</v>
       </c>
       <c r="I1351" s="1">
-        <v>3.3234031650000002E7</v>
+        <v>3.323403165E7</v>
       </c>
     </row>
     <row r="1352" spans="1:9" ht="12.75">
@@ -41806,13 +41806,13 @@
         <v>0</v>
       </c>
       <c r="G1386" s="1">
-        <v>3.2103355849999998E7</v>
+        <v>3.210335585E7</v>
       </c>
       <c r="H1386" s="1">
         <v>283032</v>
       </c>
       <c r="I1386" s="1">
-        <v>3.1820323849999998E7</v>
+        <v>3.182032385E7</v>
       </c>
     </row>
     <row r="1387" spans="1:9" ht="12.75">
@@ -42096,13 +42096,13 @@
         <v>0</v>
       </c>
       <c r="G1396" s="1">
-        <v>6689781.3</v>
+        <v>6689781.300000001</v>
       </c>
       <c r="H1396" s="1">
         <v>34552</v>
       </c>
       <c r="I1396" s="1">
-        <v>6655229.3</v>
+        <v>6655229.300000001</v>
       </c>
     </row>
     <row r="1397" spans="1:9" ht="12.75">
@@ -42386,13 +42386,13 @@
         <v>0</v>
       </c>
       <c r="G1406" s="1">
-        <v>8018272.119999999</v>
+        <v>8018272.12</v>
       </c>
       <c r="H1406" s="1">
         <v>0</v>
       </c>
       <c r="I1406" s="1">
-        <v>8018272.119999999</v>
+        <v>8018272.12</v>
       </c>
     </row>
     <row r="1407" spans="1:9" ht="12.75">
@@ -42473,13 +42473,13 @@
         <v>0</v>
       </c>
       <c r="G1409" s="1">
-        <v>4507476.45</v>
+        <v>4507476.449999999</v>
       </c>
       <c r="H1409" s="1">
         <v>0</v>
       </c>
       <c r="I1409" s="1">
-        <v>4507476.45</v>
+        <v>4507476.449999999</v>
       </c>
     </row>
     <row r="1410" spans="1:9" ht="12.75">
@@ -42589,13 +42589,13 @@
         <v>0</v>
       </c>
       <c r="G1413" s="1">
-        <v>2.4431303240000002E7</v>
+        <v>2.443130324E7</v>
       </c>
       <c r="H1413" s="1">
         <v>168699</v>
       </c>
       <c r="I1413" s="1">
-        <v>2.4262604240000002E7</v>
+        <v>2.426260424E7</v>
       </c>
     </row>
     <row r="1414" spans="1:9" ht="12.75">
@@ -42618,13 +42618,13 @@
         <v>0</v>
       </c>
       <c r="G1414" s="1">
-        <v>3242649.6500000004</v>
+        <v>3242649.65</v>
       </c>
       <c r="H1414" s="1">
         <v>0</v>
       </c>
       <c r="I1414" s="1">
-        <v>3242649.6500000004</v>
+        <v>3242649.65</v>
       </c>
     </row>
     <row r="1415" spans="1:9" ht="12.75">
@@ -42705,13 +42705,13 @@
         <v>0</v>
       </c>
       <c r="G1417" s="1">
-        <v>3088025.30</v>
+        <v>3088025.3000000003</v>
       </c>
       <c r="H1417" s="1">
         <v>0</v>
       </c>
       <c r="I1417" s="1">
-        <v>3088025.30</v>
+        <v>3088025.3000000003</v>
       </c>
     </row>
     <row r="1418" spans="1:9" ht="12.75">
@@ -45457,16 +45457,16 @@
         <v>13</v>
       </c>
       <c r="F1512" s="1">
-        <v>-1.934719700000006E7</v>
+        <v>-19347197</v>
       </c>
       <c r="G1512" s="1">
-        <v>2.3813537075000006E8</v>
+        <v>2.3813537074999997E8</v>
       </c>
       <c r="H1512" s="1">
         <v>2.263767387500001E8</v>
       </c>
       <c r="I1512" s="1">
-        <v>-7588565.000000089</v>
+        <v>-7588565.000000119</v>
       </c>
     </row>
     <row r="1513" spans="1:9" ht="12.75">
@@ -46043,10 +46043,10 @@
         <v>768503.4599999998</v>
       </c>
       <c r="H1532" s="1">
-        <v>710966.3699999999</v>
+        <v>710966.3700000002</v>
       </c>
       <c r="I1532" s="1">
-        <v>57537.08999999997</v>
+        <v>57537.08999999962</v>
       </c>
     </row>
     <row r="1533" spans="1:9" ht="12.75">
@@ -46124,7 +46124,7 @@
         <v>13</v>
       </c>
       <c r="F1535" s="1">
-        <v>-56797.000000002794</v>
+        <v>-56797.00000000186</v>
       </c>
       <c r="G1535" s="1">
         <v>3227421.94</v>
@@ -46133,7 +46133,7 @@
         <v>3624656.9399999967</v>
       </c>
       <c r="I1535" s="1">
-        <v>-454031.99999999953</v>
+        <v>-454031.9999999986</v>
       </c>
     </row>
     <row r="1536" spans="1:9" ht="12.75">
@@ -46185,13 +46185,13 @@
         <v>0</v>
       </c>
       <c r="G1537" s="1">
-        <v>1.21591783155E9</v>
+        <v>1.2159178315499997E9</v>
       </c>
       <c r="H1537" s="1">
-        <v>1.2159178315500016E9</v>
+        <v>1.2159178315500019E9</v>
       </c>
       <c r="I1537" s="1">
-        <v>-1.6689300537109375E-6</v>
+        <v>-2.1457672119140625E-6</v>
       </c>
     </row>
     <row r="1538" spans="1:9" ht="12.75">
@@ -47113,13 +47113,13 @@
         <v>2.91937089E7</v>
       </c>
       <c r="G1569" s="1">
-        <v>9.666654010000001E7</v>
+        <v>9.66665401E7</v>
       </c>
       <c r="H1569" s="1">
-        <v>8.634201064E7</v>
+        <v>8.634201063999999E7</v>
       </c>
       <c r="I1569" s="1">
-        <v>3.951823836E7</v>
+        <v>3.9518238360000014E7</v>
       </c>
     </row>
     <row r="1570" spans="1:9" ht="12.75">
@@ -47754,10 +47754,10 @@
         <v>2.3235801356E8</v>
       </c>
       <c r="H1591" s="1">
-        <v>2.0116685635999998E8</v>
+        <v>2.0116685636E8</v>
       </c>
       <c r="I1591" s="1">
-        <v>3.1191157200000018E7</v>
+        <v>3.1191157199999988E7</v>
       </c>
     </row>
     <row r="1592" spans="1:9" ht="12.75">
@@ -49230,13 +49230,13 @@
         <v>0</v>
       </c>
       <c r="G1642" s="1">
-        <v>307964.57</v>
+        <v>307964.56999999995</v>
       </c>
       <c r="H1642" s="1">
         <v>0</v>
       </c>
       <c r="I1642" s="1">
-        <v>307964.57</v>
+        <v>307964.56999999995</v>
       </c>
     </row>
     <row r="1643" spans="1:9" ht="12.75">
@@ -49926,13 +49926,13 @@
         <v>0</v>
       </c>
       <c r="G1666" s="1">
-        <v>1.3215704920000002E7</v>
+        <v>1.321570492E7</v>
       </c>
       <c r="H1666" s="1">
         <v>0</v>
       </c>
       <c r="I1666" s="1">
-        <v>1.3215704920000002E7</v>
+        <v>1.321570492E7</v>
       </c>
     </row>
     <row r="1667" spans="1:9" ht="12.75">
@@ -50477,13 +50477,13 @@
         <v>0</v>
       </c>
       <c r="G1685" s="1">
-        <v>2668824.6799999997</v>
+        <v>2668824.68</v>
       </c>
       <c r="H1685" s="1">
         <v>0</v>
       </c>
       <c r="I1685" s="1">
-        <v>2668824.6799999997</v>
+        <v>2668824.68</v>
       </c>
     </row>
     <row r="1686" spans="1:9" ht="12.75">
@@ -51263,10 +51263,10 @@
         <v>3734639.2300000004</v>
       </c>
       <c r="H1712" s="1">
-        <v>3776932.5300000007</v>
+        <v>3776932.5300000003</v>
       </c>
       <c r="I1712" s="1">
-        <v>-42293.30000000028</v>
+        <v>-42293.299999999814</v>
       </c>
     </row>
     <row r="1713" spans="1:9" ht="12.75">
@@ -51318,13 +51318,13 @@
         <v>0</v>
       </c>
       <c r="G1714" s="1">
-        <v>307784.22000000003</v>
+        <v>307784.22</v>
       </c>
       <c r="H1714" s="1">
         <v>0</v>
       </c>
       <c r="I1714" s="1">
-        <v>307784.22000000003</v>
+        <v>307784.22</v>
       </c>
     </row>
     <row r="1715" spans="1:9" ht="12.75">
@@ -51434,13 +51434,13 @@
         <v>0</v>
       </c>
       <c r="G1718" s="1">
-        <v>191355.02000000002</v>
+        <v>191355.02</v>
       </c>
       <c r="H1718" s="1">
-        <v>110023.00000000001</v>
+        <v>110023</v>
       </c>
       <c r="I1718" s="1">
-        <v>81332.02</v>
+        <v>81332.01999999999</v>
       </c>
     </row>
     <row r="1719" spans="1:9" ht="12.75">
@@ -51521,13 +51521,13 @@
         <v>0</v>
       </c>
       <c r="G1721" s="1">
-        <v>1406462.6099999999</v>
+        <v>1406462.61</v>
       </c>
       <c r="H1721" s="1">
         <v>234699.50</v>
       </c>
       <c r="I1721" s="1">
-        <v>1171763.1099999999</v>
+        <v>1171763.11</v>
       </c>
     </row>
     <row r="1722" spans="1:9" ht="12.75">
@@ -51553,7 +51553,7 @@
         <v>3389832</v>
       </c>
       <c r="H1722" s="1">
-        <v>44210.10</v>
+        <v>44210.100000000006</v>
       </c>
       <c r="I1722" s="1">
         <v>3345621.90</v>
@@ -54044,13 +54044,13 @@
         <v>0</v>
       </c>
       <c r="G1808" s="1">
-        <v>3556925.1799999997</v>
+        <v>3556925.18</v>
       </c>
       <c r="H1808" s="1">
         <v>0</v>
       </c>
       <c r="I1808" s="1">
-        <v>3556925.1799999997</v>
+        <v>3556925.18</v>
       </c>
     </row>
     <row r="1809" spans="1:9" ht="12.75">
@@ -55407,13 +55407,13 @@
         <v>0</v>
       </c>
       <c r="G1855" s="1">
-        <v>7.480875494000001E7</v>
+        <v>7.480875494E7</v>
       </c>
       <c r="H1855" s="1">
         <v>7.480879472E7</v>
       </c>
       <c r="I1855" s="1">
-        <v>-39.77999998629093</v>
+        <v>-39.78000000119209</v>
       </c>
     </row>
     <row r="1856" spans="1:9" ht="12.75">
@@ -55439,10 +55439,10 @@
         <v>211883.90</v>
       </c>
       <c r="H1856" s="1">
-        <v>270641.04</v>
+        <v>270641.04000000004</v>
       </c>
       <c r="I1856" s="1">
-        <v>-58757.139999999985</v>
+        <v>-58757.14000000004</v>
       </c>
     </row>
     <row r="1857" spans="1:9" ht="12.75">
@@ -55665,7 +55665,7 @@
         <v>381</v>
       </c>
       <c r="F1864" s="1">
-        <v>5.9604644775390625E-8</v>
+        <v>1.1920928955078125E-7</v>
       </c>
       <c r="G1864" s="1">
         <v>8.546960143279996E9</v>
@@ -55674,7 +55674,7 @@
         <v>8.546960143280002E9</v>
       </c>
       <c r="I1864" s="1">
-        <v>-3.0566006898880005E-6</v>
+        <v>-4.263594746589661E-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>